<commit_message>
Workbook Decisions: A14 decided, West EU (Ireland), 30 Sep 2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -524,7 +524,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -580,7 +579,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
@@ -11182,12 +11180,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Cloud hosting. Provider and region not chosen. Nearest Supabase region is Frankfurt.</t>
+          <t>Cloud hosting on Supabase, region West EU (Ireland).</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Open: pick region</t>
+          <t>Confirmed 30 Sep 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tests for requirement rows that had no tagged test (wave 2, item 3)
SET-003, SET-006, RPT-002, RPT-003, RPT-004, ADM-009, GST-006, RES-012 and
RES-013 (database side): 85 checks in 29_untagged_rows.sql, all passing, no
application change. Register statuses and the workbook updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -601,27 +601,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Built (database only), no tagged test</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Built+tested</t>
+          <t>Built+tested (database only)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>101</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Built+tested (database only)</t>
+          <t>Built+tested (known limit)</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -631,7 +631,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Built+tested (known limit)</t>
+          <t>Not built</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -641,40 +641,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Built, no tagged test</t>
+          <t>Partly built, no tagged test</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Not built</t>
+          <t>R1b</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Partly built, no tagged test</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>R1b</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2513,12 +2493,12 @@
       </c>
       <c r="N23" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29_untagged_rows (5)</t>
         </is>
       </c>
       <c r="O23" s="10" t="inlineStr">
         <is>
-          <t>Built, no tagged test</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P23" s="10" t="inlineStr">
@@ -2755,12 +2735,12 @@
       </c>
       <c r="N26" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29_untagged_rows (10)</t>
         </is>
       </c>
       <c r="O26" s="10" t="inlineStr">
         <is>
-          <t>Built, no tagged test</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P26" s="10" t="inlineStr"/>
@@ -2989,12 +2969,12 @@
       </c>
       <c r="N29" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29_untagged_rows (12)</t>
         </is>
       </c>
       <c r="O29" s="10" t="inlineStr">
         <is>
-          <t>Built, no tagged test</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P29" s="10" t="inlineStr"/>
@@ -4081,12 +4061,12 @@
       </c>
       <c r="N43" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29_untagged_rows (7)</t>
         </is>
       </c>
       <c r="O43" s="10" t="inlineStr">
         <is>
-          <t>Built (database only), no tagged test</t>
+          <t>Built+tested (database only)</t>
         </is>
       </c>
       <c r="P43" s="10" t="inlineStr">
@@ -4163,7 +4143,7 @@
       </c>
       <c r="N44" s="10" t="inlineStr">
         <is>
-          <t>17_more_features (2); 26_small_fixes (4)</t>
+          <t>17_more_features (2); 26_small_fixes (4); 29_untagged_rows (6)</t>
         </is>
       </c>
       <c r="O44" s="10" t="inlineStr">
@@ -5657,12 +5637,12 @@
       </c>
       <c r="N63" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29_untagged_rows (6)</t>
         </is>
       </c>
       <c r="O63" s="10" t="inlineStr">
         <is>
-          <t>Built, no tagged test</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P63" s="10" t="inlineStr"/>
@@ -8703,12 +8683,12 @@
       </c>
       <c r="N102" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29_untagged_rows (14)</t>
         </is>
       </c>
       <c r="O102" s="10" t="inlineStr">
         <is>
-          <t>Built, no tagged test</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr"/>
@@ -8781,12 +8761,12 @@
       </c>
       <c r="N103" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29_untagged_rows (11)</t>
         </is>
       </c>
       <c r="O103" s="10" t="inlineStr">
         <is>
-          <t>Built, no tagged test</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr"/>
@@ -8859,12 +8839,12 @@
       </c>
       <c r="N104" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29_untagged_rows (14)</t>
         </is>
       </c>
       <c r="O104" s="10" t="inlineStr">
         <is>
-          <t>Built, no tagged test</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr">

</xml_diff>

<commit_message>
SET-003: a room with a guest in it cannot be retired (E_ROOM_OCCUPIED)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -2735,7 +2735,7 @@
       </c>
       <c r="N26" s="10" t="inlineStr">
         <is>
-          <t>29_untagged_rows (10)</t>
+          <t>29_untagged_rows (10); 30_retire_room_guard (8)</t>
         </is>
       </c>
       <c r="O26" s="10" t="inlineStr">
@@ -2743,7 +2743,11 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P26" s="10" t="inlineStr"/>
+      <c r="P26" s="10" t="inlineStr">
+        <is>
+          <t>A room with a guest in it right now cannot be retired; check the guest out first ([E_ROOM_OCCUPIED], decision of 6 Oct 2026). Retiring a room that is already retired is safe to repeat. Future bookings assigned to a retired room are not checked yet (open question).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Register: ADM-009 and RPT-004 'Built by' describe what this app does
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -2488,7 +2488,7 @@
       </c>
       <c r="M23" s="10" t="inlineStr">
         <is>
-          <t>(needs an Edge Function or client-side export)</t>
+          <t>export_data (rpt.export: System Administrator, General Manager, Accountant) returns bookings, ledger rows or guests for one property and at most a year, and writes an audit row (action export: who, what, which property, how many rows); the Export tab on Reports downloads it as CSV through src/lib/exports.functions.ts</t>
         </is>
       </c>
       <c r="N23" s="10" t="inlineStr">
@@ -8834,7 +8834,7 @@
       </c>
       <c r="M104" s="10" t="inlineStr">
         <is>
-          <t>(views for cancellation rate, ALOS and outstanding balances still to add)</t>
+          <t>Reports screen (src/routes/_authenticated/_app/reports.tsx) on report_* functions in the database: v_kpi_daily (occupancy, average rate, revenue per room), report_revenue_by_charge_code, report_outstanding_balances, report_payments, report_cancellation_rate (cancellations and no-shows), report_length_of_stay, report_balances_by_guest; finance reports need rpt.finance.view, operations reports rpt.operations.view</t>
         </is>
       </c>
       <c r="N104" s="10" t="inlineStr">

</xml_diff>

<commit_message>
SET-003: a room with upcoming bookings cannot be retired (E_ROOM_BOOKED)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -2735,7 +2735,7 @@
       </c>
       <c r="N26" s="10" t="inlineStr">
         <is>
-          <t>29_untagged_rows (10); 30_retire_room_guard (8)</t>
+          <t>29_untagged_rows (10); 30_retire_room_guard (8); 31_retire_room_future_guard (9)</t>
         </is>
       </c>
       <c r="O26" s="10" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="P26" s="10" t="inlineStr">
         <is>
-          <t>A room with a guest in it right now cannot be retired; check the guest out first ([E_ROOM_OCCUPIED], decision of 6 Oct 2026). Retiring a room that is already retired is safe to repeat. Future bookings assigned to a retired room are not checked yet (open question).</t>
+          <t>A room cannot be retired while a guest is in it ([E_ROOM_OCCUPIED], checked first) or while upcoming bookings are assigned to it ([E_ROOM_BOOKED], names up to 5 booking numbers): confirmed, or tentative with an unexpired hold, from the business date forward (decisions of 6 Oct 2026). Retiring a room that is already retired is safe to repeat; renaming and floor changes still work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Subscription billing: database layer (PLT-012)
Plan prices on plans, payment records, one-time provider events, activation on a matching paid event, failed-payment queue for operators. Database only; checkout, webhook route and screen follow.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'R1 Requirements'!$A$1:$O$108</definedName>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Subscription billing through a payment provider (Paystack or Flutterwave).</t>
+          <t>Subscription billing through a payment provider (Paystack first). A hotel picks a plan and pays online; the price comes from the database; the provider result activates the plan once, only when the amount and currency match; failed payments show to platform operators.</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -1669,55 +1669,59 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>R1b</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>org.billing.paymentmethod</t>
+          <t>adm.subscription.manage; platform operator</t>
         </is>
       </c>
       <c r="I13" s="10" t="inlineStr">
         <is>
-          <t>A13</t>
+          <t>A13, A16</t>
         </is>
       </c>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>a hotel wants to pay online</t>
+          <t>a hotel administrator on a plan with a price</t>
         </is>
       </c>
       <c r="K13" s="10" t="inlineStr">
         <is>
-          <t>they choose a plan and pay</t>
+          <t>they start a payment and the provider confirms it</t>
         </is>
       </c>
       <c r="L13" s="10" t="inlineStr">
         <is>
-          <t>the subscription activates automatically</t>
+          <t>"the plan becomes active for a month or a year, a resent event changes nothing, a wrong amount activates nothing"</t>
         </is>
       </c>
       <c r="M13" s="10" t="inlineStr">
         <is>
-          <t>(pilots are invoiced by hand until then)</t>
+          <t>start_subscription_payment, billing_apply_event, platform_set_plan_price, platform_failed_payments</t>
         </is>
       </c>
       <c r="N13" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>32_subscription_billing (62)</t>
         </is>
       </c>
       <c r="O13" s="10" t="inlineStr">
         <is>
-          <t>R1b</t>
-        </is>
-      </c>
-      <c r="P13" s="10" t="inlineStr"/>
+          <t>Built+tested (database only)</t>
+        </is>
+      </c>
+      <c r="P13" s="10" t="inlineStr">
+        <is>
+          <t>Checkout, webhook route and Subscription screen come next. Prices are empty until A16 is decided.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Subscription billing: Paystack checkout, webhook, Subscription screen, failed-payment queue (PLT-012)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Subscription billing through a payment provider (Paystack first). A hotel picks a plan and pays online; the price comes from the database; the provider result activates the plan once, only when the amount and currency match; failed payments show to platform operators.</t>
+          <t>Subscription billing through a payment provider (Paystack first). A hotel picks a plan and pays online; the price comes from the database; the provider result activates the plan once, only when the amount and currency match; failed payments show to platform operators. Hotels pay from the Subscription tab; Paystack calls a signed webhook.</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -1704,22 +1704,22 @@
       </c>
       <c r="M13" s="10" t="inlineStr">
         <is>
-          <t>start_subscription_payment, billing_apply_event, platform_set_plan_price, platform_failed_payments</t>
+          <t>start_subscription_payment, billing_apply_event, platform_set_plan_price, platform_failed_payments, billing_options, paystack webhook gate</t>
         </is>
       </c>
       <c r="N13" s="10" t="inlineStr">
         <is>
-          <t>32_subscription_billing (62)</t>
+          <t>32_subscription_billing (62); 33_billing_options (13); paystack-webhook-unit (7)</t>
         </is>
       </c>
       <c r="O13" s="10" t="inlineStr">
         <is>
-          <t>Built+tested (database only)</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P13" s="10" t="inlineStr">
         <is>
-          <t>Checkout, webhook route and Subscription screen come next. Prices are empty until A16 is decided.</t>
+          <t>Needs PAYSTACK_SECRET_KEY and the webhook address set in Paystack. Prices are empty until A16 is decided.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cashier shifts and night audit flags, database layer (FIN-016, DAY-005)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'R1 Requirements'!$A$1:$O$108</definedName>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -8009,7 +8009,7 @@
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t>Cashier shifts and reconciliation by cashier, shift and method.</t>
+          <t>Cashier shifts: a cashier opens a shift with a float, takes payments, counts each payment method at the end; the database works out expected and difference; a manager reconciles (never the closer). A hotel can require an open shift before payments.</t>
         </is>
       </c>
       <c r="E94" s="10" t="inlineStr">
@@ -8019,55 +8019,59 @@
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G94" s="10" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="H94" s="10" t="inlineStr">
         <is>
-          <t>fin.shift.manage, fin.shift.reconcile</t>
+          <t>fin.shift.close, fin.shift.reconcile</t>
         </is>
       </c>
       <c r="I94" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>A2; decision of 7 Oct 2026</t>
         </is>
       </c>
       <c r="J94" s="10" t="inlineStr">
         <is>
-          <t>a cashier shift</t>
+          <t>a cashier with an open shift who took cash and card payments</t>
         </is>
       </c>
       <c r="K94" s="10" t="inlineStr">
         <is>
-          <t>the shift is closed</t>
+          <t>they close the shift with their counts</t>
         </is>
       </c>
       <c r="L94" s="10" t="inlineStr">
         <is>
-          <t>payments reconcile by method</t>
+          <t>the difference per method is worked out, a note is needed for a difference, and a manager reconciles it</t>
         </is>
       </c>
       <c r="M94" s="10" t="inlineStr">
         <is>
-          <t>(not in R1)</t>
+          <t>open_cashier_shift, close_cashier_shift, reconcile_cashier_shift, cashier_shift_summary, list_cashier_shifts, set_cashier_shift_required, stamp_cashier_shift</t>
         </is>
       </c>
       <c r="N94" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>34_cashier_shifts (45)</t>
         </is>
       </c>
       <c r="O94" s="10" t="inlineStr">
         <is>
-          <t>R1b</t>
-        </is>
-      </c>
-      <c r="P94" s="10" t="inlineStr"/>
+          <t>Built+tested (database only)</t>
+        </is>
+      </c>
+      <c r="P94" s="10" t="inlineStr">
+        <is>
+          <t>Shift screens come next. New permission fin.shift.reconcile goes to built-in roles only.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
@@ -8399,7 +8403,7 @@
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t>Night audit gates the roll from R2.</t>
+          <t>Night audit flags list what is still open before the day closes: open cashier shifts (blocking), unreconciled differences, guests past departure, arrivals not checked in. The flags do not stop the date rolling yet.</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr">
@@ -8414,24 +8418,24 @@
       </c>
       <c r="G99" s="10" t="inlineStr">
         <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H99" s="10" t="inlineStr">
+        <is>
+          <t>fin.nightaudit.run</t>
+        </is>
+      </c>
+      <c r="I99" s="10" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="J99" s="10" t="inlineStr">
+        <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="H99" s="10" t="inlineStr">
-        <is>
-          <t>audit.night.run</t>
-        </is>
-      </c>
-      <c r="I99" s="10" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="J99" s="10" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
       <c r="K99" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -8444,20 +8448,24 @@
       </c>
       <c r="M99" s="10" t="inlineStr">
         <is>
-          <t>(not in R1)</t>
+          <t>night_audit_flags</t>
         </is>
       </c>
       <c r="N99" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>34_cashier_shifts (7)</t>
         </is>
       </c>
       <c r="O99" s="10" t="inlineStr">
         <is>
-          <t>R1b</t>
-        </is>
-      </c>
-      <c r="P99" s="10" t="inlineStr"/>
+          <t>Partly built, no tagged test</t>
+        </is>
+      </c>
+      <c r="P99" s="10" t="inlineStr">
+        <is>
+          <t>Flags built and tested. The gate that stops the roll while a blocking flag is open is not built.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Cashier shift page and night audit flags in Admin (FIN-016, DAY-005)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C94" s="10" t="inlineStr">
         <is>
-          <t>FIN-02</t>
+          <t>/cashier</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="P94" s="10" t="inlineStr">
         <is>
-          <t>Shift screens come next. New permission fin.shift.reconcile goes to built-in roles only.</t>
+          <t>Cashier shift page built (open, close with counts, review, reconcile). Not covered by a browser test yet. New permission fin.shift.reconcile goes to built-in roles only.</t>
         </is>
       </c>
     </row>
@@ -8408,7 +8408,7 @@
       </c>
       <c r="C99" s="10" t="inlineStr">
         <is>
-          <t>FIN-03</t>
+          <t>/admin (Business date)</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="P99" s="10" t="inlineStr">
         <is>
-          <t>Flags built and tested. The gate that stops the roll while a blocking flag is open is not built.</t>
+          <t>Flags shown in Admin, Business date. The gate that stops the roll while a blocking flag is open is not built.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hotel group view: all-branches summary, Group Manager role, copy setup to a new branch
New permission rpt.group.view (System Administrator, General Manager, new Group Manager role).
group_overview() and copy_property_setup() with 31 database checks (GRP-001 to GRP-004),
the All branches screen, docs and requirement rows.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'R1 Requirements'!$A$1:$O$108</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13">
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P117"/>
+  <dimension ref="A1:P121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9870,6 +9870,318 @@
         </is>
       </c>
       <c r="P117" s="10" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t>GRP-001</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C118" s="10" t="inlineStr">
+        <is>
+          <t>All branches</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>A built-in Group Manager role and the permission rpt.group.view exist; only System Administrator, General Manager and Group Manager hold the permission.</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F118" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G118" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H118" s="10" t="inlineStr">
+        <is>
+          <t>rpt.group.view</t>
+        </is>
+      </c>
+      <c r="I118" s="10" t="inlineStr"/>
+      <c r="J118" s="10" t="inlineStr">
+        <is>
+          <t>a hotel group with several branches</t>
+        </is>
+      </c>
+      <c r="K118" s="10" t="inlineStr">
+        <is>
+          <t>an owner wants a view-only manager for the whole group</t>
+        </is>
+      </c>
+      <c r="L118" s="10" t="inlineStr">
+        <is>
+          <t>they assign the Group Manager role branch by branch, and that person can look but not post or change anything</t>
+        </is>
+      </c>
+      <c r="M118" s="10" t="inlineStr">
+        <is>
+          <t>20261013120000_group_view.sql</t>
+        </is>
+      </c>
+      <c r="N118" s="10" t="inlineStr">
+        <is>
+          <t>35_group_view (5)</t>
+        </is>
+      </c>
+      <c r="O118" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P118" s="10" t="inlineStr">
+        <is>
+          <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>GRP-002</t>
+        </is>
+      </c>
+      <c r="B119" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>All branches</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>One call shows every branch the person may see: occupancy, in house, arrivals and departures to come, approvals, repairs and last night revenue, with group totals. Revenue is totalled per currency.</t>
+        </is>
+      </c>
+      <c r="E119" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F119" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G119" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H119" s="10" t="inlineStr">
+        <is>
+          <t>rpt.group.view</t>
+        </is>
+      </c>
+      <c r="I119" s="10" t="inlineStr"/>
+      <c r="J119" s="10" t="inlineStr">
+        <is>
+          <t>a group with a Lagos and an Abuja branch</t>
+        </is>
+      </c>
+      <c r="K119" s="10" t="inlineStr">
+        <is>
+          <t>a group manager opens All branches</t>
+        </is>
+      </c>
+      <c r="L119" s="10" t="inlineStr">
+        <is>
+          <t>they see both branches with figures from the database, never another hotel group, and staff without the permission are refused</t>
+        </is>
+      </c>
+      <c r="M119" s="10" t="inlineStr">
+        <is>
+          <t>group_overview; /group screen</t>
+        </is>
+      </c>
+      <c r="N119" s="10" t="inlineStr">
+        <is>
+          <t>35_group_view (10)</t>
+        </is>
+      </c>
+      <c r="O119" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P119" s="10" t="inlineStr">
+        <is>
+          <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="inlineStr">
+        <is>
+          <t>GRP-003</t>
+        </is>
+      </c>
+      <c r="B120" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C120" s="10" t="inlineStr">
+        <is>
+          <t>All branches</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="inlineStr">
+        <is>
+          <t>A Group Manager sees only the branches they are assigned to, and cannot post charges or check guests in.</t>
+        </is>
+      </c>
+      <c r="E120" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F120" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G120" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H120" s="10" t="inlineStr">
+        <is>
+          <t>rpt.group.view</t>
+        </is>
+      </c>
+      <c r="I120" s="10" t="inlineStr"/>
+      <c r="J120" s="10" t="inlineStr">
+        <is>
+          <t>a Group Manager assigned to one branch</t>
+        </is>
+      </c>
+      <c r="K120" s="10" t="inlineStr">
+        <is>
+          <t>a second branch is assigned</t>
+        </is>
+      </c>
+      <c r="L120" s="10" t="inlineStr">
+        <is>
+          <t>the second branch appears; the role never gets write permissions</t>
+        </is>
+      </c>
+      <c r="M120" s="10" t="inlineStr">
+        <is>
+          <t>assign_role (existing); group_overview</t>
+        </is>
+      </c>
+      <c r="N120" s="10" t="inlineStr">
+        <is>
+          <t>35_group_view (3)</t>
+        </is>
+      </c>
+      <c r="O120" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P120" s="10" t="inlineStr">
+        <is>
+          <t>Access is per branch, using the existing role assignment screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="10" t="inlineStr">
+        <is>
+          <t>GRP-004</t>
+        </is>
+      </c>
+      <c r="B121" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C121" s="10" t="inlineStr">
+        <is>
+          <t>All branches (Copy setup)</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="inlineStr">
+        <is>
+          <t>A new branch can copy room types, rate plans and prices from an existing branch, once, into an empty branch.</t>
+        </is>
+      </c>
+      <c r="E121" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F121" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G121" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H121" s="10" t="inlineStr">
+        <is>
+          <t>setup.room.manage, setup.rate.manage</t>
+        </is>
+      </c>
+      <c r="I121" s="10" t="inlineStr"/>
+      <c r="J121" s="10" t="inlineStr">
+        <is>
+          <t>a new empty branch</t>
+        </is>
+      </c>
+      <c r="K121" s="10" t="inlineStr">
+        <is>
+          <t>the owner copies setup from the first branch</t>
+        </is>
+      </c>
+      <c r="L121" s="10" t="inlineStr">
+        <is>
+          <t>room types, rate plans and prices appear on the new branch and point at its own room types; rooms are not copied; a second copy is refused; the copy is audited</t>
+        </is>
+      </c>
+      <c r="M121" s="10" t="inlineStr">
+        <is>
+          <t>copy_property_setup</t>
+        </is>
+      </c>
+      <c r="N121" s="10" t="inlineStr">
+        <is>
+          <t>35_group_view (13)</t>
+        </is>
+      </c>
+      <c r="O121" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P121" s="10" t="inlineStr">
+        <is>
+          <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Reports: revenue by booking source and ageing of unpaid balances
report_revenue_by_source and report_balance_ageing, two tabs on Reports, 25 database checks
(RPT-005, RPT-006), docs and requirement rows.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'R1 Requirements'!$A$1:$O$108</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13">
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P117"/>
+  <dimension ref="A1:P119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9870,6 +9870,162 @@
         </is>
       </c>
       <c r="P117" s="10" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t>RPT-005</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C118" s="10" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>Revenue by booking source: bookings, cancellations, no-shows, room nights, room revenue and average rate for each source in a date range.</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F118" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G118" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H118" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view</t>
+        </is>
+      </c>
+      <c r="I118" s="10" t="inlineStr"/>
+      <c r="J118" s="10" t="inlineStr">
+        <is>
+          <t>bookings from direct, phone and company sources</t>
+        </is>
+      </c>
+      <c r="K118" s="10" t="inlineStr">
+        <is>
+          <t>the accountant picks a date range</t>
+        </is>
+      </c>
+      <c r="L118" s="10" t="inlineStr">
+        <is>
+          <t>each source shows its own counts and room revenue (room charges only, before tax); cancelled bookings add no nights</t>
+        </is>
+      </c>
+      <c r="M118" s="10" t="inlineStr">
+        <is>
+          <t>20261013130000_source_ageing_reports.sql: report_revenue_by_source; Reports, By booking source tab</t>
+        </is>
+      </c>
+      <c r="N118" s="10" t="inlineStr">
+        <is>
+          <t>36_source_ageing (13)</t>
+        </is>
+      </c>
+      <c r="O118" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P118" s="10" t="inlineStr">
+        <is>
+          <t>Bookings counted by arrival date; revenue by posting date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>RPT-006</t>
+        </is>
+      </c>
+      <c r="B119" s="10" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>Ageing of unpaid balances by booking source: current, 1 to 7, 8 to 30, 31 to 60 and over 60 days since the due departure, plus credit held.</t>
+        </is>
+      </c>
+      <c r="E119" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F119" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G119" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H119" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view</t>
+        </is>
+      </c>
+      <c r="I119" s="10" t="inlineStr"/>
+      <c r="J119" s="10" t="inlineStr">
+        <is>
+          <t>guests and companies who left owing money</t>
+        </is>
+      </c>
+      <c r="K119" s="10" t="inlineStr">
+        <is>
+          <t>the accountant opens the Ageing tab</t>
+        </is>
+      </c>
+      <c r="L119" s="10" t="inlineStr">
+        <is>
+          <t>each source shows what is owed in each age column; paid bills drop out; overpayments show as credit held; the total matches Outstanding balances</t>
+        </is>
+      </c>
+      <c r="M119" s="10" t="inlineStr">
+        <is>
+          <t>report_balance_ageing; Reports, Ageing tab</t>
+        </is>
+      </c>
+      <c r="N119" s="10" t="inlineStr">
+        <is>
+          <t>36_source_ageing (11)</t>
+        </is>
+      </c>
+      <c r="O119" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P119" s="10" t="inlineStr">
+        <is>
+          <t>Guests still staying count as current.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
AI helpers: owner's morning brief
Off by default, monthly limit, facts built by the database (counts and money, no personal data),
server refuses any draft with a number not in the facts. 35 database checks and 8 unit checks
(AI-001 to AI-005), Admin switch, dashboard card, docs.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'R1 Requirements'!$A$1:$O$108</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13">
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P117"/>
+  <dimension ref="A1:P122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9870,6 +9870,388 @@
         </is>
       </c>
       <c r="P117" s="10" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t>AI-001</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C118" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Admin</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F118" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G118" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H118" s="10" t="inlineStr">
+        <is>
+          <t>adm.ai.manage</t>
+        </is>
+      </c>
+      <c r="I118" s="10" t="inlineStr"/>
+      <c r="J118" s="10" t="inlineStr">
+        <is>
+          <t>a new hotel</t>
+        </is>
+      </c>
+      <c r="K118" s="10" t="inlineStr">
+        <is>
+          <t>a manager opens Admin, AI helpers</t>
+        </is>
+      </c>
+      <c r="L118" s="10" t="inlineStr">
+        <is>
+          <t>nothing runs until they switch it on and the change is in the audit log</t>
+        </is>
+      </c>
+      <c r="M118" s="10" t="inlineStr">
+        <is>
+          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
+        </is>
+      </c>
+      <c r="N118" s="10" t="inlineStr">
+        <is>
+          <t>37_ai_brief (11)</t>
+        </is>
+      </c>
+      <c r="O118" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P118" s="10" t="inlineStr">
+        <is>
+          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>AI-002</t>
+        </is>
+      </c>
+      <c r="B119" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Admin</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
+        </is>
+      </c>
+      <c r="E119" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F119" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G119" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H119" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view, rpt.operations.view</t>
+        </is>
+      </c>
+      <c r="I119" s="10" t="inlineStr"/>
+      <c r="J119" s="10" t="inlineStr">
+        <is>
+          <t>a hotel with guests, approvals and overdue bills</t>
+        </is>
+      </c>
+      <c r="K119" s="10" t="inlineStr">
+        <is>
+          <t>a brief is started</t>
+        </is>
+      </c>
+      <c r="L119" s="10" t="inlineStr">
+        <is>
+          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
+        </is>
+      </c>
+      <c r="M119" s="10" t="inlineStr">
+        <is>
+          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
+        </is>
+      </c>
+      <c r="N119" s="10" t="inlineStr">
+        <is>
+          <t>37_ai_brief (11)</t>
+        </is>
+      </c>
+      <c r="O119" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P119" s="10" t="inlineStr">
+        <is>
+          <t>Overdue means unpaid more than 30 days after departure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="inlineStr">
+        <is>
+          <t>AI-003</t>
+        </is>
+      </c>
+      <c r="B120" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C120" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Admin</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="inlineStr">
+        <is>
+          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
+        </is>
+      </c>
+      <c r="E120" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F120" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G120" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H120" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view</t>
+        </is>
+      </c>
+      <c r="I120" s="10" t="inlineStr"/>
+      <c r="J120" s="10" t="inlineStr">
+        <is>
+          <t>a limit of 2</t>
+        </is>
+      </c>
+      <c r="K120" s="10" t="inlineStr">
+        <is>
+          <t>a third brief is requested</t>
+        </is>
+      </c>
+      <c r="L120" s="10" t="inlineStr">
+        <is>
+          <t>it is refused until a failed call frees a slot or the month turns</t>
+        </is>
+      </c>
+      <c r="M120" s="10" t="inlineStr">
+        <is>
+          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
+        </is>
+      </c>
+      <c r="N120" s="10" t="inlineStr">
+        <is>
+          <t>37_ai_brief (5)</t>
+        </is>
+      </c>
+      <c r="O120" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P120" s="10" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="10" t="inlineStr">
+        <is>
+          <t>AI-004</t>
+        </is>
+      </c>
+      <c r="B121" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C121" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Admin</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="inlineStr">
+        <is>
+          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
+        </is>
+      </c>
+      <c r="E121" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F121" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G121" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H121" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view, rpt.operations.view</t>
+        </is>
+      </c>
+      <c r="I121" s="10" t="inlineStr"/>
+      <c r="J121" s="10" t="inlineStr">
+        <is>
+          <t>front desk, housekeeping, another hotel</t>
+        </is>
+      </c>
+      <c r="K121" s="10" t="inlineStr">
+        <is>
+          <t>they ask for the brief or touch the tables</t>
+        </is>
+      </c>
+      <c r="L121" s="10" t="inlineStr">
+        <is>
+          <t>they are refused</t>
+        </is>
+      </c>
+      <c r="M121" s="10" t="inlineStr">
+        <is>
+          <t>20261013140000_ai_morning_brief.sql</t>
+        </is>
+      </c>
+      <c r="N121" s="10" t="inlineStr">
+        <is>
+          <t>37_ai_brief (7)</t>
+        </is>
+      </c>
+      <c r="O121" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P121" s="10" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="10" t="inlineStr">
+        <is>
+          <t>AI-005</t>
+        </is>
+      </c>
+      <c r="B122" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C122" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Admin</t>
+        </is>
+      </c>
+      <c r="D122" s="10" t="inlineStr">
+        <is>
+          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
+        </is>
+      </c>
+      <c r="E122" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F122" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G122" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H122" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I122" s="10" t="inlineStr"/>
+      <c r="J122" s="10" t="inlineStr">
+        <is>
+          <t>a draft that rounds or invents a figure</t>
+        </is>
+      </c>
+      <c r="K122" s="10" t="inlineStr">
+        <is>
+          <t>the brief is written</t>
+        </is>
+      </c>
+      <c r="L122" s="10" t="inlineStr">
+        <is>
+          <t>the plain database lines are shown instead, with a note</t>
+        </is>
+      </c>
+      <c r="M122" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
+        </is>
+      </c>
+      <c r="N122" s="10" t="inlineStr">
+        <is>
+          <t>browser unit: ai-brief-unit (8)</t>
+        </is>
+      </c>
+      <c r="O122" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P122" s="10" t="inlineStr">
+        <is>
+          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
AI helpers: setup import assistant
Paste a room list; AI drafts room types and rooms; the database previews and adds all or nothing.
apply_setup_import and ai_import_start, 37 database checks and 9 unit checks (SET-010, AI-006, AI-007).
Pasted text with email, phone or card numbers is refused; the draft keeps only what was pasted.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13">
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P122"/>
+  <dimension ref="A1:P125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10250,6 +10250,236 @@
       <c r="P122" s="10" t="inlineStr">
         <is>
           <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t>SET-010</t>
+        </is>
+      </c>
+      <c r="B123" s="10" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="C123" s="10" t="inlineStr">
+        <is>
+          <t>Setup, Rooms</t>
+        </is>
+      </c>
+      <c r="D123" s="10" t="inlineStr">
+        <is>
+          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
+        </is>
+      </c>
+      <c r="E123" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F123" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G123" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H123" s="10" t="inlineStr">
+        <is>
+          <t>setup.room.manage</t>
+        </is>
+      </c>
+      <c r="I123" s="10" t="inlineStr"/>
+      <c r="J123" s="10" t="inlineStr">
+        <is>
+          <t>a list of room types and rooms</t>
+        </is>
+      </c>
+      <c r="K123" s="10" t="inlineStr">
+        <is>
+          <t>the manager previews and then applies it</t>
+        </is>
+      </c>
+      <c r="L123" s="10" t="inlineStr">
+        <is>
+          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
+        </is>
+      </c>
+      <c r="M123" s="10" t="inlineStr">
+        <is>
+          <t>20261013150000_setup_import.sql: apply_setup_import</t>
+        </is>
+      </c>
+      <c r="N123" s="10" t="inlineStr">
+        <is>
+          <t>38_setup_import (29)</t>
+        </is>
+      </c>
+      <c r="O123" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P123" s="10" t="inlineStr">
+        <is>
+          <t>The AI only drafts the list. This function is the check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="inlineStr">
+        <is>
+          <t>AI-006</t>
+        </is>
+      </c>
+      <c r="B124" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>Setup, Rooms</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="inlineStr">
+        <is>
+          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
+        </is>
+      </c>
+      <c r="E124" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F124" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G124" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H124" s="10" t="inlineStr">
+        <is>
+          <t>setup.room.manage</t>
+        </is>
+      </c>
+      <c r="I124" s="10" t="inlineStr"/>
+      <c r="J124" s="10" t="inlineStr">
+        <is>
+          <t>AI switched on with a limit of 1</t>
+        </is>
+      </c>
+      <c r="K124" s="10" t="inlineStr">
+        <is>
+          <t>an import draft is started twice</t>
+        </is>
+      </c>
+      <c r="L124" s="10" t="inlineStr">
+        <is>
+          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
+        </is>
+      </c>
+      <c r="M124" s="10" t="inlineStr">
+        <is>
+          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
+        </is>
+      </c>
+      <c r="N124" s="10" t="inlineStr">
+        <is>
+          <t>38_setup_import (8)</t>
+        </is>
+      </c>
+      <c r="O124" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P124" s="10" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="10" t="inlineStr">
+        <is>
+          <t>AI-007</t>
+        </is>
+      </c>
+      <c r="B125" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C125" s="10" t="inlineStr">
+        <is>
+          <t>Setup, Rooms</t>
+        </is>
+      </c>
+      <c r="D125" s="10" t="inlineStr">
+        <is>
+          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
+        </is>
+      </c>
+      <c r="E125" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F125" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G125" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H125" s="10" t="inlineStr">
+        <is>
+          <t>setup.room.manage</t>
+        </is>
+      </c>
+      <c r="I125" s="10" t="inlineStr"/>
+      <c r="J125" s="10" t="inlineStr">
+        <is>
+          <t>a pasted list</t>
+        </is>
+      </c>
+      <c r="K125" s="10" t="inlineStr">
+        <is>
+          <t>the assistant drafts it</t>
+        </is>
+      </c>
+      <c r="L125" s="10" t="inlineStr">
+        <is>
+          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
+        </is>
+      </c>
+      <c r="M125" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
+        </is>
+      </c>
+      <c r="N125" s="10" t="inlineStr">
+        <is>
+          <t>browser unit: setup-import-unit (9)</t>
+        </is>
+      </c>
+      <c r="O125" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P125" s="10" t="inlineStr">
+        <is>
+          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Group booking screen and arrival-ready flag (RES-012, RES-013)
Groups list and group page at /reservations/groups with rooms, totals,
cancel and reactivate, and Add a room. Booking page shows and toggles the
arrival-ready flag; Front Desk arrivals shows a Ready badge.
New migration 20261013160000 with list_group_bookings, get_group_booking,
set_group_booking_status and arrival_ready on v_arrivals. 31 new checks.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'R1 Requirements'!$A$1:$O$108</definedName>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -605,23 +605,23 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Built+tested (database only)</t>
+          <t>Built+tested (known limit)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Built+tested (known limit)</t>
+          <t>Not built</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -631,7 +631,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Not built</t>
+          <t>Partly built, no tagged test</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -641,20 +641,10 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Partly built, no tagged test</t>
+          <t>R1b</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>R1b</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
         <v>3</v>
       </c>
     </row>
@@ -669,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P117"/>
+  <dimension ref="A1:T117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -770,6 +760,10 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="Q1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
+      <c r="S1" s="2" t="n"/>
+      <c r="T1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -848,6 +842,10 @@
         </is>
       </c>
       <c r="P2" s="10" t="inlineStr"/>
+      <c r="Q2" s="10" t="n"/>
+      <c r="R2" s="10" t="n"/>
+      <c r="S2" s="10" t="n"/>
+      <c r="T2" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -926,6 +924,10 @@
         </is>
       </c>
       <c r="P3" s="10" t="inlineStr"/>
+      <c r="Q3" s="10" t="n"/>
+      <c r="R3" s="10" t="n"/>
+      <c r="S3" s="10" t="n"/>
+      <c r="T3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -1004,6 +1006,10 @@
         </is>
       </c>
       <c r="P4" s="10" t="inlineStr"/>
+      <c r="Q4" s="10" t="n"/>
+      <c r="R4" s="10" t="n"/>
+      <c r="S4" s="10" t="n"/>
+      <c r="T4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1082,6 +1088,10 @@
         </is>
       </c>
       <c r="P5" s="10" t="inlineStr"/>
+      <c r="Q5" s="10" t="n"/>
+      <c r="R5" s="10" t="n"/>
+      <c r="S5" s="10" t="n"/>
+      <c r="T5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -1160,6 +1170,10 @@
         </is>
       </c>
       <c r="P6" s="10" t="inlineStr"/>
+      <c r="Q6" s="10" t="n"/>
+      <c r="R6" s="10" t="n"/>
+      <c r="S6" s="10" t="n"/>
+      <c r="T6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -1238,6 +1252,10 @@
         </is>
       </c>
       <c r="P7" s="10" t="inlineStr"/>
+      <c r="Q7" s="10" t="n"/>
+      <c r="R7" s="10" t="n"/>
+      <c r="S7" s="10" t="n"/>
+      <c r="T7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1320,6 +1338,10 @@
           <t>Adding a property: System Administrator and General Manager (ADM-002), within plans.max_properties.</t>
         </is>
       </c>
+      <c r="Q8" s="10" t="n"/>
+      <c r="R8" s="10" t="n"/>
+      <c r="S8" s="10" t="n"/>
+      <c r="T8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -1402,6 +1424,10 @@
           <t>Platform console /platform (wave 2 item 2): extend trial, activate or extend paid period, suspend, change plan, cancel; each with a reason, logged in subscription_history with the operator.</t>
         </is>
       </c>
+      <c r="Q9" s="10" t="n"/>
+      <c r="R9" s="10" t="n"/>
+      <c r="S9" s="10" t="n"/>
+      <c r="T9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -1484,6 +1510,10 @@
           <t>Corrected 6 Oct 2026: before wave 2 item 2 there was no platform staff role at all; the earlier "Built, no tagged test" was wrong.</t>
         </is>
       </c>
+      <c r="Q10" s="10" t="n"/>
+      <c r="R10" s="10" t="n"/>
+      <c r="S10" s="10" t="n"/>
+      <c r="T10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -1562,6 +1592,10 @@
         </is>
       </c>
       <c r="P11" s="10" t="inlineStr"/>
+      <c r="Q11" s="10" t="n"/>
+      <c r="R11" s="10" t="n"/>
+      <c r="S11" s="10" t="n"/>
+      <c r="T11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -1640,6 +1674,10 @@
         </is>
       </c>
       <c r="P12" s="10" t="inlineStr"/>
+      <c r="Q12" s="10" t="n"/>
+      <c r="R12" s="10" t="n"/>
+      <c r="S12" s="10" t="n"/>
+      <c r="T12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -1718,6 +1756,10 @@
         </is>
       </c>
       <c r="P13" s="10" t="inlineStr"/>
+      <c r="Q13" s="10" t="n"/>
+      <c r="R13" s="10" t="n"/>
+      <c r="S13" s="10" t="n"/>
+      <c r="T13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -1796,6 +1838,10 @@
         </is>
       </c>
       <c r="P14" s="10" t="inlineStr"/>
+      <c r="Q14" s="10" t="n"/>
+      <c r="R14" s="10" t="n"/>
+      <c r="S14" s="10" t="n"/>
+      <c r="T14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -1878,6 +1924,10 @@
           <t>Invites are sent by a Vercel server function (not an Edge Function).</t>
         </is>
       </c>
+      <c r="Q15" s="10" t="n"/>
+      <c r="R15" s="10" t="n"/>
+      <c r="S15" s="10" t="n"/>
+      <c r="T15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -1956,6 +2006,10 @@
         </is>
       </c>
       <c r="P16" s="10" t="inlineStr"/>
+      <c r="Q16" s="10" t="n"/>
+      <c r="R16" s="10" t="n"/>
+      <c r="S16" s="10" t="n"/>
+      <c r="T16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -2034,6 +2088,10 @@
         </is>
       </c>
       <c r="P17" s="10" t="inlineStr"/>
+      <c r="Q17" s="10" t="n"/>
+      <c r="R17" s="10" t="n"/>
+      <c r="S17" s="10" t="n"/>
+      <c r="T17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -2112,6 +2170,10 @@
         </is>
       </c>
       <c r="P18" s="10" t="inlineStr"/>
+      <c r="Q18" s="10" t="n"/>
+      <c r="R18" s="10" t="n"/>
+      <c r="S18" s="10" t="n"/>
+      <c r="T18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -2190,6 +2252,10 @@
         </is>
       </c>
       <c r="P19" s="10" t="inlineStr"/>
+      <c r="Q19" s="10" t="n"/>
+      <c r="R19" s="10" t="n"/>
+      <c r="S19" s="10" t="n"/>
+      <c r="T19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -2268,6 +2334,10 @@
         </is>
       </c>
       <c r="P20" s="10" t="inlineStr"/>
+      <c r="Q20" s="10" t="n"/>
+      <c r="R20" s="10" t="n"/>
+      <c r="S20" s="10" t="n"/>
+      <c r="T20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
@@ -2346,6 +2416,10 @@
         </is>
       </c>
       <c r="P21" s="10" t="inlineStr"/>
+      <c r="Q21" s="10" t="n"/>
+      <c r="R21" s="10" t="n"/>
+      <c r="S21" s="10" t="n"/>
+      <c r="T21" s="10" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
@@ -2424,6 +2498,10 @@
         </is>
       </c>
       <c r="P22" s="10" t="inlineStr"/>
+      <c r="Q22" s="10" t="n"/>
+      <c r="R22" s="10" t="n"/>
+      <c r="S22" s="10" t="n"/>
+      <c r="T22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
@@ -2506,6 +2584,10 @@
           <t>export_data (audited), Reports &gt; Export.</t>
         </is>
       </c>
+      <c r="Q23" s="10" t="n"/>
+      <c r="R23" s="10" t="n"/>
+      <c r="S23" s="10" t="n"/>
+      <c r="T23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
@@ -2584,6 +2666,10 @@
         </is>
       </c>
       <c r="P24" s="10" t="inlineStr"/>
+      <c r="Q24" s="10" t="n"/>
+      <c r="R24" s="10" t="n"/>
+      <c r="S24" s="10" t="n"/>
+      <c r="T24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
@@ -2666,6 +2752,10 @@
           <t>Corrected 6 Oct 2026: room types and occupancy limits (save_room_type, max adults and children; Setup, Room types) exist; the overbooking allowance does not exist anywhere in the app.</t>
         </is>
       </c>
+      <c r="Q25" s="10" t="n"/>
+      <c r="R25" s="10" t="n"/>
+      <c r="S25" s="10" t="n"/>
+      <c r="T25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
@@ -2748,6 +2838,10 @@
           <t>A room cannot be retired while a guest is in it ([E_ROOM_OCCUPIED], checked first) or while upcoming bookings are assigned to it ([E_ROOM_BOOKED], names up to 5 booking numbers): confirmed, or tentative with an unexpired hold, from the business date forward (decisions of 6 Oct 2026). Retiring a room that is already retired is safe to repeat; renaming and floor changes still work.</t>
         </is>
       </c>
+      <c r="Q26" s="10" t="n"/>
+      <c r="R26" s="10" t="n"/>
+      <c r="S26" s="10" t="n"/>
+      <c r="T26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
@@ -2826,6 +2920,10 @@
         </is>
       </c>
       <c r="P27" s="10" t="inlineStr"/>
+      <c r="Q27" s="10" t="n"/>
+      <c r="R27" s="10" t="n"/>
+      <c r="S27" s="10" t="n"/>
+      <c r="T27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
@@ -2904,6 +3002,10 @@
         </is>
       </c>
       <c r="P28" s="10" t="inlineStr"/>
+      <c r="Q28" s="10" t="n"/>
+      <c r="R28" s="10" t="n"/>
+      <c r="S28" s="10" t="n"/>
+      <c r="T28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
@@ -2982,6 +3084,10 @@
         </is>
       </c>
       <c r="P29" s="10" t="inlineStr"/>
+      <c r="Q29" s="10" t="n"/>
+      <c r="R29" s="10" t="n"/>
+      <c r="S29" s="10" t="n"/>
+      <c r="T29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
@@ -3060,6 +3166,10 @@
         </is>
       </c>
       <c r="P30" s="10" t="inlineStr"/>
+      <c r="Q30" s="10" t="n"/>
+      <c r="R30" s="10" t="n"/>
+      <c r="S30" s="10" t="n"/>
+      <c r="T30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
@@ -3138,6 +3248,10 @@
         </is>
       </c>
       <c r="P31" s="10" t="inlineStr"/>
+      <c r="Q31" s="10" t="n"/>
+      <c r="R31" s="10" t="n"/>
+      <c r="S31" s="10" t="n"/>
+      <c r="T31" s="10" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
@@ -3216,6 +3330,10 @@
         </is>
       </c>
       <c r="P32" s="10" t="inlineStr"/>
+      <c r="Q32" s="10" t="n"/>
+      <c r="R32" s="10" t="n"/>
+      <c r="S32" s="10" t="n"/>
+      <c r="T32" s="10" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
@@ -3294,6 +3412,10 @@
         </is>
       </c>
       <c r="P33" s="10" t="inlineStr"/>
+      <c r="Q33" s="10" t="n"/>
+      <c r="R33" s="10" t="n"/>
+      <c r="S33" s="10" t="n"/>
+      <c r="T33" s="10" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
@@ -3372,6 +3494,10 @@
         </is>
       </c>
       <c r="P34" s="10" t="inlineStr"/>
+      <c r="Q34" s="10" t="n"/>
+      <c r="R34" s="10" t="n"/>
+      <c r="S34" s="10" t="n"/>
+      <c r="T34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
@@ -3450,6 +3576,10 @@
         </is>
       </c>
       <c r="P35" s="10" t="inlineStr"/>
+      <c r="Q35" s="10" t="n"/>
+      <c r="R35" s="10" t="n"/>
+      <c r="S35" s="10" t="n"/>
+      <c r="T35" s="10" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
@@ -3528,6 +3658,10 @@
         </is>
       </c>
       <c r="P36" s="10" t="inlineStr"/>
+      <c r="Q36" s="10" t="n"/>
+      <c r="R36" s="10" t="n"/>
+      <c r="S36" s="10" t="n"/>
+      <c r="T36" s="10" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
@@ -3606,6 +3740,10 @@
         </is>
       </c>
       <c r="P37" s="10" t="inlineStr"/>
+      <c r="Q37" s="10" t="n"/>
+      <c r="R37" s="10" t="n"/>
+      <c r="S37" s="10" t="n"/>
+      <c r="T37" s="10" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
@@ -3684,6 +3822,10 @@
         </is>
       </c>
       <c r="P38" s="10" t="inlineStr"/>
+      <c r="Q38" s="10" t="n"/>
+      <c r="R38" s="10" t="n"/>
+      <c r="S38" s="10" t="n"/>
+      <c r="T38" s="10" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
@@ -3762,6 +3904,10 @@
         </is>
       </c>
       <c r="P39" s="10" t="inlineStr"/>
+      <c r="Q39" s="10" t="n"/>
+      <c r="R39" s="10" t="n"/>
+      <c r="S39" s="10" t="n"/>
+      <c r="T39" s="10" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
@@ -3840,6 +3986,10 @@
         </is>
       </c>
       <c r="P40" s="10" t="inlineStr"/>
+      <c r="Q40" s="10" t="n"/>
+      <c r="R40" s="10" t="n"/>
+      <c r="S40" s="10" t="n"/>
+      <c r="T40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
@@ -3918,6 +4068,10 @@
         </is>
       </c>
       <c r="P41" s="10" t="inlineStr"/>
+      <c r="Q41" s="10" t="n"/>
+      <c r="R41" s="10" t="n"/>
+      <c r="S41" s="10" t="n"/>
+      <c r="T41" s="10" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
@@ -3996,6 +4150,10 @@
         </is>
       </c>
       <c r="P42" s="10" t="inlineStr"/>
+      <c r="Q42" s="10" t="n"/>
+      <c r="R42" s="10" t="n"/>
+      <c r="S42" s="10" t="n"/>
+      <c r="T42" s="10" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
@@ -4065,17 +4223,37 @@
       </c>
       <c r="N43" s="10" t="inlineStr">
         <is>
-          <t>29_untagged_rows (7)</t>
+          <t>29_untagged_rows (7); 39_group_booking</t>
         </is>
       </c>
       <c r="O43" s="10" t="inlineStr">
         <is>
-          <t>Built+tested (database only)</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P43" s="10" t="inlineStr">
         <is>
-          <t>save_group_booking exists and the booking form picks a group; there is no screen to create a group.</t>
+          <t>Groups list and group page (rooms</t>
+        </is>
+      </c>
+      <c r="Q43" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> totals</t>
+        </is>
+      </c>
+      <c r="R43" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> cancel</t>
+        </is>
+      </c>
+      <c r="S43" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> reactivate</t>
+        </is>
+      </c>
+      <c r="T43" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> add a room) at /reservations/groups. Groups are still created from the booking form.</t>
         </is>
       </c>
     </row>
@@ -4147,19 +4325,23 @@
       </c>
       <c r="N44" s="10" t="inlineStr">
         <is>
-          <t>17_more_features (2); 26_small_fixes (4); 29_untagged_rows (6)</t>
+          <t>17_more_features (2); 26_small_fixes (4); 29_untagged_rows (6); 39_group_booking</t>
         </is>
       </c>
       <c r="O44" s="10" t="inlineStr">
         <is>
-          <t>Built+tested (database only)</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P44" s="10" t="inlineStr">
         <is>
-          <t>set_arrival_ready exists; no screen shows the flag yet (skipped 6 Oct 2026).</t>
-        </is>
-      </c>
+          <t>Mark ready button and badge on the booking page; badge on the Front Desk arrivals list (v_arrivals.arrival_ready).</t>
+        </is>
+      </c>
+      <c r="Q44" s="10" t="n"/>
+      <c r="R44" s="10" t="n"/>
+      <c r="S44" s="10" t="n"/>
+      <c r="T44" s="10" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
@@ -4238,6 +4420,10 @@
         </is>
       </c>
       <c r="P45" s="10" t="inlineStr"/>
+      <c r="Q45" s="10" t="n"/>
+      <c r="R45" s="10" t="n"/>
+      <c r="S45" s="10" t="n"/>
+      <c r="T45" s="10" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
@@ -4316,6 +4502,10 @@
         </is>
       </c>
       <c r="P46" s="10" t="inlineStr"/>
+      <c r="Q46" s="10" t="n"/>
+      <c r="R46" s="10" t="n"/>
+      <c r="S46" s="10" t="n"/>
+      <c r="T46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
@@ -4398,6 +4588,10 @@
           <t>The check-in and walk-in screens force the registration card tick; a direct database call that omits it is not refused (decision 6 Oct 2026). Drawn signature later.</t>
         </is>
       </c>
+      <c r="Q47" s="10" t="n"/>
+      <c r="R47" s="10" t="n"/>
+      <c r="S47" s="10" t="n"/>
+      <c r="T47" s="10" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
@@ -4476,6 +4670,10 @@
         </is>
       </c>
       <c r="P48" s="10" t="inlineStr"/>
+      <c r="Q48" s="10" t="n"/>
+      <c r="R48" s="10" t="n"/>
+      <c r="S48" s="10" t="n"/>
+      <c r="T48" s="10" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
@@ -4554,6 +4752,10 @@
         </is>
       </c>
       <c r="P49" s="10" t="inlineStr"/>
+      <c r="Q49" s="10" t="n"/>
+      <c r="R49" s="10" t="n"/>
+      <c r="S49" s="10" t="n"/>
+      <c r="T49" s="10" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
@@ -4632,6 +4834,10 @@
         </is>
       </c>
       <c r="P50" s="10" t="inlineStr"/>
+      <c r="Q50" s="10" t="n"/>
+      <c r="R50" s="10" t="n"/>
+      <c r="S50" s="10" t="n"/>
+      <c r="T50" s="10" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
@@ -4714,6 +4920,10 @@
           <t>Dearer room type: front desk charges the new rate; keeping it needs fo.upgrade.complimentary (SYSADMIN, GM, FOM), audited.</t>
         </is>
       </c>
+      <c r="Q51" s="10" t="n"/>
+      <c r="R51" s="10" t="n"/>
+      <c r="S51" s="10" t="n"/>
+      <c r="T51" s="10" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
@@ -4792,6 +5002,10 @@
         </is>
       </c>
       <c r="P52" s="10" t="inlineStr"/>
+      <c r="Q52" s="10" t="n"/>
+      <c r="R52" s="10" t="n"/>
+      <c r="S52" s="10" t="n"/>
+      <c r="T52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
@@ -4870,6 +5084,10 @@
         </is>
       </c>
       <c r="P53" s="10" t="inlineStr"/>
+      <c r="Q53" s="10" t="n"/>
+      <c r="R53" s="10" t="n"/>
+      <c r="S53" s="10" t="n"/>
+      <c r="T53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
@@ -4948,6 +5166,10 @@
         </is>
       </c>
       <c r="P54" s="10" t="inlineStr"/>
+      <c r="Q54" s="10" t="n"/>
+      <c r="R54" s="10" t="n"/>
+      <c r="S54" s="10" t="n"/>
+      <c r="T54" s="10" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
@@ -5026,6 +5248,10 @@
         </is>
       </c>
       <c r="P55" s="10" t="inlineStr"/>
+      <c r="Q55" s="10" t="n"/>
+      <c r="R55" s="10" t="n"/>
+      <c r="S55" s="10" t="n"/>
+      <c r="T55" s="10" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
@@ -5104,6 +5330,10 @@
         </is>
       </c>
       <c r="P56" s="10" t="inlineStr"/>
+      <c r="Q56" s="10" t="n"/>
+      <c r="R56" s="10" t="n"/>
+      <c r="S56" s="10" t="n"/>
+      <c r="T56" s="10" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
@@ -5182,6 +5412,10 @@
         </is>
       </c>
       <c r="P57" s="10" t="inlineStr"/>
+      <c r="Q57" s="10" t="n"/>
+      <c r="R57" s="10" t="n"/>
+      <c r="S57" s="10" t="n"/>
+      <c r="T57" s="10" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
@@ -5260,6 +5494,10 @@
         </is>
       </c>
       <c r="P58" s="10" t="inlineStr"/>
+      <c r="Q58" s="10" t="n"/>
+      <c r="R58" s="10" t="n"/>
+      <c r="S58" s="10" t="n"/>
+      <c r="T58" s="10" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
@@ -5338,6 +5576,10 @@
         </is>
       </c>
       <c r="P59" s="10" t="inlineStr"/>
+      <c r="Q59" s="10" t="n"/>
+      <c r="R59" s="10" t="n"/>
+      <c r="S59" s="10" t="n"/>
+      <c r="T59" s="10" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
@@ -5416,6 +5658,10 @@
         </is>
       </c>
       <c r="P60" s="10" t="inlineStr"/>
+      <c r="Q60" s="10" t="n"/>
+      <c r="R60" s="10" t="n"/>
+      <c r="S60" s="10" t="n"/>
+      <c r="T60" s="10" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
@@ -5494,6 +5740,10 @@
         </is>
       </c>
       <c r="P61" s="10" t="inlineStr"/>
+      <c r="Q61" s="10" t="n"/>
+      <c r="R61" s="10" t="n"/>
+      <c r="S61" s="10" t="n"/>
+      <c r="T61" s="10" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
@@ -5572,6 +5822,10 @@
         </is>
       </c>
       <c r="P62" s="10" t="inlineStr"/>
+      <c r="Q62" s="10" t="n"/>
+      <c r="R62" s="10" t="n"/>
+      <c r="S62" s="10" t="n"/>
+      <c r="T62" s="10" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
@@ -5650,6 +5904,10 @@
         </is>
       </c>
       <c r="P63" s="10" t="inlineStr"/>
+      <c r="Q63" s="10" t="n"/>
+      <c r="R63" s="10" t="n"/>
+      <c r="S63" s="10" t="n"/>
+      <c r="T63" s="10" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
@@ -5728,6 +5986,10 @@
         </is>
       </c>
       <c r="P64" s="10" t="inlineStr"/>
+      <c r="Q64" s="10" t="n"/>
+      <c r="R64" s="10" t="n"/>
+      <c r="S64" s="10" t="n"/>
+      <c r="T64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
@@ -5806,6 +6068,10 @@
         </is>
       </c>
       <c r="P65" s="10" t="inlineStr"/>
+      <c r="Q65" s="10" t="n"/>
+      <c r="R65" s="10" t="n"/>
+      <c r="S65" s="10" t="n"/>
+      <c r="T65" s="10" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
@@ -5884,6 +6150,10 @@
         </is>
       </c>
       <c r="P66" s="10" t="inlineStr"/>
+      <c r="Q66" s="10" t="n"/>
+      <c r="R66" s="10" t="n"/>
+      <c r="S66" s="10" t="n"/>
+      <c r="T66" s="10" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
@@ -5962,6 +6232,10 @@
         </is>
       </c>
       <c r="P67" s="10" t="inlineStr"/>
+      <c r="Q67" s="10" t="n"/>
+      <c r="R67" s="10" t="n"/>
+      <c r="S67" s="10" t="n"/>
+      <c r="T67" s="10" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
@@ -6040,6 +6314,10 @@
         </is>
       </c>
       <c r="P68" s="10" t="inlineStr"/>
+      <c r="Q68" s="10" t="n"/>
+      <c r="R68" s="10" t="n"/>
+      <c r="S68" s="10" t="n"/>
+      <c r="T68" s="10" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
@@ -6118,6 +6396,10 @@
         </is>
       </c>
       <c r="P69" s="10" t="inlineStr"/>
+      <c r="Q69" s="10" t="n"/>
+      <c r="R69" s="10" t="n"/>
+      <c r="S69" s="10" t="n"/>
+      <c r="T69" s="10" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
@@ -6196,6 +6478,10 @@
         </is>
       </c>
       <c r="P70" s="10" t="inlineStr"/>
+      <c r="Q70" s="10" t="n"/>
+      <c r="R70" s="10" t="n"/>
+      <c r="S70" s="10" t="n"/>
+      <c r="T70" s="10" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
@@ -6274,6 +6560,10 @@
         </is>
       </c>
       <c r="P71" s="10" t="inlineStr"/>
+      <c r="Q71" s="10" t="n"/>
+      <c r="R71" s="10" t="n"/>
+      <c r="S71" s="10" t="n"/>
+      <c r="T71" s="10" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
@@ -6352,6 +6642,10 @@
         </is>
       </c>
       <c r="P72" s="10" t="inlineStr"/>
+      <c r="Q72" s="10" t="n"/>
+      <c r="R72" s="10" t="n"/>
+      <c r="S72" s="10" t="n"/>
+      <c r="T72" s="10" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
@@ -6430,6 +6724,10 @@
         </is>
       </c>
       <c r="P73" s="10" t="inlineStr"/>
+      <c r="Q73" s="10" t="n"/>
+      <c r="R73" s="10" t="n"/>
+      <c r="S73" s="10" t="n"/>
+      <c r="T73" s="10" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
@@ -6508,6 +6806,10 @@
         </is>
       </c>
       <c r="P74" s="10" t="inlineStr"/>
+      <c r="Q74" s="10" t="n"/>
+      <c r="R74" s="10" t="n"/>
+      <c r="S74" s="10" t="n"/>
+      <c r="T74" s="10" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
@@ -6586,6 +6888,10 @@
         </is>
       </c>
       <c r="P75" s="10" t="inlineStr"/>
+      <c r="Q75" s="10" t="n"/>
+      <c r="R75" s="10" t="n"/>
+      <c r="S75" s="10" t="n"/>
+      <c r="T75" s="10" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
@@ -6664,6 +6970,10 @@
         </is>
       </c>
       <c r="P76" s="10" t="inlineStr"/>
+      <c r="Q76" s="10" t="n"/>
+      <c r="R76" s="10" t="n"/>
+      <c r="S76" s="10" t="n"/>
+      <c r="T76" s="10" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
@@ -6742,6 +7052,10 @@
         </is>
       </c>
       <c r="P77" s="10" t="inlineStr"/>
+      <c r="Q77" s="10" t="n"/>
+      <c r="R77" s="10" t="n"/>
+      <c r="S77" s="10" t="n"/>
+      <c r="T77" s="10" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
@@ -6820,6 +7134,10 @@
         </is>
       </c>
       <c r="P78" s="10" t="inlineStr"/>
+      <c r="Q78" s="10" t="n"/>
+      <c r="R78" s="10" t="n"/>
+      <c r="S78" s="10" t="n"/>
+      <c r="T78" s="10" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
@@ -6898,6 +7216,10 @@
         </is>
       </c>
       <c r="P79" s="10" t="inlineStr"/>
+      <c r="Q79" s="10" t="n"/>
+      <c r="R79" s="10" t="n"/>
+      <c r="S79" s="10" t="n"/>
+      <c r="T79" s="10" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
@@ -6976,6 +7298,10 @@
         </is>
       </c>
       <c r="P80" s="10" t="inlineStr"/>
+      <c r="Q80" s="10" t="n"/>
+      <c r="R80" s="10" t="n"/>
+      <c r="S80" s="10" t="n"/>
+      <c r="T80" s="10" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
@@ -7054,6 +7380,10 @@
         </is>
       </c>
       <c r="P81" s="10" t="inlineStr"/>
+      <c r="Q81" s="10" t="n"/>
+      <c r="R81" s="10" t="n"/>
+      <c r="S81" s="10" t="n"/>
+      <c r="T81" s="10" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
@@ -7132,6 +7462,10 @@
         </is>
       </c>
       <c r="P82" s="10" t="inlineStr"/>
+      <c r="Q82" s="10" t="n"/>
+      <c r="R82" s="10" t="n"/>
+      <c r="S82" s="10" t="n"/>
+      <c r="T82" s="10" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
@@ -7210,6 +7544,10 @@
         </is>
       </c>
       <c r="P83" s="10" t="inlineStr"/>
+      <c r="Q83" s="10" t="n"/>
+      <c r="R83" s="10" t="n"/>
+      <c r="S83" s="10" t="n"/>
+      <c r="T83" s="10" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
@@ -7288,6 +7626,10 @@
         </is>
       </c>
       <c r="P84" s="10" t="inlineStr"/>
+      <c r="Q84" s="10" t="n"/>
+      <c r="R84" s="10" t="n"/>
+      <c r="S84" s="10" t="n"/>
+      <c r="T84" s="10" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
@@ -7366,6 +7708,10 @@
         </is>
       </c>
       <c r="P85" s="10" t="inlineStr"/>
+      <c r="Q85" s="10" t="n"/>
+      <c r="R85" s="10" t="n"/>
+      <c r="S85" s="10" t="n"/>
+      <c r="T85" s="10" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
@@ -7444,6 +7790,10 @@
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr"/>
+      <c r="Q86" s="10" t="n"/>
+      <c r="R86" s="10" t="n"/>
+      <c r="S86" s="10" t="n"/>
+      <c r="T86" s="10" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
@@ -7522,6 +7872,10 @@
         </is>
       </c>
       <c r="P87" s="10" t="inlineStr"/>
+      <c r="Q87" s="10" t="n"/>
+      <c r="R87" s="10" t="n"/>
+      <c r="S87" s="10" t="n"/>
+      <c r="T87" s="10" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
@@ -7600,6 +7954,10 @@
         </is>
       </c>
       <c r="P88" s="10" t="inlineStr"/>
+      <c r="Q88" s="10" t="n"/>
+      <c r="R88" s="10" t="n"/>
+      <c r="S88" s="10" t="n"/>
+      <c r="T88" s="10" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
@@ -7678,6 +8036,10 @@
         </is>
       </c>
       <c r="P89" s="10" t="inlineStr"/>
+      <c r="Q89" s="10" t="n"/>
+      <c r="R89" s="10" t="n"/>
+      <c r="S89" s="10" t="n"/>
+      <c r="T89" s="10" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
@@ -7756,6 +8118,10 @@
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr"/>
+      <c r="Q90" s="10" t="n"/>
+      <c r="R90" s="10" t="n"/>
+      <c r="S90" s="10" t="n"/>
+      <c r="T90" s="10" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
@@ -7834,6 +8200,10 @@
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr"/>
+      <c r="Q91" s="10" t="n"/>
+      <c r="R91" s="10" t="n"/>
+      <c r="S91" s="10" t="n"/>
+      <c r="T91" s="10" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
@@ -7912,6 +8282,10 @@
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr"/>
+      <c r="Q92" s="10" t="n"/>
+      <c r="R92" s="10" t="n"/>
+      <c r="S92" s="10" t="n"/>
+      <c r="T92" s="10" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
@@ -7990,6 +8364,10 @@
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr"/>
+      <c r="Q93" s="10" t="n"/>
+      <c r="R93" s="10" t="n"/>
+      <c r="S93" s="10" t="n"/>
+      <c r="T93" s="10" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
@@ -8068,6 +8446,10 @@
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr"/>
+      <c r="Q94" s="10" t="n"/>
+      <c r="R94" s="10" t="n"/>
+      <c r="S94" s="10" t="n"/>
+      <c r="T94" s="10" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
@@ -8146,6 +8528,10 @@
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr"/>
+      <c r="Q95" s="10" t="n"/>
+      <c r="R95" s="10" t="n"/>
+      <c r="S95" s="10" t="n"/>
+      <c r="T95" s="10" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
@@ -8224,6 +8610,10 @@
         </is>
       </c>
       <c r="P96" s="10" t="inlineStr"/>
+      <c r="Q96" s="10" t="n"/>
+      <c r="R96" s="10" t="n"/>
+      <c r="S96" s="10" t="n"/>
+      <c r="T96" s="10" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
@@ -8302,6 +8692,10 @@
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr"/>
+      <c r="Q97" s="10" t="n"/>
+      <c r="R97" s="10" t="n"/>
+      <c r="S97" s="10" t="n"/>
+      <c r="T97" s="10" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
@@ -8380,6 +8774,10 @@
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr"/>
+      <c r="Q98" s="10" t="n"/>
+      <c r="R98" s="10" t="n"/>
+      <c r="S98" s="10" t="n"/>
+      <c r="T98" s="10" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
@@ -8458,6 +8856,10 @@
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr"/>
+      <c r="Q99" s="10" t="n"/>
+      <c r="R99" s="10" t="n"/>
+      <c r="S99" s="10" t="n"/>
+      <c r="T99" s="10" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
@@ -8540,6 +8942,10 @@
           <t>Decided by Peter on 30 Sep 2026 (answer 5) and confirmed on 1 Oct 2026: same-day stays are charged one night; a manager can waive it with a reason.</t>
         </is>
       </c>
+      <c r="Q100" s="10" t="n"/>
+      <c r="R100" s="10" t="n"/>
+      <c r="S100" s="10" t="n"/>
+      <c r="T100" s="10" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
@@ -8618,6 +9024,10 @@
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr"/>
+      <c r="Q101" s="10" t="n"/>
+      <c r="R101" s="10" t="n"/>
+      <c r="S101" s="10" t="n"/>
+      <c r="T101" s="10" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
@@ -8696,6 +9106,10 @@
         </is>
       </c>
       <c r="P102" s="10" t="inlineStr"/>
+      <c r="Q102" s="10" t="n"/>
+      <c r="R102" s="10" t="n"/>
+      <c r="S102" s="10" t="n"/>
+      <c r="T102" s="10" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
@@ -8774,6 +9188,10 @@
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr"/>
+      <c r="Q103" s="10" t="n"/>
+      <c r="R103" s="10" t="n"/>
+      <c r="S103" s="10" t="n"/>
+      <c r="T103" s="10" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
@@ -8856,6 +9274,10 @@
           <t>Reports screen: KPIs, revenue by charge code, outstanding balances, payments, cancellations and stay length, balances by guest, export.</t>
         </is>
       </c>
+      <c r="Q104" s="10" t="n"/>
+      <c r="R104" s="10" t="n"/>
+      <c r="S104" s="10" t="n"/>
+      <c r="T104" s="10" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
@@ -8934,6 +9356,10 @@
         </is>
       </c>
       <c r="P105" s="10" t="inlineStr"/>
+      <c r="Q105" s="10" t="n"/>
+      <c r="R105" s="10" t="n"/>
+      <c r="S105" s="10" t="n"/>
+      <c r="T105" s="10" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
@@ -9012,6 +9438,10 @@
         </is>
       </c>
       <c r="P106" s="10" t="inlineStr"/>
+      <c r="Q106" s="10" t="n"/>
+      <c r="R106" s="10" t="n"/>
+      <c r="S106" s="10" t="n"/>
+      <c r="T106" s="10" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
@@ -9090,6 +9520,10 @@
         </is>
       </c>
       <c r="P107" s="10" t="inlineStr"/>
+      <c r="Q107" s="10" t="n"/>
+      <c r="R107" s="10" t="n"/>
+      <c r="S107" s="10" t="n"/>
+      <c r="T107" s="10" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
@@ -9168,6 +9602,10 @@
         </is>
       </c>
       <c r="P108" s="10" t="inlineStr"/>
+      <c r="Q108" s="10" t="n"/>
+      <c r="R108" s="10" t="n"/>
+      <c r="S108" s="10" t="n"/>
+      <c r="T108" s="10" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
@@ -9246,6 +9684,10 @@
         </is>
       </c>
       <c r="P109" s="10" t="inlineStr"/>
+      <c r="Q109" s="10" t="n"/>
+      <c r="R109" s="10" t="n"/>
+      <c r="S109" s="10" t="n"/>
+      <c r="T109" s="10" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
@@ -9324,6 +9766,10 @@
         </is>
       </c>
       <c r="P110" s="10" t="inlineStr"/>
+      <c r="Q110" s="10" t="n"/>
+      <c r="R110" s="10" t="n"/>
+      <c r="S110" s="10" t="n"/>
+      <c r="T110" s="10" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
@@ -9402,6 +9848,10 @@
         </is>
       </c>
       <c r="P111" s="10" t="inlineStr"/>
+      <c r="Q111" s="10" t="n"/>
+      <c r="R111" s="10" t="n"/>
+      <c r="S111" s="10" t="n"/>
+      <c r="T111" s="10" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
@@ -9480,6 +9930,10 @@
         </is>
       </c>
       <c r="P112" s="10" t="inlineStr"/>
+      <c r="Q112" s="10" t="n"/>
+      <c r="R112" s="10" t="n"/>
+      <c r="S112" s="10" t="n"/>
+      <c r="T112" s="10" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
@@ -9558,6 +10012,10 @@
         </is>
       </c>
       <c r="P113" s="10" t="inlineStr"/>
+      <c r="Q113" s="10" t="n"/>
+      <c r="R113" s="10" t="n"/>
+      <c r="S113" s="10" t="n"/>
+      <c r="T113" s="10" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
@@ -9636,6 +10094,10 @@
         </is>
       </c>
       <c r="P114" s="10" t="inlineStr"/>
+      <c r="Q114" s="10" t="n"/>
+      <c r="R114" s="10" t="n"/>
+      <c r="S114" s="10" t="n"/>
+      <c r="T114" s="10" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
@@ -9714,6 +10176,10 @@
         </is>
       </c>
       <c r="P115" s="10" t="inlineStr"/>
+      <c r="Q115" s="10" t="n"/>
+      <c r="R115" s="10" t="n"/>
+      <c r="S115" s="10" t="n"/>
+      <c r="T115" s="10" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
@@ -9792,6 +10258,10 @@
         </is>
       </c>
       <c r="P116" s="10" t="inlineStr"/>
+      <c r="Q116" s="10" t="n"/>
+      <c r="R116" s="10" t="n"/>
+      <c r="S116" s="10" t="n"/>
+      <c r="T116" s="10" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
@@ -9870,6 +10340,10 @@
         </is>
       </c>
       <c r="P117" s="10" t="inlineStr"/>
+      <c r="Q117" s="10" t="n"/>
+      <c r="R117" s="10" t="n"/>
+      <c r="S117" s="10" t="n"/>
+      <c r="T117" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Guided first setup (SET-011)
setup_progress() tells a hotel what is left: property details, room types,
rooms, rates, taxes, payment methods, staff. Read-only, no stored progress.
Setup opens on a checklist until everything is done; the Dashboard shows a
short card. New migration 20261013170000 and 30 new checks.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'R1 Requirements'!$A$1:$O$108</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13">
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P117"/>
+  <dimension ref="A1:P118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9870,6 +9870,88 @@
         </is>
       </c>
       <c r="P117" s="10" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t>SET-011</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="C118" s="10" t="inlineStr">
+        <is>
+          <t>/setup; /dashboard</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>A new hotel sees a checklist of what is left to set up: property details, room types, rooms, rates, taxes, payment methods and staff. Each step says what is missing and links to the right screen. The list comes from the hotel's own data, so it is always current.</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F118" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G118" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H118" s="10" t="inlineStr">
+        <is>
+          <t>any setup permission</t>
+        </is>
+      </c>
+      <c r="I118" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J118" s="10" t="inlineStr">
+        <is>
+          <t>a hotel that is part way through setup</t>
+        </is>
+      </c>
+      <c r="K118" s="10" t="inlineStr">
+        <is>
+          <t>a manager opens Setup or the Dashboard</t>
+        </is>
+      </c>
+      <c r="L118" s="10" t="inlineStr">
+        <is>
+          <t>the steps already done are ticked and the next one is linked; once all seven are done the checklist goes away</t>
+        </is>
+      </c>
+      <c r="M118" s="10" t="inlineStr">
+        <is>
+          <t>setup_progress</t>
+        </is>
+      </c>
+      <c r="N118" s="10" t="inlineStr">
+        <is>
+          <t>40_guided_setup (30)</t>
+        </is>
+      </c>
+      <c r="O118" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P118" s="10" t="inlineStr">
+        <is>
+          <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Refresh requirements workbook from the register (130 requirements)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>116</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>109</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13">
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P117"/>
+  <dimension ref="A1:P131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9882,6 +9882,1086 @@
         </is>
       </c>
       <c r="P117" s="10" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t>GRP-001</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C118" s="10" t="inlineStr">
+        <is>
+          <t>All branches</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>A built-in Group Manager role and the permission rpt.group.view exist; only System Administrator, General Manager and Group Manager hold the permission.</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F118" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G118" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H118" s="10" t="inlineStr">
+        <is>
+          <t>rpt.group.view</t>
+        </is>
+      </c>
+      <c r="I118" s="10" t="inlineStr"/>
+      <c r="J118" s="10" t="inlineStr">
+        <is>
+          <t>a hotel group with several branches</t>
+        </is>
+      </c>
+      <c r="K118" s="10" t="inlineStr">
+        <is>
+          <t>an owner wants a view-only manager for the whole group</t>
+        </is>
+      </c>
+      <c r="L118" s="10" t="inlineStr">
+        <is>
+          <t>they assign the Group Manager role branch by branch, and that person can look but not post or change anything</t>
+        </is>
+      </c>
+      <c r="M118" s="10" t="inlineStr">
+        <is>
+          <t>20261013120000_group_view.sql</t>
+        </is>
+      </c>
+      <c r="N118" s="10" t="inlineStr">
+        <is>
+          <t>35_group_view (5)</t>
+        </is>
+      </c>
+      <c r="O118" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P118" s="10" t="inlineStr">
+        <is>
+          <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>GRP-002</t>
+        </is>
+      </c>
+      <c r="B119" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>All branches</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>One call shows every branch the person may see: occupancy, in house, arrivals and departures to come, approvals, repairs and last night revenue, with group totals. Revenue is totalled per currency.</t>
+        </is>
+      </c>
+      <c r="E119" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F119" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G119" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H119" s="10" t="inlineStr">
+        <is>
+          <t>rpt.group.view</t>
+        </is>
+      </c>
+      <c r="I119" s="10" t="inlineStr"/>
+      <c r="J119" s="10" t="inlineStr">
+        <is>
+          <t>a group with a Lagos and an Abuja branch</t>
+        </is>
+      </c>
+      <c r="K119" s="10" t="inlineStr">
+        <is>
+          <t>a group manager opens All branches</t>
+        </is>
+      </c>
+      <c r="L119" s="10" t="inlineStr">
+        <is>
+          <t>they see both branches with figures from the database, never another hotel group, and staff without the permission are refused</t>
+        </is>
+      </c>
+      <c r="M119" s="10" t="inlineStr">
+        <is>
+          <t>group_overview; /group screen</t>
+        </is>
+      </c>
+      <c r="N119" s="10" t="inlineStr">
+        <is>
+          <t>35_group_view (10)</t>
+        </is>
+      </c>
+      <c r="O119" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P119" s="10" t="inlineStr">
+        <is>
+          <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="inlineStr">
+        <is>
+          <t>GRP-003</t>
+        </is>
+      </c>
+      <c r="B120" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C120" s="10" t="inlineStr">
+        <is>
+          <t>All branches</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="inlineStr">
+        <is>
+          <t>A Group Manager sees only the branches they are assigned to, and cannot post charges or check guests in.</t>
+        </is>
+      </c>
+      <c r="E120" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F120" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G120" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H120" s="10" t="inlineStr">
+        <is>
+          <t>rpt.group.view</t>
+        </is>
+      </c>
+      <c r="I120" s="10" t="inlineStr"/>
+      <c r="J120" s="10" t="inlineStr">
+        <is>
+          <t>a Group Manager assigned to one branch</t>
+        </is>
+      </c>
+      <c r="K120" s="10" t="inlineStr">
+        <is>
+          <t>a second branch is assigned</t>
+        </is>
+      </c>
+      <c r="L120" s="10" t="inlineStr">
+        <is>
+          <t>the second branch appears; the role never gets write permissions</t>
+        </is>
+      </c>
+      <c r="M120" s="10" t="inlineStr">
+        <is>
+          <t>assign_role (existing); group_overview</t>
+        </is>
+      </c>
+      <c r="N120" s="10" t="inlineStr">
+        <is>
+          <t>35_group_view (3)</t>
+        </is>
+      </c>
+      <c r="O120" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P120" s="10" t="inlineStr">
+        <is>
+          <t>Access is per branch, using the existing role assignment screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="10" t="inlineStr">
+        <is>
+          <t>GRP-004</t>
+        </is>
+      </c>
+      <c r="B121" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C121" s="10" t="inlineStr">
+        <is>
+          <t>All branches (Copy setup)</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="inlineStr">
+        <is>
+          <t>A new branch can copy room types, rate plans and prices from an existing branch, once, into an empty branch.</t>
+        </is>
+      </c>
+      <c r="E121" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F121" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G121" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H121" s="10" t="inlineStr">
+        <is>
+          <t>setup.room.manage, setup.rate.manage</t>
+        </is>
+      </c>
+      <c r="I121" s="10" t="inlineStr"/>
+      <c r="J121" s="10" t="inlineStr">
+        <is>
+          <t>a new empty branch</t>
+        </is>
+      </c>
+      <c r="K121" s="10" t="inlineStr">
+        <is>
+          <t>the owner copies setup from the first branch</t>
+        </is>
+      </c>
+      <c r="L121" s="10" t="inlineStr">
+        <is>
+          <t>room types, rate plans and prices appear on the new branch and point at its own room types; rooms are not copied; a second copy is refused; the copy is audited</t>
+        </is>
+      </c>
+      <c r="M121" s="10" t="inlineStr">
+        <is>
+          <t>copy_property_setup</t>
+        </is>
+      </c>
+      <c r="N121" s="10" t="inlineStr">
+        <is>
+          <t>35_group_view (13)</t>
+        </is>
+      </c>
+      <c r="O121" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P121" s="10" t="inlineStr">
+        <is>
+          <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="10" t="inlineStr">
+        <is>
+          <t>RPT-005</t>
+        </is>
+      </c>
+      <c r="B122" s="10" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C122" s="10" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="D122" s="10" t="inlineStr">
+        <is>
+          <t>Revenue by booking source: bookings, cancellations, no-shows, room nights, room revenue and average rate for each source in a date range.</t>
+        </is>
+      </c>
+      <c r="E122" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F122" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G122" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H122" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view</t>
+        </is>
+      </c>
+      <c r="I122" s="10" t="inlineStr"/>
+      <c r="J122" s="10" t="inlineStr">
+        <is>
+          <t>bookings from direct, phone and company sources</t>
+        </is>
+      </c>
+      <c r="K122" s="10" t="inlineStr">
+        <is>
+          <t>the accountant picks a date range</t>
+        </is>
+      </c>
+      <c r="L122" s="10" t="inlineStr">
+        <is>
+          <t>each source shows its own counts and room revenue (room charges only, before tax); cancelled bookings add no nights</t>
+        </is>
+      </c>
+      <c r="M122" s="10" t="inlineStr">
+        <is>
+          <t>20261013130000_source_ageing_reports.sql: report_revenue_by_source; Reports, By booking source tab</t>
+        </is>
+      </c>
+      <c r="N122" s="10" t="inlineStr">
+        <is>
+          <t>36_source_ageing (13)</t>
+        </is>
+      </c>
+      <c r="O122" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P122" s="10" t="inlineStr">
+        <is>
+          <t>Bookings counted by arrival date; revenue by posting date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t>RPT-006</t>
+        </is>
+      </c>
+      <c r="B123" s="10" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C123" s="10" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="D123" s="10" t="inlineStr">
+        <is>
+          <t>Ageing of unpaid balances by booking source: current, 1 to 7, 8 to 30, 31 to 60 and over 60 days since the due departure, plus credit held.</t>
+        </is>
+      </c>
+      <c r="E123" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F123" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G123" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H123" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view</t>
+        </is>
+      </c>
+      <c r="I123" s="10" t="inlineStr"/>
+      <c r="J123" s="10" t="inlineStr">
+        <is>
+          <t>guests and companies who left owing money</t>
+        </is>
+      </c>
+      <c r="K123" s="10" t="inlineStr">
+        <is>
+          <t>the accountant opens the Ageing tab</t>
+        </is>
+      </c>
+      <c r="L123" s="10" t="inlineStr">
+        <is>
+          <t>each source shows what is owed in each age column; paid bills drop out; overpayments show as credit held; the total matches Outstanding balances</t>
+        </is>
+      </c>
+      <c r="M123" s="10" t="inlineStr">
+        <is>
+          <t>report_balance_ageing; Reports, Ageing tab</t>
+        </is>
+      </c>
+      <c r="N123" s="10" t="inlineStr">
+        <is>
+          <t>36_source_ageing (11)</t>
+        </is>
+      </c>
+      <c r="O123" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P123" s="10" t="inlineStr">
+        <is>
+          <t>Guests still staying count as current.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="inlineStr">
+        <is>
+          <t>AI-001</t>
+        </is>
+      </c>
+      <c r="B124" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Admin</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
+        </is>
+      </c>
+      <c r="E124" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F124" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G124" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H124" s="10" t="inlineStr">
+        <is>
+          <t>adm.ai.manage</t>
+        </is>
+      </c>
+      <c r="I124" s="10" t="inlineStr"/>
+      <c r="J124" s="10" t="inlineStr">
+        <is>
+          <t>a new hotel</t>
+        </is>
+      </c>
+      <c r="K124" s="10" t="inlineStr">
+        <is>
+          <t>a manager opens Admin, AI helpers</t>
+        </is>
+      </c>
+      <c r="L124" s="10" t="inlineStr">
+        <is>
+          <t>nothing runs until they switch it on and the change is in the audit log</t>
+        </is>
+      </c>
+      <c r="M124" s="10" t="inlineStr">
+        <is>
+          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
+        </is>
+      </c>
+      <c r="N124" s="10" t="inlineStr">
+        <is>
+          <t>37_ai_brief (11)</t>
+        </is>
+      </c>
+      <c r="O124" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P124" s="10" t="inlineStr">
+        <is>
+          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="10" t="inlineStr">
+        <is>
+          <t>AI-002</t>
+        </is>
+      </c>
+      <c r="B125" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C125" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Admin</t>
+        </is>
+      </c>
+      <c r="D125" s="10" t="inlineStr">
+        <is>
+          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
+        </is>
+      </c>
+      <c r="E125" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F125" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G125" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H125" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view, rpt.operations.view</t>
+        </is>
+      </c>
+      <c r="I125" s="10" t="inlineStr"/>
+      <c r="J125" s="10" t="inlineStr">
+        <is>
+          <t>a hotel with guests, approvals and overdue bills</t>
+        </is>
+      </c>
+      <c r="K125" s="10" t="inlineStr">
+        <is>
+          <t>a brief is started</t>
+        </is>
+      </c>
+      <c r="L125" s="10" t="inlineStr">
+        <is>
+          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
+        </is>
+      </c>
+      <c r="M125" s="10" t="inlineStr">
+        <is>
+          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
+        </is>
+      </c>
+      <c r="N125" s="10" t="inlineStr">
+        <is>
+          <t>37_ai_brief (11)</t>
+        </is>
+      </c>
+      <c r="O125" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P125" s="10" t="inlineStr">
+        <is>
+          <t>Overdue means unpaid more than 30 days after departure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="10" t="inlineStr">
+        <is>
+          <t>AI-003</t>
+        </is>
+      </c>
+      <c r="B126" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C126" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Admin</t>
+        </is>
+      </c>
+      <c r="D126" s="10" t="inlineStr">
+        <is>
+          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
+        </is>
+      </c>
+      <c r="E126" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F126" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G126" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H126" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view</t>
+        </is>
+      </c>
+      <c r="I126" s="10" t="inlineStr"/>
+      <c r="J126" s="10" t="inlineStr">
+        <is>
+          <t>a limit of 2</t>
+        </is>
+      </c>
+      <c r="K126" s="10" t="inlineStr">
+        <is>
+          <t>a third brief is requested</t>
+        </is>
+      </c>
+      <c r="L126" s="10" t="inlineStr">
+        <is>
+          <t>it is refused until a failed call frees a slot or the month turns</t>
+        </is>
+      </c>
+      <c r="M126" s="10" t="inlineStr">
+        <is>
+          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
+        </is>
+      </c>
+      <c r="N126" s="10" t="inlineStr">
+        <is>
+          <t>37_ai_brief (5)</t>
+        </is>
+      </c>
+      <c r="O126" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P126" s="10" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="10" t="inlineStr">
+        <is>
+          <t>AI-004</t>
+        </is>
+      </c>
+      <c r="B127" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C127" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Admin</t>
+        </is>
+      </c>
+      <c r="D127" s="10" t="inlineStr">
+        <is>
+          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
+        </is>
+      </c>
+      <c r="E127" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F127" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G127" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H127" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view, rpt.operations.view</t>
+        </is>
+      </c>
+      <c r="I127" s="10" t="inlineStr"/>
+      <c r="J127" s="10" t="inlineStr">
+        <is>
+          <t>front desk, housekeeping, another hotel</t>
+        </is>
+      </c>
+      <c r="K127" s="10" t="inlineStr">
+        <is>
+          <t>they ask for the brief or touch the tables</t>
+        </is>
+      </c>
+      <c r="L127" s="10" t="inlineStr">
+        <is>
+          <t>they are refused</t>
+        </is>
+      </c>
+      <c r="M127" s="10" t="inlineStr">
+        <is>
+          <t>20261013140000_ai_morning_brief.sql</t>
+        </is>
+      </c>
+      <c r="N127" s="10" t="inlineStr">
+        <is>
+          <t>37_ai_brief (7)</t>
+        </is>
+      </c>
+      <c r="O127" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P127" s="10" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="10" t="inlineStr">
+        <is>
+          <t>AI-005</t>
+        </is>
+      </c>
+      <c r="B128" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C128" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Admin</t>
+        </is>
+      </c>
+      <c r="D128" s="10" t="inlineStr">
+        <is>
+          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
+        </is>
+      </c>
+      <c r="E128" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F128" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G128" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H128" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I128" s="10" t="inlineStr"/>
+      <c r="J128" s="10" t="inlineStr">
+        <is>
+          <t>a draft that rounds or invents a figure</t>
+        </is>
+      </c>
+      <c r="K128" s="10" t="inlineStr">
+        <is>
+          <t>the brief is written</t>
+        </is>
+      </c>
+      <c r="L128" s="10" t="inlineStr">
+        <is>
+          <t>the plain database lines are shown instead, with a note</t>
+        </is>
+      </c>
+      <c r="M128" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
+        </is>
+      </c>
+      <c r="N128" s="10" t="inlineStr">
+        <is>
+          <t>browser unit: ai-brief-unit (8)</t>
+        </is>
+      </c>
+      <c r="O128" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P128" s="10" t="inlineStr">
+        <is>
+          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="10" t="inlineStr">
+        <is>
+          <t>SET-010</t>
+        </is>
+      </c>
+      <c r="B129" s="10" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="C129" s="10" t="inlineStr">
+        <is>
+          <t>Setup, Rooms</t>
+        </is>
+      </c>
+      <c r="D129" s="10" t="inlineStr">
+        <is>
+          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
+        </is>
+      </c>
+      <c r="E129" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F129" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G129" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H129" s="10" t="inlineStr">
+        <is>
+          <t>setup.room.manage</t>
+        </is>
+      </c>
+      <c r="I129" s="10" t="inlineStr"/>
+      <c r="J129" s="10" t="inlineStr">
+        <is>
+          <t>a list of room types and rooms</t>
+        </is>
+      </c>
+      <c r="K129" s="10" t="inlineStr">
+        <is>
+          <t>the manager previews and then applies it</t>
+        </is>
+      </c>
+      <c r="L129" s="10" t="inlineStr">
+        <is>
+          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
+        </is>
+      </c>
+      <c r="M129" s="10" t="inlineStr">
+        <is>
+          <t>20261013150000_setup_import.sql: apply_setup_import</t>
+        </is>
+      </c>
+      <c r="N129" s="10" t="inlineStr">
+        <is>
+          <t>38_setup_import (29)</t>
+        </is>
+      </c>
+      <c r="O129" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P129" s="10" t="inlineStr">
+        <is>
+          <t>The AI only drafts the list. This function is the check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="10" t="inlineStr">
+        <is>
+          <t>AI-006</t>
+        </is>
+      </c>
+      <c r="B130" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C130" s="10" t="inlineStr">
+        <is>
+          <t>Setup, Rooms</t>
+        </is>
+      </c>
+      <c r="D130" s="10" t="inlineStr">
+        <is>
+          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
+        </is>
+      </c>
+      <c r="E130" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F130" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G130" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H130" s="10" t="inlineStr">
+        <is>
+          <t>setup.room.manage</t>
+        </is>
+      </c>
+      <c r="I130" s="10" t="inlineStr"/>
+      <c r="J130" s="10" t="inlineStr">
+        <is>
+          <t>AI switched on with a limit of 1</t>
+        </is>
+      </c>
+      <c r="K130" s="10" t="inlineStr">
+        <is>
+          <t>an import draft is started twice</t>
+        </is>
+      </c>
+      <c r="L130" s="10" t="inlineStr">
+        <is>
+          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
+        </is>
+      </c>
+      <c r="M130" s="10" t="inlineStr">
+        <is>
+          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
+        </is>
+      </c>
+      <c r="N130" s="10" t="inlineStr">
+        <is>
+          <t>38_setup_import (8)</t>
+        </is>
+      </c>
+      <c r="O130" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P130" s="10" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="10" t="inlineStr">
+        <is>
+          <t>AI-007</t>
+        </is>
+      </c>
+      <c r="B131" s="10" t="inlineStr">
+        <is>
+          <t>AI helpers</t>
+        </is>
+      </c>
+      <c r="C131" s="10" t="inlineStr">
+        <is>
+          <t>Setup, Rooms</t>
+        </is>
+      </c>
+      <c r="D131" s="10" t="inlineStr">
+        <is>
+          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
+        </is>
+      </c>
+      <c r="E131" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F131" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G131" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H131" s="10" t="inlineStr">
+        <is>
+          <t>setup.room.manage</t>
+        </is>
+      </c>
+      <c r="I131" s="10" t="inlineStr"/>
+      <c r="J131" s="10" t="inlineStr">
+        <is>
+          <t>a pasted list</t>
+        </is>
+      </c>
+      <c r="K131" s="10" t="inlineStr">
+        <is>
+          <t>the assistant drafts it</t>
+        </is>
+      </c>
+      <c r="L131" s="10" t="inlineStr">
+        <is>
+          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
+        </is>
+      </c>
+      <c r="M131" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
+        </is>
+      </c>
+      <c r="N131" s="10" t="inlineStr">
+        <is>
+          <t>browser unit: setup-import-unit (9)</t>
+        </is>
+      </c>
+      <c r="O131" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P131" s="10" t="inlineStr">
+        <is>
+          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Last-room load test (NFR-006)
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13">
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P132"/>
+  <dimension ref="A1:P133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11042,6 +11042,88 @@
       <c r="P132" s="10" t="inlineStr">
         <is>
           <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="10" t="inlineStr">
+        <is>
+          <t>NFR-006</t>
+        </is>
+      </c>
+      <c r="B133" s="10" t="inlineStr">
+        <is>
+          <t>Non-functional</t>
+        </is>
+      </c>
+      <c r="C133" s="10" t="inlineStr">
+        <is>
+          <t>(all)</t>
+        </is>
+      </c>
+      <c r="D133" s="10" t="inlineStr">
+        <is>
+          <t>The last room of a type is sold once, however many desks book at the same moment, and a repeated booking never doubles.</t>
+        </is>
+      </c>
+      <c r="E133" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F133" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G133" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H133" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I133" s="10" t="inlineStr">
+        <is>
+          <t>Rule: Safe last-room booking</t>
+        </is>
+      </c>
+      <c r="J133" s="10" t="inlineStr">
+        <is>
+          <t>one room of a type is left and several desks book it together</t>
+        </is>
+      </c>
+      <c r="K133" s="10" t="inlineStr">
+        <is>
+          <t>all of them submit at the same moment</t>
+        </is>
+      </c>
+      <c r="L133" s="10" t="inlineStr">
+        <is>
+          <t>exactly one booking succeeds, the rest get E_NO_AVAILABILITY, and nothing is oversold</t>
+        </is>
+      </c>
+      <c r="M133" s="10" t="inlineStr">
+        <is>
+          <t>create_reservation, assert_available</t>
+        </is>
+      </c>
+      <c r="N133" s="10" t="inlineStr">
+        <is>
+          <t>concurrency/last_room.sh (6)</t>
+        </is>
+      </c>
+      <c r="O133" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P133" s="10" t="inlineStr">
+        <is>
+          <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Support access with the hotel's consent (PLT-010): database, tests, docs
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13">
@@ -631,7 +631,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Not built</t>
+          <t>Partly built (flags only)</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -641,20 +641,10 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Partly built (flags only)</t>
+          <t>Partly built, no tagged test</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Partly built, no tagged test</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1503,7 +1493,7 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Time-boxed break-glass support access, with reason, tenant notice and audit entry.</t>
+          <t>Time-boxed support access with the hotel's consent: the operator asks with a reason, the hotel's administrator says yes for 1 to 72 hours or no, can stop it at any time, and every step is in the hotel audit log. The support view is read-only and holds no guest, booking, money or contact data.</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -1523,7 +1513,7 @@
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>platform.support.access</t>
+          <t>platform operator; adm.support.manage</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
@@ -1533,35 +1523,39 @@
       </c>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>a platform user needs to help a hotel</t>
+          <t>a platform operator needs to help a hotel</t>
         </is>
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
-          <t>they request support access with a reason</t>
+          <t>they ask for support access with a reason and the hotel says yes</t>
         </is>
       </c>
       <c r="L11" s="10" t="inlineStr">
         <is>
-          <t>access is limited in time, written to the hotel's audit log and the hotel is told</t>
+          <t>they can open a read-only support view until the time ends or the hotel stops it; the hotel is told and every step is audited</t>
         </is>
       </c>
       <c r="M11" s="10" t="inlineStr">
         <is>
-          <t>(not written)</t>
+          <t>platform_request_support_access, decide_support_access, revoke_support_access, platform_support_snapshot, list_support_access</t>
         </is>
       </c>
       <c r="N11" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>41_support_access</t>
         </is>
       </c>
       <c r="O11" s="10" t="inlineStr">
         <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="P11" s="10" t="inlineStr"/>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P11" s="10" t="inlineStr">
+        <is>
+          <t>Database done 8 Oct 2026. Screens for the hotel (Admin) and the operator (platform console) follow. New permission adm.support.manage reaches System Administrator and General Manager only.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Add printable downtime pack (FO-014)
A /downtime page lists arrivals due, in-house guests with balance, departures due, blank paper walk-in lines and a short paper routine. No database change.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P133"/>
+  <dimension ref="A1:P134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11118,6 +11118,84 @@
       <c r="P133" s="10" t="inlineStr">
         <is>
           <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="10" t="inlineStr">
+        <is>
+          <t>FO-014</t>
+        </is>
+      </c>
+      <c r="B134" s="10" t="inlineStr">
+        <is>
+          <t>Front Office</t>
+        </is>
+      </c>
+      <c r="C134" s="10" t="inlineStr">
+        <is>
+          <t>/downtime</t>
+        </is>
+      </c>
+      <c r="D134" s="10" t="inlineStr">
+        <is>
+          <t>A printable downtime pack: arrivals due, in-house guests with balance, departures due, ten blank lines for new guests on paper, and a short paper routine. Staff print it when the internet or system is down.</t>
+        </is>
+      </c>
+      <c r="E134" s="10" t="inlineStr">
+        <is>
+          <t>BR-006</t>
+        </is>
+      </c>
+      <c r="F134" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G134" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H134" s="10" t="inlineStr">
+        <is>
+          <t>fo.view</t>
+        </is>
+      </c>
+      <c r="I134" s="10" t="inlineStr"/>
+      <c r="J134" s="10" t="inlineStr">
+        <is>
+          <t>a hotel with guests in house</t>
+        </is>
+      </c>
+      <c r="K134" s="10" t="inlineStr">
+        <is>
+          <t>a front desk user opens Downtime pack and prints</t>
+        </is>
+      </c>
+      <c r="L134" s="10" t="inlineStr">
+        <is>
+          <t>the lists show room, guest, phone, departure and the folio balance from the database, with blank lines and the paper routine</t>
+        </is>
+      </c>
+      <c r="M134" s="10" t="inlineStr">
+        <is>
+          <t>src/routes/_authenticated/_app/downtime.tsx</t>
+        </is>
+      </c>
+      <c r="N134" s="10" t="inlineStr">
+        <is>
+          <t>browser: downtime-pack.spec (1)</t>
+        </is>
+      </c>
+      <c r="O134" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P134" s="10" t="inlineStr">
+        <is>
+          <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add booking rules screen and set_booking_rules (SET-012)
Longest stay and tentative hold hours become editable on Setup, Property. New function, audited, with tests.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P133"/>
+  <dimension ref="A1:P134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11118,6 +11118,84 @@
       <c r="P133" s="10" t="inlineStr">
         <is>
           <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="10" t="inlineStr">
+        <is>
+          <t>SET-012</t>
+        </is>
+      </c>
+      <c r="B134" s="10" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="C134" s="10" t="inlineStr">
+        <is>
+          <t>/setup/property</t>
+        </is>
+      </c>
+      <c r="D134" s="10" t="inlineStr">
+        <is>
+          <t>A manager sets the longest stay (1 to 365 nights) and how long a tentative booking holds its room (1 to 720 hours) for each property.</t>
+        </is>
+      </c>
+      <c r="E134" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F134" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G134" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H134" s="10" t="inlineStr">
+        <is>
+          <t>setup.property.edit</t>
+        </is>
+      </c>
+      <c r="I134" s="10" t="inlineStr"/>
+      <c r="J134" s="10" t="inlineStr">
+        <is>
+          <t>a property with the default rules (30 nights, 24 hours)</t>
+        </is>
+      </c>
+      <c r="K134" s="10" t="inlineStr">
+        <is>
+          <t>a manager saves new booking rules</t>
+        </is>
+      </c>
+      <c r="L134" s="10" t="inlineStr">
+        <is>
+          <t>new bookings use them, bad values are refused with E_INVALID, and the change is audited with old and new values</t>
+        </is>
+      </c>
+      <c r="M134" s="10" t="inlineStr">
+        <is>
+          <t>set_booking_rules; Booking rules on Setup, Property</t>
+        </is>
+      </c>
+      <c r="N134" s="10" t="inlineStr">
+        <is>
+          <t>42_booking_rules (9)</t>
+        </is>
+      </c>
+      <c r="O134" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P134" s="10" t="inlineStr">
+        <is>
+          <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Warn night audit users before the business date rolls (DAY-007)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P135"/>
+  <dimension ref="A1:P136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11274,6 +11274,88 @@
       <c r="P135" s="10" t="inlineStr">
         <is>
           <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="10" t="inlineStr">
+        <is>
+          <t>DAY-007</t>
+        </is>
+      </c>
+      <c r="B136" s="10" t="inlineStr">
+        <is>
+          <t>Business Date</t>
+        </is>
+      </c>
+      <c r="C136" s="10" t="inlineStr">
+        <is>
+          <t>Notifications bell</t>
+        </is>
+      </c>
+      <c r="D136" s="10" t="inlineStr">
+        <is>
+          <t>In the last hour before a property rolls its business date, if a cashier shift is still open, users who can run the night audit get one warning that night. The roll does not wait.</t>
+        </is>
+      </c>
+      <c r="E136" s="10" t="inlineStr">
+        <is>
+          <t>BR-016</t>
+        </is>
+      </c>
+      <c r="F136" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G136" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H136" s="10" t="inlineStr">
+        <is>
+          <t>fin.nightaudit.run</t>
+        </is>
+      </c>
+      <c r="I136" s="10" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="J136" s="10" t="inlineStr">
+        <is>
+          <t>a cashier shift is still open</t>
+        </is>
+      </c>
+      <c r="K136" s="10" t="inlineStr">
+        <is>
+          <t>the roll time is less than 60 minutes away</t>
+        </is>
+      </c>
+      <c r="L136" s="10" t="inlineStr">
+        <is>
+          <t>each night audit user gets one rollover_warning notification for that business date; none earlier, none after the roll time, none if no shift is open, none twice</t>
+        </is>
+      </c>
+      <c r="M136" s="10" t="inlineStr">
+        <is>
+          <t>app.warn_before_rollover; cron job rollover-warning</t>
+        </is>
+      </c>
+      <c r="N136" s="10" t="inlineStr">
+        <is>
+          <t>43_rollover_warning (7)</t>
+        </is>
+      </c>
+      <c r="O136" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P136" s="10" t="inlineStr">
+        <is>
+          <t>Added 8 Oct 2026. Warning only; the hard gate stays in R2 (DAY-005).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Prove the sample folio tax method with setup only (FIN-018)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P136"/>
+  <dimension ref="A1:P137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9412,22 +9412,22 @@
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>GST-007</t>
+          <t>FIN-018</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t>Guests</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
         <is>
-          <t>/guests/$id; check-in; walk-in</t>
+          <t>/setup/taxes</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t>A photo or scan of an ID document is kept in private storage, shrunk and stripped of hidden data in the browser, and opened only through a 60-second link.</t>
+          <t>A hotel can match the tax method of its existing folio using setup alone: each tax on the room price only, food and drink untaxed. A sample bill of 45,000 room plus 12,001 bar totals 67,126.</t>
         </is>
       </c>
       <c r="E112" s="10" t="inlineStr">
@@ -9447,37 +9447,37 @@
       </c>
       <c r="H112" s="10" t="inlineStr">
         <is>
-          <t>guest.document.file.upload / view / delete</t>
+          <t>setup.tax.manage</t>
         </is>
       </c>
       <c r="I112" s="10" t="inlineStr">
         <is>
-          <t>SET-009 switch</t>
+          <t>Tax rates compounds_on_previous; charge code is_taxable</t>
         </is>
       </c>
       <c r="J112" s="10" t="inlineStr">
         <is>
-          <t>a hotel that allows ID photos</t>
+          <t>a property with service charge 10%, VAT 7.5% and state tax 5%, none compounding, and a non-taxable bar code</t>
         </is>
       </c>
       <c r="K112" s="10" t="inlineStr">
         <is>
-          <t>front desk adds an ID photo</t>
+          <t>a room charge of 45,000 and a bar charge of 12,001 are posted</t>
         </is>
       </c>
       <c r="L112" s="10" t="inlineStr">
         <is>
-          <t>it is stored privately and opens only through a short-lived link</t>
+          <t>the taxes are 4,500, 3,375 and 2,250, the bar has no tax and the bill is 67,126</t>
         </is>
       </c>
       <c r="M112" s="10" t="inlineStr">
         <is>
-          <t>begin_id_photo_upload, finish_id_photo_upload, open_id_photo</t>
+          <t>save_tax_rate, save_charge_code, post_charge</t>
         </is>
       </c>
       <c r="N112" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (30)</t>
+          <t>44_folio_sample_method (5)</t>
         </is>
       </c>
       <c r="O112" s="10" t="inlineStr">
@@ -9485,12 +9485,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P112" s="10" t="inlineStr"/>
+      <c r="P112" s="10" t="inlineStr">
+        <is>
+          <t>Method only; the accountant still signs off the rates (A11)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>GST-008</t>
+          <t>GST-007</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
@@ -9500,12 +9504,12 @@
       </c>
       <c r="C113" s="10" t="inlineStr">
         <is>
-          <t>/guests/$id</t>
+          <t>/guests/$id; check-in; walk-in</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t>Every upload, view and deletion of an ID photo is audited with ids only, no personal data.</t>
+          <t>A photo or scan of an ID document is kept in private storage, shrunk and stripped of hidden data in the browser, and opened only through a 60-second link.</t>
         </is>
       </c>
       <c r="E113" s="10" t="inlineStr">
@@ -9525,37 +9529,37 @@
       </c>
       <c r="H113" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>guest.document.file.upload / view / delete</t>
         </is>
       </c>
       <c r="I113" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SET-009 switch</t>
         </is>
       </c>
       <c r="J113" s="10" t="inlineStr">
         <is>
-          <t>an ID photo</t>
+          <t>a hotel that allows ID photos</t>
         </is>
       </c>
       <c r="K113" s="10" t="inlineStr">
         <is>
-          <t>it is uploaded, opened or deleted</t>
+          <t>front desk adds an ID photo</t>
         </is>
       </c>
       <c r="L113" s="10" t="inlineStr">
         <is>
-          <t>an audit row records who and which file, with no personal data</t>
+          <t>it is stored privately and opens only through a short-lived link</t>
         </is>
       </c>
       <c r="M113" s="10" t="inlineStr">
         <is>
-          <t>app.audit_id_photo</t>
+          <t>begin_id_photo_upload, finish_id_photo_upload, open_id_photo</t>
         </is>
       </c>
       <c r="N113" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (9)</t>
+          <t>24_id_photos (30)</t>
         </is>
       </c>
       <c r="O113" s="10" t="inlineStr">
@@ -9568,7 +9572,7 @@
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>GST-009</t>
+          <t>GST-008</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
@@ -9583,7 +9587,7 @@
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t>ID photos are removed from storage when the guest is anonymised or the document is removed, and move with the guest when two profiles are merged.</t>
+          <t>Every upload, view and deletion of an ID photo is audited with ids only, no personal data.</t>
         </is>
       </c>
       <c r="E114" s="10" t="inlineStr">
@@ -9613,27 +9617,27 @@
       </c>
       <c r="J114" s="10" t="inlineStr">
         <is>
-          <t>a guest with ID photos</t>
+          <t>an ID photo</t>
         </is>
       </c>
       <c r="K114" s="10" t="inlineStr">
         <is>
-          <t>the guest is anonymised, the document removed, or the profile merged</t>
+          <t>it is uploaded, opened or deleted</t>
         </is>
       </c>
       <c r="L114" s="10" t="inlineStr">
         <is>
-          <t>the files are removed, or move to the kept profile</t>
+          <t>an audit row records who and which file, with no personal data</t>
         </is>
       </c>
       <c r="M114" s="10" t="inlineStr">
         <is>
-          <t>anonymise_guest, merge_guests, delete_id_photo</t>
+          <t>app.audit_id_photo</t>
         </is>
       </c>
       <c r="N114" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (4)</t>
+          <t>24_id_photos (9)</t>
         </is>
       </c>
       <c r="O114" s="10" t="inlineStr">
@@ -9646,7 +9650,7 @@
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>GST-010</t>
+          <t>GST-009</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
@@ -9656,12 +9660,12 @@
       </c>
       <c r="C115" s="10" t="inlineStr">
         <is>
-          <t>(daily clean-up)</t>
+          <t>/guests/$id</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t>ID photos are deleted automatically a set number of months (one setting, now 12) after the guest's last check-out, unless the guest has a booking that is not over.</t>
+          <t>ID photos are removed from storage when the guest is anonymised or the document is removed, and move with the guest when two profiles are merged.</t>
         </is>
       </c>
       <c r="E115" s="10" t="inlineStr">
@@ -9686,32 +9690,32 @@
       </c>
       <c r="I115" s="10" t="inlineStr">
         <is>
-          <t>Setting id_photo_keep_months; daily cron</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J115" s="10" t="inlineStr">
         <is>
-          <t>a guest whose last check-out was more than the keep period ago</t>
+          <t>a guest with ID photos</t>
         </is>
       </c>
       <c r="K115" s="10" t="inlineStr">
         <is>
-          <t>the daily clean-up runs</t>
+          <t>the guest is anonymised, the document removed, or the profile merged</t>
         </is>
       </c>
       <c r="L115" s="10" t="inlineStr">
         <is>
-          <t>their ID photos are deleted</t>
+          <t>the files are removed, or move to the kept profile</t>
         </is>
       </c>
       <c r="M115" s="10" t="inlineStr">
         <is>
-          <t>/api/cron/id-photo-cleanup</t>
+          <t>anonymise_guest, merge_guests, delete_id_photo</t>
         </is>
       </c>
       <c r="N115" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (5)</t>
+          <t>24_id_photos (4)</t>
         </is>
       </c>
       <c r="O115" s="10" t="inlineStr">
@@ -9724,22 +9728,22 @@
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
         <is>
-          <t>ROOM-005</t>
+          <t>GST-010</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t>Rooms</t>
+          <t>Guests</t>
         </is>
       </c>
       <c r="C116" s="10" t="inlineStr">
         <is>
-          <t>/rooms</t>
+          <t>(daily clean-up)</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t>Rooms are added one at a time or several by number or by name, with a preview; labels are free text up to 30 characters, unique per hotel ignoring case and extra spaces, shown as typed and sorted in natural order.</t>
+          <t>ID photos are deleted automatically a set number of months (one setting, now 12) after the guest's last check-out, unless the guest has a booking that is not over.</t>
         </is>
       </c>
       <c r="E116" s="10" t="inlineStr">
@@ -9759,37 +9763,37 @@
       </c>
       <c r="H116" s="10" t="inlineStr">
         <is>
-          <t>setup.room.edit</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I116" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Setting id_photo_keep_months; daily cron</t>
         </is>
       </c>
       <c r="J116" s="10" t="inlineStr">
         <is>
-          <t>an administrator on the Rooms page</t>
+          <t>a guest whose last check-out was more than the keep period ago</t>
         </is>
       </c>
       <c r="K116" s="10" t="inlineStr">
         <is>
-          <t>they add rooms by number range or by names</t>
+          <t>the daily clean-up runs</t>
         </is>
       </c>
       <c r="L116" s="10" t="inlineStr">
         <is>
-          <t>valid new rooms are created, duplicates skipped and invalid names shown</t>
+          <t>their ID photos are deleted</t>
         </is>
       </c>
       <c r="M116" s="10" t="inlineStr">
         <is>
-          <t>add_rooms_range, add_rooms_named, save_room</t>
+          <t>/api/cron/id-photo-cleanup</t>
         </is>
       </c>
       <c r="N116" s="10" t="inlineStr">
         <is>
-          <t>23_room_labels (46); 26_small_fixes (1); browser: rooms-add</t>
+          <t>24_id_photos (5)</t>
         </is>
       </c>
       <c r="O116" s="10" t="inlineStr">
@@ -9802,22 +9806,22 @@
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>SET-009</t>
+          <t>ROOM-005</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Rooms</t>
         </is>
       </c>
       <c r="C117" s="10" t="inlineStr">
         <is>
-          <t>/setup/property</t>
+          <t>/rooms</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t>Per hotel: "Allow ID photos" (off by default) and "Require ID photo at check-in" (only when allowed). While Allow is off, uploading and opening ID photos are refused.</t>
+          <t>Rooms are added one at a time or several by number or by name, with a preview; labels are free text up to 30 characters, unique per hotel ignoring case and extra spaces, shown as typed and sorted in natural order.</t>
         </is>
       </c>
       <c r="E117" s="10" t="inlineStr">
@@ -9837,7 +9841,7 @@
       </c>
       <c r="H117" s="10" t="inlineStr">
         <is>
-          <t>setup.property.edit</t>
+          <t>setup.room.edit</t>
         </is>
       </c>
       <c r="I117" s="10" t="inlineStr">
@@ -9847,27 +9851,27 @@
       </c>
       <c r="J117" s="10" t="inlineStr">
         <is>
-          <t>a hotel with ID photos off</t>
+          <t>an administrator on the Rooms page</t>
         </is>
       </c>
       <c r="K117" s="10" t="inlineStr">
         <is>
-          <t>staff try to add or open an ID photo</t>
+          <t>they add rooms by number range or by names</t>
         </is>
       </c>
       <c r="L117" s="10" t="inlineStr">
         <is>
-          <t>it is refused; when Require is on, check-in waits for an ID photo</t>
+          <t>valid new rooms are created, duplicates skipped and invalid names shown</t>
         </is>
       </c>
       <c r="M117" s="10" t="inlineStr">
         <is>
-          <t>set_id_photo_settings</t>
+          <t>add_rooms_range, add_rooms_named, save_room</t>
         </is>
       </c>
       <c r="N117" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (10)</t>
+          <t>23_room_labels (46); 26_small_fixes (1); browser: rooms-add</t>
         </is>
       </c>
       <c r="O117" s="10" t="inlineStr">
@@ -9880,32 +9884,32 @@
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
         <is>
-          <t>GRP-001</t>
+          <t>SET-009</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t>Platform &amp; Tenancy</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C118" s="10" t="inlineStr">
         <is>
-          <t>All branches</t>
+          <t>/setup/property</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t>A built-in Group Manager role and the permission rpt.group.view exist; only System Administrator, General Manager and Group Manager hold the permission.</t>
+          <t>Per hotel: "Allow ID photos" (off by default) and "Require ID photo at check-in" (only when allowed). While Allow is off, uploading and opening ID photos are refused.</t>
         </is>
       </c>
       <c r="E118" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F118" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G118" s="10" t="inlineStr">
@@ -9915,33 +9919,37 @@
       </c>
       <c r="H118" s="10" t="inlineStr">
         <is>
-          <t>rpt.group.view</t>
-        </is>
-      </c>
-      <c r="I118" s="10" t="inlineStr"/>
+          <t>setup.property.edit</t>
+        </is>
+      </c>
+      <c r="I118" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="J118" s="10" t="inlineStr">
         <is>
-          <t>a hotel group with several branches</t>
+          <t>a hotel with ID photos off</t>
         </is>
       </c>
       <c r="K118" s="10" t="inlineStr">
         <is>
-          <t>an owner wants a view-only manager for the whole group</t>
+          <t>staff try to add or open an ID photo</t>
         </is>
       </c>
       <c r="L118" s="10" t="inlineStr">
         <is>
-          <t>they assign the Group Manager role branch by branch, and that person can look but not post or change anything</t>
+          <t>it is refused; when Require is on, check-in waits for an ID photo</t>
         </is>
       </c>
       <c r="M118" s="10" t="inlineStr">
         <is>
-          <t>20261013120000_group_view.sql</t>
+          <t>set_id_photo_settings</t>
         </is>
       </c>
       <c r="N118" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (5)</t>
+          <t>24_id_photos (10)</t>
         </is>
       </c>
       <c r="O118" s="10" t="inlineStr">
@@ -9949,16 +9957,12 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P118" s="10" t="inlineStr">
-        <is>
-          <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
-        </is>
-      </c>
+      <c r="P118" s="10" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>GRP-002</t>
+          <t>GRP-001</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
@@ -9973,7 +9977,7 @@
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t>One call shows every branch the person may see: occupancy, in house, arrivals and departures to come, approvals, repairs and last night revenue, with group totals. Revenue is totalled per currency.</t>
+          <t>A built-in Group Manager role and the permission rpt.group.view exist; only System Administrator, General Manager and Group Manager hold the permission.</t>
         </is>
       </c>
       <c r="E119" s="10" t="inlineStr">
@@ -9999,27 +10003,27 @@
       <c r="I119" s="10" t="inlineStr"/>
       <c r="J119" s="10" t="inlineStr">
         <is>
-          <t>a group with a Lagos and an Abuja branch</t>
+          <t>a hotel group with several branches</t>
         </is>
       </c>
       <c r="K119" s="10" t="inlineStr">
         <is>
-          <t>a group manager opens All branches</t>
+          <t>an owner wants a view-only manager for the whole group</t>
         </is>
       </c>
       <c r="L119" s="10" t="inlineStr">
         <is>
-          <t>they see both branches with figures from the database, never another hotel group, and staff without the permission are refused</t>
+          <t>they assign the Group Manager role branch by branch, and that person can look but not post or change anything</t>
         </is>
       </c>
       <c r="M119" s="10" t="inlineStr">
         <is>
-          <t>group_overview; /group screen</t>
+          <t>20261013120000_group_view.sql</t>
         </is>
       </c>
       <c r="N119" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (10)</t>
+          <t>35_group_view (5)</t>
         </is>
       </c>
       <c r="O119" s="10" t="inlineStr">
@@ -10029,14 +10033,14 @@
       </c>
       <c r="P119" s="10" t="inlineStr">
         <is>
-          <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
+          <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
         <is>
-          <t>GRP-003</t>
+          <t>GRP-002</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
@@ -10051,7 +10055,7 @@
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t>A Group Manager sees only the branches they are assigned to, and cannot post charges or check guests in.</t>
+          <t>One call shows every branch the person may see: occupancy, in house, arrivals and departures to come, approvals, repairs and last night revenue, with group totals. Revenue is totalled per currency.</t>
         </is>
       </c>
       <c r="E120" s="10" t="inlineStr">
@@ -10077,27 +10081,27 @@
       <c r="I120" s="10" t="inlineStr"/>
       <c r="J120" s="10" t="inlineStr">
         <is>
-          <t>a Group Manager assigned to one branch</t>
+          <t>a group with a Lagos and an Abuja branch</t>
         </is>
       </c>
       <c r="K120" s="10" t="inlineStr">
         <is>
-          <t>a second branch is assigned</t>
+          <t>a group manager opens All branches</t>
         </is>
       </c>
       <c r="L120" s="10" t="inlineStr">
         <is>
-          <t>the second branch appears; the role never gets write permissions</t>
+          <t>they see both branches with figures from the database, never another hotel group, and staff without the permission are refused</t>
         </is>
       </c>
       <c r="M120" s="10" t="inlineStr">
         <is>
-          <t>assign_role (existing); group_overview</t>
+          <t>group_overview; /group screen</t>
         </is>
       </c>
       <c r="N120" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (3)</t>
+          <t>35_group_view (10)</t>
         </is>
       </c>
       <c r="O120" s="10" t="inlineStr">
@@ -10107,14 +10111,14 @@
       </c>
       <c r="P120" s="10" t="inlineStr">
         <is>
-          <t>Access is per branch, using the existing role assignment screen.</t>
+          <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>GRP-004</t>
+          <t>GRP-003</t>
         </is>
       </c>
       <c r="B121" s="10" t="inlineStr">
@@ -10124,12 +10128,12 @@
       </c>
       <c r="C121" s="10" t="inlineStr">
         <is>
-          <t>All branches (Copy setup)</t>
+          <t>All branches</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t>A new branch can copy room types, rate plans and prices from an existing branch, once, into an empty branch.</t>
+          <t>A Group Manager sees only the branches they are assigned to, and cannot post charges or check guests in.</t>
         </is>
       </c>
       <c r="E121" s="10" t="inlineStr">
@@ -10149,33 +10153,33 @@
       </c>
       <c r="H121" s="10" t="inlineStr">
         <is>
-          <t>setup.room.manage, setup.rate.manage</t>
+          <t>rpt.group.view</t>
         </is>
       </c>
       <c r="I121" s="10" t="inlineStr"/>
       <c r="J121" s="10" t="inlineStr">
         <is>
-          <t>a new empty branch</t>
+          <t>a Group Manager assigned to one branch</t>
         </is>
       </c>
       <c r="K121" s="10" t="inlineStr">
         <is>
-          <t>the owner copies setup from the first branch</t>
+          <t>a second branch is assigned</t>
         </is>
       </c>
       <c r="L121" s="10" t="inlineStr">
         <is>
-          <t>room types, rate plans and prices appear on the new branch and point at its own room types; rooms are not copied; a second copy is refused; the copy is audited</t>
+          <t>the second branch appears; the role never gets write permissions</t>
         </is>
       </c>
       <c r="M121" s="10" t="inlineStr">
         <is>
-          <t>copy_property_setup</t>
+          <t>assign_role (existing); group_overview</t>
         </is>
       </c>
       <c r="N121" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (13)</t>
+          <t>35_group_view (3)</t>
         </is>
       </c>
       <c r="O121" s="10" t="inlineStr">
@@ -10185,29 +10189,29 @@
       </c>
       <c r="P121" s="10" t="inlineStr">
         <is>
-          <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
+          <t>Access is per branch, using the existing role assignment screen.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="10" t="inlineStr">
         <is>
-          <t>RPT-005</t>
+          <t>GRP-004</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Platform &amp; Tenancy</t>
         </is>
       </c>
       <c r="C122" s="10" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>All branches (Copy setup)</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t>Revenue by booking source: bookings, cancellations, no-shows, room nights, room revenue and average rate for each source in a date range.</t>
+          <t>A new branch can copy room types, rate plans and prices from an existing branch, once, into an empty branch.</t>
         </is>
       </c>
       <c r="E122" s="10" t="inlineStr">
@@ -10227,33 +10231,33 @@
       </c>
       <c r="H122" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view</t>
+          <t>setup.room.manage, setup.rate.manage</t>
         </is>
       </c>
       <c r="I122" s="10" t="inlineStr"/>
       <c r="J122" s="10" t="inlineStr">
         <is>
-          <t>bookings from direct, phone and company sources</t>
+          <t>a new empty branch</t>
         </is>
       </c>
       <c r="K122" s="10" t="inlineStr">
         <is>
-          <t>the accountant picks a date range</t>
+          <t>the owner copies setup from the first branch</t>
         </is>
       </c>
       <c r="L122" s="10" t="inlineStr">
         <is>
-          <t>each source shows its own counts and room revenue (room charges only, before tax); cancelled bookings add no nights</t>
+          <t>room types, rate plans and prices appear on the new branch and point at its own room types; rooms are not copied; a second copy is refused; the copy is audited</t>
         </is>
       </c>
       <c r="M122" s="10" t="inlineStr">
         <is>
-          <t>20261013130000_source_ageing_reports.sql: report_revenue_by_source; Reports, By booking source tab</t>
+          <t>copy_property_setup</t>
         </is>
       </c>
       <c r="N122" s="10" t="inlineStr">
         <is>
-          <t>36_source_ageing (13)</t>
+          <t>35_group_view (13)</t>
         </is>
       </c>
       <c r="O122" s="10" t="inlineStr">
@@ -10263,14 +10267,14 @@
       </c>
       <c r="P122" s="10" t="inlineStr">
         <is>
-          <t>Bookings counted by arrival date; revenue by posting date.</t>
+          <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>RPT-006</t>
+          <t>RPT-005</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
@@ -10285,7 +10289,7 @@
       </c>
       <c r="D123" s="10" t="inlineStr">
         <is>
-          <t>Ageing of unpaid balances by booking source: current, 1 to 7, 8 to 30, 31 to 60 and over 60 days since the due departure, plus credit held.</t>
+          <t>Revenue by booking source: bookings, cancellations, no-shows, room nights, room revenue and average rate for each source in a date range.</t>
         </is>
       </c>
       <c r="E123" s="10" t="inlineStr">
@@ -10311,27 +10315,27 @@
       <c r="I123" s="10" t="inlineStr"/>
       <c r="J123" s="10" t="inlineStr">
         <is>
-          <t>guests and companies who left owing money</t>
+          <t>bookings from direct, phone and company sources</t>
         </is>
       </c>
       <c r="K123" s="10" t="inlineStr">
         <is>
-          <t>the accountant opens the Ageing tab</t>
+          <t>the accountant picks a date range</t>
         </is>
       </c>
       <c r="L123" s="10" t="inlineStr">
         <is>
-          <t>each source shows what is owed in each age column; paid bills drop out; overpayments show as credit held; the total matches Outstanding balances</t>
+          <t>each source shows its own counts and room revenue (room charges only, before tax); cancelled bookings add no nights</t>
         </is>
       </c>
       <c r="M123" s="10" t="inlineStr">
         <is>
-          <t>report_balance_ageing; Reports, Ageing tab</t>
+          <t>20261013130000_source_ageing_reports.sql: report_revenue_by_source; Reports, By booking source tab</t>
         </is>
       </c>
       <c r="N123" s="10" t="inlineStr">
         <is>
-          <t>36_source_ageing (11)</t>
+          <t>36_source_ageing (13)</t>
         </is>
       </c>
       <c r="O123" s="10" t="inlineStr">
@@ -10341,29 +10345,29 @@
       </c>
       <c r="P123" s="10" t="inlineStr">
         <is>
-          <t>Guests still staying count as current.</t>
+          <t>Bookings counted by arrival date; revenue by posting date.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="10" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>RPT-006</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
         <is>
-          <t>AI helpers</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C124" s="10" t="inlineStr">
         <is>
-          <t>Dashboard, Admin</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr">
         <is>
-          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
+          <t>Ageing of unpaid balances by booking source: current, 1 to 7, 8 to 30, 31 to 60 and over 60 days since the due departure, plus credit held.</t>
         </is>
       </c>
       <c r="E124" s="10" t="inlineStr">
@@ -10383,33 +10387,33 @@
       </c>
       <c r="H124" s="10" t="inlineStr">
         <is>
-          <t>adm.ai.manage</t>
+          <t>rpt.finance.view</t>
         </is>
       </c>
       <c r="I124" s="10" t="inlineStr"/>
       <c r="J124" s="10" t="inlineStr">
         <is>
-          <t>a new hotel</t>
+          <t>guests and companies who left owing money</t>
         </is>
       </c>
       <c r="K124" s="10" t="inlineStr">
         <is>
-          <t>a manager opens Admin, AI helpers</t>
+          <t>the accountant opens the Ageing tab</t>
         </is>
       </c>
       <c r="L124" s="10" t="inlineStr">
         <is>
-          <t>nothing runs until they switch it on and the change is in the audit log</t>
+          <t>each source shows what is owed in each age column; paid bills drop out; overpayments show as credit held; the total matches Outstanding balances</t>
         </is>
       </c>
       <c r="M124" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
+          <t>report_balance_ageing; Reports, Ageing tab</t>
         </is>
       </c>
       <c r="N124" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (11)</t>
+          <t>36_source_ageing (11)</t>
         </is>
       </c>
       <c r="O124" s="10" t="inlineStr">
@@ -10419,14 +10423,14 @@
       </c>
       <c r="P124" s="10" t="inlineStr">
         <is>
-          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
+          <t>Guests still staying count as current.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>AI-002</t>
+          <t>AI-001</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
@@ -10441,7 +10445,7 @@
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
+          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
         </is>
       </c>
       <c r="E125" s="10" t="inlineStr">
@@ -10461,28 +10465,28 @@
       </c>
       <c r="H125" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view, rpt.operations.view</t>
+          <t>adm.ai.manage</t>
         </is>
       </c>
       <c r="I125" s="10" t="inlineStr"/>
       <c r="J125" s="10" t="inlineStr">
         <is>
-          <t>a hotel with guests, approvals and overdue bills</t>
+          <t>a new hotel</t>
         </is>
       </c>
       <c r="K125" s="10" t="inlineStr">
         <is>
-          <t>a brief is started</t>
+          <t>a manager opens Admin, AI helpers</t>
         </is>
       </c>
       <c r="L125" s="10" t="inlineStr">
         <is>
-          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
+          <t>nothing runs until they switch it on and the change is in the audit log</t>
         </is>
       </c>
       <c r="M125" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
+          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
         </is>
       </c>
       <c r="N125" s="10" t="inlineStr">
@@ -10497,14 +10501,14 @@
       </c>
       <c r="P125" s="10" t="inlineStr">
         <is>
-          <t>Overdue means unpaid more than 30 days after departure.</t>
+          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="10" t="inlineStr">
         <is>
-          <t>AI-003</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
@@ -10519,7 +10523,7 @@
       </c>
       <c r="D126" s="10" t="inlineStr">
         <is>
-          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
+          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
         </is>
       </c>
       <c r="E126" s="10" t="inlineStr">
@@ -10539,33 +10543,33 @@
       </c>
       <c r="H126" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view</t>
+          <t>rpt.finance.view, rpt.operations.view</t>
         </is>
       </c>
       <c r="I126" s="10" t="inlineStr"/>
       <c r="J126" s="10" t="inlineStr">
         <is>
-          <t>a limit of 2</t>
+          <t>a hotel with guests, approvals and overdue bills</t>
         </is>
       </c>
       <c r="K126" s="10" t="inlineStr">
         <is>
-          <t>a third brief is requested</t>
+          <t>a brief is started</t>
         </is>
       </c>
       <c r="L126" s="10" t="inlineStr">
         <is>
-          <t>it is refused until a failed call frees a slot or the month turns</t>
+          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
         </is>
       </c>
       <c r="M126" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
+          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
         </is>
       </c>
       <c r="N126" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (5)</t>
+          <t>37_ai_brief (11)</t>
         </is>
       </c>
       <c r="O126" s="10" t="inlineStr">
@@ -10573,12 +10577,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P126" s="10" t="inlineStr"/>
+      <c r="P126" s="10" t="inlineStr">
+        <is>
+          <t>Overdue means unpaid more than 30 days after departure.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
         <is>
-          <t>AI-004</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
@@ -10593,7 +10601,7 @@
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
+          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
         </is>
       </c>
       <c r="E127" s="10" t="inlineStr">
@@ -10613,33 +10621,33 @@
       </c>
       <c r="H127" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view, rpt.operations.view</t>
+          <t>rpt.finance.view</t>
         </is>
       </c>
       <c r="I127" s="10" t="inlineStr"/>
       <c r="J127" s="10" t="inlineStr">
         <is>
-          <t>front desk, housekeeping, another hotel</t>
+          <t>a limit of 2</t>
         </is>
       </c>
       <c r="K127" s="10" t="inlineStr">
         <is>
-          <t>they ask for the brief or touch the tables</t>
+          <t>a third brief is requested</t>
         </is>
       </c>
       <c r="L127" s="10" t="inlineStr">
         <is>
-          <t>they are refused</t>
+          <t>it is refused until a failed call frees a slot or the month turns</t>
         </is>
       </c>
       <c r="M127" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql</t>
+          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
         </is>
       </c>
       <c r="N127" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (7)</t>
+          <t>37_ai_brief (5)</t>
         </is>
       </c>
       <c r="O127" s="10" t="inlineStr">
@@ -10652,7 +10660,7 @@
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
         <is>
-          <t>AI-005</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
@@ -10667,7 +10675,7 @@
       </c>
       <c r="D128" s="10" t="inlineStr">
         <is>
-          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
+          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
         </is>
       </c>
       <c r="E128" s="10" t="inlineStr">
@@ -10687,33 +10695,33 @@
       </c>
       <c r="H128" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>rpt.finance.view, rpt.operations.view</t>
         </is>
       </c>
       <c r="I128" s="10" t="inlineStr"/>
       <c r="J128" s="10" t="inlineStr">
         <is>
-          <t>a draft that rounds or invents a figure</t>
+          <t>front desk, housekeeping, another hotel</t>
         </is>
       </c>
       <c r="K128" s="10" t="inlineStr">
         <is>
-          <t>the brief is written</t>
+          <t>they ask for the brief or touch the tables</t>
         </is>
       </c>
       <c r="L128" s="10" t="inlineStr">
         <is>
-          <t>the plain database lines are shown instead, with a note</t>
+          <t>they are refused</t>
         </is>
       </c>
       <c r="M128" s="10" t="inlineStr">
         <is>
-          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
+          <t>20261013140000_ai_morning_brief.sql</t>
         </is>
       </c>
       <c r="N128" s="10" t="inlineStr">
         <is>
-          <t>browser unit: ai-brief-unit (8)</t>
+          <t>37_ai_brief (7)</t>
         </is>
       </c>
       <c r="O128" s="10" t="inlineStr">
@@ -10721,31 +10729,27 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P128" s="10" t="inlineStr">
-        <is>
-          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
-        </is>
-      </c>
+      <c r="P128" s="10" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
         <is>
-          <t>SET-010</t>
+          <t>AI-005</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>AI helpers</t>
         </is>
       </c>
       <c r="C129" s="10" t="inlineStr">
         <is>
-          <t>Setup, Rooms</t>
+          <t>Dashboard, Admin</t>
         </is>
       </c>
       <c r="D129" s="10" t="inlineStr">
         <is>
-          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
+          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
         </is>
       </c>
       <c r="E129" s="10" t="inlineStr">
@@ -10765,33 +10769,33 @@
       </c>
       <c r="H129" s="10" t="inlineStr">
         <is>
-          <t>setup.room.manage</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I129" s="10" t="inlineStr"/>
       <c r="J129" s="10" t="inlineStr">
         <is>
-          <t>a list of room types and rooms</t>
+          <t>a draft that rounds or invents a figure</t>
         </is>
       </c>
       <c r="K129" s="10" t="inlineStr">
         <is>
-          <t>the manager previews and then applies it</t>
+          <t>the brief is written</t>
         </is>
       </c>
       <c r="L129" s="10" t="inlineStr">
         <is>
-          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
+          <t>the plain database lines are shown instead, with a note</t>
         </is>
       </c>
       <c r="M129" s="10" t="inlineStr">
         <is>
-          <t>20261013150000_setup_import.sql: apply_setup_import</t>
+          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
         </is>
       </c>
       <c r="N129" s="10" t="inlineStr">
         <is>
-          <t>38_setup_import (29)</t>
+          <t>browser unit: ai-brief-unit (8)</t>
         </is>
       </c>
       <c r="O129" s="10" t="inlineStr">
@@ -10801,19 +10805,19 @@
       </c>
       <c r="P129" s="10" t="inlineStr">
         <is>
-          <t>The AI only drafts the list. This function is the check.</t>
+          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
         <is>
-          <t>AI-006</t>
+          <t>SET-010</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
         <is>
-          <t>AI helpers</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C130" s="10" t="inlineStr">
@@ -10823,7 +10827,7 @@
       </c>
       <c r="D130" s="10" t="inlineStr">
         <is>
-          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
+          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
         </is>
       </c>
       <c r="E130" s="10" t="inlineStr">
@@ -10849,27 +10853,27 @@
       <c r="I130" s="10" t="inlineStr"/>
       <c r="J130" s="10" t="inlineStr">
         <is>
-          <t>AI switched on with a limit of 1</t>
+          <t>a list of room types and rooms</t>
         </is>
       </c>
       <c r="K130" s="10" t="inlineStr">
         <is>
-          <t>an import draft is started twice</t>
+          <t>the manager previews and then applies it</t>
         </is>
       </c>
       <c r="L130" s="10" t="inlineStr">
         <is>
-          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
+          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
         </is>
       </c>
       <c r="M130" s="10" t="inlineStr">
         <is>
-          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
+          <t>20261013150000_setup_import.sql: apply_setup_import</t>
         </is>
       </c>
       <c r="N130" s="10" t="inlineStr">
         <is>
-          <t>38_setup_import (8)</t>
+          <t>38_setup_import (29)</t>
         </is>
       </c>
       <c r="O130" s="10" t="inlineStr">
@@ -10877,12 +10881,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P130" s="10" t="inlineStr"/>
+      <c r="P130" s="10" t="inlineStr">
+        <is>
+          <t>The AI only drafts the list. This function is the check.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
         <is>
-          <t>AI-007</t>
+          <t>AI-006</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
@@ -10897,7 +10905,7 @@
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
+          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
         </is>
       </c>
       <c r="E131" s="10" t="inlineStr">
@@ -10923,27 +10931,27 @@
       <c r="I131" s="10" t="inlineStr"/>
       <c r="J131" s="10" t="inlineStr">
         <is>
-          <t>a pasted list</t>
+          <t>AI switched on with a limit of 1</t>
         </is>
       </c>
       <c r="K131" s="10" t="inlineStr">
         <is>
-          <t>the assistant drafts it</t>
+          <t>an import draft is started twice</t>
         </is>
       </c>
       <c r="L131" s="10" t="inlineStr">
         <is>
-          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
+          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
         </is>
       </c>
       <c r="M131" s="10" t="inlineStr">
         <is>
-          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
+          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
         </is>
       </c>
       <c r="N131" s="10" t="inlineStr">
         <is>
-          <t>browser unit: setup-import-unit (9)</t>
+          <t>38_setup_import (8)</t>
         </is>
       </c>
       <c r="O131" s="10" t="inlineStr">
@@ -10951,36 +10959,32 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P131" s="10" t="inlineStr">
-        <is>
-          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
-        </is>
-      </c>
+      <c r="P131" s="10" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="10" t="inlineStr">
         <is>
-          <t>SET-011</t>
+          <t>AI-007</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>AI helpers</t>
         </is>
       </c>
       <c r="C132" s="10" t="inlineStr">
         <is>
-          <t>/setup; /dashboard</t>
+          <t>Setup, Rooms</t>
         </is>
       </c>
       <c r="D132" s="10" t="inlineStr">
         <is>
-          <t>A new hotel sees a checklist of what is left to set up: property details, room types, rooms, rates, taxes, payment methods and staff. Each step says what is missing and links to the right screen. The list comes from the hotel's own data, so it is always current.</t>
+          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
         </is>
       </c>
       <c r="E132" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F132" s="10" t="inlineStr">
@@ -10995,37 +10999,33 @@
       </c>
       <c r="H132" s="10" t="inlineStr">
         <is>
-          <t>any setup permission</t>
-        </is>
-      </c>
-      <c r="I132" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>setup.room.manage</t>
+        </is>
+      </c>
+      <c r="I132" s="10" t="inlineStr"/>
       <c r="J132" s="10" t="inlineStr">
         <is>
-          <t>a hotel that is part way through setup</t>
+          <t>a pasted list</t>
         </is>
       </c>
       <c r="K132" s="10" t="inlineStr">
         <is>
-          <t>a manager opens Setup or the Dashboard</t>
+          <t>the assistant drafts it</t>
         </is>
       </c>
       <c r="L132" s="10" t="inlineStr">
         <is>
-          <t>the steps already done are ticked and the next one is linked; once all seven are done the checklist goes away</t>
+          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
         </is>
       </c>
       <c r="M132" s="10" t="inlineStr">
         <is>
-          <t>setup_progress</t>
+          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
         </is>
       </c>
       <c r="N132" s="10" t="inlineStr">
         <is>
-          <t>40_guided_setup (30)</t>
+          <t>browser unit: setup-import-unit (9)</t>
         </is>
       </c>
       <c r="O132" s="10" t="inlineStr">
@@ -11035,39 +11035,39 @@
       </c>
       <c r="P132" s="10" t="inlineStr">
         <is>
-          <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
+          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
         <is>
-          <t>NFR-006</t>
+          <t>SET-011</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
         <is>
-          <t>Non-functional</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C133" s="10" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/setup; /dashboard</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr">
         <is>
-          <t>The last room of a type is sold once, however many desks book at the same moment, and a repeated booking never doubles.</t>
+          <t>A new hotel sees a checklist of what is left to set up: property details, room types, rooms, rates, taxes, payment methods and staff. Each step says what is missing and links to the right screen. The list comes from the hotel's own data, so it is always current.</t>
         </is>
       </c>
       <c r="E133" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F133" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G133" s="10" t="inlineStr">
@@ -11077,37 +11077,37 @@
       </c>
       <c r="H133" s="10" t="inlineStr">
         <is>
+          <t>any setup permission</t>
+        </is>
+      </c>
+      <c r="I133" s="10" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I133" s="10" t="inlineStr">
-        <is>
-          <t>Rule: Safe last-room booking</t>
-        </is>
-      </c>
       <c r="J133" s="10" t="inlineStr">
         <is>
-          <t>one room of a type is left and several desks book it together</t>
+          <t>a hotel that is part way through setup</t>
         </is>
       </c>
       <c r="K133" s="10" t="inlineStr">
         <is>
-          <t>all of them submit at the same moment</t>
+          <t>a manager opens Setup or the Dashboard</t>
         </is>
       </c>
       <c r="L133" s="10" t="inlineStr">
         <is>
-          <t>exactly one booking succeeds, the rest get E_NO_AVAILABILITY, and nothing is oversold</t>
+          <t>the steps already done are ticked and the next one is linked; once all seven are done the checklist goes away</t>
         </is>
       </c>
       <c r="M133" s="10" t="inlineStr">
         <is>
-          <t>create_reservation, assert_available</t>
+          <t>setup_progress</t>
         </is>
       </c>
       <c r="N133" s="10" t="inlineStr">
         <is>
-          <t>concurrency/last_room.sh (6)</t>
+          <t>40_guided_setup (30)</t>
         </is>
       </c>
       <c r="O133" s="10" t="inlineStr">
@@ -11117,29 +11117,29 @@
       </c>
       <c r="P133" s="10" t="inlineStr">
         <is>
-          <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
+          <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
         <is>
-          <t>SET-012</t>
+          <t>NFR-006</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Non-functional</t>
         </is>
       </c>
       <c r="C134" s="10" t="inlineStr">
         <is>
-          <t>/setup/property</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
         <is>
-          <t>A manager sets the longest stay (1 to 365 nights) and how long a tentative booking holds its room (1 to 720 hours) for each property.</t>
+          <t>The last room of a type is sold once, however many desks book at the same moment, and a repeated booking never doubles.</t>
         </is>
       </c>
       <c r="E134" s="10" t="inlineStr">
@@ -11149,7 +11149,7 @@
       </c>
       <c r="F134" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G134" s="10" t="inlineStr">
@@ -11159,33 +11159,37 @@
       </c>
       <c r="H134" s="10" t="inlineStr">
         <is>
-          <t>setup.property.edit</t>
-        </is>
-      </c>
-      <c r="I134" s="10" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I134" s="10" t="inlineStr">
+        <is>
+          <t>Rule: Safe last-room booking</t>
+        </is>
+      </c>
       <c r="J134" s="10" t="inlineStr">
         <is>
-          <t>a property with the default rules (30 nights, 24 hours)</t>
+          <t>one room of a type is left and several desks book it together</t>
         </is>
       </c>
       <c r="K134" s="10" t="inlineStr">
         <is>
-          <t>a manager saves new booking rules</t>
+          <t>all of them submit at the same moment</t>
         </is>
       </c>
       <c r="L134" s="10" t="inlineStr">
         <is>
-          <t>new bookings use them, bad values are refused with E_INVALID, and the change is audited with old and new values</t>
+          <t>exactly one booking succeeds, the rest get E_NO_AVAILABILITY, and nothing is oversold</t>
         </is>
       </c>
       <c r="M134" s="10" t="inlineStr">
         <is>
-          <t>set_booking_rules; Booking rules on Setup, Property</t>
+          <t>create_reservation, assert_available</t>
         </is>
       </c>
       <c r="N134" s="10" t="inlineStr">
         <is>
-          <t>42_booking_rules (9)</t>
+          <t>concurrency/last_room.sh (6)</t>
         </is>
       </c>
       <c r="O134" s="10" t="inlineStr">
@@ -11195,39 +11199,39 @@
       </c>
       <c r="P134" s="10" t="inlineStr">
         <is>
-          <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
+          <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
         <is>
-          <t>FO-014</t>
+          <t>SET-012</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
         <is>
-          <t>Front Office</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C135" s="10" t="inlineStr">
         <is>
-          <t>/downtime</t>
+          <t>/setup/property</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr">
         <is>
-          <t>A printable downtime pack: arrivals due, in-house guests with balance, departures due, ten blank lines for new guests on paper, and a short paper routine. Staff print it when the internet or system is down.</t>
+          <t>A manager sets the longest stay (1 to 365 nights) and how long a tentative booking holds its room (1 to 720 hours) for each property.</t>
         </is>
       </c>
       <c r="E135" s="10" t="inlineStr">
         <is>
-          <t>BR-006</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F135" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G135" s="10" t="inlineStr">
@@ -11237,33 +11241,33 @@
       </c>
       <c r="H135" s="10" t="inlineStr">
         <is>
-          <t>fo.view</t>
+          <t>setup.property.edit</t>
         </is>
       </c>
       <c r="I135" s="10" t="inlineStr"/>
       <c r="J135" s="10" t="inlineStr">
         <is>
-          <t>a hotel with guests in house</t>
+          <t>a property with the default rules (30 nights, 24 hours)</t>
         </is>
       </c>
       <c r="K135" s="10" t="inlineStr">
         <is>
-          <t>a front desk user opens Downtime pack and prints</t>
+          <t>a manager saves new booking rules</t>
         </is>
       </c>
       <c r="L135" s="10" t="inlineStr">
         <is>
-          <t>the lists show room, guest, phone, departure and the folio balance from the database, with blank lines and the paper routine</t>
+          <t>new bookings use them, bad values are refused with E_INVALID, and the change is audited with old and new values</t>
         </is>
       </c>
       <c r="M135" s="10" t="inlineStr">
         <is>
-          <t>src/routes/_authenticated/_app/downtime.tsx</t>
+          <t>set_booking_rules; Booking rules on Setup, Property</t>
         </is>
       </c>
       <c r="N135" s="10" t="inlineStr">
         <is>
-          <t>browser: downtime-pack.spec (1)</t>
+          <t>42_booking_rules (9)</t>
         </is>
       </c>
       <c r="O135" s="10" t="inlineStr">
@@ -11273,87 +11277,165 @@
       </c>
       <c r="P135" s="10" t="inlineStr">
         <is>
-          <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
+          <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
         <is>
+          <t>FO-014</t>
+        </is>
+      </c>
+      <c r="B136" s="10" t="inlineStr">
+        <is>
+          <t>Front Office</t>
+        </is>
+      </c>
+      <c r="C136" s="10" t="inlineStr">
+        <is>
+          <t>/downtime</t>
+        </is>
+      </c>
+      <c r="D136" s="10" t="inlineStr">
+        <is>
+          <t>A printable downtime pack: arrivals due, in-house guests with balance, departures due, ten blank lines for new guests on paper, and a short paper routine. Staff print it when the internet or system is down.</t>
+        </is>
+      </c>
+      <c r="E136" s="10" t="inlineStr">
+        <is>
+          <t>BR-006</t>
+        </is>
+      </c>
+      <c r="F136" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G136" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H136" s="10" t="inlineStr">
+        <is>
+          <t>fo.view</t>
+        </is>
+      </c>
+      <c r="I136" s="10" t="inlineStr"/>
+      <c r="J136" s="10" t="inlineStr">
+        <is>
+          <t>a hotel with guests in house</t>
+        </is>
+      </c>
+      <c r="K136" s="10" t="inlineStr">
+        <is>
+          <t>a front desk user opens Downtime pack and prints</t>
+        </is>
+      </c>
+      <c r="L136" s="10" t="inlineStr">
+        <is>
+          <t>the lists show room, guest, phone, departure and the folio balance from the database, with blank lines and the paper routine</t>
+        </is>
+      </c>
+      <c r="M136" s="10" t="inlineStr">
+        <is>
+          <t>src/routes/_authenticated/_app/downtime.tsx</t>
+        </is>
+      </c>
+      <c r="N136" s="10" t="inlineStr">
+        <is>
+          <t>browser: downtime-pack.spec (1)</t>
+        </is>
+      </c>
+      <c r="O136" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P136" s="10" t="inlineStr">
+        <is>
+          <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="10" t="inlineStr">
+        <is>
           <t>DAY-007</t>
         </is>
       </c>
-      <c r="B136" s="10" t="inlineStr">
+      <c r="B137" s="10" t="inlineStr">
         <is>
           <t>Business Date</t>
         </is>
       </c>
-      <c r="C136" s="10" t="inlineStr">
+      <c r="C137" s="10" t="inlineStr">
         <is>
           <t>Notifications bell</t>
         </is>
       </c>
-      <c r="D136" s="10" t="inlineStr">
+      <c r="D137" s="10" t="inlineStr">
         <is>
           <t>In the last hour before a property rolls its business date, if a cashier shift is still open, users who can run the night audit get one warning that night. The roll does not wait.</t>
         </is>
       </c>
-      <c r="E136" s="10" t="inlineStr">
+      <c r="E137" s="10" t="inlineStr">
         <is>
           <t>BR-016</t>
         </is>
       </c>
-      <c r="F136" s="10" t="inlineStr">
+      <c r="F137" s="10" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="G136" s="10" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H136" s="10" t="inlineStr">
+      <c r="G137" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H137" s="10" t="inlineStr">
         <is>
           <t>fin.nightaudit.run</t>
         </is>
       </c>
-      <c r="I136" s="10" t="inlineStr">
+      <c r="I137" s="10" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="J136" s="10" t="inlineStr">
+      <c r="J137" s="10" t="inlineStr">
         <is>
           <t>a cashier shift is still open</t>
         </is>
       </c>
-      <c r="K136" s="10" t="inlineStr">
+      <c r="K137" s="10" t="inlineStr">
         <is>
           <t>the roll time is less than 60 minutes away</t>
         </is>
       </c>
-      <c r="L136" s="10" t="inlineStr">
+      <c r="L137" s="10" t="inlineStr">
         <is>
           <t>each night audit user gets one rollover_warning notification for that business date; none earlier, none after the roll time, none if no shift is open, none twice</t>
         </is>
       </c>
-      <c r="M136" s="10" t="inlineStr">
+      <c r="M137" s="10" t="inlineStr">
         <is>
           <t>app.warn_before_rollover; cron job rollover-warning</t>
         </is>
       </c>
-      <c r="N136" s="10" t="inlineStr">
+      <c r="N137" s="10" t="inlineStr">
         <is>
           <t>43_rollover_warning (9)</t>
         </is>
       </c>
-      <c r="O136" s="10" t="inlineStr">
+      <c r="O137" s="10" t="inlineStr">
         <is>
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P136" s="10" t="inlineStr">
+      <c r="P137" s="10" t="inlineStr">
         <is>
           <t>Added 8 Oct 2026. Warning only; the hard gate stays in R2 (DAY-005).</t>
         </is>

</xml_diff>

<commit_message>
Add nights, guests, check-in time, day totals and receipt references to invoices (FIN-019)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P137"/>
+  <dimension ref="A1:P138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9494,22 +9494,22 @@
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>GST-007</t>
+          <t>FIN-019</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t>Guests</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C113" s="10" t="inlineStr">
         <is>
-          <t>/guests/$id; check-in; walk-in</t>
+          <t>/invoices/$id</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t>A photo or scan of an ID document is kept in private storage, shrunk and stripped of hidden data in the browser, and opened only through a 60-second link.</t>
+          <t>An invoice shows the check-in time, number of guests, number of nights, a total for each day, and the receipt reference of each charge. Invoices issued earlier stay as issued.</t>
         </is>
       </c>
       <c r="E113" s="10" t="inlineStr">
@@ -9519,7 +9519,7 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G113" s="10" t="inlineStr">
@@ -9529,37 +9529,37 @@
       </c>
       <c r="H113" s="10" t="inlineStr">
         <is>
-          <t>guest.document.file.upload / view / delete</t>
+          <t>fin.invoice.issue</t>
         </is>
       </c>
       <c r="I113" s="10" t="inlineStr">
         <is>
-          <t>SET-009 switch</t>
+          <t>Invoice snapshot is insert-only</t>
         </is>
       </c>
       <c r="J113" s="10" t="inlineStr">
         <is>
-          <t>a hotel that allows ID photos</t>
+          <t>a stay with charges, one with a receipt reference</t>
         </is>
       </c>
       <c r="K113" s="10" t="inlineStr">
         <is>
-          <t>front desk adds an ID photo</t>
+          <t>an invoice is issued</t>
         </is>
       </c>
       <c r="L113" s="10" t="inlineStr">
         <is>
-          <t>it is stored privately and opens only through a short-lived link</t>
+          <t>the invoice shows nights, guests, check-in time, a total per day and the receipt reference, all worked out in the database</t>
         </is>
       </c>
       <c r="M113" s="10" t="inlineStr">
         <is>
-          <t>begin_id_photo_upload, finish_id_photo_upload, open_id_photo</t>
+          <t>issue_invoice</t>
         </is>
       </c>
       <c r="N113" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (30)</t>
+          <t>45_invoice_layout (6)</t>
         </is>
       </c>
       <c r="O113" s="10" t="inlineStr">
@@ -9567,12 +9567,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P113" s="10" t="inlineStr"/>
+      <c r="P113" s="10" t="inlineStr">
+        <is>
+          <t>Day totals and fields are stored in the invoice header when it is issued</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>GST-008</t>
+          <t>GST-007</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
@@ -9582,12 +9586,12 @@
       </c>
       <c r="C114" s="10" t="inlineStr">
         <is>
-          <t>/guests/$id</t>
+          <t>/guests/$id; check-in; walk-in</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t>Every upload, view and deletion of an ID photo is audited with ids only, no personal data.</t>
+          <t>A photo or scan of an ID document is kept in private storage, shrunk and stripped of hidden data in the browser, and opened only through a 60-second link.</t>
         </is>
       </c>
       <c r="E114" s="10" t="inlineStr">
@@ -9607,37 +9611,37 @@
       </c>
       <c r="H114" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>guest.document.file.upload / view / delete</t>
         </is>
       </c>
       <c r="I114" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SET-009 switch</t>
         </is>
       </c>
       <c r="J114" s="10" t="inlineStr">
         <is>
-          <t>an ID photo</t>
+          <t>a hotel that allows ID photos</t>
         </is>
       </c>
       <c r="K114" s="10" t="inlineStr">
         <is>
-          <t>it is uploaded, opened or deleted</t>
+          <t>front desk adds an ID photo</t>
         </is>
       </c>
       <c r="L114" s="10" t="inlineStr">
         <is>
-          <t>an audit row records who and which file, with no personal data</t>
+          <t>it is stored privately and opens only through a short-lived link</t>
         </is>
       </c>
       <c r="M114" s="10" t="inlineStr">
         <is>
-          <t>app.audit_id_photo</t>
+          <t>begin_id_photo_upload, finish_id_photo_upload, open_id_photo</t>
         </is>
       </c>
       <c r="N114" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (9)</t>
+          <t>24_id_photos (30)</t>
         </is>
       </c>
       <c r="O114" s="10" t="inlineStr">
@@ -9650,7 +9654,7 @@
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>GST-009</t>
+          <t>GST-008</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
@@ -9665,7 +9669,7 @@
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t>ID photos are removed from storage when the guest is anonymised or the document is removed, and move with the guest when two profiles are merged.</t>
+          <t>Every upload, view and deletion of an ID photo is audited with ids only, no personal data.</t>
         </is>
       </c>
       <c r="E115" s="10" t="inlineStr">
@@ -9695,27 +9699,27 @@
       </c>
       <c r="J115" s="10" t="inlineStr">
         <is>
-          <t>a guest with ID photos</t>
+          <t>an ID photo</t>
         </is>
       </c>
       <c r="K115" s="10" t="inlineStr">
         <is>
-          <t>the guest is anonymised, the document removed, or the profile merged</t>
+          <t>it is uploaded, opened or deleted</t>
         </is>
       </c>
       <c r="L115" s="10" t="inlineStr">
         <is>
-          <t>the files are removed, or move to the kept profile</t>
+          <t>an audit row records who and which file, with no personal data</t>
         </is>
       </c>
       <c r="M115" s="10" t="inlineStr">
         <is>
-          <t>anonymise_guest, merge_guests, delete_id_photo</t>
+          <t>app.audit_id_photo</t>
         </is>
       </c>
       <c r="N115" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (4)</t>
+          <t>24_id_photos (9)</t>
         </is>
       </c>
       <c r="O115" s="10" t="inlineStr">
@@ -9728,7 +9732,7 @@
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
         <is>
-          <t>GST-010</t>
+          <t>GST-009</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
@@ -9738,12 +9742,12 @@
       </c>
       <c r="C116" s="10" t="inlineStr">
         <is>
-          <t>(daily clean-up)</t>
+          <t>/guests/$id</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t>ID photos are deleted automatically a set number of months (one setting, now 12) after the guest's last check-out, unless the guest has a booking that is not over.</t>
+          <t>ID photos are removed from storage when the guest is anonymised or the document is removed, and move with the guest when two profiles are merged.</t>
         </is>
       </c>
       <c r="E116" s="10" t="inlineStr">
@@ -9768,32 +9772,32 @@
       </c>
       <c r="I116" s="10" t="inlineStr">
         <is>
-          <t>Setting id_photo_keep_months; daily cron</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J116" s="10" t="inlineStr">
         <is>
-          <t>a guest whose last check-out was more than the keep period ago</t>
+          <t>a guest with ID photos</t>
         </is>
       </c>
       <c r="K116" s="10" t="inlineStr">
         <is>
-          <t>the daily clean-up runs</t>
+          <t>the guest is anonymised, the document removed, or the profile merged</t>
         </is>
       </c>
       <c r="L116" s="10" t="inlineStr">
         <is>
-          <t>their ID photos are deleted</t>
+          <t>the files are removed, or move to the kept profile</t>
         </is>
       </c>
       <c r="M116" s="10" t="inlineStr">
         <is>
-          <t>/api/cron/id-photo-cleanup</t>
+          <t>anonymise_guest, merge_guests, delete_id_photo</t>
         </is>
       </c>
       <c r="N116" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (5)</t>
+          <t>24_id_photos (4)</t>
         </is>
       </c>
       <c r="O116" s="10" t="inlineStr">
@@ -9806,22 +9810,22 @@
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>ROOM-005</t>
+          <t>GST-010</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t>Rooms</t>
+          <t>Guests</t>
         </is>
       </c>
       <c r="C117" s="10" t="inlineStr">
         <is>
-          <t>/rooms</t>
+          <t>(daily clean-up)</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t>Rooms are added one at a time or several by number or by name, with a preview; labels are free text up to 30 characters, unique per hotel ignoring case and extra spaces, shown as typed and sorted in natural order.</t>
+          <t>ID photos are deleted automatically a set number of months (one setting, now 12) after the guest's last check-out, unless the guest has a booking that is not over.</t>
         </is>
       </c>
       <c r="E117" s="10" t="inlineStr">
@@ -9841,37 +9845,37 @@
       </c>
       <c r="H117" s="10" t="inlineStr">
         <is>
-          <t>setup.room.edit</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I117" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Setting id_photo_keep_months; daily cron</t>
         </is>
       </c>
       <c r="J117" s="10" t="inlineStr">
         <is>
-          <t>an administrator on the Rooms page</t>
+          <t>a guest whose last check-out was more than the keep period ago</t>
         </is>
       </c>
       <c r="K117" s="10" t="inlineStr">
         <is>
-          <t>they add rooms by number range or by names</t>
+          <t>the daily clean-up runs</t>
         </is>
       </c>
       <c r="L117" s="10" t="inlineStr">
         <is>
-          <t>valid new rooms are created, duplicates skipped and invalid names shown</t>
+          <t>their ID photos are deleted</t>
         </is>
       </c>
       <c r="M117" s="10" t="inlineStr">
         <is>
-          <t>add_rooms_range, add_rooms_named, save_room</t>
+          <t>/api/cron/id-photo-cleanup</t>
         </is>
       </c>
       <c r="N117" s="10" t="inlineStr">
         <is>
-          <t>23_room_labels (46); 26_small_fixes (1); browser: rooms-add</t>
+          <t>24_id_photos (5)</t>
         </is>
       </c>
       <c r="O117" s="10" t="inlineStr">
@@ -9884,22 +9888,22 @@
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
         <is>
-          <t>SET-009</t>
+          <t>ROOM-005</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Rooms</t>
         </is>
       </c>
       <c r="C118" s="10" t="inlineStr">
         <is>
-          <t>/setup/property</t>
+          <t>/rooms</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t>Per hotel: "Allow ID photos" (off by default) and "Require ID photo at check-in" (only when allowed). While Allow is off, uploading and opening ID photos are refused.</t>
+          <t>Rooms are added one at a time or several by number or by name, with a preview; labels are free text up to 30 characters, unique per hotel ignoring case and extra spaces, shown as typed and sorted in natural order.</t>
         </is>
       </c>
       <c r="E118" s="10" t="inlineStr">
@@ -9919,7 +9923,7 @@
       </c>
       <c r="H118" s="10" t="inlineStr">
         <is>
-          <t>setup.property.edit</t>
+          <t>setup.room.edit</t>
         </is>
       </c>
       <c r="I118" s="10" t="inlineStr">
@@ -9929,27 +9933,27 @@
       </c>
       <c r="J118" s="10" t="inlineStr">
         <is>
-          <t>a hotel with ID photos off</t>
+          <t>an administrator on the Rooms page</t>
         </is>
       </c>
       <c r="K118" s="10" t="inlineStr">
         <is>
-          <t>staff try to add or open an ID photo</t>
+          <t>they add rooms by number range or by names</t>
         </is>
       </c>
       <c r="L118" s="10" t="inlineStr">
         <is>
-          <t>it is refused; when Require is on, check-in waits for an ID photo</t>
+          <t>valid new rooms are created, duplicates skipped and invalid names shown</t>
         </is>
       </c>
       <c r="M118" s="10" t="inlineStr">
         <is>
-          <t>set_id_photo_settings</t>
+          <t>add_rooms_range, add_rooms_named, save_room</t>
         </is>
       </c>
       <c r="N118" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (10)</t>
+          <t>23_room_labels (46); 26_small_fixes (1); browser: rooms-add</t>
         </is>
       </c>
       <c r="O118" s="10" t="inlineStr">
@@ -9962,32 +9966,32 @@
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>GRP-001</t>
+          <t>SET-009</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
         <is>
-          <t>Platform &amp; Tenancy</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C119" s="10" t="inlineStr">
         <is>
-          <t>All branches</t>
+          <t>/setup/property</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t>A built-in Group Manager role and the permission rpt.group.view exist; only System Administrator, General Manager and Group Manager hold the permission.</t>
+          <t>Per hotel: "Allow ID photos" (off by default) and "Require ID photo at check-in" (only when allowed). While Allow is off, uploading and opening ID photos are refused.</t>
         </is>
       </c>
       <c r="E119" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G119" s="10" t="inlineStr">
@@ -9997,33 +10001,37 @@
       </c>
       <c r="H119" s="10" t="inlineStr">
         <is>
-          <t>rpt.group.view</t>
-        </is>
-      </c>
-      <c r="I119" s="10" t="inlineStr"/>
+          <t>setup.property.edit</t>
+        </is>
+      </c>
+      <c r="I119" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="J119" s="10" t="inlineStr">
         <is>
-          <t>a hotel group with several branches</t>
+          <t>a hotel with ID photos off</t>
         </is>
       </c>
       <c r="K119" s="10" t="inlineStr">
         <is>
-          <t>an owner wants a view-only manager for the whole group</t>
+          <t>staff try to add or open an ID photo</t>
         </is>
       </c>
       <c r="L119" s="10" t="inlineStr">
         <is>
-          <t>they assign the Group Manager role branch by branch, and that person can look but not post or change anything</t>
+          <t>it is refused; when Require is on, check-in waits for an ID photo</t>
         </is>
       </c>
       <c r="M119" s="10" t="inlineStr">
         <is>
-          <t>20261013120000_group_view.sql</t>
+          <t>set_id_photo_settings</t>
         </is>
       </c>
       <c r="N119" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (5)</t>
+          <t>24_id_photos (10)</t>
         </is>
       </c>
       <c r="O119" s="10" t="inlineStr">
@@ -10031,16 +10039,12 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P119" s="10" t="inlineStr">
-        <is>
-          <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
-        </is>
-      </c>
+      <c r="P119" s="10" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
         <is>
-          <t>GRP-002</t>
+          <t>GRP-001</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
@@ -10055,7 +10059,7 @@
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t>One call shows every branch the person may see: occupancy, in house, arrivals and departures to come, approvals, repairs and last night revenue, with group totals. Revenue is totalled per currency.</t>
+          <t>A built-in Group Manager role and the permission rpt.group.view exist; only System Administrator, General Manager and Group Manager hold the permission.</t>
         </is>
       </c>
       <c r="E120" s="10" t="inlineStr">
@@ -10081,27 +10085,27 @@
       <c r="I120" s="10" t="inlineStr"/>
       <c r="J120" s="10" t="inlineStr">
         <is>
-          <t>a group with a Lagos and an Abuja branch</t>
+          <t>a hotel group with several branches</t>
         </is>
       </c>
       <c r="K120" s="10" t="inlineStr">
         <is>
-          <t>a group manager opens All branches</t>
+          <t>an owner wants a view-only manager for the whole group</t>
         </is>
       </c>
       <c r="L120" s="10" t="inlineStr">
         <is>
-          <t>they see both branches with figures from the database, never another hotel group, and staff without the permission are refused</t>
+          <t>they assign the Group Manager role branch by branch, and that person can look but not post or change anything</t>
         </is>
       </c>
       <c r="M120" s="10" t="inlineStr">
         <is>
-          <t>group_overview; /group screen</t>
+          <t>20261013120000_group_view.sql</t>
         </is>
       </c>
       <c r="N120" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (10)</t>
+          <t>35_group_view (5)</t>
         </is>
       </c>
       <c r="O120" s="10" t="inlineStr">
@@ -10111,14 +10115,14 @@
       </c>
       <c r="P120" s="10" t="inlineStr">
         <is>
-          <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
+          <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>GRP-003</t>
+          <t>GRP-002</t>
         </is>
       </c>
       <c r="B121" s="10" t="inlineStr">
@@ -10133,7 +10137,7 @@
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t>A Group Manager sees only the branches they are assigned to, and cannot post charges or check guests in.</t>
+          <t>One call shows every branch the person may see: occupancy, in house, arrivals and departures to come, approvals, repairs and last night revenue, with group totals. Revenue is totalled per currency.</t>
         </is>
       </c>
       <c r="E121" s="10" t="inlineStr">
@@ -10159,27 +10163,27 @@
       <c r="I121" s="10" t="inlineStr"/>
       <c r="J121" s="10" t="inlineStr">
         <is>
-          <t>a Group Manager assigned to one branch</t>
+          <t>a group with a Lagos and an Abuja branch</t>
         </is>
       </c>
       <c r="K121" s="10" t="inlineStr">
         <is>
-          <t>a second branch is assigned</t>
+          <t>a group manager opens All branches</t>
         </is>
       </c>
       <c r="L121" s="10" t="inlineStr">
         <is>
-          <t>the second branch appears; the role never gets write permissions</t>
+          <t>they see both branches with figures from the database, never another hotel group, and staff without the permission are refused</t>
         </is>
       </c>
       <c r="M121" s="10" t="inlineStr">
         <is>
-          <t>assign_role (existing); group_overview</t>
+          <t>group_overview; /group screen</t>
         </is>
       </c>
       <c r="N121" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (3)</t>
+          <t>35_group_view (10)</t>
         </is>
       </c>
       <c r="O121" s="10" t="inlineStr">
@@ -10189,14 +10193,14 @@
       </c>
       <c r="P121" s="10" t="inlineStr">
         <is>
-          <t>Access is per branch, using the existing role assignment screen.</t>
+          <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="10" t="inlineStr">
         <is>
-          <t>GRP-004</t>
+          <t>GRP-003</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
@@ -10206,12 +10210,12 @@
       </c>
       <c r="C122" s="10" t="inlineStr">
         <is>
-          <t>All branches (Copy setup)</t>
+          <t>All branches</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t>A new branch can copy room types, rate plans and prices from an existing branch, once, into an empty branch.</t>
+          <t>A Group Manager sees only the branches they are assigned to, and cannot post charges or check guests in.</t>
         </is>
       </c>
       <c r="E122" s="10" t="inlineStr">
@@ -10231,33 +10235,33 @@
       </c>
       <c r="H122" s="10" t="inlineStr">
         <is>
-          <t>setup.room.manage, setup.rate.manage</t>
+          <t>rpt.group.view</t>
         </is>
       </c>
       <c r="I122" s="10" t="inlineStr"/>
       <c r="J122" s="10" t="inlineStr">
         <is>
-          <t>a new empty branch</t>
+          <t>a Group Manager assigned to one branch</t>
         </is>
       </c>
       <c r="K122" s="10" t="inlineStr">
         <is>
-          <t>the owner copies setup from the first branch</t>
+          <t>a second branch is assigned</t>
         </is>
       </c>
       <c r="L122" s="10" t="inlineStr">
         <is>
-          <t>room types, rate plans and prices appear on the new branch and point at its own room types; rooms are not copied; a second copy is refused; the copy is audited</t>
+          <t>the second branch appears; the role never gets write permissions</t>
         </is>
       </c>
       <c r="M122" s="10" t="inlineStr">
         <is>
-          <t>copy_property_setup</t>
+          <t>assign_role (existing); group_overview</t>
         </is>
       </c>
       <c r="N122" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (13)</t>
+          <t>35_group_view (3)</t>
         </is>
       </c>
       <c r="O122" s="10" t="inlineStr">
@@ -10267,29 +10271,29 @@
       </c>
       <c r="P122" s="10" t="inlineStr">
         <is>
-          <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
+          <t>Access is per branch, using the existing role assignment screen.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>RPT-005</t>
+          <t>GRP-004</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Platform &amp; Tenancy</t>
         </is>
       </c>
       <c r="C123" s="10" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>All branches (Copy setup)</t>
         </is>
       </c>
       <c r="D123" s="10" t="inlineStr">
         <is>
-          <t>Revenue by booking source: bookings, cancellations, no-shows, room nights, room revenue and average rate for each source in a date range.</t>
+          <t>A new branch can copy room types, rate plans and prices from an existing branch, once, into an empty branch.</t>
         </is>
       </c>
       <c r="E123" s="10" t="inlineStr">
@@ -10309,33 +10313,33 @@
       </c>
       <c r="H123" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view</t>
+          <t>setup.room.manage, setup.rate.manage</t>
         </is>
       </c>
       <c r="I123" s="10" t="inlineStr"/>
       <c r="J123" s="10" t="inlineStr">
         <is>
-          <t>bookings from direct, phone and company sources</t>
+          <t>a new empty branch</t>
         </is>
       </c>
       <c r="K123" s="10" t="inlineStr">
         <is>
-          <t>the accountant picks a date range</t>
+          <t>the owner copies setup from the first branch</t>
         </is>
       </c>
       <c r="L123" s="10" t="inlineStr">
         <is>
-          <t>each source shows its own counts and room revenue (room charges only, before tax); cancelled bookings add no nights</t>
+          <t>room types, rate plans and prices appear on the new branch and point at its own room types; rooms are not copied; a second copy is refused; the copy is audited</t>
         </is>
       </c>
       <c r="M123" s="10" t="inlineStr">
         <is>
-          <t>20261013130000_source_ageing_reports.sql: report_revenue_by_source; Reports, By booking source tab</t>
+          <t>copy_property_setup</t>
         </is>
       </c>
       <c r="N123" s="10" t="inlineStr">
         <is>
-          <t>36_source_ageing (13)</t>
+          <t>35_group_view (13)</t>
         </is>
       </c>
       <c r="O123" s="10" t="inlineStr">
@@ -10345,14 +10349,14 @@
       </c>
       <c r="P123" s="10" t="inlineStr">
         <is>
-          <t>Bookings counted by arrival date; revenue by posting date.</t>
+          <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="10" t="inlineStr">
         <is>
-          <t>RPT-006</t>
+          <t>RPT-005</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
@@ -10367,7 +10371,7 @@
       </c>
       <c r="D124" s="10" t="inlineStr">
         <is>
-          <t>Ageing of unpaid balances by booking source: current, 1 to 7, 8 to 30, 31 to 60 and over 60 days since the due departure, plus credit held.</t>
+          <t>Revenue by booking source: bookings, cancellations, no-shows, room nights, room revenue and average rate for each source in a date range.</t>
         </is>
       </c>
       <c r="E124" s="10" t="inlineStr">
@@ -10393,27 +10397,27 @@
       <c r="I124" s="10" t="inlineStr"/>
       <c r="J124" s="10" t="inlineStr">
         <is>
-          <t>guests and companies who left owing money</t>
+          <t>bookings from direct, phone and company sources</t>
         </is>
       </c>
       <c r="K124" s="10" t="inlineStr">
         <is>
-          <t>the accountant opens the Ageing tab</t>
+          <t>the accountant picks a date range</t>
         </is>
       </c>
       <c r="L124" s="10" t="inlineStr">
         <is>
-          <t>each source shows what is owed in each age column; paid bills drop out; overpayments show as credit held; the total matches Outstanding balances</t>
+          <t>each source shows its own counts and room revenue (room charges only, before tax); cancelled bookings add no nights</t>
         </is>
       </c>
       <c r="M124" s="10" t="inlineStr">
         <is>
-          <t>report_balance_ageing; Reports, Ageing tab</t>
+          <t>20261013130000_source_ageing_reports.sql: report_revenue_by_source; Reports, By booking source tab</t>
         </is>
       </c>
       <c r="N124" s="10" t="inlineStr">
         <is>
-          <t>36_source_ageing (11)</t>
+          <t>36_source_ageing (13)</t>
         </is>
       </c>
       <c r="O124" s="10" t="inlineStr">
@@ -10423,29 +10427,29 @@
       </c>
       <c r="P124" s="10" t="inlineStr">
         <is>
-          <t>Guests still staying count as current.</t>
+          <t>Bookings counted by arrival date; revenue by posting date.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>RPT-006</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
         <is>
-          <t>AI helpers</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C125" s="10" t="inlineStr">
         <is>
-          <t>Dashboard, Admin</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
+          <t>Ageing of unpaid balances by booking source: current, 1 to 7, 8 to 30, 31 to 60 and over 60 days since the due departure, plus credit held.</t>
         </is>
       </c>
       <c r="E125" s="10" t="inlineStr">
@@ -10465,33 +10469,33 @@
       </c>
       <c r="H125" s="10" t="inlineStr">
         <is>
-          <t>adm.ai.manage</t>
+          <t>rpt.finance.view</t>
         </is>
       </c>
       <c r="I125" s="10" t="inlineStr"/>
       <c r="J125" s="10" t="inlineStr">
         <is>
-          <t>a new hotel</t>
+          <t>guests and companies who left owing money</t>
         </is>
       </c>
       <c r="K125" s="10" t="inlineStr">
         <is>
-          <t>a manager opens Admin, AI helpers</t>
+          <t>the accountant opens the Ageing tab</t>
         </is>
       </c>
       <c r="L125" s="10" t="inlineStr">
         <is>
-          <t>nothing runs until they switch it on and the change is in the audit log</t>
+          <t>each source shows what is owed in each age column; paid bills drop out; overpayments show as credit held; the total matches Outstanding balances</t>
         </is>
       </c>
       <c r="M125" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
+          <t>report_balance_ageing; Reports, Ageing tab</t>
         </is>
       </c>
       <c r="N125" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (11)</t>
+          <t>36_source_ageing (11)</t>
         </is>
       </c>
       <c r="O125" s="10" t="inlineStr">
@@ -10501,14 +10505,14 @@
       </c>
       <c r="P125" s="10" t="inlineStr">
         <is>
-          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
+          <t>Guests still staying count as current.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="10" t="inlineStr">
         <is>
-          <t>AI-002</t>
+          <t>AI-001</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
@@ -10523,7 +10527,7 @@
       </c>
       <c r="D126" s="10" t="inlineStr">
         <is>
-          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
+          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
         </is>
       </c>
       <c r="E126" s="10" t="inlineStr">
@@ -10543,28 +10547,28 @@
       </c>
       <c r="H126" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view, rpt.operations.view</t>
+          <t>adm.ai.manage</t>
         </is>
       </c>
       <c r="I126" s="10" t="inlineStr"/>
       <c r="J126" s="10" t="inlineStr">
         <is>
-          <t>a hotel with guests, approvals and overdue bills</t>
+          <t>a new hotel</t>
         </is>
       </c>
       <c r="K126" s="10" t="inlineStr">
         <is>
-          <t>a brief is started</t>
+          <t>a manager opens Admin, AI helpers</t>
         </is>
       </c>
       <c r="L126" s="10" t="inlineStr">
         <is>
-          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
+          <t>nothing runs until they switch it on and the change is in the audit log</t>
         </is>
       </c>
       <c r="M126" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
+          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
         </is>
       </c>
       <c r="N126" s="10" t="inlineStr">
@@ -10579,14 +10583,14 @@
       </c>
       <c r="P126" s="10" t="inlineStr">
         <is>
-          <t>Overdue means unpaid more than 30 days after departure.</t>
+          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
         <is>
-          <t>AI-003</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
@@ -10601,7 +10605,7 @@
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
+          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
         </is>
       </c>
       <c r="E127" s="10" t="inlineStr">
@@ -10621,33 +10625,33 @@
       </c>
       <c r="H127" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view</t>
+          <t>rpt.finance.view, rpt.operations.view</t>
         </is>
       </c>
       <c r="I127" s="10" t="inlineStr"/>
       <c r="J127" s="10" t="inlineStr">
         <is>
-          <t>a limit of 2</t>
+          <t>a hotel with guests, approvals and overdue bills</t>
         </is>
       </c>
       <c r="K127" s="10" t="inlineStr">
         <is>
-          <t>a third brief is requested</t>
+          <t>a brief is started</t>
         </is>
       </c>
       <c r="L127" s="10" t="inlineStr">
         <is>
-          <t>it is refused until a failed call frees a slot or the month turns</t>
+          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
         </is>
       </c>
       <c r="M127" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
+          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
         </is>
       </c>
       <c r="N127" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (5)</t>
+          <t>37_ai_brief (11)</t>
         </is>
       </c>
       <c r="O127" s="10" t="inlineStr">
@@ -10655,12 +10659,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P127" s="10" t="inlineStr"/>
+      <c r="P127" s="10" t="inlineStr">
+        <is>
+          <t>Overdue means unpaid more than 30 days after departure.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
         <is>
-          <t>AI-004</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
@@ -10675,7 +10683,7 @@
       </c>
       <c r="D128" s="10" t="inlineStr">
         <is>
-          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
+          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
         </is>
       </c>
       <c r="E128" s="10" t="inlineStr">
@@ -10695,33 +10703,33 @@
       </c>
       <c r="H128" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view, rpt.operations.view</t>
+          <t>rpt.finance.view</t>
         </is>
       </c>
       <c r="I128" s="10" t="inlineStr"/>
       <c r="J128" s="10" t="inlineStr">
         <is>
-          <t>front desk, housekeeping, another hotel</t>
+          <t>a limit of 2</t>
         </is>
       </c>
       <c r="K128" s="10" t="inlineStr">
         <is>
-          <t>they ask for the brief or touch the tables</t>
+          <t>a third brief is requested</t>
         </is>
       </c>
       <c r="L128" s="10" t="inlineStr">
         <is>
-          <t>they are refused</t>
+          <t>it is refused until a failed call frees a slot or the month turns</t>
         </is>
       </c>
       <c r="M128" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql</t>
+          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
         </is>
       </c>
       <c r="N128" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (7)</t>
+          <t>37_ai_brief (5)</t>
         </is>
       </c>
       <c r="O128" s="10" t="inlineStr">
@@ -10734,7 +10742,7 @@
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
         <is>
-          <t>AI-005</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
@@ -10749,7 +10757,7 @@
       </c>
       <c r="D129" s="10" t="inlineStr">
         <is>
-          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
+          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
         </is>
       </c>
       <c r="E129" s="10" t="inlineStr">
@@ -10769,33 +10777,33 @@
       </c>
       <c r="H129" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>rpt.finance.view, rpt.operations.view</t>
         </is>
       </c>
       <c r="I129" s="10" t="inlineStr"/>
       <c r="J129" s="10" t="inlineStr">
         <is>
-          <t>a draft that rounds or invents a figure</t>
+          <t>front desk, housekeeping, another hotel</t>
         </is>
       </c>
       <c r="K129" s="10" t="inlineStr">
         <is>
-          <t>the brief is written</t>
+          <t>they ask for the brief or touch the tables</t>
         </is>
       </c>
       <c r="L129" s="10" t="inlineStr">
         <is>
-          <t>the plain database lines are shown instead, with a note</t>
+          <t>they are refused</t>
         </is>
       </c>
       <c r="M129" s="10" t="inlineStr">
         <is>
-          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
+          <t>20261013140000_ai_morning_brief.sql</t>
         </is>
       </c>
       <c r="N129" s="10" t="inlineStr">
         <is>
-          <t>browser unit: ai-brief-unit (8)</t>
+          <t>37_ai_brief (7)</t>
         </is>
       </c>
       <c r="O129" s="10" t="inlineStr">
@@ -10803,31 +10811,27 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P129" s="10" t="inlineStr">
-        <is>
-          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
-        </is>
-      </c>
+      <c r="P129" s="10" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
         <is>
-          <t>SET-010</t>
+          <t>AI-005</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>AI helpers</t>
         </is>
       </c>
       <c r="C130" s="10" t="inlineStr">
         <is>
-          <t>Setup, Rooms</t>
+          <t>Dashboard, Admin</t>
         </is>
       </c>
       <c r="D130" s="10" t="inlineStr">
         <is>
-          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
+          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
         </is>
       </c>
       <c r="E130" s="10" t="inlineStr">
@@ -10847,33 +10851,33 @@
       </c>
       <c r="H130" s="10" t="inlineStr">
         <is>
-          <t>setup.room.manage</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I130" s="10" t="inlineStr"/>
       <c r="J130" s="10" t="inlineStr">
         <is>
-          <t>a list of room types and rooms</t>
+          <t>a draft that rounds or invents a figure</t>
         </is>
       </c>
       <c r="K130" s="10" t="inlineStr">
         <is>
-          <t>the manager previews and then applies it</t>
+          <t>the brief is written</t>
         </is>
       </c>
       <c r="L130" s="10" t="inlineStr">
         <is>
-          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
+          <t>the plain database lines are shown instead, with a note</t>
         </is>
       </c>
       <c r="M130" s="10" t="inlineStr">
         <is>
-          <t>20261013150000_setup_import.sql: apply_setup_import</t>
+          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
         </is>
       </c>
       <c r="N130" s="10" t="inlineStr">
         <is>
-          <t>38_setup_import (29)</t>
+          <t>browser unit: ai-brief-unit (8)</t>
         </is>
       </c>
       <c r="O130" s="10" t="inlineStr">
@@ -10883,19 +10887,19 @@
       </c>
       <c r="P130" s="10" t="inlineStr">
         <is>
-          <t>The AI only drafts the list. This function is the check.</t>
+          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
         <is>
-          <t>AI-006</t>
+          <t>SET-010</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
         <is>
-          <t>AI helpers</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C131" s="10" t="inlineStr">
@@ -10905,7 +10909,7 @@
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
+          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
         </is>
       </c>
       <c r="E131" s="10" t="inlineStr">
@@ -10931,27 +10935,27 @@
       <c r="I131" s="10" t="inlineStr"/>
       <c r="J131" s="10" t="inlineStr">
         <is>
-          <t>AI switched on with a limit of 1</t>
+          <t>a list of room types and rooms</t>
         </is>
       </c>
       <c r="K131" s="10" t="inlineStr">
         <is>
-          <t>an import draft is started twice</t>
+          <t>the manager previews and then applies it</t>
         </is>
       </c>
       <c r="L131" s="10" t="inlineStr">
         <is>
-          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
+          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
         </is>
       </c>
       <c r="M131" s="10" t="inlineStr">
         <is>
-          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
+          <t>20261013150000_setup_import.sql: apply_setup_import</t>
         </is>
       </c>
       <c r="N131" s="10" t="inlineStr">
         <is>
-          <t>38_setup_import (8)</t>
+          <t>38_setup_import (29)</t>
         </is>
       </c>
       <c r="O131" s="10" t="inlineStr">
@@ -10959,12 +10963,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P131" s="10" t="inlineStr"/>
+      <c r="P131" s="10" t="inlineStr">
+        <is>
+          <t>The AI only drafts the list. This function is the check.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="10" t="inlineStr">
         <is>
-          <t>AI-007</t>
+          <t>AI-006</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
@@ -10979,7 +10987,7 @@
       </c>
       <c r="D132" s="10" t="inlineStr">
         <is>
-          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
+          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
         </is>
       </c>
       <c r="E132" s="10" t="inlineStr">
@@ -11005,27 +11013,27 @@
       <c r="I132" s="10" t="inlineStr"/>
       <c r="J132" s="10" t="inlineStr">
         <is>
-          <t>a pasted list</t>
+          <t>AI switched on with a limit of 1</t>
         </is>
       </c>
       <c r="K132" s="10" t="inlineStr">
         <is>
-          <t>the assistant drafts it</t>
+          <t>an import draft is started twice</t>
         </is>
       </c>
       <c r="L132" s="10" t="inlineStr">
         <is>
-          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
+          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
         </is>
       </c>
       <c r="M132" s="10" t="inlineStr">
         <is>
-          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
+          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
         </is>
       </c>
       <c r="N132" s="10" t="inlineStr">
         <is>
-          <t>browser unit: setup-import-unit (9)</t>
+          <t>38_setup_import (8)</t>
         </is>
       </c>
       <c r="O132" s="10" t="inlineStr">
@@ -11033,36 +11041,32 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P132" s="10" t="inlineStr">
-        <is>
-          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
-        </is>
-      </c>
+      <c r="P132" s="10" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
         <is>
-          <t>SET-011</t>
+          <t>AI-007</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>AI helpers</t>
         </is>
       </c>
       <c r="C133" s="10" t="inlineStr">
         <is>
-          <t>/setup; /dashboard</t>
+          <t>Setup, Rooms</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr">
         <is>
-          <t>A new hotel sees a checklist of what is left to set up: property details, room types, rooms, rates, taxes, payment methods and staff. Each step says what is missing and links to the right screen. The list comes from the hotel's own data, so it is always current.</t>
+          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
         </is>
       </c>
       <c r="E133" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F133" s="10" t="inlineStr">
@@ -11077,37 +11081,33 @@
       </c>
       <c r="H133" s="10" t="inlineStr">
         <is>
-          <t>any setup permission</t>
-        </is>
-      </c>
-      <c r="I133" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>setup.room.manage</t>
+        </is>
+      </c>
+      <c r="I133" s="10" t="inlineStr"/>
       <c r="J133" s="10" t="inlineStr">
         <is>
-          <t>a hotel that is part way through setup</t>
+          <t>a pasted list</t>
         </is>
       </c>
       <c r="K133" s="10" t="inlineStr">
         <is>
-          <t>a manager opens Setup or the Dashboard</t>
+          <t>the assistant drafts it</t>
         </is>
       </c>
       <c r="L133" s="10" t="inlineStr">
         <is>
-          <t>the steps already done are ticked and the next one is linked; once all seven are done the checklist goes away</t>
+          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
         </is>
       </c>
       <c r="M133" s="10" t="inlineStr">
         <is>
-          <t>setup_progress</t>
+          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
         </is>
       </c>
       <c r="N133" s="10" t="inlineStr">
         <is>
-          <t>40_guided_setup (30)</t>
+          <t>browser unit: setup-import-unit (9)</t>
         </is>
       </c>
       <c r="O133" s="10" t="inlineStr">
@@ -11117,39 +11117,39 @@
       </c>
       <c r="P133" s="10" t="inlineStr">
         <is>
-          <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
+          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
         <is>
-          <t>NFR-006</t>
+          <t>SET-011</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
         <is>
-          <t>Non-functional</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C134" s="10" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/setup; /dashboard</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
         <is>
-          <t>The last room of a type is sold once, however many desks book at the same moment, and a repeated booking never doubles.</t>
+          <t>A new hotel sees a checklist of what is left to set up: property details, room types, rooms, rates, taxes, payment methods and staff. Each step says what is missing and links to the right screen. The list comes from the hotel's own data, so it is always current.</t>
         </is>
       </c>
       <c r="E134" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F134" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G134" s="10" t="inlineStr">
@@ -11159,37 +11159,37 @@
       </c>
       <c r="H134" s="10" t="inlineStr">
         <is>
+          <t>any setup permission</t>
+        </is>
+      </c>
+      <c r="I134" s="10" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I134" s="10" t="inlineStr">
-        <is>
-          <t>Rule: Safe last-room booking</t>
-        </is>
-      </c>
       <c r="J134" s="10" t="inlineStr">
         <is>
-          <t>one room of a type is left and several desks book it together</t>
+          <t>a hotel that is part way through setup</t>
         </is>
       </c>
       <c r="K134" s="10" t="inlineStr">
         <is>
-          <t>all of them submit at the same moment</t>
+          <t>a manager opens Setup or the Dashboard</t>
         </is>
       </c>
       <c r="L134" s="10" t="inlineStr">
         <is>
-          <t>exactly one booking succeeds, the rest get E_NO_AVAILABILITY, and nothing is oversold</t>
+          <t>the steps already done are ticked and the next one is linked; once all seven are done the checklist goes away</t>
         </is>
       </c>
       <c r="M134" s="10" t="inlineStr">
         <is>
-          <t>create_reservation, assert_available</t>
+          <t>setup_progress</t>
         </is>
       </c>
       <c r="N134" s="10" t="inlineStr">
         <is>
-          <t>concurrency/last_room.sh (6)</t>
+          <t>40_guided_setup (30)</t>
         </is>
       </c>
       <c r="O134" s="10" t="inlineStr">
@@ -11199,29 +11199,29 @@
       </c>
       <c r="P134" s="10" t="inlineStr">
         <is>
-          <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
+          <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
         <is>
-          <t>SET-012</t>
+          <t>NFR-006</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Non-functional</t>
         </is>
       </c>
       <c r="C135" s="10" t="inlineStr">
         <is>
-          <t>/setup/property</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr">
         <is>
-          <t>A manager sets the longest stay (1 to 365 nights) and how long a tentative booking holds its room (1 to 720 hours) for each property.</t>
+          <t>The last room of a type is sold once, however many desks book at the same moment, and a repeated booking never doubles.</t>
         </is>
       </c>
       <c r="E135" s="10" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="F135" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G135" s="10" t="inlineStr">
@@ -11241,33 +11241,37 @@
       </c>
       <c r="H135" s="10" t="inlineStr">
         <is>
-          <t>setup.property.edit</t>
-        </is>
-      </c>
-      <c r="I135" s="10" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I135" s="10" t="inlineStr">
+        <is>
+          <t>Rule: Safe last-room booking</t>
+        </is>
+      </c>
       <c r="J135" s="10" t="inlineStr">
         <is>
-          <t>a property with the default rules (30 nights, 24 hours)</t>
+          <t>one room of a type is left and several desks book it together</t>
         </is>
       </c>
       <c r="K135" s="10" t="inlineStr">
         <is>
-          <t>a manager saves new booking rules</t>
+          <t>all of them submit at the same moment</t>
         </is>
       </c>
       <c r="L135" s="10" t="inlineStr">
         <is>
-          <t>new bookings use them, bad values are refused with E_INVALID, and the change is audited with old and new values</t>
+          <t>exactly one booking succeeds, the rest get E_NO_AVAILABILITY, and nothing is oversold</t>
         </is>
       </c>
       <c r="M135" s="10" t="inlineStr">
         <is>
-          <t>set_booking_rules; Booking rules on Setup, Property</t>
+          <t>create_reservation, assert_available</t>
         </is>
       </c>
       <c r="N135" s="10" t="inlineStr">
         <is>
-          <t>42_booking_rules (9)</t>
+          <t>concurrency/last_room.sh (6)</t>
         </is>
       </c>
       <c r="O135" s="10" t="inlineStr">
@@ -11277,39 +11281,39 @@
       </c>
       <c r="P135" s="10" t="inlineStr">
         <is>
-          <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
+          <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
         <is>
-          <t>FO-014</t>
+          <t>SET-012</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
         <is>
-          <t>Front Office</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C136" s="10" t="inlineStr">
         <is>
-          <t>/downtime</t>
+          <t>/setup/property</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr">
         <is>
-          <t>A printable downtime pack: arrivals due, in-house guests with balance, departures due, ten blank lines for new guests on paper, and a short paper routine. Staff print it when the internet or system is down.</t>
+          <t>A manager sets the longest stay (1 to 365 nights) and how long a tentative booking holds its room (1 to 720 hours) for each property.</t>
         </is>
       </c>
       <c r="E136" s="10" t="inlineStr">
         <is>
-          <t>BR-006</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F136" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G136" s="10" t="inlineStr">
@@ -11319,33 +11323,33 @@
       </c>
       <c r="H136" s="10" t="inlineStr">
         <is>
-          <t>fo.view</t>
+          <t>setup.property.edit</t>
         </is>
       </c>
       <c r="I136" s="10" t="inlineStr"/>
       <c r="J136" s="10" t="inlineStr">
         <is>
-          <t>a hotel with guests in house</t>
+          <t>a property with the default rules (30 nights, 24 hours)</t>
         </is>
       </c>
       <c r="K136" s="10" t="inlineStr">
         <is>
-          <t>a front desk user opens Downtime pack and prints</t>
+          <t>a manager saves new booking rules</t>
         </is>
       </c>
       <c r="L136" s="10" t="inlineStr">
         <is>
-          <t>the lists show room, guest, phone, departure and the folio balance from the database, with blank lines and the paper routine</t>
+          <t>new bookings use them, bad values are refused with E_INVALID, and the change is audited with old and new values</t>
         </is>
       </c>
       <c r="M136" s="10" t="inlineStr">
         <is>
-          <t>src/routes/_authenticated/_app/downtime.tsx</t>
+          <t>set_booking_rules; Booking rules on Setup, Property</t>
         </is>
       </c>
       <c r="N136" s="10" t="inlineStr">
         <is>
-          <t>browser: downtime-pack.spec (1)</t>
+          <t>42_booking_rules (9)</t>
         </is>
       </c>
       <c r="O136" s="10" t="inlineStr">
@@ -11355,87 +11359,165 @@
       </c>
       <c r="P136" s="10" t="inlineStr">
         <is>
-          <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
+          <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
         <is>
+          <t>FO-014</t>
+        </is>
+      </c>
+      <c r="B137" s="10" t="inlineStr">
+        <is>
+          <t>Front Office</t>
+        </is>
+      </c>
+      <c r="C137" s="10" t="inlineStr">
+        <is>
+          <t>/downtime</t>
+        </is>
+      </c>
+      <c r="D137" s="10" t="inlineStr">
+        <is>
+          <t>A printable downtime pack: arrivals due, in-house guests with balance, departures due, ten blank lines for new guests on paper, and a short paper routine. Staff print it when the internet or system is down.</t>
+        </is>
+      </c>
+      <c r="E137" s="10" t="inlineStr">
+        <is>
+          <t>BR-006</t>
+        </is>
+      </c>
+      <c r="F137" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G137" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H137" s="10" t="inlineStr">
+        <is>
+          <t>fo.view</t>
+        </is>
+      </c>
+      <c r="I137" s="10" t="inlineStr"/>
+      <c r="J137" s="10" t="inlineStr">
+        <is>
+          <t>a hotel with guests in house</t>
+        </is>
+      </c>
+      <c r="K137" s="10" t="inlineStr">
+        <is>
+          <t>a front desk user opens Downtime pack and prints</t>
+        </is>
+      </c>
+      <c r="L137" s="10" t="inlineStr">
+        <is>
+          <t>the lists show room, guest, phone, departure and the folio balance from the database, with blank lines and the paper routine</t>
+        </is>
+      </c>
+      <c r="M137" s="10" t="inlineStr">
+        <is>
+          <t>src/routes/_authenticated/_app/downtime.tsx</t>
+        </is>
+      </c>
+      <c r="N137" s="10" t="inlineStr">
+        <is>
+          <t>browser: downtime-pack.spec (1)</t>
+        </is>
+      </c>
+      <c r="O137" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P137" s="10" t="inlineStr">
+        <is>
+          <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="10" t="inlineStr">
+        <is>
           <t>DAY-007</t>
         </is>
       </c>
-      <c r="B137" s="10" t="inlineStr">
+      <c r="B138" s="10" t="inlineStr">
         <is>
           <t>Business Date</t>
         </is>
       </c>
-      <c r="C137" s="10" t="inlineStr">
+      <c r="C138" s="10" t="inlineStr">
         <is>
           <t>Notifications bell</t>
         </is>
       </c>
-      <c r="D137" s="10" t="inlineStr">
+      <c r="D138" s="10" t="inlineStr">
         <is>
           <t>In the last hour before a property rolls its business date, if a cashier shift is still open, users who can run the night audit get one warning that night. The roll does not wait.</t>
         </is>
       </c>
-      <c r="E137" s="10" t="inlineStr">
+      <c r="E138" s="10" t="inlineStr">
         <is>
           <t>BR-016</t>
         </is>
       </c>
-      <c r="F137" s="10" t="inlineStr">
+      <c r="F138" s="10" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="G137" s="10" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H137" s="10" t="inlineStr">
+      <c r="G138" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H138" s="10" t="inlineStr">
         <is>
           <t>fin.nightaudit.run</t>
         </is>
       </c>
-      <c r="I137" s="10" t="inlineStr">
+      <c r="I138" s="10" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="J137" s="10" t="inlineStr">
+      <c r="J138" s="10" t="inlineStr">
         <is>
           <t>a cashier shift is still open</t>
         </is>
       </c>
-      <c r="K137" s="10" t="inlineStr">
+      <c r="K138" s="10" t="inlineStr">
         <is>
           <t>the roll time is less than 60 minutes away</t>
         </is>
       </c>
-      <c r="L137" s="10" t="inlineStr">
+      <c r="L138" s="10" t="inlineStr">
         <is>
           <t>each night audit user gets one rollover_warning notification for that business date; none earlier, none after the roll time, none if no shift is open, none twice</t>
         </is>
       </c>
-      <c r="M137" s="10" t="inlineStr">
+      <c r="M138" s="10" t="inlineStr">
         <is>
           <t>app.warn_before_rollover; cron job rollover-warning</t>
         </is>
       </c>
-      <c r="N137" s="10" t="inlineStr">
+      <c r="N138" s="10" t="inlineStr">
         <is>
           <t>43_rollover_warning (9)</t>
         </is>
       </c>
-      <c r="O137" s="10" t="inlineStr">
+      <c r="O138" s="10" t="inlineStr">
         <is>
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P137" s="10" t="inlineStr">
+      <c r="P138" s="10" t="inlineStr">
         <is>
           <t>Added 8 Oct 2026. Warning only; the hard gate stays in R2 (DAY-005).</t>
         </is>

</xml_diff>

<commit_message>
Put year and month in invoice numbers (FIN-020)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P138"/>
+  <dimension ref="A1:P139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9576,22 +9576,22 @@
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>GST-007</t>
+          <t>FIN-020</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t>Guests</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C114" s="10" t="inlineStr">
         <is>
-          <t>/guests/$id; check-in; walk-in</t>
+          <t>/invoices/$id</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t>A photo or scan of an ID document is kept in private storage, shrunk and stripped of hidden data in the browser, and opened only through a 60-second link.</t>
+          <t>Invoice and interim invoice numbers carry the year and month of the hotel business date, then a count that restarts each month with no gaps (INV-202610-000001, INT-202610-000001). Invoices already issued keep their numbers.</t>
         </is>
       </c>
       <c r="E114" s="10" t="inlineStr">
@@ -9601,7 +9601,7 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G114" s="10" t="inlineStr">
@@ -9611,37 +9611,37 @@
       </c>
       <c r="H114" s="10" t="inlineStr">
         <is>
-          <t>guest.document.file.upload / view / delete</t>
+          <t>fin.invoice.issue</t>
         </is>
       </c>
       <c r="I114" s="10" t="inlineStr">
         <is>
-          <t>SET-009 switch</t>
+          <t>document_sequences period_key</t>
         </is>
       </c>
       <c r="J114" s="10" t="inlineStr">
         <is>
-          <t>a hotel that allows ID photos</t>
+          <t>a hotel with invoices issued in one month</t>
         </is>
       </c>
       <c r="K114" s="10" t="inlineStr">
         <is>
-          <t>front desk adds an ID photo</t>
+          <t>an invoice is issued in the next month</t>
         </is>
       </c>
       <c r="L114" s="10" t="inlineStr">
         <is>
-          <t>it is stored privately and opens only through a short-lived link</t>
+          <t>its number starts with the new year and month and the count restarts at 1; the INT and INV series stay separate; reservation and folio numbers are unchanged</t>
         </is>
       </c>
       <c r="M114" s="10" t="inlineStr">
         <is>
-          <t>begin_id_photo_upload, finish_id_photo_upload, open_id_photo</t>
+          <t>next_document_number, issue_invoice</t>
         </is>
       </c>
       <c r="N114" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (30)</t>
+          <t>46_invoice_number_month (8); 17_more_features</t>
         </is>
       </c>
       <c r="O114" s="10" t="inlineStr">
@@ -9649,12 +9649,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P114" s="10" t="inlineStr"/>
+      <c r="P114" s="10" t="inlineStr">
+        <is>
+          <t>Month comes from the business date, not the clock. No hotel code in the number yet.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>GST-008</t>
+          <t>GST-007</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
@@ -9664,12 +9668,12 @@
       </c>
       <c r="C115" s="10" t="inlineStr">
         <is>
-          <t>/guests/$id</t>
+          <t>/guests/$id; check-in; walk-in</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t>Every upload, view and deletion of an ID photo is audited with ids only, no personal data.</t>
+          <t>A photo or scan of an ID document is kept in private storage, shrunk and stripped of hidden data in the browser, and opened only through a 60-second link.</t>
         </is>
       </c>
       <c r="E115" s="10" t="inlineStr">
@@ -9689,37 +9693,37 @@
       </c>
       <c r="H115" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>guest.document.file.upload / view / delete</t>
         </is>
       </c>
       <c r="I115" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SET-009 switch</t>
         </is>
       </c>
       <c r="J115" s="10" t="inlineStr">
         <is>
-          <t>an ID photo</t>
+          <t>a hotel that allows ID photos</t>
         </is>
       </c>
       <c r="K115" s="10" t="inlineStr">
         <is>
-          <t>it is uploaded, opened or deleted</t>
+          <t>front desk adds an ID photo</t>
         </is>
       </c>
       <c r="L115" s="10" t="inlineStr">
         <is>
-          <t>an audit row records who and which file, with no personal data</t>
+          <t>it is stored privately and opens only through a short-lived link</t>
         </is>
       </c>
       <c r="M115" s="10" t="inlineStr">
         <is>
-          <t>app.audit_id_photo</t>
+          <t>begin_id_photo_upload, finish_id_photo_upload, open_id_photo</t>
         </is>
       </c>
       <c r="N115" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (9)</t>
+          <t>24_id_photos (30)</t>
         </is>
       </c>
       <c r="O115" s="10" t="inlineStr">
@@ -9732,7 +9736,7 @@
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
         <is>
-          <t>GST-009</t>
+          <t>GST-008</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
@@ -9747,7 +9751,7 @@
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t>ID photos are removed from storage when the guest is anonymised or the document is removed, and move with the guest when two profiles are merged.</t>
+          <t>Every upload, view and deletion of an ID photo is audited with ids only, no personal data.</t>
         </is>
       </c>
       <c r="E116" s="10" t="inlineStr">
@@ -9777,27 +9781,27 @@
       </c>
       <c r="J116" s="10" t="inlineStr">
         <is>
-          <t>a guest with ID photos</t>
+          <t>an ID photo</t>
         </is>
       </c>
       <c r="K116" s="10" t="inlineStr">
         <is>
-          <t>the guest is anonymised, the document removed, or the profile merged</t>
+          <t>it is uploaded, opened or deleted</t>
         </is>
       </c>
       <c r="L116" s="10" t="inlineStr">
         <is>
-          <t>the files are removed, or move to the kept profile</t>
+          <t>an audit row records who and which file, with no personal data</t>
         </is>
       </c>
       <c r="M116" s="10" t="inlineStr">
         <is>
-          <t>anonymise_guest, merge_guests, delete_id_photo</t>
+          <t>app.audit_id_photo</t>
         </is>
       </c>
       <c r="N116" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (4)</t>
+          <t>24_id_photos (9)</t>
         </is>
       </c>
       <c r="O116" s="10" t="inlineStr">
@@ -9810,7 +9814,7 @@
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>GST-010</t>
+          <t>GST-009</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
@@ -9820,12 +9824,12 @@
       </c>
       <c r="C117" s="10" t="inlineStr">
         <is>
-          <t>(daily clean-up)</t>
+          <t>/guests/$id</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t>ID photos are deleted automatically a set number of months (one setting, now 12) after the guest's last check-out, unless the guest has a booking that is not over.</t>
+          <t>ID photos are removed from storage when the guest is anonymised or the document is removed, and move with the guest when two profiles are merged.</t>
         </is>
       </c>
       <c r="E117" s="10" t="inlineStr">
@@ -9850,32 +9854,32 @@
       </c>
       <c r="I117" s="10" t="inlineStr">
         <is>
-          <t>Setting id_photo_keep_months; daily cron</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J117" s="10" t="inlineStr">
         <is>
-          <t>a guest whose last check-out was more than the keep period ago</t>
+          <t>a guest with ID photos</t>
         </is>
       </c>
       <c r="K117" s="10" t="inlineStr">
         <is>
-          <t>the daily clean-up runs</t>
+          <t>the guest is anonymised, the document removed, or the profile merged</t>
         </is>
       </c>
       <c r="L117" s="10" t="inlineStr">
         <is>
-          <t>their ID photos are deleted</t>
+          <t>the files are removed, or move to the kept profile</t>
         </is>
       </c>
       <c r="M117" s="10" t="inlineStr">
         <is>
-          <t>/api/cron/id-photo-cleanup</t>
+          <t>anonymise_guest, merge_guests, delete_id_photo</t>
         </is>
       </c>
       <c r="N117" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (5)</t>
+          <t>24_id_photos (4)</t>
         </is>
       </c>
       <c r="O117" s="10" t="inlineStr">
@@ -9888,22 +9892,22 @@
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
         <is>
-          <t>ROOM-005</t>
+          <t>GST-010</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t>Rooms</t>
+          <t>Guests</t>
         </is>
       </c>
       <c r="C118" s="10" t="inlineStr">
         <is>
-          <t>/rooms</t>
+          <t>(daily clean-up)</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t>Rooms are added one at a time or several by number or by name, with a preview; labels are free text up to 30 characters, unique per hotel ignoring case and extra spaces, shown as typed and sorted in natural order.</t>
+          <t>ID photos are deleted automatically a set number of months (one setting, now 12) after the guest's last check-out, unless the guest has a booking that is not over.</t>
         </is>
       </c>
       <c r="E118" s="10" t="inlineStr">
@@ -9923,37 +9927,37 @@
       </c>
       <c r="H118" s="10" t="inlineStr">
         <is>
-          <t>setup.room.edit</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I118" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Setting id_photo_keep_months; daily cron</t>
         </is>
       </c>
       <c r="J118" s="10" t="inlineStr">
         <is>
-          <t>an administrator on the Rooms page</t>
+          <t>a guest whose last check-out was more than the keep period ago</t>
         </is>
       </c>
       <c r="K118" s="10" t="inlineStr">
         <is>
-          <t>they add rooms by number range or by names</t>
+          <t>the daily clean-up runs</t>
         </is>
       </c>
       <c r="L118" s="10" t="inlineStr">
         <is>
-          <t>valid new rooms are created, duplicates skipped and invalid names shown</t>
+          <t>their ID photos are deleted</t>
         </is>
       </c>
       <c r="M118" s="10" t="inlineStr">
         <is>
-          <t>add_rooms_range, add_rooms_named, save_room</t>
+          <t>/api/cron/id-photo-cleanup</t>
         </is>
       </c>
       <c r="N118" s="10" t="inlineStr">
         <is>
-          <t>23_room_labels (46); 26_small_fixes (1); browser: rooms-add</t>
+          <t>24_id_photos (5)</t>
         </is>
       </c>
       <c r="O118" s="10" t="inlineStr">
@@ -9966,22 +9970,22 @@
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>SET-009</t>
+          <t>ROOM-005</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Rooms</t>
         </is>
       </c>
       <c r="C119" s="10" t="inlineStr">
         <is>
-          <t>/setup/property</t>
+          <t>/rooms</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t>Per hotel: "Allow ID photos" (off by default) and "Require ID photo at check-in" (only when allowed). While Allow is off, uploading and opening ID photos are refused.</t>
+          <t>Rooms are added one at a time or several by number or by name, with a preview; labels are free text up to 30 characters, unique per hotel ignoring case and extra spaces, shown as typed and sorted in natural order.</t>
         </is>
       </c>
       <c r="E119" s="10" t="inlineStr">
@@ -10001,7 +10005,7 @@
       </c>
       <c r="H119" s="10" t="inlineStr">
         <is>
-          <t>setup.property.edit</t>
+          <t>setup.room.edit</t>
         </is>
       </c>
       <c r="I119" s="10" t="inlineStr">
@@ -10011,27 +10015,27 @@
       </c>
       <c r="J119" s="10" t="inlineStr">
         <is>
-          <t>a hotel with ID photos off</t>
+          <t>an administrator on the Rooms page</t>
         </is>
       </c>
       <c r="K119" s="10" t="inlineStr">
         <is>
-          <t>staff try to add or open an ID photo</t>
+          <t>they add rooms by number range or by names</t>
         </is>
       </c>
       <c r="L119" s="10" t="inlineStr">
         <is>
-          <t>it is refused; when Require is on, check-in waits for an ID photo</t>
+          <t>valid new rooms are created, duplicates skipped and invalid names shown</t>
         </is>
       </c>
       <c r="M119" s="10" t="inlineStr">
         <is>
-          <t>set_id_photo_settings</t>
+          <t>add_rooms_range, add_rooms_named, save_room</t>
         </is>
       </c>
       <c r="N119" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (10)</t>
+          <t>23_room_labels (46); 26_small_fixes (1); browser: rooms-add</t>
         </is>
       </c>
       <c r="O119" s="10" t="inlineStr">
@@ -10044,32 +10048,32 @@
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
         <is>
-          <t>GRP-001</t>
+          <t>SET-009</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
         <is>
-          <t>Platform &amp; Tenancy</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C120" s="10" t="inlineStr">
         <is>
-          <t>All branches</t>
+          <t>/setup/property</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t>A built-in Group Manager role and the permission rpt.group.view exist; only System Administrator, General Manager and Group Manager hold the permission.</t>
+          <t>Per hotel: "Allow ID photos" (off by default) and "Require ID photo at check-in" (only when allowed). While Allow is off, uploading and opening ID photos are refused.</t>
         </is>
       </c>
       <c r="E120" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F120" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G120" s="10" t="inlineStr">
@@ -10079,33 +10083,37 @@
       </c>
       <c r="H120" s="10" t="inlineStr">
         <is>
-          <t>rpt.group.view</t>
-        </is>
-      </c>
-      <c r="I120" s="10" t="inlineStr"/>
+          <t>setup.property.edit</t>
+        </is>
+      </c>
+      <c r="I120" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="J120" s="10" t="inlineStr">
         <is>
-          <t>a hotel group with several branches</t>
+          <t>a hotel with ID photos off</t>
         </is>
       </c>
       <c r="K120" s="10" t="inlineStr">
         <is>
-          <t>an owner wants a view-only manager for the whole group</t>
+          <t>staff try to add or open an ID photo</t>
         </is>
       </c>
       <c r="L120" s="10" t="inlineStr">
         <is>
-          <t>they assign the Group Manager role branch by branch, and that person can look but not post or change anything</t>
+          <t>it is refused; when Require is on, check-in waits for an ID photo</t>
         </is>
       </c>
       <c r="M120" s="10" t="inlineStr">
         <is>
-          <t>20261013120000_group_view.sql</t>
+          <t>set_id_photo_settings</t>
         </is>
       </c>
       <c r="N120" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (5)</t>
+          <t>24_id_photos (10)</t>
         </is>
       </c>
       <c r="O120" s="10" t="inlineStr">
@@ -10113,16 +10121,12 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P120" s="10" t="inlineStr">
-        <is>
-          <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
-        </is>
-      </c>
+      <c r="P120" s="10" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>GRP-002</t>
+          <t>GRP-001</t>
         </is>
       </c>
       <c r="B121" s="10" t="inlineStr">
@@ -10137,7 +10141,7 @@
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t>One call shows every branch the person may see: occupancy, in house, arrivals and departures to come, approvals, repairs and last night revenue, with group totals. Revenue is totalled per currency.</t>
+          <t>A built-in Group Manager role and the permission rpt.group.view exist; only System Administrator, General Manager and Group Manager hold the permission.</t>
         </is>
       </c>
       <c r="E121" s="10" t="inlineStr">
@@ -10163,27 +10167,27 @@
       <c r="I121" s="10" t="inlineStr"/>
       <c r="J121" s="10" t="inlineStr">
         <is>
-          <t>a group with a Lagos and an Abuja branch</t>
+          <t>a hotel group with several branches</t>
         </is>
       </c>
       <c r="K121" s="10" t="inlineStr">
         <is>
-          <t>a group manager opens All branches</t>
+          <t>an owner wants a view-only manager for the whole group</t>
         </is>
       </c>
       <c r="L121" s="10" t="inlineStr">
         <is>
-          <t>they see both branches with figures from the database, never another hotel group, and staff without the permission are refused</t>
+          <t>they assign the Group Manager role branch by branch, and that person can look but not post or change anything</t>
         </is>
       </c>
       <c r="M121" s="10" t="inlineStr">
         <is>
-          <t>group_overview; /group screen</t>
+          <t>20261013120000_group_view.sql</t>
         </is>
       </c>
       <c r="N121" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (10)</t>
+          <t>35_group_view (5)</t>
         </is>
       </c>
       <c r="O121" s="10" t="inlineStr">
@@ -10193,14 +10197,14 @@
       </c>
       <c r="P121" s="10" t="inlineStr">
         <is>
-          <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
+          <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="10" t="inlineStr">
         <is>
-          <t>GRP-003</t>
+          <t>GRP-002</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
@@ -10215,7 +10219,7 @@
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t>A Group Manager sees only the branches they are assigned to, and cannot post charges or check guests in.</t>
+          <t>One call shows every branch the person may see: occupancy, in house, arrivals and departures to come, approvals, repairs and last night revenue, with group totals. Revenue is totalled per currency.</t>
         </is>
       </c>
       <c r="E122" s="10" t="inlineStr">
@@ -10241,27 +10245,27 @@
       <c r="I122" s="10" t="inlineStr"/>
       <c r="J122" s="10" t="inlineStr">
         <is>
-          <t>a Group Manager assigned to one branch</t>
+          <t>a group with a Lagos and an Abuja branch</t>
         </is>
       </c>
       <c r="K122" s="10" t="inlineStr">
         <is>
-          <t>a second branch is assigned</t>
+          <t>a group manager opens All branches</t>
         </is>
       </c>
       <c r="L122" s="10" t="inlineStr">
         <is>
-          <t>the second branch appears; the role never gets write permissions</t>
+          <t>they see both branches with figures from the database, never another hotel group, and staff without the permission are refused</t>
         </is>
       </c>
       <c r="M122" s="10" t="inlineStr">
         <is>
-          <t>assign_role (existing); group_overview</t>
+          <t>group_overview; /group screen</t>
         </is>
       </c>
       <c r="N122" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (3)</t>
+          <t>35_group_view (10)</t>
         </is>
       </c>
       <c r="O122" s="10" t="inlineStr">
@@ -10271,14 +10275,14 @@
       </c>
       <c r="P122" s="10" t="inlineStr">
         <is>
-          <t>Access is per branch, using the existing role assignment screen.</t>
+          <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>GRP-004</t>
+          <t>GRP-003</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
@@ -10288,12 +10292,12 @@
       </c>
       <c r="C123" s="10" t="inlineStr">
         <is>
-          <t>All branches (Copy setup)</t>
+          <t>All branches</t>
         </is>
       </c>
       <c r="D123" s="10" t="inlineStr">
         <is>
-          <t>A new branch can copy room types, rate plans and prices from an existing branch, once, into an empty branch.</t>
+          <t>A Group Manager sees only the branches they are assigned to, and cannot post charges or check guests in.</t>
         </is>
       </c>
       <c r="E123" s="10" t="inlineStr">
@@ -10313,33 +10317,33 @@
       </c>
       <c r="H123" s="10" t="inlineStr">
         <is>
-          <t>setup.room.manage, setup.rate.manage</t>
+          <t>rpt.group.view</t>
         </is>
       </c>
       <c r="I123" s="10" t="inlineStr"/>
       <c r="J123" s="10" t="inlineStr">
         <is>
-          <t>a new empty branch</t>
+          <t>a Group Manager assigned to one branch</t>
         </is>
       </c>
       <c r="K123" s="10" t="inlineStr">
         <is>
-          <t>the owner copies setup from the first branch</t>
+          <t>a second branch is assigned</t>
         </is>
       </c>
       <c r="L123" s="10" t="inlineStr">
         <is>
-          <t>room types, rate plans and prices appear on the new branch and point at its own room types; rooms are not copied; a second copy is refused; the copy is audited</t>
+          <t>the second branch appears; the role never gets write permissions</t>
         </is>
       </c>
       <c r="M123" s="10" t="inlineStr">
         <is>
-          <t>copy_property_setup</t>
+          <t>assign_role (existing); group_overview</t>
         </is>
       </c>
       <c r="N123" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (13)</t>
+          <t>35_group_view (3)</t>
         </is>
       </c>
       <c r="O123" s="10" t="inlineStr">
@@ -10349,29 +10353,29 @@
       </c>
       <c r="P123" s="10" t="inlineStr">
         <is>
-          <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
+          <t>Access is per branch, using the existing role assignment screen.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="10" t="inlineStr">
         <is>
-          <t>RPT-005</t>
+          <t>GRP-004</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Platform &amp; Tenancy</t>
         </is>
       </c>
       <c r="C124" s="10" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>All branches (Copy setup)</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr">
         <is>
-          <t>Revenue by booking source: bookings, cancellations, no-shows, room nights, room revenue and average rate for each source in a date range.</t>
+          <t>A new branch can copy room types, rate plans and prices from an existing branch, once, into an empty branch.</t>
         </is>
       </c>
       <c r="E124" s="10" t="inlineStr">
@@ -10391,33 +10395,33 @@
       </c>
       <c r="H124" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view</t>
+          <t>setup.room.manage, setup.rate.manage</t>
         </is>
       </c>
       <c r="I124" s="10" t="inlineStr"/>
       <c r="J124" s="10" t="inlineStr">
         <is>
-          <t>bookings from direct, phone and company sources</t>
+          <t>a new empty branch</t>
         </is>
       </c>
       <c r="K124" s="10" t="inlineStr">
         <is>
-          <t>the accountant picks a date range</t>
+          <t>the owner copies setup from the first branch</t>
         </is>
       </c>
       <c r="L124" s="10" t="inlineStr">
         <is>
-          <t>each source shows its own counts and room revenue (room charges only, before tax); cancelled bookings add no nights</t>
+          <t>room types, rate plans and prices appear on the new branch and point at its own room types; rooms are not copied; a second copy is refused; the copy is audited</t>
         </is>
       </c>
       <c r="M124" s="10" t="inlineStr">
         <is>
-          <t>20261013130000_source_ageing_reports.sql: report_revenue_by_source; Reports, By booking source tab</t>
+          <t>copy_property_setup</t>
         </is>
       </c>
       <c r="N124" s="10" t="inlineStr">
         <is>
-          <t>36_source_ageing (13)</t>
+          <t>35_group_view (13)</t>
         </is>
       </c>
       <c r="O124" s="10" t="inlineStr">
@@ -10427,14 +10431,14 @@
       </c>
       <c r="P124" s="10" t="inlineStr">
         <is>
-          <t>Bookings counted by arrival date; revenue by posting date.</t>
+          <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>RPT-006</t>
+          <t>RPT-005</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
@@ -10449,7 +10453,7 @@
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t>Ageing of unpaid balances by booking source: current, 1 to 7, 8 to 30, 31 to 60 and over 60 days since the due departure, plus credit held.</t>
+          <t>Revenue by booking source: bookings, cancellations, no-shows, room nights, room revenue and average rate for each source in a date range.</t>
         </is>
       </c>
       <c r="E125" s="10" t="inlineStr">
@@ -10475,27 +10479,27 @@
       <c r="I125" s="10" t="inlineStr"/>
       <c r="J125" s="10" t="inlineStr">
         <is>
-          <t>guests and companies who left owing money</t>
+          <t>bookings from direct, phone and company sources</t>
         </is>
       </c>
       <c r="K125" s="10" t="inlineStr">
         <is>
-          <t>the accountant opens the Ageing tab</t>
+          <t>the accountant picks a date range</t>
         </is>
       </c>
       <c r="L125" s="10" t="inlineStr">
         <is>
-          <t>each source shows what is owed in each age column; paid bills drop out; overpayments show as credit held; the total matches Outstanding balances</t>
+          <t>each source shows its own counts and room revenue (room charges only, before tax); cancelled bookings add no nights</t>
         </is>
       </c>
       <c r="M125" s="10" t="inlineStr">
         <is>
-          <t>report_balance_ageing; Reports, Ageing tab</t>
+          <t>20261013130000_source_ageing_reports.sql: report_revenue_by_source; Reports, By booking source tab</t>
         </is>
       </c>
       <c r="N125" s="10" t="inlineStr">
         <is>
-          <t>36_source_ageing (11)</t>
+          <t>36_source_ageing (13)</t>
         </is>
       </c>
       <c r="O125" s="10" t="inlineStr">
@@ -10505,29 +10509,29 @@
       </c>
       <c r="P125" s="10" t="inlineStr">
         <is>
-          <t>Guests still staying count as current.</t>
+          <t>Bookings counted by arrival date; revenue by posting date.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="10" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>RPT-006</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
         <is>
-          <t>AI helpers</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C126" s="10" t="inlineStr">
         <is>
-          <t>Dashboard, Admin</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="D126" s="10" t="inlineStr">
         <is>
-          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
+          <t>Ageing of unpaid balances by booking source: current, 1 to 7, 8 to 30, 31 to 60 and over 60 days since the due departure, plus credit held.</t>
         </is>
       </c>
       <c r="E126" s="10" t="inlineStr">
@@ -10547,33 +10551,33 @@
       </c>
       <c r="H126" s="10" t="inlineStr">
         <is>
-          <t>adm.ai.manage</t>
+          <t>rpt.finance.view</t>
         </is>
       </c>
       <c r="I126" s="10" t="inlineStr"/>
       <c r="J126" s="10" t="inlineStr">
         <is>
-          <t>a new hotel</t>
+          <t>guests and companies who left owing money</t>
         </is>
       </c>
       <c r="K126" s="10" t="inlineStr">
         <is>
-          <t>a manager opens Admin, AI helpers</t>
+          <t>the accountant opens the Ageing tab</t>
         </is>
       </c>
       <c r="L126" s="10" t="inlineStr">
         <is>
-          <t>nothing runs until they switch it on and the change is in the audit log</t>
+          <t>each source shows what is owed in each age column; paid bills drop out; overpayments show as credit held; the total matches Outstanding balances</t>
         </is>
       </c>
       <c r="M126" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
+          <t>report_balance_ageing; Reports, Ageing tab</t>
         </is>
       </c>
       <c r="N126" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (11)</t>
+          <t>36_source_ageing (11)</t>
         </is>
       </c>
       <c r="O126" s="10" t="inlineStr">
@@ -10583,14 +10587,14 @@
       </c>
       <c r="P126" s="10" t="inlineStr">
         <is>
-          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
+          <t>Guests still staying count as current.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
         <is>
-          <t>AI-002</t>
+          <t>AI-001</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
@@ -10605,7 +10609,7 @@
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
+          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
         </is>
       </c>
       <c r="E127" s="10" t="inlineStr">
@@ -10625,28 +10629,28 @@
       </c>
       <c r="H127" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view, rpt.operations.view</t>
+          <t>adm.ai.manage</t>
         </is>
       </c>
       <c r="I127" s="10" t="inlineStr"/>
       <c r="J127" s="10" t="inlineStr">
         <is>
-          <t>a hotel with guests, approvals and overdue bills</t>
+          <t>a new hotel</t>
         </is>
       </c>
       <c r="K127" s="10" t="inlineStr">
         <is>
-          <t>a brief is started</t>
+          <t>a manager opens Admin, AI helpers</t>
         </is>
       </c>
       <c r="L127" s="10" t="inlineStr">
         <is>
-          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
+          <t>nothing runs until they switch it on and the change is in the audit log</t>
         </is>
       </c>
       <c r="M127" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
+          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
         </is>
       </c>
       <c r="N127" s="10" t="inlineStr">
@@ -10661,14 +10665,14 @@
       </c>
       <c r="P127" s="10" t="inlineStr">
         <is>
-          <t>Overdue means unpaid more than 30 days after departure.</t>
+          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
         <is>
-          <t>AI-003</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
@@ -10683,7 +10687,7 @@
       </c>
       <c r="D128" s="10" t="inlineStr">
         <is>
-          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
+          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
         </is>
       </c>
       <c r="E128" s="10" t="inlineStr">
@@ -10703,33 +10707,33 @@
       </c>
       <c r="H128" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view</t>
+          <t>rpt.finance.view, rpt.operations.view</t>
         </is>
       </c>
       <c r="I128" s="10" t="inlineStr"/>
       <c r="J128" s="10" t="inlineStr">
         <is>
-          <t>a limit of 2</t>
+          <t>a hotel with guests, approvals and overdue bills</t>
         </is>
       </c>
       <c r="K128" s="10" t="inlineStr">
         <is>
-          <t>a third brief is requested</t>
+          <t>a brief is started</t>
         </is>
       </c>
       <c r="L128" s="10" t="inlineStr">
         <is>
-          <t>it is refused until a failed call frees a slot or the month turns</t>
+          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
         </is>
       </c>
       <c r="M128" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
+          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
         </is>
       </c>
       <c r="N128" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (5)</t>
+          <t>37_ai_brief (11)</t>
         </is>
       </c>
       <c r="O128" s="10" t="inlineStr">
@@ -10737,12 +10741,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P128" s="10" t="inlineStr"/>
+      <c r="P128" s="10" t="inlineStr">
+        <is>
+          <t>Overdue means unpaid more than 30 days after departure.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
         <is>
-          <t>AI-004</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
@@ -10757,7 +10765,7 @@
       </c>
       <c r="D129" s="10" t="inlineStr">
         <is>
-          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
+          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
         </is>
       </c>
       <c r="E129" s="10" t="inlineStr">
@@ -10777,33 +10785,33 @@
       </c>
       <c r="H129" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view, rpt.operations.view</t>
+          <t>rpt.finance.view</t>
         </is>
       </c>
       <c r="I129" s="10" t="inlineStr"/>
       <c r="J129" s="10" t="inlineStr">
         <is>
-          <t>front desk, housekeeping, another hotel</t>
+          <t>a limit of 2</t>
         </is>
       </c>
       <c r="K129" s="10" t="inlineStr">
         <is>
-          <t>they ask for the brief or touch the tables</t>
+          <t>a third brief is requested</t>
         </is>
       </c>
       <c r="L129" s="10" t="inlineStr">
         <is>
-          <t>they are refused</t>
+          <t>it is refused until a failed call frees a slot or the month turns</t>
         </is>
       </c>
       <c r="M129" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql</t>
+          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
         </is>
       </c>
       <c r="N129" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (7)</t>
+          <t>37_ai_brief (5)</t>
         </is>
       </c>
       <c r="O129" s="10" t="inlineStr">
@@ -10816,7 +10824,7 @@
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
         <is>
-          <t>AI-005</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
@@ -10831,7 +10839,7 @@
       </c>
       <c r="D130" s="10" t="inlineStr">
         <is>
-          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
+          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
         </is>
       </c>
       <c r="E130" s="10" t="inlineStr">
@@ -10851,33 +10859,33 @@
       </c>
       <c r="H130" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>rpt.finance.view, rpt.operations.view</t>
         </is>
       </c>
       <c r="I130" s="10" t="inlineStr"/>
       <c r="J130" s="10" t="inlineStr">
         <is>
-          <t>a draft that rounds or invents a figure</t>
+          <t>front desk, housekeeping, another hotel</t>
         </is>
       </c>
       <c r="K130" s="10" t="inlineStr">
         <is>
-          <t>the brief is written</t>
+          <t>they ask for the brief or touch the tables</t>
         </is>
       </c>
       <c r="L130" s="10" t="inlineStr">
         <is>
-          <t>the plain database lines are shown instead, with a note</t>
+          <t>they are refused</t>
         </is>
       </c>
       <c r="M130" s="10" t="inlineStr">
         <is>
-          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
+          <t>20261013140000_ai_morning_brief.sql</t>
         </is>
       </c>
       <c r="N130" s="10" t="inlineStr">
         <is>
-          <t>browser unit: ai-brief-unit (8)</t>
+          <t>37_ai_brief (7)</t>
         </is>
       </c>
       <c r="O130" s="10" t="inlineStr">
@@ -10885,31 +10893,27 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P130" s="10" t="inlineStr">
-        <is>
-          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
-        </is>
-      </c>
+      <c r="P130" s="10" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
         <is>
-          <t>SET-010</t>
+          <t>AI-005</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>AI helpers</t>
         </is>
       </c>
       <c r="C131" s="10" t="inlineStr">
         <is>
-          <t>Setup, Rooms</t>
+          <t>Dashboard, Admin</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
+          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
         </is>
       </c>
       <c r="E131" s="10" t="inlineStr">
@@ -10929,33 +10933,33 @@
       </c>
       <c r="H131" s="10" t="inlineStr">
         <is>
-          <t>setup.room.manage</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I131" s="10" t="inlineStr"/>
       <c r="J131" s="10" t="inlineStr">
         <is>
-          <t>a list of room types and rooms</t>
+          <t>a draft that rounds or invents a figure</t>
         </is>
       </c>
       <c r="K131" s="10" t="inlineStr">
         <is>
-          <t>the manager previews and then applies it</t>
+          <t>the brief is written</t>
         </is>
       </c>
       <c r="L131" s="10" t="inlineStr">
         <is>
-          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
+          <t>the plain database lines are shown instead, with a note</t>
         </is>
       </c>
       <c r="M131" s="10" t="inlineStr">
         <is>
-          <t>20261013150000_setup_import.sql: apply_setup_import</t>
+          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
         </is>
       </c>
       <c r="N131" s="10" t="inlineStr">
         <is>
-          <t>38_setup_import (29)</t>
+          <t>browser unit: ai-brief-unit (8)</t>
         </is>
       </c>
       <c r="O131" s="10" t="inlineStr">
@@ -10965,19 +10969,19 @@
       </c>
       <c r="P131" s="10" t="inlineStr">
         <is>
-          <t>The AI only drafts the list. This function is the check.</t>
+          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="10" t="inlineStr">
         <is>
-          <t>AI-006</t>
+          <t>SET-010</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
         <is>
-          <t>AI helpers</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C132" s="10" t="inlineStr">
@@ -10987,7 +10991,7 @@
       </c>
       <c r="D132" s="10" t="inlineStr">
         <is>
-          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
+          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
         </is>
       </c>
       <c r="E132" s="10" t="inlineStr">
@@ -11013,27 +11017,27 @@
       <c r="I132" s="10" t="inlineStr"/>
       <c r="J132" s="10" t="inlineStr">
         <is>
-          <t>AI switched on with a limit of 1</t>
+          <t>a list of room types and rooms</t>
         </is>
       </c>
       <c r="K132" s="10" t="inlineStr">
         <is>
-          <t>an import draft is started twice</t>
+          <t>the manager previews and then applies it</t>
         </is>
       </c>
       <c r="L132" s="10" t="inlineStr">
         <is>
-          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
+          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
         </is>
       </c>
       <c r="M132" s="10" t="inlineStr">
         <is>
-          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
+          <t>20261013150000_setup_import.sql: apply_setup_import</t>
         </is>
       </c>
       <c r="N132" s="10" t="inlineStr">
         <is>
-          <t>38_setup_import (8)</t>
+          <t>38_setup_import (29)</t>
         </is>
       </c>
       <c r="O132" s="10" t="inlineStr">
@@ -11041,12 +11045,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P132" s="10" t="inlineStr"/>
+      <c r="P132" s="10" t="inlineStr">
+        <is>
+          <t>The AI only drafts the list. This function is the check.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
         <is>
-          <t>AI-007</t>
+          <t>AI-006</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
@@ -11061,7 +11069,7 @@
       </c>
       <c r="D133" s="10" t="inlineStr">
         <is>
-          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
+          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
         </is>
       </c>
       <c r="E133" s="10" t="inlineStr">
@@ -11087,27 +11095,27 @@
       <c r="I133" s="10" t="inlineStr"/>
       <c r="J133" s="10" t="inlineStr">
         <is>
-          <t>a pasted list</t>
+          <t>AI switched on with a limit of 1</t>
         </is>
       </c>
       <c r="K133" s="10" t="inlineStr">
         <is>
-          <t>the assistant drafts it</t>
+          <t>an import draft is started twice</t>
         </is>
       </c>
       <c r="L133" s="10" t="inlineStr">
         <is>
-          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
+          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
         </is>
       </c>
       <c r="M133" s="10" t="inlineStr">
         <is>
-          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
+          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
         </is>
       </c>
       <c r="N133" s="10" t="inlineStr">
         <is>
-          <t>browser unit: setup-import-unit (9)</t>
+          <t>38_setup_import (8)</t>
         </is>
       </c>
       <c r="O133" s="10" t="inlineStr">
@@ -11115,36 +11123,32 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P133" s="10" t="inlineStr">
-        <is>
-          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
-        </is>
-      </c>
+      <c r="P133" s="10" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
         <is>
-          <t>SET-011</t>
+          <t>AI-007</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>AI helpers</t>
         </is>
       </c>
       <c r="C134" s="10" t="inlineStr">
         <is>
-          <t>/setup; /dashboard</t>
+          <t>Setup, Rooms</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
         <is>
-          <t>A new hotel sees a checklist of what is left to set up: property details, room types, rooms, rates, taxes, payment methods and staff. Each step says what is missing and links to the right screen. The list comes from the hotel's own data, so it is always current.</t>
+          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
         </is>
       </c>
       <c r="E134" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F134" s="10" t="inlineStr">
@@ -11159,37 +11163,33 @@
       </c>
       <c r="H134" s="10" t="inlineStr">
         <is>
-          <t>any setup permission</t>
-        </is>
-      </c>
-      <c r="I134" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>setup.room.manage</t>
+        </is>
+      </c>
+      <c r="I134" s="10" t="inlineStr"/>
       <c r="J134" s="10" t="inlineStr">
         <is>
-          <t>a hotel that is part way through setup</t>
+          <t>a pasted list</t>
         </is>
       </c>
       <c r="K134" s="10" t="inlineStr">
         <is>
-          <t>a manager opens Setup or the Dashboard</t>
+          <t>the assistant drafts it</t>
         </is>
       </c>
       <c r="L134" s="10" t="inlineStr">
         <is>
-          <t>the steps already done are ticked and the next one is linked; once all seven are done the checklist goes away</t>
+          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
         </is>
       </c>
       <c r="M134" s="10" t="inlineStr">
         <is>
-          <t>setup_progress</t>
+          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
         </is>
       </c>
       <c r="N134" s="10" t="inlineStr">
         <is>
-          <t>40_guided_setup (30)</t>
+          <t>browser unit: setup-import-unit (9)</t>
         </is>
       </c>
       <c r="O134" s="10" t="inlineStr">
@@ -11199,39 +11199,39 @@
       </c>
       <c r="P134" s="10" t="inlineStr">
         <is>
-          <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
+          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
         <is>
-          <t>NFR-006</t>
+          <t>SET-011</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
         <is>
-          <t>Non-functional</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C135" s="10" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/setup; /dashboard</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr">
         <is>
-          <t>The last room of a type is sold once, however many desks book at the same moment, and a repeated booking never doubles.</t>
+          <t>A new hotel sees a checklist of what is left to set up: property details, room types, rooms, rates, taxes, payment methods and staff. Each step says what is missing and links to the right screen. The list comes from the hotel's own data, so it is always current.</t>
         </is>
       </c>
       <c r="E135" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F135" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G135" s="10" t="inlineStr">
@@ -11241,37 +11241,37 @@
       </c>
       <c r="H135" s="10" t="inlineStr">
         <is>
+          <t>any setup permission</t>
+        </is>
+      </c>
+      <c r="I135" s="10" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I135" s="10" t="inlineStr">
-        <is>
-          <t>Rule: Safe last-room booking</t>
-        </is>
-      </c>
       <c r="J135" s="10" t="inlineStr">
         <is>
-          <t>one room of a type is left and several desks book it together</t>
+          <t>a hotel that is part way through setup</t>
         </is>
       </c>
       <c r="K135" s="10" t="inlineStr">
         <is>
-          <t>all of them submit at the same moment</t>
+          <t>a manager opens Setup or the Dashboard</t>
         </is>
       </c>
       <c r="L135" s="10" t="inlineStr">
         <is>
-          <t>exactly one booking succeeds, the rest get E_NO_AVAILABILITY, and nothing is oversold</t>
+          <t>the steps already done are ticked and the next one is linked; once all seven are done the checklist goes away</t>
         </is>
       </c>
       <c r="M135" s="10" t="inlineStr">
         <is>
-          <t>create_reservation, assert_available</t>
+          <t>setup_progress</t>
         </is>
       </c>
       <c r="N135" s="10" t="inlineStr">
         <is>
-          <t>concurrency/last_room.sh (6)</t>
+          <t>40_guided_setup (30)</t>
         </is>
       </c>
       <c r="O135" s="10" t="inlineStr">
@@ -11281,29 +11281,29 @@
       </c>
       <c r="P135" s="10" t="inlineStr">
         <is>
-          <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
+          <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
         <is>
-          <t>SET-012</t>
+          <t>NFR-006</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Non-functional</t>
         </is>
       </c>
       <c r="C136" s="10" t="inlineStr">
         <is>
-          <t>/setup/property</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr">
         <is>
-          <t>A manager sets the longest stay (1 to 365 nights) and how long a tentative booking holds its room (1 to 720 hours) for each property.</t>
+          <t>The last room of a type is sold once, however many desks book at the same moment, and a repeated booking never doubles.</t>
         </is>
       </c>
       <c r="E136" s="10" t="inlineStr">
@@ -11313,7 +11313,7 @@
       </c>
       <c r="F136" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G136" s="10" t="inlineStr">
@@ -11323,33 +11323,37 @@
       </c>
       <c r="H136" s="10" t="inlineStr">
         <is>
-          <t>setup.property.edit</t>
-        </is>
-      </c>
-      <c r="I136" s="10" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I136" s="10" t="inlineStr">
+        <is>
+          <t>Rule: Safe last-room booking</t>
+        </is>
+      </c>
       <c r="J136" s="10" t="inlineStr">
         <is>
-          <t>a property with the default rules (30 nights, 24 hours)</t>
+          <t>one room of a type is left and several desks book it together</t>
         </is>
       </c>
       <c r="K136" s="10" t="inlineStr">
         <is>
-          <t>a manager saves new booking rules</t>
+          <t>all of them submit at the same moment</t>
         </is>
       </c>
       <c r="L136" s="10" t="inlineStr">
         <is>
-          <t>new bookings use them, bad values are refused with E_INVALID, and the change is audited with old and new values</t>
+          <t>exactly one booking succeeds, the rest get E_NO_AVAILABILITY, and nothing is oversold</t>
         </is>
       </c>
       <c r="M136" s="10" t="inlineStr">
         <is>
-          <t>set_booking_rules; Booking rules on Setup, Property</t>
+          <t>create_reservation, assert_available</t>
         </is>
       </c>
       <c r="N136" s="10" t="inlineStr">
         <is>
-          <t>42_booking_rules (9)</t>
+          <t>concurrency/last_room.sh (6)</t>
         </is>
       </c>
       <c r="O136" s="10" t="inlineStr">
@@ -11359,39 +11363,39 @@
       </c>
       <c r="P136" s="10" t="inlineStr">
         <is>
-          <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
+          <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
         <is>
-          <t>FO-014</t>
+          <t>SET-012</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t>Front Office</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C137" s="10" t="inlineStr">
         <is>
-          <t>/downtime</t>
+          <t>/setup/property</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
         <is>
-          <t>A printable downtime pack: arrivals due, in-house guests with balance, departures due, ten blank lines for new guests on paper, and a short paper routine. Staff print it when the internet or system is down.</t>
+          <t>A manager sets the longest stay (1 to 365 nights) and how long a tentative booking holds its room (1 to 720 hours) for each property.</t>
         </is>
       </c>
       <c r="E137" s="10" t="inlineStr">
         <is>
-          <t>BR-006</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G137" s="10" t="inlineStr">
@@ -11401,33 +11405,33 @@
       </c>
       <c r="H137" s="10" t="inlineStr">
         <is>
-          <t>fo.view</t>
+          <t>setup.property.edit</t>
         </is>
       </c>
       <c r="I137" s="10" t="inlineStr"/>
       <c r="J137" s="10" t="inlineStr">
         <is>
-          <t>a hotel with guests in house</t>
+          <t>a property with the default rules (30 nights, 24 hours)</t>
         </is>
       </c>
       <c r="K137" s="10" t="inlineStr">
         <is>
-          <t>a front desk user opens Downtime pack and prints</t>
+          <t>a manager saves new booking rules</t>
         </is>
       </c>
       <c r="L137" s="10" t="inlineStr">
         <is>
-          <t>the lists show room, guest, phone, departure and the folio balance from the database, with blank lines and the paper routine</t>
+          <t>new bookings use them, bad values are refused with E_INVALID, and the change is audited with old and new values</t>
         </is>
       </c>
       <c r="M137" s="10" t="inlineStr">
         <is>
-          <t>src/routes/_authenticated/_app/downtime.tsx</t>
+          <t>set_booking_rules; Booking rules on Setup, Property</t>
         </is>
       </c>
       <c r="N137" s="10" t="inlineStr">
         <is>
-          <t>browser: downtime-pack.spec (1)</t>
+          <t>42_booking_rules (9)</t>
         </is>
       </c>
       <c r="O137" s="10" t="inlineStr">
@@ -11437,87 +11441,165 @@
       </c>
       <c r="P137" s="10" t="inlineStr">
         <is>
-          <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
+          <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="10" t="inlineStr">
         <is>
+          <t>FO-014</t>
+        </is>
+      </c>
+      <c r="B138" s="10" t="inlineStr">
+        <is>
+          <t>Front Office</t>
+        </is>
+      </c>
+      <c r="C138" s="10" t="inlineStr">
+        <is>
+          <t>/downtime</t>
+        </is>
+      </c>
+      <c r="D138" s="10" t="inlineStr">
+        <is>
+          <t>A printable downtime pack: arrivals due, in-house guests with balance, departures due, ten blank lines for new guests on paper, and a short paper routine. Staff print it when the internet or system is down.</t>
+        </is>
+      </c>
+      <c r="E138" s="10" t="inlineStr">
+        <is>
+          <t>BR-006</t>
+        </is>
+      </c>
+      <c r="F138" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G138" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H138" s="10" t="inlineStr">
+        <is>
+          <t>fo.view</t>
+        </is>
+      </c>
+      <c r="I138" s="10" t="inlineStr"/>
+      <c r="J138" s="10" t="inlineStr">
+        <is>
+          <t>a hotel with guests in house</t>
+        </is>
+      </c>
+      <c r="K138" s="10" t="inlineStr">
+        <is>
+          <t>a front desk user opens Downtime pack and prints</t>
+        </is>
+      </c>
+      <c r="L138" s="10" t="inlineStr">
+        <is>
+          <t>the lists show room, guest, phone, departure and the folio balance from the database, with blank lines and the paper routine</t>
+        </is>
+      </c>
+      <c r="M138" s="10" t="inlineStr">
+        <is>
+          <t>src/routes/_authenticated/_app/downtime.tsx</t>
+        </is>
+      </c>
+      <c r="N138" s="10" t="inlineStr">
+        <is>
+          <t>browser: downtime-pack.spec (1)</t>
+        </is>
+      </c>
+      <c r="O138" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P138" s="10" t="inlineStr">
+        <is>
+          <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="10" t="inlineStr">
+        <is>
           <t>DAY-007</t>
         </is>
       </c>
-      <c r="B138" s="10" t="inlineStr">
+      <c r="B139" s="10" t="inlineStr">
         <is>
           <t>Business Date</t>
         </is>
       </c>
-      <c r="C138" s="10" t="inlineStr">
+      <c r="C139" s="10" t="inlineStr">
         <is>
           <t>Notifications bell</t>
         </is>
       </c>
-      <c r="D138" s="10" t="inlineStr">
+      <c r="D139" s="10" t="inlineStr">
         <is>
           <t>In the last hour before a property rolls its business date, if a cashier shift is still open, users who can run the night audit get one warning that night. The roll does not wait.</t>
         </is>
       </c>
-      <c r="E138" s="10" t="inlineStr">
+      <c r="E139" s="10" t="inlineStr">
         <is>
           <t>BR-016</t>
         </is>
       </c>
-      <c r="F138" s="10" t="inlineStr">
+      <c r="F139" s="10" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="G138" s="10" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H138" s="10" t="inlineStr">
+      <c r="G139" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H139" s="10" t="inlineStr">
         <is>
           <t>fin.nightaudit.run</t>
         </is>
       </c>
-      <c r="I138" s="10" t="inlineStr">
+      <c r="I139" s="10" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="J138" s="10" t="inlineStr">
+      <c r="J139" s="10" t="inlineStr">
         <is>
           <t>a cashier shift is still open</t>
         </is>
       </c>
-      <c r="K138" s="10" t="inlineStr">
+      <c r="K139" s="10" t="inlineStr">
         <is>
           <t>the roll time is less than 60 minutes away</t>
         </is>
       </c>
-      <c r="L138" s="10" t="inlineStr">
+      <c r="L139" s="10" t="inlineStr">
         <is>
           <t>each night audit user gets one rollover_warning notification for that business date; none earlier, none after the roll time, none if no shift is open, none twice</t>
         </is>
       </c>
-      <c r="M138" s="10" t="inlineStr">
+      <c r="M139" s="10" t="inlineStr">
         <is>
           <t>app.warn_before_rollover; cron job rollover-warning</t>
         </is>
       </c>
-      <c r="N138" s="10" t="inlineStr">
+      <c r="N139" s="10" t="inlineStr">
         <is>
           <t>43_rollover_warning (9)</t>
         </is>
       </c>
-      <c r="O138" s="10" t="inlineStr">
+      <c r="O139" s="10" t="inlineStr">
         <is>
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P138" s="10" t="inlineStr">
+      <c r="P139" s="10" t="inlineStr">
         <is>
           <t>Added 8 Oct 2026. Warning only; the hard gate stays in R2 (DAY-005).</t>
         </is>

</xml_diff>

<commit_message>
Add the owner summary: yesterday at a glance on the dashboard (RPT-007)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P139"/>
+  <dimension ref="A1:P140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10594,27 +10594,27 @@
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>RPT-007</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
         <is>
-          <t>AI helpers</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C127" s="10" t="inlineStr">
         <is>
-          <t>Dashboard, Admin</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
+          <t>The owner summary: last night's occupancy and revenue, money collected by payment method, today's arrivals, departures and rooms, what is waiting, and old unpaid bills, as plain sentences built in the database. Works with AI off; a later daily email can send the same text.</t>
         </is>
       </c>
       <c r="E127" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F127" s="10" t="inlineStr">
@@ -10629,33 +10629,37 @@
       </c>
       <c r="H127" s="10" t="inlineStr">
         <is>
-          <t>adm.ai.manage</t>
-        </is>
-      </c>
-      <c r="I127" s="10" t="inlineStr"/>
+          <t>rpt.finance.view, rpt.operations.view</t>
+        </is>
+      </c>
+      <c r="I127" s="10" t="inlineStr">
+        <is>
+          <t>Reads the morning brief facts</t>
+        </is>
+      </c>
       <c r="J127" s="10" t="inlineStr">
         <is>
-          <t>a new hotel</t>
+          <t>a hotel with a closed day and payments on it</t>
         </is>
       </c>
       <c r="K127" s="10" t="inlineStr">
         <is>
-          <t>a manager opens Admin, AI helpers</t>
+          <t>the owner opens the dashboard</t>
         </is>
       </c>
       <c r="L127" s="10" t="inlineStr">
         <is>
-          <t>nothing runs until they switch it on and the change is in the audit log</t>
+          <t>sees yesterday at a glance with the money collected by method; front desk without finance reports is refused</t>
         </is>
       </c>
       <c r="M127" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
+          <t>owner_summary</t>
         </is>
       </c>
       <c r="N127" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (11)</t>
+          <t>47_owner_summary (8); browser: owner-summary</t>
         </is>
       </c>
       <c r="O127" s="10" t="inlineStr">
@@ -10665,14 +10669,14 @@
       </c>
       <c r="P127" s="10" t="inlineStr">
         <is>
-          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
+          <t>Email delivery waits on the sending domain and email account.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
         <is>
-          <t>AI-002</t>
+          <t>AI-001</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
@@ -10687,7 +10691,7 @@
       </c>
       <c r="D128" s="10" t="inlineStr">
         <is>
-          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
+          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
         </is>
       </c>
       <c r="E128" s="10" t="inlineStr">
@@ -10707,28 +10711,28 @@
       </c>
       <c r="H128" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view, rpt.operations.view</t>
+          <t>adm.ai.manage</t>
         </is>
       </c>
       <c r="I128" s="10" t="inlineStr"/>
       <c r="J128" s="10" t="inlineStr">
         <is>
-          <t>a hotel with guests, approvals and overdue bills</t>
+          <t>a new hotel</t>
         </is>
       </c>
       <c r="K128" s="10" t="inlineStr">
         <is>
-          <t>a brief is started</t>
+          <t>a manager opens Admin, AI helpers</t>
         </is>
       </c>
       <c r="L128" s="10" t="inlineStr">
         <is>
-          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
+          <t>nothing runs until they switch it on and the change is in the audit log</t>
         </is>
       </c>
       <c r="M128" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
+          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
         </is>
       </c>
       <c r="N128" s="10" t="inlineStr">
@@ -10743,14 +10747,14 @@
       </c>
       <c r="P128" s="10" t="inlineStr">
         <is>
-          <t>Overdue means unpaid more than 30 days after departure.</t>
+          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
         <is>
-          <t>AI-003</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
@@ -10765,7 +10769,7 @@
       </c>
       <c r="D129" s="10" t="inlineStr">
         <is>
-          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
+          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
         </is>
       </c>
       <c r="E129" s="10" t="inlineStr">
@@ -10785,33 +10789,33 @@
       </c>
       <c r="H129" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view</t>
+          <t>rpt.finance.view, rpt.operations.view</t>
         </is>
       </c>
       <c r="I129" s="10" t="inlineStr"/>
       <c r="J129" s="10" t="inlineStr">
         <is>
-          <t>a limit of 2</t>
+          <t>a hotel with guests, approvals and overdue bills</t>
         </is>
       </c>
       <c r="K129" s="10" t="inlineStr">
         <is>
-          <t>a third brief is requested</t>
+          <t>a brief is started</t>
         </is>
       </c>
       <c r="L129" s="10" t="inlineStr">
         <is>
-          <t>it is refused until a failed call frees a slot or the month turns</t>
+          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
         </is>
       </c>
       <c r="M129" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
+          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
         </is>
       </c>
       <c r="N129" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (5)</t>
+          <t>37_ai_brief (11)</t>
         </is>
       </c>
       <c r="O129" s="10" t="inlineStr">
@@ -10819,12 +10823,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P129" s="10" t="inlineStr"/>
+      <c r="P129" s="10" t="inlineStr">
+        <is>
+          <t>Overdue means unpaid more than 30 days after departure.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
         <is>
-          <t>AI-004</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
@@ -10839,7 +10847,7 @@
       </c>
       <c r="D130" s="10" t="inlineStr">
         <is>
-          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
+          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
         </is>
       </c>
       <c r="E130" s="10" t="inlineStr">
@@ -10859,33 +10867,33 @@
       </c>
       <c r="H130" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view, rpt.operations.view</t>
+          <t>rpt.finance.view</t>
         </is>
       </c>
       <c r="I130" s="10" t="inlineStr"/>
       <c r="J130" s="10" t="inlineStr">
         <is>
-          <t>front desk, housekeeping, another hotel</t>
+          <t>a limit of 2</t>
         </is>
       </c>
       <c r="K130" s="10" t="inlineStr">
         <is>
-          <t>they ask for the brief or touch the tables</t>
+          <t>a third brief is requested</t>
         </is>
       </c>
       <c r="L130" s="10" t="inlineStr">
         <is>
-          <t>they are refused</t>
+          <t>it is refused until a failed call frees a slot or the month turns</t>
         </is>
       </c>
       <c r="M130" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql</t>
+          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
         </is>
       </c>
       <c r="N130" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (7)</t>
+          <t>37_ai_brief (5)</t>
         </is>
       </c>
       <c r="O130" s="10" t="inlineStr">
@@ -10898,7 +10906,7 @@
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
         <is>
-          <t>AI-005</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
@@ -10913,7 +10921,7 @@
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
+          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
         </is>
       </c>
       <c r="E131" s="10" t="inlineStr">
@@ -10933,33 +10941,33 @@
       </c>
       <c r="H131" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>rpt.finance.view, rpt.operations.view</t>
         </is>
       </c>
       <c r="I131" s="10" t="inlineStr"/>
       <c r="J131" s="10" t="inlineStr">
         <is>
-          <t>a draft that rounds or invents a figure</t>
+          <t>front desk, housekeeping, another hotel</t>
         </is>
       </c>
       <c r="K131" s="10" t="inlineStr">
         <is>
-          <t>the brief is written</t>
+          <t>they ask for the brief or touch the tables</t>
         </is>
       </c>
       <c r="L131" s="10" t="inlineStr">
         <is>
-          <t>the plain database lines are shown instead, with a note</t>
+          <t>they are refused</t>
         </is>
       </c>
       <c r="M131" s="10" t="inlineStr">
         <is>
-          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
+          <t>20261013140000_ai_morning_brief.sql</t>
         </is>
       </c>
       <c r="N131" s="10" t="inlineStr">
         <is>
-          <t>browser unit: ai-brief-unit (8)</t>
+          <t>37_ai_brief (7)</t>
         </is>
       </c>
       <c r="O131" s="10" t="inlineStr">
@@ -10967,31 +10975,27 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P131" s="10" t="inlineStr">
-        <is>
-          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
-        </is>
-      </c>
+      <c r="P131" s="10" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="10" t="inlineStr">
         <is>
-          <t>SET-010</t>
+          <t>AI-005</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>AI helpers</t>
         </is>
       </c>
       <c r="C132" s="10" t="inlineStr">
         <is>
-          <t>Setup, Rooms</t>
+          <t>Dashboard, Admin</t>
         </is>
       </c>
       <c r="D132" s="10" t="inlineStr">
         <is>
-          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
+          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
         </is>
       </c>
       <c r="E132" s="10" t="inlineStr">
@@ -11011,33 +11015,33 @@
       </c>
       <c r="H132" s="10" t="inlineStr">
         <is>
-          <t>setup.room.manage</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I132" s="10" t="inlineStr"/>
       <c r="J132" s="10" t="inlineStr">
         <is>
-          <t>a list of room types and rooms</t>
+          <t>a draft that rounds or invents a figure</t>
         </is>
       </c>
       <c r="K132" s="10" t="inlineStr">
         <is>
-          <t>the manager previews and then applies it</t>
+          <t>the brief is written</t>
         </is>
       </c>
       <c r="L132" s="10" t="inlineStr">
         <is>
-          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
+          <t>the plain database lines are shown instead, with a note</t>
         </is>
       </c>
       <c r="M132" s="10" t="inlineStr">
         <is>
-          <t>20261013150000_setup_import.sql: apply_setup_import</t>
+          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
         </is>
       </c>
       <c r="N132" s="10" t="inlineStr">
         <is>
-          <t>38_setup_import (29)</t>
+          <t>browser unit: ai-brief-unit (8)</t>
         </is>
       </c>
       <c r="O132" s="10" t="inlineStr">
@@ -11047,19 +11051,19 @@
       </c>
       <c r="P132" s="10" t="inlineStr">
         <is>
-          <t>The AI only drafts the list. This function is the check.</t>
+          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
         <is>
-          <t>AI-006</t>
+          <t>SET-010</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
         <is>
-          <t>AI helpers</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C133" s="10" t="inlineStr">
@@ -11069,7 +11073,7 @@
       </c>
       <c r="D133" s="10" t="inlineStr">
         <is>
-          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
+          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
         </is>
       </c>
       <c r="E133" s="10" t="inlineStr">
@@ -11095,27 +11099,27 @@
       <c r="I133" s="10" t="inlineStr"/>
       <c r="J133" s="10" t="inlineStr">
         <is>
-          <t>AI switched on with a limit of 1</t>
+          <t>a list of room types and rooms</t>
         </is>
       </c>
       <c r="K133" s="10" t="inlineStr">
         <is>
-          <t>an import draft is started twice</t>
+          <t>the manager previews and then applies it</t>
         </is>
       </c>
       <c r="L133" s="10" t="inlineStr">
         <is>
-          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
+          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
         </is>
       </c>
       <c r="M133" s="10" t="inlineStr">
         <is>
-          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
+          <t>20261013150000_setup_import.sql: apply_setup_import</t>
         </is>
       </c>
       <c r="N133" s="10" t="inlineStr">
         <is>
-          <t>38_setup_import (8)</t>
+          <t>38_setup_import (29)</t>
         </is>
       </c>
       <c r="O133" s="10" t="inlineStr">
@@ -11123,12 +11127,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P133" s="10" t="inlineStr"/>
+      <c r="P133" s="10" t="inlineStr">
+        <is>
+          <t>The AI only drafts the list. This function is the check.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
         <is>
-          <t>AI-007</t>
+          <t>AI-006</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
@@ -11143,7 +11151,7 @@
       </c>
       <c r="D134" s="10" t="inlineStr">
         <is>
-          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
+          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
         </is>
       </c>
       <c r="E134" s="10" t="inlineStr">
@@ -11169,27 +11177,27 @@
       <c r="I134" s="10" t="inlineStr"/>
       <c r="J134" s="10" t="inlineStr">
         <is>
-          <t>a pasted list</t>
+          <t>AI switched on with a limit of 1</t>
         </is>
       </c>
       <c r="K134" s="10" t="inlineStr">
         <is>
-          <t>the assistant drafts it</t>
+          <t>an import draft is started twice</t>
         </is>
       </c>
       <c r="L134" s="10" t="inlineStr">
         <is>
-          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
+          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
         </is>
       </c>
       <c r="M134" s="10" t="inlineStr">
         <is>
-          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
+          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
         </is>
       </c>
       <c r="N134" s="10" t="inlineStr">
         <is>
-          <t>browser unit: setup-import-unit (9)</t>
+          <t>38_setup_import (8)</t>
         </is>
       </c>
       <c r="O134" s="10" t="inlineStr">
@@ -11197,36 +11205,32 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P134" s="10" t="inlineStr">
-        <is>
-          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
-        </is>
-      </c>
+      <c r="P134" s="10" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
         <is>
-          <t>SET-011</t>
+          <t>AI-007</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>AI helpers</t>
         </is>
       </c>
       <c r="C135" s="10" t="inlineStr">
         <is>
-          <t>/setup; /dashboard</t>
+          <t>Setup, Rooms</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr">
         <is>
-          <t>A new hotel sees a checklist of what is left to set up: property details, room types, rooms, rates, taxes, payment methods and staff. Each step says what is missing and links to the right screen. The list comes from the hotel's own data, so it is always current.</t>
+          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
         </is>
       </c>
       <c r="E135" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F135" s="10" t="inlineStr">
@@ -11241,37 +11245,33 @@
       </c>
       <c r="H135" s="10" t="inlineStr">
         <is>
-          <t>any setup permission</t>
-        </is>
-      </c>
-      <c r="I135" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>setup.room.manage</t>
+        </is>
+      </c>
+      <c r="I135" s="10" t="inlineStr"/>
       <c r="J135" s="10" t="inlineStr">
         <is>
-          <t>a hotel that is part way through setup</t>
+          <t>a pasted list</t>
         </is>
       </c>
       <c r="K135" s="10" t="inlineStr">
         <is>
-          <t>a manager opens Setup or the Dashboard</t>
+          <t>the assistant drafts it</t>
         </is>
       </c>
       <c r="L135" s="10" t="inlineStr">
         <is>
-          <t>the steps already done are ticked and the next one is linked; once all seven are done the checklist goes away</t>
+          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
         </is>
       </c>
       <c r="M135" s="10" t="inlineStr">
         <is>
-          <t>setup_progress</t>
+          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
         </is>
       </c>
       <c r="N135" s="10" t="inlineStr">
         <is>
-          <t>40_guided_setup (30)</t>
+          <t>browser unit: setup-import-unit (9)</t>
         </is>
       </c>
       <c r="O135" s="10" t="inlineStr">
@@ -11281,39 +11281,39 @@
       </c>
       <c r="P135" s="10" t="inlineStr">
         <is>
-          <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
+          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
         <is>
-          <t>NFR-006</t>
+          <t>SET-011</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
         <is>
-          <t>Non-functional</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C136" s="10" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/setup; /dashboard</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr">
         <is>
-          <t>The last room of a type is sold once, however many desks book at the same moment, and a repeated booking never doubles.</t>
+          <t>A new hotel sees a checklist of what is left to set up: property details, room types, rooms, rates, taxes, payment methods and staff. Each step says what is missing and links to the right screen. The list comes from the hotel's own data, so it is always current.</t>
         </is>
       </c>
       <c r="E136" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F136" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G136" s="10" t="inlineStr">
@@ -11323,37 +11323,37 @@
       </c>
       <c r="H136" s="10" t="inlineStr">
         <is>
+          <t>any setup permission</t>
+        </is>
+      </c>
+      <c r="I136" s="10" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I136" s="10" t="inlineStr">
-        <is>
-          <t>Rule: Safe last-room booking</t>
-        </is>
-      </c>
       <c r="J136" s="10" t="inlineStr">
         <is>
-          <t>one room of a type is left and several desks book it together</t>
+          <t>a hotel that is part way through setup</t>
         </is>
       </c>
       <c r="K136" s="10" t="inlineStr">
         <is>
-          <t>all of them submit at the same moment</t>
+          <t>a manager opens Setup or the Dashboard</t>
         </is>
       </c>
       <c r="L136" s="10" t="inlineStr">
         <is>
-          <t>exactly one booking succeeds, the rest get E_NO_AVAILABILITY, and nothing is oversold</t>
+          <t>the steps already done are ticked and the next one is linked; once all seven are done the checklist goes away</t>
         </is>
       </c>
       <c r="M136" s="10" t="inlineStr">
         <is>
-          <t>create_reservation, assert_available</t>
+          <t>setup_progress</t>
         </is>
       </c>
       <c r="N136" s="10" t="inlineStr">
         <is>
-          <t>concurrency/last_room.sh (6)</t>
+          <t>40_guided_setup (30)</t>
         </is>
       </c>
       <c r="O136" s="10" t="inlineStr">
@@ -11363,29 +11363,29 @@
       </c>
       <c r="P136" s="10" t="inlineStr">
         <is>
-          <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
+          <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
         <is>
-          <t>SET-012</t>
+          <t>NFR-006</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Non-functional</t>
         </is>
       </c>
       <c r="C137" s="10" t="inlineStr">
         <is>
-          <t>/setup/property</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
         <is>
-          <t>A manager sets the longest stay (1 to 365 nights) and how long a tentative booking holds its room (1 to 720 hours) for each property.</t>
+          <t>The last room of a type is sold once, however many desks book at the same moment, and a repeated booking never doubles.</t>
         </is>
       </c>
       <c r="E137" s="10" t="inlineStr">
@@ -11395,7 +11395,7 @@
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G137" s="10" t="inlineStr">
@@ -11405,33 +11405,37 @@
       </c>
       <c r="H137" s="10" t="inlineStr">
         <is>
-          <t>setup.property.edit</t>
-        </is>
-      </c>
-      <c r="I137" s="10" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I137" s="10" t="inlineStr">
+        <is>
+          <t>Rule: Safe last-room booking</t>
+        </is>
+      </c>
       <c r="J137" s="10" t="inlineStr">
         <is>
-          <t>a property with the default rules (30 nights, 24 hours)</t>
+          <t>one room of a type is left and several desks book it together</t>
         </is>
       </c>
       <c r="K137" s="10" t="inlineStr">
         <is>
-          <t>a manager saves new booking rules</t>
+          <t>all of them submit at the same moment</t>
         </is>
       </c>
       <c r="L137" s="10" t="inlineStr">
         <is>
-          <t>new bookings use them, bad values are refused with E_INVALID, and the change is audited with old and new values</t>
+          <t>exactly one booking succeeds, the rest get E_NO_AVAILABILITY, and nothing is oversold</t>
         </is>
       </c>
       <c r="M137" s="10" t="inlineStr">
         <is>
-          <t>set_booking_rules; Booking rules on Setup, Property</t>
+          <t>create_reservation, assert_available</t>
         </is>
       </c>
       <c r="N137" s="10" t="inlineStr">
         <is>
-          <t>42_booking_rules (9)</t>
+          <t>concurrency/last_room.sh (6)</t>
         </is>
       </c>
       <c r="O137" s="10" t="inlineStr">
@@ -11441,39 +11445,39 @@
       </c>
       <c r="P137" s="10" t="inlineStr">
         <is>
-          <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
+          <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="10" t="inlineStr">
         <is>
-          <t>FO-014</t>
+          <t>SET-012</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
         <is>
-          <t>Front Office</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C138" s="10" t="inlineStr">
         <is>
-          <t>/downtime</t>
+          <t>/setup/property</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr">
         <is>
-          <t>A printable downtime pack: arrivals due, in-house guests with balance, departures due, ten blank lines for new guests on paper, and a short paper routine. Staff print it when the internet or system is down.</t>
+          <t>A manager sets the longest stay (1 to 365 nights) and how long a tentative booking holds its room (1 to 720 hours) for each property.</t>
         </is>
       </c>
       <c r="E138" s="10" t="inlineStr">
         <is>
-          <t>BR-006</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F138" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G138" s="10" t="inlineStr">
@@ -11483,33 +11487,33 @@
       </c>
       <c r="H138" s="10" t="inlineStr">
         <is>
-          <t>fo.view</t>
+          <t>setup.property.edit</t>
         </is>
       </c>
       <c r="I138" s="10" t="inlineStr"/>
       <c r="J138" s="10" t="inlineStr">
         <is>
-          <t>a hotel with guests in house</t>
+          <t>a property with the default rules (30 nights, 24 hours)</t>
         </is>
       </c>
       <c r="K138" s="10" t="inlineStr">
         <is>
-          <t>a front desk user opens Downtime pack and prints</t>
+          <t>a manager saves new booking rules</t>
         </is>
       </c>
       <c r="L138" s="10" t="inlineStr">
         <is>
-          <t>the lists show room, guest, phone, departure and the folio balance from the database, with blank lines and the paper routine</t>
+          <t>new bookings use them, bad values are refused with E_INVALID, and the change is audited with old and new values</t>
         </is>
       </c>
       <c r="M138" s="10" t="inlineStr">
         <is>
-          <t>src/routes/_authenticated/_app/downtime.tsx</t>
+          <t>set_booking_rules; Booking rules on Setup, Property</t>
         </is>
       </c>
       <c r="N138" s="10" t="inlineStr">
         <is>
-          <t>browser: downtime-pack.spec (1)</t>
+          <t>42_booking_rules (9)</t>
         </is>
       </c>
       <c r="O138" s="10" t="inlineStr">
@@ -11519,87 +11523,165 @@
       </c>
       <c r="P138" s="10" t="inlineStr">
         <is>
-          <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
+          <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="10" t="inlineStr">
         <is>
+          <t>FO-014</t>
+        </is>
+      </c>
+      <c r="B139" s="10" t="inlineStr">
+        <is>
+          <t>Front Office</t>
+        </is>
+      </c>
+      <c r="C139" s="10" t="inlineStr">
+        <is>
+          <t>/downtime</t>
+        </is>
+      </c>
+      <c r="D139" s="10" t="inlineStr">
+        <is>
+          <t>A printable downtime pack: arrivals due, in-house guests with balance, departures due, ten blank lines for new guests on paper, and a short paper routine. Staff print it when the internet or system is down.</t>
+        </is>
+      </c>
+      <c r="E139" s="10" t="inlineStr">
+        <is>
+          <t>BR-006</t>
+        </is>
+      </c>
+      <c r="F139" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G139" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H139" s="10" t="inlineStr">
+        <is>
+          <t>fo.view</t>
+        </is>
+      </c>
+      <c r="I139" s="10" t="inlineStr"/>
+      <c r="J139" s="10" t="inlineStr">
+        <is>
+          <t>a hotel with guests in house</t>
+        </is>
+      </c>
+      <c r="K139" s="10" t="inlineStr">
+        <is>
+          <t>a front desk user opens Downtime pack and prints</t>
+        </is>
+      </c>
+      <c r="L139" s="10" t="inlineStr">
+        <is>
+          <t>the lists show room, guest, phone, departure and the folio balance from the database, with blank lines and the paper routine</t>
+        </is>
+      </c>
+      <c r="M139" s="10" t="inlineStr">
+        <is>
+          <t>src/routes/_authenticated/_app/downtime.tsx</t>
+        </is>
+      </c>
+      <c r="N139" s="10" t="inlineStr">
+        <is>
+          <t>browser: downtime-pack.spec (1)</t>
+        </is>
+      </c>
+      <c r="O139" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P139" s="10" t="inlineStr">
+        <is>
+          <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="10" t="inlineStr">
+        <is>
           <t>DAY-007</t>
         </is>
       </c>
-      <c r="B139" s="10" t="inlineStr">
+      <c r="B140" s="10" t="inlineStr">
         <is>
           <t>Business Date</t>
         </is>
       </c>
-      <c r="C139" s="10" t="inlineStr">
+      <c r="C140" s="10" t="inlineStr">
         <is>
           <t>Notifications bell</t>
         </is>
       </c>
-      <c r="D139" s="10" t="inlineStr">
+      <c r="D140" s="10" t="inlineStr">
         <is>
           <t>In the last hour before a property rolls its business date, if a cashier shift is still open, users who can run the night audit get one warning that night. The roll does not wait.</t>
         </is>
       </c>
-      <c r="E139" s="10" t="inlineStr">
+      <c r="E140" s="10" t="inlineStr">
         <is>
           <t>BR-016</t>
         </is>
       </c>
-      <c r="F139" s="10" t="inlineStr">
+      <c r="F140" s="10" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="G139" s="10" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H139" s="10" t="inlineStr">
+      <c r="G140" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H140" s="10" t="inlineStr">
         <is>
           <t>fin.nightaudit.run</t>
         </is>
       </c>
-      <c r="I139" s="10" t="inlineStr">
+      <c r="I140" s="10" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="J139" s="10" t="inlineStr">
+      <c r="J140" s="10" t="inlineStr">
         <is>
           <t>a cashier shift is still open</t>
         </is>
       </c>
-      <c r="K139" s="10" t="inlineStr">
+      <c r="K140" s="10" t="inlineStr">
         <is>
           <t>the roll time is less than 60 minutes away</t>
         </is>
       </c>
-      <c r="L139" s="10" t="inlineStr">
+      <c r="L140" s="10" t="inlineStr">
         <is>
           <t>each night audit user gets one rollover_warning notification for that business date; none earlier, none after the roll time, none if no shift is open, none twice</t>
         </is>
       </c>
-      <c r="M139" s="10" t="inlineStr">
+      <c r="M140" s="10" t="inlineStr">
         <is>
           <t>app.warn_before_rollover; cron job rollover-warning</t>
         </is>
       </c>
-      <c r="N139" s="10" t="inlineStr">
+      <c r="N140" s="10" t="inlineStr">
         <is>
           <t>43_rollover_warning (9)</t>
         </is>
       </c>
-      <c r="O139" s="10" t="inlineStr">
+      <c r="O140" s="10" t="inlineStr">
         <is>
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P139" s="10" t="inlineStr">
+      <c r="P140" s="10" t="inlineStr">
         <is>
           <t>Added 8 Oct 2026. Warning only; the hard gate stays in R2 (DAY-005).</t>
         </is>

</xml_diff>

<commit_message>
Owner summary: a payment reversed the same day nets to zero (RPT-007)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -10659,7 +10659,7 @@
       </c>
       <c r="N127" s="10" t="inlineStr">
         <is>
-          <t>47_owner_summary (8); browser: owner-summary</t>
+          <t>47_owner_summary (9); browser: owner-summary</t>
         </is>
       </c>
       <c r="O127" s="10" t="inlineStr">
@@ -10669,7 +10669,7 @@
       </c>
       <c r="P127" s="10" t="inlineStr">
         <is>
-          <t>Email delivery waits on the sending domain and email account.</t>
+          <t>Email delivery waits on the sending domain and email account. Collected money nets payment reversals the same day (migration 20261015130000).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Photos on maintenance tickets (MNT-004)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P141"/>
+  <dimension ref="A1:P142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6744,27 +6744,27 @@
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
         <is>
-          <t>SVC-001</t>
+          <t>MNT-004</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>Guest Service</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>FO-01</t>
+          <t>MNT-02</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>Guest requests are captured, assigned, progressed and completed.</t>
+          <t>Staff add up to 5 photos to a maintenance ticket from the phone. Photos are private, and uploads and views are audited by ids only.</t>
         </is>
       </c>
       <c r="E78" s="10" t="inlineStr">
         <is>
-          <t>BR-006</t>
+          <t>BR-012</t>
         </is>
       </c>
       <c r="F78" s="10" t="inlineStr">
@@ -6779,37 +6779,37 @@
       </c>
       <c r="H78" s="10" t="inlineStr">
         <is>
-          <t>svc.request.create, svc.request.manage</t>
+          <t>mnt.ticket.create, mnt.ticket.work, mnt.view, mnt.ticket.assign</t>
         </is>
       </c>
       <c r="I78" s="10" t="inlineStr">
         <is>
-          <t>Workflow WF05</t>
+          <t>Rule: Private storage</t>
         </is>
       </c>
       <c r="J78" s="10" t="inlineStr">
         <is>
-          <t>a guest in house</t>
+          <t>an open ticket</t>
         </is>
       </c>
       <c r="K78" s="10" t="inlineStr">
         <is>
-          <t>staff log a request and it is assigned, started and completed</t>
+          <t>an attendant adds a photo, others view it, a supervisor removes it</t>
         </is>
       </c>
       <c r="L78" s="10" t="inlineStr">
         <is>
-          <t>it is tied to the guest's room and finishes once</t>
+          <t>only people tied to the ticket can add or view, the limit is 5, a removed photo is cleaned from storage, and a finished ticket takes no new photos</t>
         </is>
       </c>
       <c r="M78" s="10" t="inlineStr">
         <is>
-          <t>create_service_request, assign_service_request, start_service_request, complete_service_request</t>
+          <t>begin_ticket_photo_upload, finish_ticket_photo_upload, list_ticket_photos, open_ticket_photo, delete_ticket_photo</t>
         </is>
       </c>
       <c r="N78" s="10" t="inlineStr">
         <is>
-          <t>17_more_features (3)</t>
+          <t>49_ticket_photos (17)</t>
         </is>
       </c>
       <c r="O78" s="10" t="inlineStr">
@@ -6822,7 +6822,7 @@
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>SVC-002</t>
+          <t>SVC-001</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
@@ -6832,17 +6832,17 @@
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>FO-01, FIN-01</t>
+          <t>FO-01</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>A chargeable request posts its charge, with tax, to the folio when completed.</t>
+          <t>Guest requests are captured, assigned, progressed and completed.</t>
         </is>
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
-          <t>BR-013</t>
+          <t>BR-006</t>
         </is>
       </c>
       <c r="F79" s="10" t="inlineStr">
@@ -6857,7 +6857,7 @@
       </c>
       <c r="H79" s="10" t="inlineStr">
         <is>
-          <t>svc.request.manage, fin.charge.post</t>
+          <t>svc.request.create, svc.request.manage</t>
         </is>
       </c>
       <c r="I79" s="10" t="inlineStr">
@@ -6867,22 +6867,22 @@
       </c>
       <c r="J79" s="10" t="inlineStr">
         <is>
-          <t>a chargeable laundry request of 3,000</t>
+          <t>a guest in house</t>
         </is>
       </c>
       <c r="K79" s="10" t="inlineStr">
         <is>
-          <t>it is completed</t>
+          <t>staff log a request and it is assigned, started and completed</t>
         </is>
       </c>
       <c r="L79" s="10" t="inlineStr">
         <is>
-          <t>3,000 plus tax is posted once to the guest's folio</t>
+          <t>it is tied to the guest's room and finishes once</t>
         </is>
       </c>
       <c r="M79" s="10" t="inlineStr">
         <is>
-          <t>complete_service_request</t>
+          <t>create_service_request, assign_service_request, start_service_request, complete_service_request</t>
         </is>
       </c>
       <c r="N79" s="10" t="inlineStr">
@@ -6900,22 +6900,22 @@
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>FIN-001</t>
+          <t>SVC-002</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Guest Service</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
         <is>
-          <t>FIN-01</t>
+          <t>FO-01, FIN-01</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t>Charges post with their tax lines; prices can include or exclude tax; the remainder of a rounding goes on the last tax line.</t>
+          <t>A chargeable request posts its charge, with tax, to the folio when completed.</t>
         </is>
       </c>
       <c r="E80" s="10" t="inlineStr">
@@ -6925,7 +6925,7 @@
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G80" s="10" t="inlineStr">
@@ -6935,37 +6935,37 @@
       </c>
       <c r="H80" s="10" t="inlineStr">
         <is>
-          <t>fin.charge.post</t>
+          <t>svc.request.manage, fin.charge.post</t>
         </is>
       </c>
       <c r="I80" s="10" t="inlineStr">
         <is>
-          <t>Rule: Business date</t>
+          <t>Workflow WF05</t>
         </is>
       </c>
       <c r="J80" s="10" t="inlineStr">
         <is>
-          <t>service charge 10% and VAT 7.5%</t>
+          <t>a chargeable laundry request of 3,000</t>
         </is>
       </c>
       <c r="K80" s="10" t="inlineStr">
         <is>
-          <t>a charge of 10,000 or an inclusive 11,825 is posted</t>
+          <t>it is completed</t>
         </is>
       </c>
       <c r="L80" s="10" t="inlineStr">
         <is>
-          <t>the folio owes 11,825 with a net of 10,000 either way</t>
+          <t>3,000 plus tax is posted once to the guest's folio</t>
         </is>
       </c>
       <c r="M80" s="10" t="inlineStr">
         <is>
-          <t>post_charge, compute_taxes, insert_with_tax</t>
+          <t>complete_service_request</t>
         </is>
       </c>
       <c r="N80" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (6)</t>
+          <t>17_more_features (3)</t>
         </is>
       </c>
       <c r="O80" s="10" t="inlineStr">
@@ -6978,7 +6978,7 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>FIN-002</t>
+          <t>FIN-001</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
@@ -6993,7 +6993,7 @@
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>Payments and deposits are recorded against a folio with a method; payments are taken outside the system in R1.</t>
+          <t>Charges post with their tax lines; prices can include or exclude tax; the remainder of a rounding goes on the last tax line.</t>
         </is>
       </c>
       <c r="E81" s="10" t="inlineStr">
@@ -7013,37 +7013,37 @@
       </c>
       <c r="H81" s="10" t="inlineStr">
         <is>
-          <t>fin.payment.post, fin.deposit.take</t>
+          <t>fin.charge.post</t>
         </is>
       </c>
       <c r="I81" s="10" t="inlineStr">
         <is>
-          <t>Rule: Payments in R1</t>
+          <t>Rule: Business date</t>
         </is>
       </c>
       <c r="J81" s="10" t="inlineStr">
         <is>
-          <t>a folio with a balance</t>
+          <t>service charge 10% and VAT 7.5%</t>
         </is>
       </c>
       <c r="K81" s="10" t="inlineStr">
         <is>
-          <t>staff record a cash payment or a deposit</t>
+          <t>a charge of 10,000 or an inclusive 11,825 is posted</t>
         </is>
       </c>
       <c r="L81" s="10" t="inlineStr">
         <is>
-          <t>the balance falls; a role without the matching permission is refused</t>
+          <t>the folio owes 11,825 with a net of 10,000 either way</t>
         </is>
       </c>
       <c r="M81" s="10" t="inlineStr">
         <is>
-          <t>post_payment</t>
+          <t>post_charge, compute_taxes, insert_with_tax</t>
         </is>
       </c>
       <c r="N81" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (2)</t>
+          <t>12_ledger (6)</t>
         </is>
       </c>
       <c r="O81" s="10" t="inlineStr">
@@ -7056,7 +7056,7 @@
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>FIN-003</t>
+          <t>FIN-002</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t>Foreign-currency postings store the amount, currency, exchange rate and base amount.</t>
+          <t>Payments and deposits are recorded against a folio with a method; payments are taken outside the system in R1.</t>
         </is>
       </c>
       <c r="E82" s="10" t="inlineStr">
@@ -7081,7 +7081,7 @@
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G82" s="10" t="inlineStr">
@@ -7091,32 +7091,32 @@
       </c>
       <c r="H82" s="10" t="inlineStr">
         <is>
-          <t>fin.payment.post</t>
+          <t>fin.payment.post, fin.deposit.take</t>
         </is>
       </c>
       <c r="I82" s="10" t="inlineStr">
         <is>
-          <t>Rule: Multi-currency</t>
+          <t>Rule: Payments in R1</t>
         </is>
       </c>
       <c r="J82" s="10" t="inlineStr">
         <is>
-          <t>USD 10 at 1,500</t>
+          <t>a folio with a balance</t>
         </is>
       </c>
       <c r="K82" s="10" t="inlineStr">
         <is>
-          <t>it is posted</t>
+          <t>staff record a cash payment or a deposit</t>
         </is>
       </c>
       <c r="L82" s="10" t="inlineStr">
         <is>
-          <t>the row shows the rate and 15,000 in the base currency; the amount must respect the currency's decimals</t>
+          <t>the balance falls; a role without the matching permission is refused</t>
         </is>
       </c>
       <c r="M82" s="10" t="inlineStr">
         <is>
-          <t>insert_txn, fx_rate</t>
+          <t>post_payment</t>
         </is>
       </c>
       <c r="N82" s="10" t="inlineStr">
@@ -7134,7 +7134,7 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>FIN-004</t>
+          <t>FIN-003</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
@@ -7149,17 +7149,17 @@
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t>A discount within the user's limit posts at once; above the limit it waits for an approver who is not the requester.</t>
+          <t>Foreign-currency postings store the amount, currency, exchange rate and base amount.</t>
         </is>
       </c>
       <c r="E83" s="10" t="inlineStr">
         <is>
-          <t>BR-015</t>
+          <t>BR-013</t>
         </is>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G83" s="10" t="inlineStr">
@@ -7169,37 +7169,37 @@
       </c>
       <c r="H83" s="10" t="inlineStr">
         <is>
-          <t>fin.discount.apply, fin.discount.approve</t>
+          <t>fin.payment.post</t>
         </is>
       </c>
       <c r="I83" s="10" t="inlineStr">
         <is>
-          <t>Rule: Limits; Separation of duties</t>
+          <t>Rule: Multi-currency</t>
         </is>
       </c>
       <c r="J83" s="10" t="inlineStr">
         <is>
-          <t>a front desk limit of 5,000</t>
+          <t>USD 10 at 1,500</t>
         </is>
       </c>
       <c r="K83" s="10" t="inlineStr">
         <is>
-          <t>they apply 3,000 then 8,000</t>
+          <t>it is posted</t>
         </is>
       </c>
       <c r="L83" s="10" t="inlineStr">
         <is>
-          <t>the first posts; the second is pending, does not change the balance and can be approved or rejected (with a reason) by a manager</t>
+          <t>the row shows the rate and 15,000 in the base currency; the amount must respect the currency's decimals</t>
         </is>
       </c>
       <c r="M83" s="10" t="inlineStr">
         <is>
-          <t>apply_discount, decide_approval</t>
+          <t>insert_txn, fx_rate</t>
         </is>
       </c>
       <c r="N83" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (6)</t>
+          <t>12_ledger (2)</t>
         </is>
       </c>
       <c r="O83" s="10" t="inlineStr">
@@ -7212,7 +7212,7 @@
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>FIN-005</t>
+          <t>FIN-004</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t>Adjustments, reversals and refunds always need a second person and stay within the approver's limit.</t>
+          <t>A discount within the user's limit posts at once; above the limit it waits for an approver who is not the requester.</t>
         </is>
       </c>
       <c r="E84" s="10" t="inlineStr">
@@ -7247,37 +7247,37 @@
       </c>
       <c r="H84" s="10" t="inlineStr">
         <is>
-          <t>fin.adjust.post, fin.adjust.approve, fin.reverse.post, fin.refund.post, fin.refund.approve</t>
+          <t>fin.discount.apply, fin.discount.approve</t>
         </is>
       </c>
       <c r="I84" s="10" t="inlineStr">
         <is>
-          <t>Rule: Separation of duties, Limits</t>
+          <t>Rule: Limits; Separation of duties</t>
         </is>
       </c>
       <c r="J84" s="10" t="inlineStr">
         <is>
-          <t>an adjustment of 50,000 requested by a cashier</t>
+          <t>a front desk limit of 5,000</t>
         </is>
       </c>
       <c r="K84" s="10" t="inlineStr">
         <is>
-          <t>a manager with a 20,000 limit approves</t>
+          <t>they apply 3,000 then 8,000</t>
         </is>
       </c>
       <c r="L84" s="10" t="inlineStr">
         <is>
-          <t>it is refused with E_LIMIT; a senior approver can; nobody approves their own request</t>
+          <t>the first posts; the second is pending, does not change the balance and can be approved or rejected (with a reason) by a manager</t>
         </is>
       </c>
       <c r="M84" s="10" t="inlineStr">
         <is>
-          <t>request_adjustment, request_reversal, request_refund, decide_approval; check constraint approver_is_not_requester</t>
+          <t>apply_discount, decide_approval</t>
         </is>
       </c>
       <c r="N84" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (2)</t>
+          <t>12_ledger (6)</t>
         </is>
       </c>
       <c r="O84" s="10" t="inlineStr">
@@ -7290,7 +7290,7 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>FIN-006</t>
+          <t>FIN-005</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
@@ -7305,12 +7305,12 @@
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>A posted transaction is never edited or deleted; corrections are linked reversal, adjustment or refund rows.</t>
+          <t>Adjustments, reversals and refunds always need a second person and stay within the approver's limit.</t>
         </is>
       </c>
       <c r="E85" s="10" t="inlineStr">
         <is>
-          <t>BR-014, BR-015</t>
+          <t>BR-015</t>
         </is>
       </c>
       <c r="F85" s="10" t="inlineStr">
@@ -7325,37 +7325,37 @@
       </c>
       <c r="H85" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fin.adjust.post, fin.adjust.approve, fin.reverse.post, fin.refund.post, fin.refund.approve</t>
         </is>
       </c>
       <c r="I85" s="10" t="inlineStr">
         <is>
-          <t>Rule: Immutability</t>
+          <t>Rule: Separation of duties, Limits</t>
         </is>
       </c>
       <c r="J85" s="10" t="inlineStr">
         <is>
-          <t>a posted charge</t>
+          <t>an adjustment of 50,000 requested by a cashier</t>
         </is>
       </c>
       <c r="K85" s="10" t="inlineStr">
         <is>
-          <t>anyone, including the database owner, changes or deletes it</t>
+          <t>a manager with a 20,000 limit approves</t>
         </is>
       </c>
       <c r="L85" s="10" t="inlineStr">
         <is>
-          <t>the change is refused with E_IMMUTABLE; a reversal posts a linked row (with its tax lines) and a charge reverses only once</t>
+          <t>it is refused with E_LIMIT; a senior approver can; nobody approves their own request</t>
         </is>
       </c>
       <c r="M85" s="10" t="inlineStr">
         <is>
-          <t>txn_guard triggers; request_reversal</t>
+          <t>request_adjustment, request_reversal, request_refund, decide_approval; check constraint approver_is_not_requester</t>
         </is>
       </c>
       <c r="N85" s="10" t="inlineStr">
         <is>
-          <t>10_security (1); 12_ledger (13)</t>
+          <t>12_ledger (2)</t>
         </is>
       </c>
       <c r="O85" s="10" t="inlineStr">
@@ -7368,7 +7368,7 @@
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>FIN-007</t>
+          <t>FIN-006</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
@@ -7383,12 +7383,12 @@
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t>A refund cannot exceed the credit on the folio.</t>
+          <t>A posted transaction is never edited or deleted; corrections are linked reversal, adjustment or refund rows.</t>
         </is>
       </c>
       <c r="E86" s="10" t="inlineStr">
         <is>
-          <t>BR-015</t>
+          <t>BR-014, BR-015</t>
         </is>
       </c>
       <c r="F86" s="10" t="inlineStr">
@@ -7403,37 +7403,37 @@
       </c>
       <c r="H86" s="10" t="inlineStr">
         <is>
-          <t>fin.refund.post</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I86" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Rule: Immutability</t>
         </is>
       </c>
       <c r="J86" s="10" t="inlineStr">
         <is>
-          <t>a folio with a small credit</t>
+          <t>a posted charge</t>
         </is>
       </c>
       <c r="K86" s="10" t="inlineStr">
         <is>
-          <t>staff request a bigger refund</t>
+          <t>anyone, including the database owner, changes or deletes it</t>
         </is>
       </c>
       <c r="L86" s="10" t="inlineStr">
         <is>
-          <t>it is refused with E_REFUND_LIMIT; a refund within the credit is approved and pays out</t>
+          <t>the change is refused with E_IMMUTABLE; a reversal posts a linked row (with its tax lines) and a charge reverses only once</t>
         </is>
       </c>
       <c r="M86" s="10" t="inlineStr">
         <is>
-          <t>request_refund</t>
+          <t>txn_guard triggers; request_reversal</t>
         </is>
       </c>
       <c r="N86" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (2)</t>
+          <t>10_security (1); 12_ledger (13)</t>
         </is>
       </c>
       <c r="O86" s="10" t="inlineStr">
@@ -7446,7 +7446,7 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>FIN-008</t>
+          <t>FIN-007</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
@@ -7461,12 +7461,12 @@
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t>Repeating the same request cannot double post (idempotency keys).</t>
+          <t>A refund cannot exceed the credit on the folio.</t>
         </is>
       </c>
       <c r="E87" s="10" t="inlineStr">
         <is>
-          <t>BR-013</t>
+          <t>BR-015</t>
         </is>
       </c>
       <c r="F87" s="10" t="inlineStr">
@@ -7481,32 +7481,32 @@
       </c>
       <c r="H87" s="10" t="inlineStr">
         <is>
+          <t>fin.refund.post</t>
+        </is>
+      </c>
+      <c r="I87" s="10" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I87" s="10" t="inlineStr">
-        <is>
-          <t>Rule: Offline-ready design; A12</t>
-        </is>
-      </c>
       <c r="J87" s="10" t="inlineStr">
         <is>
-          <t>a charge posted with a key</t>
+          <t>a folio with a small credit</t>
         </is>
       </c>
       <c r="K87" s="10" t="inlineStr">
         <is>
-          <t>the same request arrives again</t>
+          <t>staff request a bigger refund</t>
         </is>
       </c>
       <c r="L87" s="10" t="inlineStr">
         <is>
-          <t>the second returns the first and the balance is unchanged</t>
+          <t>it is refused with E_REFUND_LIMIT; a refund within the credit is approved and pays out</t>
         </is>
       </c>
       <c r="M87" s="10" t="inlineStr">
         <is>
-          <t>idempotency_key unique per tenant</t>
+          <t>request_refund</t>
         </is>
       </c>
       <c r="N87" s="10" t="inlineStr">
@@ -7524,7 +7524,7 @@
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>FIN-009</t>
+          <t>FIN-008</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
@@ -7539,7 +7539,7 @@
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t>Move a posted charge, with its tax, to another folio of the same booking; revenue does not change.</t>
+          <t>Repeating the same request cannot double post (idempotency keys).</t>
         </is>
       </c>
       <c r="E88" s="10" t="inlineStr">
@@ -7549,7 +7549,7 @@
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G88" s="10" t="inlineStr">
@@ -7559,37 +7559,37 @@
       </c>
       <c r="H88" s="10" t="inlineStr">
         <is>
-          <t>fin.folio.transfer</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I88" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Rule: Offline-ready design; A12</t>
         </is>
       </c>
       <c r="J88" s="10" t="inlineStr">
         <is>
-          <t>a charge on the guest folio</t>
+          <t>a charge posted with a key</t>
         </is>
       </c>
       <c r="K88" s="10" t="inlineStr">
         <is>
-          <t>a manager transfers it to a company folio</t>
+          <t>the same request arrives again</t>
         </is>
       </c>
       <c r="L88" s="10" t="inlineStr">
         <is>
-          <t>the target owes the charge and tax, the source is relieved, the total is unchanged and the charge moves once</t>
+          <t>the second returns the first and the balance is unchanged</t>
         </is>
       </c>
       <c r="M88" s="10" t="inlineStr">
         <is>
-          <t>transfer_transaction</t>
+          <t>idempotency_key unique per tenant</t>
         </is>
       </c>
       <c r="N88" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (6)</t>
+          <t>12_ledger (2)</t>
         </is>
       </c>
       <c r="O88" s="10" t="inlineStr">
@@ -7602,7 +7602,7 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>FIN-010</t>
+          <t>FIN-009</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
@@ -7617,7 +7617,7 @@
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t>Split folios per reservation.</t>
+          <t>Move a posted charge, with its tax, to another folio of the same booking; revenue does not change.</t>
         </is>
       </c>
       <c r="E89" s="10" t="inlineStr">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="H89" s="10" t="inlineStr">
         <is>
-          <t>fin.folio.split</t>
+          <t>fin.folio.transfer</t>
         </is>
       </c>
       <c r="I89" s="10" t="inlineStr">
@@ -7647,27 +7647,27 @@
       </c>
       <c r="J89" s="10" t="inlineStr">
         <is>
-          <t>a reservation</t>
+          <t>a charge on the guest folio</t>
         </is>
       </c>
       <c r="K89" s="10" t="inlineStr">
         <is>
-          <t>staff add a Company folio</t>
+          <t>a manager transfers it to a company folio</t>
         </is>
       </c>
       <c r="L89" s="10" t="inlineStr">
         <is>
-          <t>charges can be posted to either folio and check-out settles both</t>
+          <t>the target owes the charge and tax, the source is relieved, the total is unchanged and the charge moves once</t>
         </is>
       </c>
       <c r="M89" s="10" t="inlineStr">
         <is>
-          <t>split_folio</t>
+          <t>transfer_transaction</t>
         </is>
       </c>
       <c r="N89" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (1)</t>
+          <t>12_ledger (6)</t>
         </is>
       </c>
       <c r="O89" s="10" t="inlineStr">
@@ -7680,7 +7680,7 @@
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>FIN-011</t>
+          <t>FIN-010</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
@@ -7695,17 +7695,17 @@
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t>A folio closes only at a zero balance and reopens only for the accountant with a reason; a closed folio takes no postings.</t>
+          <t>Split folios per reservation.</t>
         </is>
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>BR-013, BR-015</t>
+          <t>BR-013</t>
         </is>
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G90" s="10" t="inlineStr">
@@ -7715,37 +7715,37 @@
       </c>
       <c r="H90" s="10" t="inlineStr">
         <is>
-          <t>fin.invoice.issue, fin.folio.reopen</t>
+          <t>fin.folio.split</t>
         </is>
       </c>
       <c r="I90" s="10" t="inlineStr">
         <is>
-          <t>Rule: Reasons</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J90" s="10" t="inlineStr">
         <is>
-          <t>a settled folio</t>
+          <t>a reservation</t>
         </is>
       </c>
       <c r="K90" s="10" t="inlineStr">
         <is>
-          <t>it is closed and then a posting is attempted</t>
+          <t>staff add a Company folio</t>
         </is>
       </c>
       <c r="L90" s="10" t="inlineStr">
         <is>
-          <t>the posting is refused with E_FOLIO_CLOSED; reopening needs the permission and a reason and is audited</t>
+          <t>charges can be posted to either folio and check-out settles both</t>
         </is>
       </c>
       <c r="M90" s="10" t="inlineStr">
         <is>
-          <t>close_folio, reopen_folio</t>
+          <t>split_folio</t>
         </is>
       </c>
       <c r="N90" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (5)</t>
+          <t>12_ledger (1)</t>
         </is>
       </c>
       <c r="O90" s="10" t="inlineStr">
@@ -7758,7 +7758,7 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>FIN-012</t>
+          <t>FIN-011</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
@@ -7768,17 +7768,17 @@
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>FIN-01, FO-03</t>
+          <t>FIN-01</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>Invoices and receipts are numbered documents built from posted rows; they cannot be changed once issued.</t>
+          <t>A folio closes only at a zero balance and reopens only for the accountant with a reason; a closed folio takes no postings.</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
-          <t>BR-013</t>
+          <t>BR-013, BR-015</t>
         </is>
       </c>
       <c r="F91" s="10" t="inlineStr">
@@ -7793,12 +7793,12 @@
       </c>
       <c r="H91" s="10" t="inlineStr">
         <is>
-          <t>fin.invoice.issue</t>
+          <t>fin.invoice.issue, fin.folio.reopen</t>
         </is>
       </c>
       <c r="I91" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Rule: Reasons</t>
         </is>
       </c>
       <c r="J91" s="10" t="inlineStr">
@@ -7808,22 +7808,22 @@
       </c>
       <c r="K91" s="10" t="inlineStr">
         <is>
-          <t>an invoice is issued</t>
+          <t>it is closed and then a posting is attempted</t>
         </is>
       </c>
       <c r="L91" s="10" t="inlineStr">
         <is>
-          <t>the total, tax and balance match the folio and the invoice cannot be edited; interim receipts have their own number series</t>
+          <t>the posting is refused with E_FOLIO_CLOSED; reopening needs the permission and a reason and is audited</t>
         </is>
       </c>
       <c r="M91" s="10" t="inlineStr">
         <is>
-          <t>issue_invoice</t>
+          <t>close_folio, reopen_folio</t>
         </is>
       </c>
       <c r="N91" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (4); 17_more_features (4)</t>
+          <t>12_ledger (5)</t>
         </is>
       </c>
       <c r="O91" s="10" t="inlineStr">
@@ -7836,7 +7836,7 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>FIN-013</t>
+          <t>FIN-012</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
@@ -7846,12 +7846,12 @@
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>FIN-01</t>
+          <t>FIN-01, FO-03</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>Balances are calculated from posted rows and never stored; pending approvals do not change them.</t>
+          <t>Invoices and receipts are numbered documents built from posted rows; they cannot be changed once issued.</t>
         </is>
       </c>
       <c r="E92" s="10" t="inlineStr">
@@ -7871,37 +7871,37 @@
       </c>
       <c r="H92" s="10" t="inlineStr">
         <is>
-          <t>fin.folio.view</t>
+          <t>fin.invoice.issue</t>
         </is>
       </c>
       <c r="I92" s="10" t="inlineStr">
         <is>
-          <t>Rule: Immutability</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J92" s="10" t="inlineStr">
         <is>
-          <t>a pending discount</t>
+          <t>a settled folio</t>
         </is>
       </c>
       <c r="K92" s="10" t="inlineStr">
         <is>
-          <t>the balance is read</t>
+          <t>an invoice is issued</t>
         </is>
       </c>
       <c r="L92" s="10" t="inlineStr">
         <is>
-          <t>it is unchanged until the approval posts</t>
+          <t>the total, tax and balance match the folio and the invoice cannot be edited; interim receipts have their own number series</t>
         </is>
       </c>
       <c r="M92" s="10" t="inlineStr">
         <is>
-          <t>v_folio_balances</t>
+          <t>issue_invoice</t>
         </is>
       </c>
       <c r="N92" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (2)</t>
+          <t>12_ledger (4); 17_more_features (4)</t>
         </is>
       </c>
       <c r="O92" s="10" t="inlineStr">
@@ -7914,7 +7914,7 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>FIN-014</t>
+          <t>FIN-013</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>Every posting takes the open business date, and a past date is refused.</t>
+          <t>Balances are calculated from posted rows and never stored; pending approvals do not change them.</t>
         </is>
       </c>
       <c r="E93" s="10" t="inlineStr">
@@ -7949,37 +7949,37 @@
       </c>
       <c r="H93" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fin.folio.view</t>
         </is>
       </c>
       <c r="I93" s="10" t="inlineStr">
         <is>
-          <t>Rule: Business date</t>
+          <t>Rule: Immutability</t>
         </is>
       </c>
       <c r="J93" s="10" t="inlineStr">
         <is>
-          <t>a posting for a past date</t>
+          <t>a pending discount</t>
         </is>
       </c>
       <c r="K93" s="10" t="inlineStr">
         <is>
-          <t>it is inserted</t>
+          <t>the balance is read</t>
         </is>
       </c>
       <c r="L93" s="10" t="inlineStr">
         <is>
-          <t>it is refused with E_DATE</t>
+          <t>it is unchanged until the approval posts</t>
         </is>
       </c>
       <c r="M93" s="10" t="inlineStr">
         <is>
-          <t>txn_guard</t>
+          <t>v_folio_balances</t>
         </is>
       </c>
       <c r="N93" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (2); 14_lifecycle (1); upgrade (2)</t>
+          <t>12_ledger (2)</t>
         </is>
       </c>
       <c r="O93" s="10" t="inlineStr">
@@ -7992,7 +7992,7 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>FIN-015</t>
+          <t>FIN-014</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
@@ -8007,12 +8007,12 @@
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t>Folio visibility follows the role: managers see all folios, a reservation officer sees only those of their own bookings.</t>
+          <t>Every posting takes the open business date, and a past date is refused.</t>
         </is>
       </c>
       <c r="E94" s="10" t="inlineStr">
         <is>
-          <t>BR-017</t>
+          <t>BR-013</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
@@ -8027,37 +8027,37 @@
       </c>
       <c r="H94" s="10" t="inlineStr">
         <is>
-          <t>fin.folio.view</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I94" s="10" t="inlineStr">
         <is>
-          <t>Own-record scope</t>
+          <t>Rule: Business date</t>
         </is>
       </c>
       <c r="J94" s="10" t="inlineStr">
         <is>
-          <t>a reservation officer</t>
+          <t>a posting for a past date</t>
         </is>
       </c>
       <c r="K94" s="10" t="inlineStr">
         <is>
-          <t>they read a colleague's folio</t>
+          <t>it is inserted</t>
         </is>
       </c>
       <c r="L94" s="10" t="inlineStr">
         <is>
-          <t>they see nothing; they can still take a deposit</t>
+          <t>it is refused with E_DATE</t>
         </is>
       </c>
       <c r="M94" s="10" t="inlineStr">
         <is>
-          <t>can_see_folio</t>
+          <t>txn_guard</t>
         </is>
       </c>
       <c r="N94" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (6)</t>
+          <t>12_ledger (2); 14_lifecycle (1); upgrade (2)</t>
         </is>
       </c>
       <c r="O94" s="10" t="inlineStr">
@@ -8070,7 +8070,7 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>FIN-016</t>
+          <t>FIN-015</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
@@ -8080,17 +8080,17 @@
       </c>
       <c r="C95" s="10" t="inlineStr">
         <is>
-          <t>/cashier</t>
+          <t>FIN-01</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t>Cashier shifts: a cashier opens a shift with a float, takes payments, counts each payment method at the end; the database works out expected and difference; a manager reconciles (never the closer). A hotel can require an open shift before payments.</t>
+          <t>Folio visibility follows the role: managers see all folios, a reservation officer sees only those of their own bookings.</t>
         </is>
       </c>
       <c r="E95" s="10" t="inlineStr">
         <is>
-          <t>BR-016</t>
+          <t>BR-017</t>
         </is>
       </c>
       <c r="F95" s="10" t="inlineStr">
@@ -8105,74 +8105,70 @@
       </c>
       <c r="H95" s="10" t="inlineStr">
         <is>
-          <t>fin.shift.close, fin.shift.reconcile</t>
+          <t>fin.folio.view</t>
         </is>
       </c>
       <c r="I95" s="10" t="inlineStr">
         <is>
-          <t>A2; decision of 7 Oct 2026</t>
+          <t>Own-record scope</t>
         </is>
       </c>
       <c r="J95" s="10" t="inlineStr">
         <is>
-          <t>a cashier with an open shift who took cash and card payments</t>
+          <t>a reservation officer</t>
         </is>
       </c>
       <c r="K95" s="10" t="inlineStr">
         <is>
-          <t>they close the shift with their counts</t>
+          <t>they read a colleague's folio</t>
         </is>
       </c>
       <c r="L95" s="10" t="inlineStr">
         <is>
-          <t>the difference per method is worked out, a note is needed for a difference, and a manager reconciles it</t>
+          <t>they see nothing; they can still take a deposit</t>
         </is>
       </c>
       <c r="M95" s="10" t="inlineStr">
         <is>
-          <t>open_cashier_shift, close_cashier_shift, reconcile_cashier_shift, cashier_shift_summary, list_cashier_shifts, set_cashier_shift_required, stamp_cashier_shift</t>
+          <t>can_see_folio</t>
         </is>
       </c>
       <c r="N95" s="10" t="inlineStr">
         <is>
-          <t>34_cashier_shifts (45)</t>
+          <t>12_ledger (6)</t>
         </is>
       </c>
       <c r="O95" s="10" t="inlineStr">
         <is>
-          <t>Built+tested (database only)</t>
-        </is>
-      </c>
-      <c r="P95" s="10" t="inlineStr">
-        <is>
-          <t>Cashier shift page built (open, close with counts, review, reconcile). Not covered by a browser test yet. New permission fin.shift.reconcile goes to built-in roles only.</t>
-        </is>
-      </c>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P95" s="10" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>DAY-001</t>
+          <t>FIN-016</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>Business Date</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
         <is>
-          <t>(system)</t>
+          <t>/cashier</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t>The business date rolls automatically at each property's cut-off time.</t>
+          <t>Cashier shifts: a cashier opens a shift with a float, takes payments, counts each payment method at the end; the database works out expected and difference; a manager reconciles (never the closer). A hotel can require an open shift before payments.</t>
         </is>
       </c>
       <c r="E96" s="10" t="inlineStr">
         <is>
-          <t>BR-019</t>
+          <t>BR-016</t>
         </is>
       </c>
       <c r="F96" s="10" t="inlineStr">
@@ -8187,50 +8183,54 @@
       </c>
       <c r="H96" s="10" t="inlineStr">
         <is>
-          <t>audit.businessdate.view</t>
+          <t>fin.shift.close, fin.shift.reconcile</t>
         </is>
       </c>
       <c r="I96" s="10" t="inlineStr">
         <is>
-          <t>Rule: Business date; A2</t>
+          <t>A2; decision of 7 Oct 2026</t>
         </is>
       </c>
       <c r="J96" s="10" t="inlineStr">
         <is>
-          <t>a property whose cut-off has passed</t>
+          <t>a cashier with an open shift who took cash and card payments</t>
         </is>
       </c>
       <c r="K96" s="10" t="inlineStr">
         <is>
-          <t>the scheduler runs</t>
+          <t>they close the shift with their counts</t>
         </is>
       </c>
       <c r="L96" s="10" t="inlineStr">
         <is>
-          <t>the date advances one day, up to three days per run; the roll is logged</t>
+          <t>the difference per method is worked out, a note is needed for a difference, and a manager reconciles it</t>
         </is>
       </c>
       <c r="M96" s="10" t="inlineStr">
         <is>
-          <t>roll_business_date, run_due_rollovers (pg_cron)</t>
+          <t>open_cashier_shift, close_cashier_shift, reconcile_cashier_shift, cashier_shift_summary, list_cashier_shifts, set_cashier_shift_required, stamp_cashier_shift</t>
         </is>
       </c>
       <c r="N96" s="10" t="inlineStr">
         <is>
-          <t>14_lifecycle (4); upgrade (5)</t>
+          <t>34_cashier_shifts (45)</t>
         </is>
       </c>
       <c r="O96" s="10" t="inlineStr">
         <is>
-          <t>Built+tested</t>
-        </is>
-      </c>
-      <c r="P96" s="10" t="inlineStr"/>
+          <t>Built+tested (database only)</t>
+        </is>
+      </c>
+      <c r="P96" s="10" t="inlineStr">
+        <is>
+          <t>Cashier shift page built (open, close with counts, review, reconcile). Not covered by a browser test yet. New permission fin.shift.reconcile goes to built-in roles only.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>DAY-002</t>
+          <t>DAY-001</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
@@ -8245,12 +8245,12 @@
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t>At the roll, each guest in house is charged the night's room rate and tax exactly once.</t>
+          <t>The business date rolls automatically at each property's cut-off time.</t>
         </is>
       </c>
       <c r="E97" s="10" t="inlineStr">
         <is>
-          <t>BR-013</t>
+          <t>BR-019</t>
         </is>
       </c>
       <c r="F97" s="10" t="inlineStr">
@@ -8265,37 +8265,37 @@
       </c>
       <c r="H97" s="10" t="inlineStr">
         <is>
-          <t>(system)</t>
+          <t>audit.businessdate.view</t>
         </is>
       </c>
       <c r="I97" s="10" t="inlineStr">
         <is>
-          <t>Rule: Business date</t>
+          <t>Rule: Business date; A2</t>
         </is>
       </c>
       <c r="J97" s="10" t="inlineStr">
         <is>
-          <t>two guests in house</t>
+          <t>a property whose cut-off has passed</t>
         </is>
       </c>
       <c r="K97" s="10" t="inlineStr">
         <is>
-          <t>the roll runs</t>
+          <t>the scheduler runs</t>
         </is>
       </c>
       <c r="L97" s="10" t="inlineStr">
         <is>
-          <t>each folio gets one room charge for the closing date, with tax; running it again for the same night cannot repeat it</t>
+          <t>the date advances one day, up to three days per run; the roll is logged</t>
         </is>
       </c>
       <c r="M97" s="10" t="inlineStr">
         <is>
-          <t>roll_business_date; idempotency keys room:&lt;reservation&gt;:&lt;date&gt;</t>
+          <t>roll_business_date, run_due_rollovers (pg_cron)</t>
         </is>
       </c>
       <c r="N97" s="10" t="inlineStr">
         <is>
-          <t>14_lifecycle (3)</t>
+          <t>14_lifecycle (4); upgrade (5)</t>
         </is>
       </c>
       <c r="O97" s="10" t="inlineStr">
@@ -8308,7 +8308,7 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>DAY-003</t>
+          <t>DAY-002</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
@@ -8323,7 +8323,7 @@
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t>A guest still in house past departure is charged and extended a night if the room allows; otherwise managers are told.</t>
+          <t>At the roll, each guest in house is charged the night's room rate and tax exactly once.</t>
         </is>
       </c>
       <c r="E98" s="10" t="inlineStr">
@@ -8333,7 +8333,7 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G98" s="10" t="inlineStr">
@@ -8348,12 +8348,12 @@
       </c>
       <c r="I98" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Rule: Business date</t>
         </is>
       </c>
       <c r="J98" s="10" t="inlineStr">
         <is>
-          <t>a guest due out today who is still in house</t>
+          <t>two guests in house</t>
         </is>
       </c>
       <c r="K98" s="10" t="inlineStr">
@@ -8363,17 +8363,17 @@
       </c>
       <c r="L98" s="10" t="inlineStr">
         <is>
-          <t>the departure moves one day and the night is charged</t>
+          <t>each folio gets one room charge for the closing date, with tax; running it again for the same night cannot repeat it</t>
         </is>
       </c>
       <c r="M98" s="10" t="inlineStr">
         <is>
-          <t>roll_business_date</t>
+          <t>roll_business_date; idempotency keys room:&lt;reservation&gt;:&lt;date&gt;</t>
         </is>
       </c>
       <c r="N98" s="10" t="inlineStr">
         <is>
-          <t>14_lifecycle (12); upgrade (2)</t>
+          <t>14_lifecycle (3)</t>
         </is>
       </c>
       <c r="O98" s="10" t="inlineStr">
@@ -8386,7 +8386,7 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>DAY-004</t>
+          <t>DAY-003</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
@@ -8401,7 +8401,7 @@
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t>A failed roll changes nothing and notifies managers; other properties are not blocked.</t>
+          <t>A guest still in house past departure is charged and extended a night if the room allows; otherwise managers are told.</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G99" s="10" t="inlineStr">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="H99" s="10" t="inlineStr">
         <is>
-          <t>audit.businessdate.view</t>
+          <t>(system)</t>
         </is>
       </c>
       <c r="I99" s="10" t="inlineStr">
@@ -8431,27 +8431,27 @@
       </c>
       <c r="J99" s="10" t="inlineStr">
         <is>
-          <t>a property whose roll fails</t>
+          <t>a guest due out today who is still in house</t>
         </is>
       </c>
       <c r="K99" s="10" t="inlineStr">
         <is>
-          <t>the scheduler runs</t>
+          <t>the roll runs</t>
         </is>
       </c>
       <c r="L99" s="10" t="inlineStr">
         <is>
-          <t>its date is unchanged and managers get a notification</t>
+          <t>the departure moves one day and the night is charged</t>
         </is>
       </c>
       <c r="M99" s="10" t="inlineStr">
         <is>
-          <t>run_due_rollovers</t>
+          <t>roll_business_date</t>
         </is>
       </c>
       <c r="N99" s="10" t="inlineStr">
         <is>
-          <t>17_more_features (2)</t>
+          <t>14_lifecycle (12); upgrade (2)</t>
         </is>
       </c>
       <c r="O99" s="10" t="inlineStr">
@@ -8464,7 +8464,7 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>DAY-005</t>
+          <t>DAY-004</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
@@ -8474,22 +8474,22 @@
       </c>
       <c r="C100" s="10" t="inlineStr">
         <is>
-          <t>/admin (Business date)</t>
+          <t>(system)</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t>Night audit flags list what is still open before the day closes: open cashier shifts (blocking), unreconciled differences, guests past departure, arrivals not checked in. The flags do not stop the date rolling yet.</t>
+          <t>A failed roll changes nothing and notifies managers; other properties are not blocked.</t>
         </is>
       </c>
       <c r="E100" s="10" t="inlineStr">
         <is>
-          <t>BR-016</t>
+          <t>BR-013</t>
         </is>
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G100" s="10" t="inlineStr">
@@ -8499,54 +8499,50 @@
       </c>
       <c r="H100" s="10" t="inlineStr">
         <is>
-          <t>fin.nightaudit.run</t>
+          <t>audit.businessdate.view</t>
         </is>
       </c>
       <c r="I100" s="10" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J100" s="10" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>a property whose roll fails</t>
         </is>
       </c>
       <c r="K100" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>the scheduler runs</t>
         </is>
       </c>
       <c r="L100" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>its date is unchanged and managers get a notification</t>
         </is>
       </c>
       <c r="M100" s="10" t="inlineStr">
         <is>
-          <t>night_audit_flags</t>
+          <t>run_due_rollovers</t>
         </is>
       </c>
       <c r="N100" s="10" t="inlineStr">
         <is>
-          <t>34_cashier_shifts (7)</t>
+          <t>17_more_features (2)</t>
         </is>
       </c>
       <c r="O100" s="10" t="inlineStr">
         <is>
-          <t>Partly built (flags only)</t>
-        </is>
-      </c>
-      <c r="P100" s="10" t="inlineStr">
-        <is>
-          <t>Flags shown in Admin, Business date. The gate that stops the roll while a blocking flag is open is not built.</t>
-        </is>
-      </c>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P100" s="10" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>DAY-006</t>
+          <t>DAY-005</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
@@ -8556,17 +8552,17 @@
       </c>
       <c r="C101" s="10" t="inlineStr">
         <is>
-          <t>(system)</t>
+          <t>/admin (Business date)</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t>A same-day arrival and departure: decide whether a night or day-use charge applies.</t>
+          <t>Night audit flags list what is still open before the day closes: open cashier shifts (blocking), unreconciled differences, guests past departure, arrivals not checked in. The flags do not stop the date rolling yet.</t>
         </is>
       </c>
       <c r="E101" s="10" t="inlineStr">
         <is>
-          <t>BR-013</t>
+          <t>BR-016</t>
         </is>
       </c>
       <c r="F101" s="10" t="inlineStr">
@@ -8581,79 +8577,79 @@
       </c>
       <c r="H101" s="10" t="inlineStr">
         <is>
-          <t>(decision)</t>
+          <t>fin.nightaudit.run</t>
         </is>
       </c>
       <c r="I101" s="10" t="inlineStr">
         <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="J101" s="10" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="K101" s="10" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J101" s="10" t="inlineStr">
-        <is>
-          <t>a guest checks in and out on the same business date</t>
-        </is>
-      </c>
-      <c r="K101" s="10" t="inlineStr">
-        <is>
-          <t>they leave before the roll</t>
-        </is>
-      </c>
       <c r="L101" s="10" t="inlineStr">
         <is>
-          <t>today no room charge is made; the desk can post a manual charge</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M101" s="10" t="inlineStr">
         <is>
-          <t>check_out</t>
+          <t>night_audit_flags</t>
         </is>
       </c>
       <c r="N101" s="10" t="inlineStr">
         <is>
-          <t>19_same_day (21); upgrade (2); browser: desk-journey</t>
+          <t>34_cashier_shifts (7)</t>
         </is>
       </c>
       <c r="O101" s="10" t="inlineStr">
         <is>
-          <t>Built+tested</t>
+          <t>Partly built (flags only)</t>
         </is>
       </c>
       <c r="P101" s="10" t="inlineStr">
         <is>
-          <t>Decided by Peter on 30 Sep 2026 (answer 5) and confirmed on 1 Oct 2026: same-day stays are charged one night; a manager can waive it with a reason.</t>
+          <t>Flags shown in Admin, Business date. The gate that stops the roll while a blocking flag is open is not built.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>RPT-001</t>
+          <t>DAY-006</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t>Reporting</t>
+          <t>Business Date</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
         <is>
-          <t>DASH-01, REP-01</t>
+          <t>(system)</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t>Occupancy, ADR and RevPAR use one definition: rooms sold over rooms available (out-of-order rooms excluded), revenue net of tax.</t>
+          <t>A same-day arrival and departure: decide whether a night or day-use charge applies.</t>
         </is>
       </c>
       <c r="E102" s="10" t="inlineStr">
         <is>
-          <t>BR-019</t>
+          <t>BR-013</t>
         </is>
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G102" s="10" t="inlineStr">
@@ -8663,37 +8659,37 @@
       </c>
       <c r="H102" s="10" t="inlineStr">
         <is>
-          <t>dash.view_exec, rep.ops.view</t>
+          <t>(decision)</t>
         </is>
       </c>
       <c r="I102" s="10" t="inlineStr">
         <is>
-          <t>KPI Dictionary</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J102" s="10" t="inlineStr">
         <is>
-          <t>a closed day</t>
+          <t>a guest checks in and out on the same business date</t>
         </is>
       </c>
       <c r="K102" s="10" t="inlineStr">
         <is>
-          <t>management opens the KPI view</t>
+          <t>they leave before the roll</t>
         </is>
       </c>
       <c r="L102" s="10" t="inlineStr">
         <is>
-          <t>occupancy, ADR and RevPAR equal sold, revenue and available as defined; tax is shown apart</t>
+          <t>today no room charge is made; the desk can post a manual charge</t>
         </is>
       </c>
       <c r="M102" s="10" t="inlineStr">
         <is>
-          <t>daily_stats, v_kpi_daily</t>
+          <t>check_out</t>
         </is>
       </c>
       <c r="N102" s="10" t="inlineStr">
         <is>
-          <t>14_lifecycle (4)</t>
+          <t>19_same_day (21); upgrade (2); browser: desk-journey</t>
         </is>
       </c>
       <c r="O102" s="10" t="inlineStr">
@@ -8701,12 +8697,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P102" s="10" t="inlineStr"/>
+      <c r="P102" s="10" t="inlineStr">
+        <is>
+          <t>Decided by Peter on 30 Sep 2026 (answer 5) and confirmed on 1 Oct 2026: same-day stays are charged one night; a manager can waive it with a reason.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>RPT-002</t>
+          <t>RPT-001</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
@@ -8716,17 +8716,17 @@
       </c>
       <c r="C103" s="10" t="inlineStr">
         <is>
-          <t>DASH-02</t>
+          <t>DASH-01, REP-01</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>Live operations views: arrivals, in-house, room board, housekeeping board.</t>
+          <t>Occupancy, ADR and RevPAR use one definition: rooms sold over rooms available (out-of-order rooms excluded), revenue net of tax.</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>BR-006, BR-019</t>
+          <t>BR-019</t>
         </is>
       </c>
       <c r="F103" s="10" t="inlineStr">
@@ -8741,37 +8741,37 @@
       </c>
       <c r="H103" s="10" t="inlineStr">
         <is>
-          <t>dash.view_ops</t>
+          <t>dash.view_exec, rep.ops.view</t>
         </is>
       </c>
       <c r="I103" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>KPI Dictionary</t>
         </is>
       </c>
       <c r="J103" s="10" t="inlineStr">
         <is>
-          <t>activity in the hotel</t>
+          <t>a closed day</t>
         </is>
       </c>
       <c r="K103" s="10" t="inlineStr">
         <is>
-          <t>staff open the operations dashboard</t>
+          <t>management opens the KPI view</t>
         </is>
       </c>
       <c r="L103" s="10" t="inlineStr">
         <is>
-          <t>the views return only rows the user may see</t>
+          <t>occupancy, ADR and RevPAR equal sold, revenue and available as defined; tax is shown apart</t>
         </is>
       </c>
       <c r="M103" s="10" t="inlineStr">
         <is>
-          <t>v_arrivals, v_in_house, v_room_board, v_hk_board</t>
+          <t>daily_stats, v_kpi_daily</t>
         </is>
       </c>
       <c r="N103" s="10" t="inlineStr">
         <is>
-          <t>29_untagged_rows (14)</t>
+          <t>14_lifecycle (4)</t>
         </is>
       </c>
       <c r="O103" s="10" t="inlineStr">
@@ -8784,7 +8784,7 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>RPT-003</t>
+          <t>RPT-002</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
@@ -8794,17 +8794,17 @@
       </c>
       <c r="C104" s="10" t="inlineStr">
         <is>
-          <t>REP-01, REP-02</t>
+          <t>DASH-02</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t>Every reported figure traces to ledger rows or operational records.</t>
+          <t>Live operations views: arrivals, in-house, room board, housekeeping board.</t>
         </is>
       </c>
       <c r="E104" s="10" t="inlineStr">
         <is>
-          <t>BR-020</t>
+          <t>BR-006, BR-019</t>
         </is>
       </c>
       <c r="F104" s="10" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="H104" s="10" t="inlineStr">
         <is>
-          <t>rep.ops.view, rep.fin.view</t>
+          <t>dash.view_ops</t>
         </is>
       </c>
       <c r="I104" s="10" t="inlineStr">
@@ -8829,27 +8829,27 @@
       </c>
       <c r="J104" s="10" t="inlineStr">
         <is>
-          <t>a daily figure</t>
+          <t>activity in the hotel</t>
         </is>
       </c>
       <c r="K104" s="10" t="inlineStr">
         <is>
-          <t>an auditor recomputes it from folio_transactions</t>
+          <t>staff open the operations dashboard</t>
         </is>
       </c>
       <c r="L104" s="10" t="inlineStr">
         <is>
-          <t>the figures agree</t>
+          <t>the views return only rows the user may see</t>
         </is>
       </c>
       <c r="M104" s="10" t="inlineStr">
         <is>
-          <t>daily_stats computed from folio_transactions</t>
+          <t>v_arrivals, v_in_house, v_room_board, v_hk_board</t>
         </is>
       </c>
       <c r="N104" s="10" t="inlineStr">
         <is>
-          <t>29_untagged_rows (11)</t>
+          <t>29_untagged_rows (14)</t>
         </is>
       </c>
       <c r="O104" s="10" t="inlineStr">
@@ -8862,7 +8862,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>RPT-004</t>
+          <t>RPT-003</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
@@ -8877,12 +8877,12 @@
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t>Report screens (occupancy trend, revenue by group, outstanding balances, cancellation and no-show rates).</t>
+          <t>Every reported figure traces to ledger rows or operational records.</t>
         </is>
       </c>
       <c r="E105" s="10" t="inlineStr">
         <is>
-          <t>BR-019</t>
+          <t>BR-020</t>
         </is>
       </c>
       <c r="F105" s="10" t="inlineStr">
@@ -8902,32 +8902,32 @@
       </c>
       <c r="I105" s="10" t="inlineStr">
         <is>
-          <t>KPI Dictionary</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J105" s="10" t="inlineStr">
         <is>
-          <t>a date range</t>
+          <t>a daily figure</t>
         </is>
       </c>
       <c r="K105" s="10" t="inlineStr">
         <is>
-          <t>a manager opens a report</t>
+          <t>an auditor recomputes it from folio_transactions</t>
         </is>
       </c>
       <c r="L105" s="10" t="inlineStr">
         <is>
-          <t>the numbers match the KPI definitions</t>
+          <t>the figures agree</t>
         </is>
       </c>
       <c r="M105" s="10" t="inlineStr">
         <is>
-          <t>Reports screen (src/routes/_authenticated/_app/reports.tsx) on report_* functions in the database: v_kpi_daily (occupancy, average rate, revenue per room), report_revenue_by_charge_code, report_outstanding_balances, report_payments, report_cancellation_rate (cancellations and no-shows), report_length_of_stay, report_balances_by_guest; finance reports need rpt.finance.view, operations reports rpt.operations.view</t>
+          <t>daily_stats computed from folio_transactions</t>
         </is>
       </c>
       <c r="N105" s="10" t="inlineStr">
         <is>
-          <t>29_untagged_rows (14)</t>
+          <t>29_untagged_rows (11)</t>
         </is>
       </c>
       <c r="O105" s="10" t="inlineStr">
@@ -8935,36 +8935,32 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P105" s="10" t="inlineStr">
-        <is>
-          <t>Reports screen: KPIs, revenue by charge code, outstanding balances, payments, cancellations and stay length, balances by guest, export.</t>
-        </is>
-      </c>
+      <c r="P105" s="10" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>NFR-001</t>
+          <t>RPT-004</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t>Non-functional</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>REP-01, REP-02</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t>Every table has row-level security and tenant_id; security definer functions pin their search path.</t>
+          <t>Report screens (occupancy trend, revenue by group, outstanding balances, cancellation and no-show rates).</t>
         </is>
       </c>
       <c r="E106" s="10" t="inlineStr">
         <is>
-          <t>BR-017</t>
+          <t>BR-019</t>
         </is>
       </c>
       <c r="F106" s="10" t="inlineStr">
@@ -8979,37 +8975,37 @@
       </c>
       <c r="H106" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>rep.ops.view, rep.fin.view</t>
         </is>
       </c>
       <c r="I106" s="10" t="inlineStr">
         <is>
-          <t>Rule: Tenant isolation</t>
+          <t>KPI Dictionary</t>
         </is>
       </c>
       <c r="J106" s="10" t="inlineStr">
         <is>
-          <t>a migration adds a table or function</t>
+          <t>a date range</t>
         </is>
       </c>
       <c r="K106" s="10" t="inlineStr">
         <is>
-          <t>the test suite runs</t>
+          <t>a manager opens a report</t>
         </is>
       </c>
       <c r="L106" s="10" t="inlineStr">
         <is>
-          <t>it fails if RLS, tenant_id or search_path is missing</t>
+          <t>the numbers match the KPI definitions</t>
         </is>
       </c>
       <c r="M106" s="10" t="inlineStr">
         <is>
-          <t>structure tests</t>
+          <t>Reports screen (src/routes/_authenticated/_app/reports.tsx) on report_* functions in the database: v_kpi_daily (occupancy, average rate, revenue per room), report_revenue_by_charge_code, report_outstanding_balances, report_payments, report_cancellation_rate (cancellations and no-shows), report_length_of_stay, report_balances_by_guest; finance reports need rpt.finance.view, operations reports rpt.operations.view</t>
         </is>
       </c>
       <c r="N106" s="10" t="inlineStr">
         <is>
-          <t>10_security (3)</t>
+          <t>29_untagged_rows (14)</t>
         </is>
       </c>
       <c r="O106" s="10" t="inlineStr">
@@ -9017,12 +9013,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P106" s="10" t="inlineStr"/>
+      <c r="P106" s="10" t="inlineStr">
+        <is>
+          <t>Reports screen: KPIs, revenue by charge code, outstanding balances, payments, cancellations and stay length, balances by guest, export.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>NFR-002</t>
+          <t>NFR-001</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
@@ -9037,12 +9037,12 @@
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t>The browser can write directly only to plain configuration tables; ledger, reservations, stays, tasks and blocks change only through functions.</t>
+          <t>Every table has row-level security and tenant_id; security definer functions pin their search path.</t>
         </is>
       </c>
       <c r="E107" s="10" t="inlineStr">
         <is>
-          <t>BR-014, BR-017</t>
+          <t>BR-017</t>
         </is>
       </c>
       <c r="F107" s="10" t="inlineStr">
@@ -9062,32 +9062,32 @@
       </c>
       <c r="I107" s="10" t="inlineStr">
         <is>
-          <t>Rule: Immutability</t>
+          <t>Rule: Tenant isolation</t>
         </is>
       </c>
       <c r="J107" s="10" t="inlineStr">
         <is>
-          <t>any user</t>
+          <t>a migration adds a table or function</t>
         </is>
       </c>
       <c r="K107" s="10" t="inlineStr">
         <is>
-          <t>they write to a ledger or state table</t>
+          <t>the test suite runs</t>
         </is>
       </c>
       <c r="L107" s="10" t="inlineStr">
         <is>
-          <t>permission denied; the list of directly writable tables is asserted by a test</t>
+          <t>it fails if RLS, tenant_id or search_path is missing</t>
         </is>
       </c>
       <c r="M107" s="10" t="inlineStr">
         <is>
-          <t>20260928001100_grants.sql</t>
+          <t>structure tests</t>
         </is>
       </c>
       <c r="N107" s="10" t="inlineStr">
         <is>
-          <t>10_security (2)</t>
+          <t>10_security (3)</t>
         </is>
       </c>
       <c r="O107" s="10" t="inlineStr">
@@ -9100,7 +9100,7 @@
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>NFR-003</t>
+          <t>NFR-002</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
@@ -9115,17 +9115,17 @@
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t>Create actions accept client-generated ids and idempotency keys so an offline queue can be added later.</t>
+          <t>The browser can write directly only to plain configuration tables; ledger, reservations, stays, tasks and blocks change only through functions.</t>
         </is>
       </c>
       <c r="E108" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>BR-014, BR-017</t>
         </is>
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G108" s="10" t="inlineStr">
@@ -9140,32 +9140,32 @@
       </c>
       <c r="I108" s="10" t="inlineStr">
         <is>
-          <t>Rule: Offline-ready design; A12</t>
+          <t>Rule: Immutability</t>
         </is>
       </c>
       <c r="J108" s="10" t="inlineStr">
         <is>
-          <t>a repeated create request</t>
+          <t>any user</t>
         </is>
       </c>
       <c r="K108" s="10" t="inlineStr">
         <is>
-          <t>it arrives twice</t>
+          <t>they write to a ledger or state table</t>
         </is>
       </c>
       <c r="L108" s="10" t="inlineStr">
         <is>
-          <t>only one record exists</t>
+          <t>permission denied; the list of directly writable tables is asserted by a test</t>
         </is>
       </c>
       <c r="M108" s="10" t="inlineStr">
         <is>
-          <t>idempotency keys; client ids allowed on insert</t>
+          <t>20260928001100_grants.sql</t>
         </is>
       </c>
       <c r="N108" s="10" t="inlineStr">
         <is>
-          <t>13_reservations (1)</t>
+          <t>10_security (2)</t>
         </is>
       </c>
       <c r="O108" s="10" t="inlineStr">
@@ -9178,7 +9178,7 @@
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>NFR-004</t>
+          <t>NFR-003</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
@@ -9193,17 +9193,17 @@
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t>Money uses fixed decimals per currency (naira 2, CFA franc 0), never floating point.</t>
+          <t>Create actions accept client-generated ids and idempotency keys so an offline queue can be added later.</t>
         </is>
       </c>
       <c r="E109" s="10" t="inlineStr">
         <is>
-          <t>BR-013</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G109" s="10" t="inlineStr">
@@ -9218,32 +9218,32 @@
       </c>
       <c r="I109" s="10" t="inlineStr">
         <is>
-          <t>A10</t>
+          <t>Rule: Offline-ready design; A12</t>
         </is>
       </c>
       <c r="J109" s="10" t="inlineStr">
         <is>
-          <t>an amount with too many decimals</t>
+          <t>a repeated create request</t>
         </is>
       </c>
       <c r="K109" s="10" t="inlineStr">
         <is>
-          <t>it is posted</t>
+          <t>it arrives twice</t>
         </is>
       </c>
       <c r="L109" s="10" t="inlineStr">
         <is>
-          <t>it is refused with E_PRECISION</t>
+          <t>only one record exists</t>
         </is>
       </c>
       <c r="M109" s="10" t="inlineStr">
         <is>
-          <t>numeric(20,4), currencies.decimals</t>
+          <t>idempotency keys; client ids allowed on insert</t>
         </is>
       </c>
       <c r="N109" s="10" t="inlineStr">
         <is>
-          <t>12_ledger (2)</t>
+          <t>13_reservations (1)</t>
         </is>
       </c>
       <c r="O109" s="10" t="inlineStr">
@@ -9256,7 +9256,7 @@
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
         <is>
-          <t>NFR-005</t>
+          <t>NFR-004</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
@@ -9271,12 +9271,12 @@
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t>Business date and cut-off follow the property's timezone.</t>
+          <t>Money uses fixed decimals per currency (naira 2, CFA franc 0), never floating point.</t>
         </is>
       </c>
       <c r="E110" s="10" t="inlineStr">
         <is>
-          <t>BR-019</t>
+          <t>BR-013</t>
         </is>
       </c>
       <c r="F110" s="10" t="inlineStr">
@@ -9296,32 +9296,32 @@
       </c>
       <c r="I110" s="10" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A10</t>
         </is>
       </c>
       <c r="J110" s="10" t="inlineStr">
         <is>
-          <t>a property in Lagos</t>
+          <t>an amount with too many decimals</t>
         </is>
       </c>
       <c r="K110" s="10" t="inlineStr">
         <is>
-          <t>it is created just before or after cut-off</t>
+          <t>it is posted</t>
         </is>
       </c>
       <c r="L110" s="10" t="inlineStr">
         <is>
-          <t>the business date is the local hotel day, not the server's day</t>
+          <t>it is refused with E_PRECISION</t>
         </is>
       </c>
       <c r="M110" s="10" t="inlineStr">
         <is>
-          <t>local_business_date</t>
+          <t>numeric(20,4), currencies.decimals</t>
         </is>
       </c>
       <c r="N110" s="10" t="inlineStr">
         <is>
-          <t>17_more_features (1)</t>
+          <t>12_ledger (2)</t>
         </is>
       </c>
       <c r="O110" s="10" t="inlineStr">
@@ -9334,72 +9334,72 @@
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>DAY-006b</t>
+          <t>NFR-005</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t>Business Date</t>
+          <t>Non-functional</t>
         </is>
       </c>
       <c r="C111" s="10" t="inlineStr">
         <is>
-          <t>/checkout/$id</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t>A guest leaving on the arrival day is charged one night at check-out; a manager can waive it with a reason.</t>
+          <t>Business date and cut-off follow the property's timezone.</t>
         </is>
       </c>
       <c r="E111" s="10" t="inlineStr">
         <is>
+          <t>BR-019</t>
+        </is>
+      </c>
+      <c r="F111" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G111" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H111" s="10" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F111" s="10" t="inlineStr">
-        <is>
-          <t>Must</t>
-        </is>
-      </c>
-      <c r="G111" s="10" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H111" s="10" t="inlineStr">
-        <is>
-          <t>fo.checkout; fo.sameday.waive</t>
-        </is>
-      </c>
       <c r="I111" s="10" t="inlineStr">
         <is>
-          <t>Rule: DAY-006 decision</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="J111" s="10" t="inlineStr">
         <is>
-          <t>an in-house guest whose arrival and departure are today</t>
+          <t>a property in Lagos</t>
         </is>
       </c>
       <c r="K111" s="10" t="inlineStr">
         <is>
-          <t>they are checked out</t>
+          <t>it is created just before or after cut-off</t>
         </is>
       </c>
       <c r="L111" s="10" t="inlineStr">
         <is>
-          <t>one night (with tax) is posted unless a manager waives it with a reason</t>
+          <t>the business date is the local hotel day, not the server's day</t>
         </is>
       </c>
       <c r="M111" s="10" t="inlineStr">
         <is>
-          <t>preview_check_out_charge, check_out</t>
+          <t>local_business_date</t>
         </is>
       </c>
       <c r="N111" s="10" t="inlineStr">
         <is>
-          <t>21_same_day_checkout (28); upgrade (2)</t>
+          <t>17_more_features (1)</t>
         </is>
       </c>
       <c r="O111" s="10" t="inlineStr">
@@ -9412,22 +9412,22 @@
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>FIN-017</t>
+          <t>DAY-006b</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Business Date</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
         <is>
-          <t>/folios/$id</t>
+          <t>/checkout/$id</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t>A payment matching one on the same bill (amount, currency, method, reference) within 10 minutes is refused unless the cashier confirms it with a reason; the refusal names the earlier payment and the confirmation is audited.</t>
+          <t>A guest leaving on the arrival day is charged one night at check-out; a manager can waive it with a reason.</t>
         </is>
       </c>
       <c r="E112" s="10" t="inlineStr">
@@ -9447,37 +9447,37 @@
       </c>
       <c r="H112" s="10" t="inlineStr">
         <is>
-          <t>fin.payment.post</t>
+          <t>fo.checkout; fo.sameday.waive</t>
         </is>
       </c>
       <c r="I112" s="10" t="inlineStr">
         <is>
-          <t>Setting duplicate_payment_window_minutes</t>
+          <t>Rule: DAY-006 decision</t>
         </is>
       </c>
       <c r="J112" s="10" t="inlineStr">
         <is>
-          <t>a payment recorded on a bill a few minutes ago</t>
+          <t>an in-house guest whose arrival and departure are today</t>
         </is>
       </c>
       <c r="K112" s="10" t="inlineStr">
         <is>
-          <t>the same payment is recorded again with a new key</t>
+          <t>they are checked out</t>
         </is>
       </c>
       <c r="L112" s="10" t="inlineStr">
         <is>
-          <t>it is refused naming the earlier payment; with a reason it is recorded and audited as payment_duplicate_confirmed</t>
+          <t>one night (with tax) is posted unless a manager waives it with a reason</t>
         </is>
       </c>
       <c r="M112" s="10" t="inlineStr">
         <is>
-          <t>post_payment</t>
+          <t>preview_check_out_charge, check_out</t>
         </is>
       </c>
       <c r="N112" s="10" t="inlineStr">
         <is>
-          <t>25_duplicate_payments (20); browser: duplicate-payment</t>
+          <t>21_same_day_checkout (28); upgrade (2)</t>
         </is>
       </c>
       <c r="O112" s="10" t="inlineStr">
@@ -9490,7 +9490,7 @@
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>FIN-018</t>
+          <t>FIN-017</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
@@ -9500,12 +9500,12 @@
       </c>
       <c r="C113" s="10" t="inlineStr">
         <is>
-          <t>/setup/taxes</t>
+          <t>/folios/$id</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t>A hotel can match the tax method of its existing folio using setup alone: each tax on the room price only, food and drink untaxed. A sample bill of 45,000 room plus 12,001 bar totals 67,126.</t>
+          <t>A payment matching one on the same bill (amount, currency, method, reference) within 10 minutes is refused unless the cashier confirms it with a reason; the refusal names the earlier payment and the confirmation is audited.</t>
         </is>
       </c>
       <c r="E113" s="10" t="inlineStr">
@@ -9525,37 +9525,37 @@
       </c>
       <c r="H113" s="10" t="inlineStr">
         <is>
-          <t>setup.tax.manage</t>
+          <t>fin.payment.post</t>
         </is>
       </c>
       <c r="I113" s="10" t="inlineStr">
         <is>
-          <t>Tax rates compounds_on_previous; charge code is_taxable</t>
+          <t>Setting duplicate_payment_window_minutes</t>
         </is>
       </c>
       <c r="J113" s="10" t="inlineStr">
         <is>
-          <t>a property with service charge 10%, VAT 7.5% and state tax 5%, none compounding, and a non-taxable bar code</t>
+          <t>a payment recorded on a bill a few minutes ago</t>
         </is>
       </c>
       <c r="K113" s="10" t="inlineStr">
         <is>
-          <t>a room charge of 45,000 and a bar charge of 12,001 are posted</t>
+          <t>the same payment is recorded again with a new key</t>
         </is>
       </c>
       <c r="L113" s="10" t="inlineStr">
         <is>
-          <t>the taxes are 4,500, 3,375 and 2,250, the bar has no tax and the bill is 67,126</t>
+          <t>it is refused naming the earlier payment; with a reason it is recorded and audited as payment_duplicate_confirmed</t>
         </is>
       </c>
       <c r="M113" s="10" t="inlineStr">
         <is>
-          <t>save_tax_rate, save_charge_code, post_charge</t>
+          <t>post_payment</t>
         </is>
       </c>
       <c r="N113" s="10" t="inlineStr">
         <is>
-          <t>44_folio_sample_method (5)</t>
+          <t>25_duplicate_payments (20); browser: duplicate-payment</t>
         </is>
       </c>
       <c r="O113" s="10" t="inlineStr">
@@ -9563,16 +9563,12 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P113" s="10" t="inlineStr">
-        <is>
-          <t>Method only; the accountant still signs off the rates (A11)</t>
-        </is>
-      </c>
+      <c r="P113" s="10" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>FIN-019</t>
+          <t>FIN-018</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
@@ -9582,12 +9578,12 @@
       </c>
       <c r="C114" s="10" t="inlineStr">
         <is>
-          <t>/invoices/$id</t>
+          <t>/setup/taxes</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t>An invoice shows the check-in time, number of guests, number of nights, a total for each day, and the receipt reference of each charge. Invoices issued earlier stay as issued.</t>
+          <t>A hotel can match the tax method of its existing folio using setup alone: each tax on the room price only, food and drink untaxed. A sample bill of 45,000 room plus 12,001 bar totals 67,126.</t>
         </is>
       </c>
       <c r="E114" s="10" t="inlineStr">
@@ -9597,7 +9593,7 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G114" s="10" t="inlineStr">
@@ -9607,37 +9603,37 @@
       </c>
       <c r="H114" s="10" t="inlineStr">
         <is>
-          <t>fin.invoice.issue</t>
+          <t>setup.tax.manage</t>
         </is>
       </c>
       <c r="I114" s="10" t="inlineStr">
         <is>
-          <t>Invoice snapshot is insert-only</t>
+          <t>Tax rates compounds_on_previous; charge code is_taxable</t>
         </is>
       </c>
       <c r="J114" s="10" t="inlineStr">
         <is>
-          <t>a stay with charges, one with a receipt reference</t>
+          <t>a property with service charge 10%, VAT 7.5% and state tax 5%, none compounding, and a non-taxable bar code</t>
         </is>
       </c>
       <c r="K114" s="10" t="inlineStr">
         <is>
-          <t>an invoice is issued</t>
+          <t>a room charge of 45,000 and a bar charge of 12,001 are posted</t>
         </is>
       </c>
       <c r="L114" s="10" t="inlineStr">
         <is>
-          <t>the invoice shows nights, guests, check-in time, a total per day and the receipt reference, all worked out in the database</t>
+          <t>the taxes are 4,500, 3,375 and 2,250, the bar has no tax and the bill is 67,126</t>
         </is>
       </c>
       <c r="M114" s="10" t="inlineStr">
         <is>
-          <t>issue_invoice</t>
+          <t>save_tax_rate, save_charge_code, post_charge</t>
         </is>
       </c>
       <c r="N114" s="10" t="inlineStr">
         <is>
-          <t>45_invoice_layout (6)</t>
+          <t>44_folio_sample_method (5)</t>
         </is>
       </c>
       <c r="O114" s="10" t="inlineStr">
@@ -9647,14 +9643,14 @@
       </c>
       <c r="P114" s="10" t="inlineStr">
         <is>
-          <t>Day totals and fields are stored in the invoice header when it is issued</t>
+          <t>Method only; the accountant still signs off the rates (A11)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>FIN-020</t>
+          <t>FIN-019</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
@@ -9669,7 +9665,7 @@
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t>Invoice and interim invoice numbers carry the year and month of the hotel business date, then a count that restarts each month with no gaps (INV-202610-000001, INT-202610-000001). Invoices already issued keep their numbers.</t>
+          <t>An invoice shows the check-in time, number of guests, number of nights, a total for each day, and the receipt reference of each charge. Invoices issued earlier stay as issued.</t>
         </is>
       </c>
       <c r="E115" s="10" t="inlineStr">
@@ -9694,32 +9690,32 @@
       </c>
       <c r="I115" s="10" t="inlineStr">
         <is>
-          <t>document_sequences period_key</t>
+          <t>Invoice snapshot is insert-only</t>
         </is>
       </c>
       <c r="J115" s="10" t="inlineStr">
         <is>
-          <t>a hotel with invoices issued in one month</t>
+          <t>a stay with charges, one with a receipt reference</t>
         </is>
       </c>
       <c r="K115" s="10" t="inlineStr">
         <is>
-          <t>an invoice is issued in the next month</t>
+          <t>an invoice is issued</t>
         </is>
       </c>
       <c r="L115" s="10" t="inlineStr">
         <is>
-          <t>its number starts with the new year and month and the count restarts at 1; the INT and INV series stay separate; reservation and folio numbers are unchanged</t>
+          <t>the invoice shows nights, guests, check-in time, a total per day and the receipt reference, all worked out in the database</t>
         </is>
       </c>
       <c r="M115" s="10" t="inlineStr">
         <is>
-          <t>next_document_number, issue_invoice</t>
+          <t>issue_invoice</t>
         </is>
       </c>
       <c r="N115" s="10" t="inlineStr">
         <is>
-          <t>46_invoice_number_month (8); 17_more_features</t>
+          <t>45_invoice_layout (6)</t>
         </is>
       </c>
       <c r="O115" s="10" t="inlineStr">
@@ -9729,29 +9725,29 @@
       </c>
       <c r="P115" s="10" t="inlineStr">
         <is>
-          <t>Month comes from the business date, not the clock. No hotel code in the number yet.</t>
+          <t>Day totals and fields are stored in the invoice header when it is issued</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
         <is>
-          <t>GST-007</t>
+          <t>FIN-020</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t>Guests</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C116" s="10" t="inlineStr">
         <is>
-          <t>/guests/$id; check-in; walk-in</t>
+          <t>/invoices/$id</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t>A photo or scan of an ID document is kept in private storage, shrunk and stripped of hidden data in the browser, and opened only through a 60-second link.</t>
+          <t>Invoice and interim invoice numbers carry the year and month of the hotel business date, then a count that restarts each month with no gaps (INV-202610-000001, INT-202610-000001). Invoices already issued keep their numbers.</t>
         </is>
       </c>
       <c r="E116" s="10" t="inlineStr">
@@ -9761,7 +9757,7 @@
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G116" s="10" t="inlineStr">
@@ -9771,37 +9767,37 @@
       </c>
       <c r="H116" s="10" t="inlineStr">
         <is>
-          <t>guest.document.file.upload / view / delete</t>
+          <t>fin.invoice.issue</t>
         </is>
       </c>
       <c r="I116" s="10" t="inlineStr">
         <is>
-          <t>SET-009 switch</t>
+          <t>document_sequences period_key</t>
         </is>
       </c>
       <c r="J116" s="10" t="inlineStr">
         <is>
-          <t>a hotel that allows ID photos</t>
+          <t>a hotel with invoices issued in one month</t>
         </is>
       </c>
       <c r="K116" s="10" t="inlineStr">
         <is>
-          <t>front desk adds an ID photo</t>
+          <t>an invoice is issued in the next month</t>
         </is>
       </c>
       <c r="L116" s="10" t="inlineStr">
         <is>
-          <t>it is stored privately and opens only through a short-lived link</t>
+          <t>its number starts with the new year and month and the count restarts at 1; the INT and INV series stay separate; reservation and folio numbers are unchanged</t>
         </is>
       </c>
       <c r="M116" s="10" t="inlineStr">
         <is>
-          <t>begin_id_photo_upload, finish_id_photo_upload, open_id_photo</t>
+          <t>next_document_number, issue_invoice</t>
         </is>
       </c>
       <c r="N116" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (30)</t>
+          <t>46_invoice_number_month (8); 17_more_features</t>
         </is>
       </c>
       <c r="O116" s="10" t="inlineStr">
@@ -9809,12 +9805,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P116" s="10" t="inlineStr"/>
+      <c r="P116" s="10" t="inlineStr">
+        <is>
+          <t>Month comes from the business date, not the clock. No hotel code in the number yet.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>GST-008</t>
+          <t>GST-007</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
@@ -9824,12 +9824,12 @@
       </c>
       <c r="C117" s="10" t="inlineStr">
         <is>
-          <t>/guests/$id</t>
+          <t>/guests/$id; check-in; walk-in</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t>Every upload, view and deletion of an ID photo is audited with ids only, no personal data.</t>
+          <t>A photo or scan of an ID document is kept in private storage, shrunk and stripped of hidden data in the browser, and opened only through a 60-second link.</t>
         </is>
       </c>
       <c r="E117" s="10" t="inlineStr">
@@ -9849,37 +9849,37 @@
       </c>
       <c r="H117" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>guest.document.file.upload / view / delete</t>
         </is>
       </c>
       <c r="I117" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SET-009 switch</t>
         </is>
       </c>
       <c r="J117" s="10" t="inlineStr">
         <is>
-          <t>an ID photo</t>
+          <t>a hotel that allows ID photos</t>
         </is>
       </c>
       <c r="K117" s="10" t="inlineStr">
         <is>
-          <t>it is uploaded, opened or deleted</t>
+          <t>front desk adds an ID photo</t>
         </is>
       </c>
       <c r="L117" s="10" t="inlineStr">
         <is>
-          <t>an audit row records who and which file, with no personal data</t>
+          <t>it is stored privately and opens only through a short-lived link</t>
         </is>
       </c>
       <c r="M117" s="10" t="inlineStr">
         <is>
-          <t>app.audit_id_photo</t>
+          <t>begin_id_photo_upload, finish_id_photo_upload, open_id_photo</t>
         </is>
       </c>
       <c r="N117" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (9)</t>
+          <t>24_id_photos (30)</t>
         </is>
       </c>
       <c r="O117" s="10" t="inlineStr">
@@ -9892,7 +9892,7 @@
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
         <is>
-          <t>GST-009</t>
+          <t>GST-008</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
@@ -9907,7 +9907,7 @@
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t>ID photos are removed from storage when the guest is anonymised or the document is removed, and move with the guest when two profiles are merged.</t>
+          <t>Every upload, view and deletion of an ID photo is audited with ids only, no personal data.</t>
         </is>
       </c>
       <c r="E118" s="10" t="inlineStr">
@@ -9937,27 +9937,27 @@
       </c>
       <c r="J118" s="10" t="inlineStr">
         <is>
-          <t>a guest with ID photos</t>
+          <t>an ID photo</t>
         </is>
       </c>
       <c r="K118" s="10" t="inlineStr">
         <is>
-          <t>the guest is anonymised, the document removed, or the profile merged</t>
+          <t>it is uploaded, opened or deleted</t>
         </is>
       </c>
       <c r="L118" s="10" t="inlineStr">
         <is>
-          <t>the files are removed, or move to the kept profile</t>
+          <t>an audit row records who and which file, with no personal data</t>
         </is>
       </c>
       <c r="M118" s="10" t="inlineStr">
         <is>
-          <t>anonymise_guest, merge_guests, delete_id_photo</t>
+          <t>app.audit_id_photo</t>
         </is>
       </c>
       <c r="N118" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (4)</t>
+          <t>24_id_photos (9)</t>
         </is>
       </c>
       <c r="O118" s="10" t="inlineStr">
@@ -9970,7 +9970,7 @@
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>GST-010</t>
+          <t>GST-009</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
@@ -9980,12 +9980,12 @@
       </c>
       <c r="C119" s="10" t="inlineStr">
         <is>
-          <t>(daily clean-up)</t>
+          <t>/guests/$id</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t>ID photos are deleted automatically a set number of months (one setting, now 12) after the guest's last check-out, unless the guest has a booking that is not over.</t>
+          <t>ID photos are removed from storage when the guest is anonymised or the document is removed, and move with the guest when two profiles are merged.</t>
         </is>
       </c>
       <c r="E119" s="10" t="inlineStr">
@@ -10010,32 +10010,32 @@
       </c>
       <c r="I119" s="10" t="inlineStr">
         <is>
-          <t>Setting id_photo_keep_months; daily cron</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J119" s="10" t="inlineStr">
         <is>
-          <t>a guest whose last check-out was more than the keep period ago</t>
+          <t>a guest with ID photos</t>
         </is>
       </c>
       <c r="K119" s="10" t="inlineStr">
         <is>
-          <t>the daily clean-up runs</t>
+          <t>the guest is anonymised, the document removed, or the profile merged</t>
         </is>
       </c>
       <c r="L119" s="10" t="inlineStr">
         <is>
-          <t>their ID photos are deleted</t>
+          <t>the files are removed, or move to the kept profile</t>
         </is>
       </c>
       <c r="M119" s="10" t="inlineStr">
         <is>
-          <t>/api/cron/id-photo-cleanup</t>
+          <t>anonymise_guest, merge_guests, delete_id_photo</t>
         </is>
       </c>
       <c r="N119" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (5)</t>
+          <t>24_id_photos (4)</t>
         </is>
       </c>
       <c r="O119" s="10" t="inlineStr">
@@ -10048,22 +10048,22 @@
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
         <is>
-          <t>ROOM-005</t>
+          <t>GST-010</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
         <is>
-          <t>Rooms</t>
+          <t>Guests</t>
         </is>
       </c>
       <c r="C120" s="10" t="inlineStr">
         <is>
-          <t>/rooms</t>
+          <t>(daily clean-up)</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t>Rooms are added one at a time or several by number or by name, with a preview; labels are free text up to 30 characters, unique per hotel ignoring case and extra spaces, shown as typed and sorted in natural order.</t>
+          <t>ID photos are deleted automatically a set number of months (one setting, now 12) after the guest's last check-out, unless the guest has a booking that is not over.</t>
         </is>
       </c>
       <c r="E120" s="10" t="inlineStr">
@@ -10083,37 +10083,37 @@
       </c>
       <c r="H120" s="10" t="inlineStr">
         <is>
-          <t>setup.room.edit</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I120" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Setting id_photo_keep_months; daily cron</t>
         </is>
       </c>
       <c r="J120" s="10" t="inlineStr">
         <is>
-          <t>an administrator on the Rooms page</t>
+          <t>a guest whose last check-out was more than the keep period ago</t>
         </is>
       </c>
       <c r="K120" s="10" t="inlineStr">
         <is>
-          <t>they add rooms by number range or by names</t>
+          <t>the daily clean-up runs</t>
         </is>
       </c>
       <c r="L120" s="10" t="inlineStr">
         <is>
-          <t>valid new rooms are created, duplicates skipped and invalid names shown</t>
+          <t>their ID photos are deleted</t>
         </is>
       </c>
       <c r="M120" s="10" t="inlineStr">
         <is>
-          <t>add_rooms_range, add_rooms_named, save_room</t>
+          <t>/api/cron/id-photo-cleanup</t>
         </is>
       </c>
       <c r="N120" s="10" t="inlineStr">
         <is>
-          <t>23_room_labels (46); 26_small_fixes (1); browser: rooms-add</t>
+          <t>24_id_photos (5)</t>
         </is>
       </c>
       <c r="O120" s="10" t="inlineStr">
@@ -10126,22 +10126,22 @@
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>SET-009</t>
+          <t>ROOM-005</t>
         </is>
       </c>
       <c r="B121" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Rooms</t>
         </is>
       </c>
       <c r="C121" s="10" t="inlineStr">
         <is>
-          <t>/setup/property</t>
+          <t>/rooms</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t>Per hotel: "Allow ID photos" (off by default) and "Require ID photo at check-in" (only when allowed). While Allow is off, uploading and opening ID photos are refused.</t>
+          <t>Rooms are added one at a time or several by number or by name, with a preview; labels are free text up to 30 characters, unique per hotel ignoring case and extra spaces, shown as typed and sorted in natural order.</t>
         </is>
       </c>
       <c r="E121" s="10" t="inlineStr">
@@ -10161,7 +10161,7 @@
       </c>
       <c r="H121" s="10" t="inlineStr">
         <is>
-          <t>setup.property.edit</t>
+          <t>setup.room.edit</t>
         </is>
       </c>
       <c r="I121" s="10" t="inlineStr">
@@ -10171,27 +10171,27 @@
       </c>
       <c r="J121" s="10" t="inlineStr">
         <is>
-          <t>a hotel with ID photos off</t>
+          <t>an administrator on the Rooms page</t>
         </is>
       </c>
       <c r="K121" s="10" t="inlineStr">
         <is>
-          <t>staff try to add or open an ID photo</t>
+          <t>they add rooms by number range or by names</t>
         </is>
       </c>
       <c r="L121" s="10" t="inlineStr">
         <is>
-          <t>it is refused; when Require is on, check-in waits for an ID photo</t>
+          <t>valid new rooms are created, duplicates skipped and invalid names shown</t>
         </is>
       </c>
       <c r="M121" s="10" t="inlineStr">
         <is>
-          <t>set_id_photo_settings</t>
+          <t>add_rooms_range, add_rooms_named, save_room</t>
         </is>
       </c>
       <c r="N121" s="10" t="inlineStr">
         <is>
-          <t>24_id_photos (10)</t>
+          <t>23_room_labels (46); 26_small_fixes (1); browser: rooms-add</t>
         </is>
       </c>
       <c r="O121" s="10" t="inlineStr">
@@ -10204,32 +10204,32 @@
     <row r="122">
       <c r="A122" s="10" t="inlineStr">
         <is>
-          <t>GRP-001</t>
+          <t>SET-009</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
         <is>
-          <t>Platform &amp; Tenancy</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C122" s="10" t="inlineStr">
         <is>
-          <t>All branches</t>
+          <t>/setup/property</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t>A built-in Group Manager role and the permission rpt.group.view exist; only System Administrator, General Manager and Group Manager hold the permission.</t>
+          <t>Per hotel: "Allow ID photos" (off by default) and "Require ID photo at check-in" (only when allowed). While Allow is off, uploading and opening ID photos are refused.</t>
         </is>
       </c>
       <c r="E122" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F122" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G122" s="10" t="inlineStr">
@@ -10239,33 +10239,37 @@
       </c>
       <c r="H122" s="10" t="inlineStr">
         <is>
-          <t>rpt.group.view</t>
-        </is>
-      </c>
-      <c r="I122" s="10" t="inlineStr"/>
+          <t>setup.property.edit</t>
+        </is>
+      </c>
+      <c r="I122" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="J122" s="10" t="inlineStr">
         <is>
-          <t>a hotel group with several branches</t>
+          <t>a hotel with ID photos off</t>
         </is>
       </c>
       <c r="K122" s="10" t="inlineStr">
         <is>
-          <t>an owner wants a view-only manager for the whole group</t>
+          <t>staff try to add or open an ID photo</t>
         </is>
       </c>
       <c r="L122" s="10" t="inlineStr">
         <is>
-          <t>they assign the Group Manager role branch by branch, and that person can look but not post or change anything</t>
+          <t>it is refused; when Require is on, check-in waits for an ID photo</t>
         </is>
       </c>
       <c r="M122" s="10" t="inlineStr">
         <is>
-          <t>20261013120000_group_view.sql</t>
+          <t>set_id_photo_settings</t>
         </is>
       </c>
       <c r="N122" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (5)</t>
+          <t>24_id_photos (10)</t>
         </is>
       </c>
       <c r="O122" s="10" t="inlineStr">
@@ -10273,16 +10277,12 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P122" s="10" t="inlineStr">
-        <is>
-          <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
-        </is>
-      </c>
+      <c r="P122" s="10" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>GRP-002</t>
+          <t>GRP-001</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
@@ -10297,7 +10297,7 @@
       </c>
       <c r="D123" s="10" t="inlineStr">
         <is>
-          <t>One call shows every branch the person may see: occupancy, in house, arrivals and departures to come, approvals, repairs and last night revenue, with group totals. Revenue is totalled per currency.</t>
+          <t>A built-in Group Manager role and the permission rpt.group.view exist; only System Administrator, General Manager and Group Manager hold the permission.</t>
         </is>
       </c>
       <c r="E123" s="10" t="inlineStr">
@@ -10323,27 +10323,27 @@
       <c r="I123" s="10" t="inlineStr"/>
       <c r="J123" s="10" t="inlineStr">
         <is>
-          <t>a group with a Lagos and an Abuja branch</t>
+          <t>a hotel group with several branches</t>
         </is>
       </c>
       <c r="K123" s="10" t="inlineStr">
         <is>
-          <t>a group manager opens All branches</t>
+          <t>an owner wants a view-only manager for the whole group</t>
         </is>
       </c>
       <c r="L123" s="10" t="inlineStr">
         <is>
-          <t>they see both branches with figures from the database, never another hotel group, and staff without the permission are refused</t>
+          <t>they assign the Group Manager role branch by branch, and that person can look but not post or change anything</t>
         </is>
       </c>
       <c r="M123" s="10" t="inlineStr">
         <is>
-          <t>group_overview; /group screen</t>
+          <t>20261013120000_group_view.sql</t>
         </is>
       </c>
       <c r="N123" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (10)</t>
+          <t>35_group_view (5)</t>
         </is>
       </c>
       <c r="O123" s="10" t="inlineStr">
@@ -10353,14 +10353,14 @@
       </c>
       <c r="P123" s="10" t="inlineStr">
         <is>
-          <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
+          <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="10" t="inlineStr">
         <is>
-          <t>GRP-003</t>
+          <t>GRP-002</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
@@ -10375,7 +10375,7 @@
       </c>
       <c r="D124" s="10" t="inlineStr">
         <is>
-          <t>A Group Manager sees only the branches they are assigned to, and cannot post charges or check guests in.</t>
+          <t>One call shows every branch the person may see: occupancy, in house, arrivals and departures to come, approvals, repairs and last night revenue, with group totals. Revenue is totalled per currency.</t>
         </is>
       </c>
       <c r="E124" s="10" t="inlineStr">
@@ -10401,27 +10401,27 @@
       <c r="I124" s="10" t="inlineStr"/>
       <c r="J124" s="10" t="inlineStr">
         <is>
-          <t>a Group Manager assigned to one branch</t>
+          <t>a group with a Lagos and an Abuja branch</t>
         </is>
       </c>
       <c r="K124" s="10" t="inlineStr">
         <is>
-          <t>a second branch is assigned</t>
+          <t>a group manager opens All branches</t>
         </is>
       </c>
       <c r="L124" s="10" t="inlineStr">
         <is>
-          <t>the second branch appears; the role never gets write permissions</t>
+          <t>they see both branches with figures from the database, never another hotel group, and staff without the permission are refused</t>
         </is>
       </c>
       <c r="M124" s="10" t="inlineStr">
         <is>
-          <t>assign_role (existing); group_overview</t>
+          <t>group_overview; /group screen</t>
         </is>
       </c>
       <c r="N124" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (3)</t>
+          <t>35_group_view (10)</t>
         </is>
       </c>
       <c r="O124" s="10" t="inlineStr">
@@ -10431,14 +10431,14 @@
       </c>
       <c r="P124" s="10" t="inlineStr">
         <is>
-          <t>Access is per branch, using the existing role assignment screen.</t>
+          <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>GRP-004</t>
+          <t>GRP-003</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
@@ -10448,12 +10448,12 @@
       </c>
       <c r="C125" s="10" t="inlineStr">
         <is>
-          <t>All branches (Copy setup)</t>
+          <t>All branches</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t>A new branch can copy room types, rate plans and prices from an existing branch, once, into an empty branch.</t>
+          <t>A Group Manager sees only the branches they are assigned to, and cannot post charges or check guests in.</t>
         </is>
       </c>
       <c r="E125" s="10" t="inlineStr">
@@ -10473,33 +10473,33 @@
       </c>
       <c r="H125" s="10" t="inlineStr">
         <is>
-          <t>setup.room.manage, setup.rate.manage</t>
+          <t>rpt.group.view</t>
         </is>
       </c>
       <c r="I125" s="10" t="inlineStr"/>
       <c r="J125" s="10" t="inlineStr">
         <is>
-          <t>a new empty branch</t>
+          <t>a Group Manager assigned to one branch</t>
         </is>
       </c>
       <c r="K125" s="10" t="inlineStr">
         <is>
-          <t>the owner copies setup from the first branch</t>
+          <t>a second branch is assigned</t>
         </is>
       </c>
       <c r="L125" s="10" t="inlineStr">
         <is>
-          <t>room types, rate plans and prices appear on the new branch and point at its own room types; rooms are not copied; a second copy is refused; the copy is audited</t>
+          <t>the second branch appears; the role never gets write permissions</t>
         </is>
       </c>
       <c r="M125" s="10" t="inlineStr">
         <is>
-          <t>copy_property_setup</t>
+          <t>assign_role (existing); group_overview</t>
         </is>
       </c>
       <c r="N125" s="10" t="inlineStr">
         <is>
-          <t>35_group_view (13)</t>
+          <t>35_group_view (3)</t>
         </is>
       </c>
       <c r="O125" s="10" t="inlineStr">
@@ -10509,29 +10509,29 @@
       </c>
       <c r="P125" s="10" t="inlineStr">
         <is>
-          <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
+          <t>Access is per branch, using the existing role assignment screen.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="10" t="inlineStr">
         <is>
-          <t>RPT-005</t>
+          <t>GRP-004</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Platform &amp; Tenancy</t>
         </is>
       </c>
       <c r="C126" s="10" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>All branches (Copy setup)</t>
         </is>
       </c>
       <c r="D126" s="10" t="inlineStr">
         <is>
-          <t>Revenue by booking source: bookings, cancellations, no-shows, room nights, room revenue and average rate for each source in a date range.</t>
+          <t>A new branch can copy room types, rate plans and prices from an existing branch, once, into an empty branch.</t>
         </is>
       </c>
       <c r="E126" s="10" t="inlineStr">
@@ -10551,33 +10551,33 @@
       </c>
       <c r="H126" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view</t>
+          <t>setup.room.manage, setup.rate.manage</t>
         </is>
       </c>
       <c r="I126" s="10" t="inlineStr"/>
       <c r="J126" s="10" t="inlineStr">
         <is>
-          <t>bookings from direct, phone and company sources</t>
+          <t>a new empty branch</t>
         </is>
       </c>
       <c r="K126" s="10" t="inlineStr">
         <is>
-          <t>the accountant picks a date range</t>
+          <t>the owner copies setup from the first branch</t>
         </is>
       </c>
       <c r="L126" s="10" t="inlineStr">
         <is>
-          <t>each source shows its own counts and room revenue (room charges only, before tax); cancelled bookings add no nights</t>
+          <t>room types, rate plans and prices appear on the new branch and point at its own room types; rooms are not copied; a second copy is refused; the copy is audited</t>
         </is>
       </c>
       <c r="M126" s="10" t="inlineStr">
         <is>
-          <t>20261013130000_source_ageing_reports.sql: report_revenue_by_source; Reports, By booking source tab</t>
+          <t>copy_property_setup</t>
         </is>
       </c>
       <c r="N126" s="10" t="inlineStr">
         <is>
-          <t>36_source_ageing (13)</t>
+          <t>35_group_view (13)</t>
         </is>
       </c>
       <c r="O126" s="10" t="inlineStr">
@@ -10587,14 +10587,14 @@
       </c>
       <c r="P126" s="10" t="inlineStr">
         <is>
-          <t>Bookings counted by arrival date; revenue by posting date.</t>
+          <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
         <is>
-          <t>RPT-006</t>
+          <t>RPT-005</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
@@ -10609,7 +10609,7 @@
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t>Ageing of unpaid balances by booking source: current, 1 to 7, 8 to 30, 31 to 60 and over 60 days since the due departure, plus credit held.</t>
+          <t>Revenue by booking source: bookings, cancellations, no-shows, room nights, room revenue and average rate for each source in a date range.</t>
         </is>
       </c>
       <c r="E127" s="10" t="inlineStr">
@@ -10635,27 +10635,27 @@
       <c r="I127" s="10" t="inlineStr"/>
       <c r="J127" s="10" t="inlineStr">
         <is>
-          <t>guests and companies who left owing money</t>
+          <t>bookings from direct, phone and company sources</t>
         </is>
       </c>
       <c r="K127" s="10" t="inlineStr">
         <is>
-          <t>the accountant opens the Ageing tab</t>
+          <t>the accountant picks a date range</t>
         </is>
       </c>
       <c r="L127" s="10" t="inlineStr">
         <is>
-          <t>each source shows what is owed in each age column; paid bills drop out; overpayments show as credit held; the total matches Outstanding balances</t>
+          <t>each source shows its own counts and room revenue (room charges only, before tax); cancelled bookings add no nights</t>
         </is>
       </c>
       <c r="M127" s="10" t="inlineStr">
         <is>
-          <t>report_balance_ageing; Reports, Ageing tab</t>
+          <t>20261013130000_source_ageing_reports.sql: report_revenue_by_source; Reports, By booking source tab</t>
         </is>
       </c>
       <c r="N127" s="10" t="inlineStr">
         <is>
-          <t>36_source_ageing (11)</t>
+          <t>36_source_ageing (13)</t>
         </is>
       </c>
       <c r="O127" s="10" t="inlineStr">
@@ -10665,14 +10665,14 @@
       </c>
       <c r="P127" s="10" t="inlineStr">
         <is>
-          <t>Guests still staying count as current.</t>
+          <t>Bookings counted by arrival date; revenue by posting date.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
         <is>
-          <t>RPT-007</t>
+          <t>RPT-006</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
@@ -10682,17 +10682,17 @@
       </c>
       <c r="C128" s="10" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="D128" s="10" t="inlineStr">
         <is>
-          <t>The owner summary: last night's occupancy and revenue, money collected by payment method, today's arrivals, departures and rooms, what is waiting, and old unpaid bills, as plain sentences built in the database. Works with AI off; a later daily email can send the same text.</t>
+          <t>Ageing of unpaid balances by booking source: current, 1 to 7, 8 to 30, 31 to 60 and over 60 days since the due departure, plus credit held.</t>
         </is>
       </c>
       <c r="E128" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F128" s="10" t="inlineStr">
@@ -10707,37 +10707,33 @@
       </c>
       <c r="H128" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view, rpt.operations.view</t>
-        </is>
-      </c>
-      <c r="I128" s="10" t="inlineStr">
-        <is>
-          <t>Reads the morning brief facts</t>
-        </is>
-      </c>
+          <t>rpt.finance.view</t>
+        </is>
+      </c>
+      <c r="I128" s="10" t="inlineStr"/>
       <c r="J128" s="10" t="inlineStr">
         <is>
-          <t>a hotel with a closed day and payments on it</t>
+          <t>guests and companies who left owing money</t>
         </is>
       </c>
       <c r="K128" s="10" t="inlineStr">
         <is>
-          <t>the owner opens the dashboard</t>
+          <t>the accountant opens the Ageing tab</t>
         </is>
       </c>
       <c r="L128" s="10" t="inlineStr">
         <is>
-          <t>sees yesterday at a glance with the money collected by method; front desk without finance reports is refused</t>
+          <t>each source shows what is owed in each age column; paid bills drop out; overpayments show as credit held; the total matches Outstanding balances</t>
         </is>
       </c>
       <c r="M128" s="10" t="inlineStr">
         <is>
-          <t>owner_summary</t>
+          <t>report_balance_ageing; Reports, Ageing tab</t>
         </is>
       </c>
       <c r="N128" s="10" t="inlineStr">
         <is>
-          <t>47_owner_summary (9); browser: owner-summary</t>
+          <t>36_source_ageing (11)</t>
         </is>
       </c>
       <c r="O128" s="10" t="inlineStr">
@@ -10747,34 +10743,34 @@
       </c>
       <c r="P128" s="10" t="inlineStr">
         <is>
-          <t>Email delivery waits on the sending domain and email account. Collected money nets payment reversals the same day (migration 20261015130000).</t>
+          <t>Guests still staying count as current.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>RPT-007</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
         <is>
-          <t>AI helpers</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C129" s="10" t="inlineStr">
         <is>
-          <t>Dashboard, Admin</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D129" s="10" t="inlineStr">
         <is>
-          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
+          <t>The owner summary: last night's occupancy and revenue, money collected by payment method, today's arrivals, departures and rooms, what is waiting, and old unpaid bills, as plain sentences built in the database. Works with AI off; a later daily email can send the same text.</t>
         </is>
       </c>
       <c r="E129" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F129" s="10" t="inlineStr">
@@ -10789,33 +10785,37 @@
       </c>
       <c r="H129" s="10" t="inlineStr">
         <is>
-          <t>adm.ai.manage</t>
-        </is>
-      </c>
-      <c r="I129" s="10" t="inlineStr"/>
+          <t>rpt.finance.view, rpt.operations.view</t>
+        </is>
+      </c>
+      <c r="I129" s="10" t="inlineStr">
+        <is>
+          <t>Reads the morning brief facts</t>
+        </is>
+      </c>
       <c r="J129" s="10" t="inlineStr">
         <is>
-          <t>a new hotel</t>
+          <t>a hotel with a closed day and payments on it</t>
         </is>
       </c>
       <c r="K129" s="10" t="inlineStr">
         <is>
-          <t>a manager opens Admin, AI helpers</t>
+          <t>the owner opens the dashboard</t>
         </is>
       </c>
       <c r="L129" s="10" t="inlineStr">
         <is>
-          <t>nothing runs until they switch it on and the change is in the audit log</t>
+          <t>sees yesterday at a glance with the money collected by method; front desk without finance reports is refused</t>
         </is>
       </c>
       <c r="M129" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
+          <t>owner_summary</t>
         </is>
       </c>
       <c r="N129" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (11)</t>
+          <t>47_owner_summary (9); browser: owner-summary</t>
         </is>
       </c>
       <c r="O129" s="10" t="inlineStr">
@@ -10825,14 +10825,14 @@
       </c>
       <c r="P129" s="10" t="inlineStr">
         <is>
-          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
+          <t>Email delivery waits on the sending domain and email account. Collected money nets payment reversals the same day (migration 20261015130000).</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
         <is>
-          <t>AI-002</t>
+          <t>AI-001</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="D130" s="10" t="inlineStr">
         <is>
-          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
+          <t>AI helpers are off for every hotel until a System Administrator or General Manager switches them on, with a monthly limit; the switch is audited.</t>
         </is>
       </c>
       <c r="E130" s="10" t="inlineStr">
@@ -10867,28 +10867,28 @@
       </c>
       <c r="H130" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view, rpt.operations.view</t>
+          <t>adm.ai.manage</t>
         </is>
       </c>
       <c r="I130" s="10" t="inlineStr"/>
       <c r="J130" s="10" t="inlineStr">
         <is>
-          <t>a hotel with guests, approvals and overdue bills</t>
+          <t>a new hotel</t>
         </is>
       </c>
       <c r="K130" s="10" t="inlineStr">
         <is>
-          <t>a brief is started</t>
+          <t>a manager opens Admin, AI helpers</t>
         </is>
       </c>
       <c r="L130" s="10" t="inlineStr">
         <is>
-          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
+          <t>nothing runs until they switch it on and the change is in the audit log</t>
         </is>
       </c>
       <c r="M130" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
+          <t>20261013140000_ai_morning_brief.sql: set_ai_settings, ai_status; Admin, AI helpers tab</t>
         </is>
       </c>
       <c r="N130" s="10" t="inlineStr">
@@ -10903,14 +10903,14 @@
       </c>
       <c r="P130" s="10" t="inlineStr">
         <is>
-          <t>Overdue means unpaid more than 30 days after departure.</t>
+          <t>Custom roles copied earlier do not get adm.ai.manage.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
         <is>
-          <t>AI-003</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
@@ -10925,7 +10925,7 @@
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
+          <t>The facts sent to the AI are counts and money lines built by the database: no guest names, ID details, room numbers or card data.</t>
         </is>
       </c>
       <c r="E131" s="10" t="inlineStr">
@@ -10945,33 +10945,33 @@
       </c>
       <c r="H131" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view</t>
+          <t>rpt.finance.view, rpt.operations.view</t>
         </is>
       </c>
       <c r="I131" s="10" t="inlineStr"/>
       <c r="J131" s="10" t="inlineStr">
         <is>
-          <t>a limit of 2</t>
+          <t>a hotel with guests, approvals and overdue bills</t>
         </is>
       </c>
       <c r="K131" s="10" t="inlineStr">
         <is>
-          <t>a third brief is requested</t>
+          <t>a brief is started</t>
         </is>
       </c>
       <c r="L131" s="10" t="inlineStr">
         <is>
-          <t>it is refused until a failed call frees a slot or the month turns</t>
+          <t>the facts hold only business date, last night, today, attention figures and plain lines, and overdue money matches the ledger</t>
         </is>
       </c>
       <c r="M131" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
+          <t>20261013140000_ai_morning_brief.sql: ai_morning_brief_start, app.morning_brief_facts</t>
         </is>
       </c>
       <c r="N131" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (5)</t>
+          <t>37_ai_brief (11)</t>
         </is>
       </c>
       <c r="O131" s="10" t="inlineStr">
@@ -10979,12 +10979,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P131" s="10" t="inlineStr"/>
+      <c r="P131" s="10" t="inlineStr">
+        <is>
+          <t>Overdue means unpaid more than 30 days after departure.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="10" t="inlineStr">
         <is>
-          <t>AI-004</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
@@ -10999,7 +11003,7 @@
       </c>
       <c r="D132" s="10" t="inlineStr">
         <is>
-          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
+          <t>Each hotel has a monthly limit on AI drafts; failed calls do not count; a call can be finished once, by the person who started it.</t>
         </is>
       </c>
       <c r="E132" s="10" t="inlineStr">
@@ -11019,33 +11023,33 @@
       </c>
       <c r="H132" s="10" t="inlineStr">
         <is>
-          <t>rpt.finance.view, rpt.operations.view</t>
+          <t>rpt.finance.view</t>
         </is>
       </c>
       <c r="I132" s="10" t="inlineStr"/>
       <c r="J132" s="10" t="inlineStr">
         <is>
-          <t>front desk, housekeeping, another hotel</t>
+          <t>a limit of 2</t>
         </is>
       </c>
       <c r="K132" s="10" t="inlineStr">
         <is>
-          <t>they ask for the brief or touch the tables</t>
+          <t>a third brief is requested</t>
         </is>
       </c>
       <c r="L132" s="10" t="inlineStr">
         <is>
-          <t>they are refused</t>
+          <t>it is refused until a failed call frees a slot or the month turns</t>
         </is>
       </c>
       <c r="M132" s="10" t="inlineStr">
         <is>
-          <t>20261013140000_ai_morning_brief.sql</t>
+          <t>20261013140000_ai_morning_brief.sql: ai_call_finish</t>
         </is>
       </c>
       <c r="N132" s="10" t="inlineStr">
         <is>
-          <t>37_ai_brief (7)</t>
+          <t>37_ai_brief (5)</t>
         </is>
       </c>
       <c r="O132" s="10" t="inlineStr">
@@ -11058,7 +11062,7 @@
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
         <is>
-          <t>AI-005</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
@@ -11073,7 +11077,7 @@
       </c>
       <c r="D133" s="10" t="inlineStr">
         <is>
-          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
+          <t>Only finance and operations viewers can ask for the brief; the usage log and settings cannot be written or read directly by the browser.</t>
         </is>
       </c>
       <c r="E133" s="10" t="inlineStr">
@@ -11093,33 +11097,33 @@
       </c>
       <c r="H133" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>rpt.finance.view, rpt.operations.view</t>
         </is>
       </c>
       <c r="I133" s="10" t="inlineStr"/>
       <c r="J133" s="10" t="inlineStr">
         <is>
-          <t>a draft that rounds or invents a figure</t>
+          <t>front desk, housekeeping, another hotel</t>
         </is>
       </c>
       <c r="K133" s="10" t="inlineStr">
         <is>
-          <t>the brief is written</t>
+          <t>they ask for the brief or touch the tables</t>
         </is>
       </c>
       <c r="L133" s="10" t="inlineStr">
         <is>
-          <t>the plain database lines are shown instead, with a note</t>
+          <t>they are refused</t>
         </is>
       </c>
       <c r="M133" s="10" t="inlineStr">
         <is>
-          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
+          <t>20261013140000_ai_morning_brief.sql</t>
         </is>
       </c>
       <c r="N133" s="10" t="inlineStr">
         <is>
-          <t>browser unit: ai-brief-unit (8)</t>
+          <t>37_ai_brief (7)</t>
         </is>
       </c>
       <c r="O133" s="10" t="inlineStr">
@@ -11127,31 +11131,27 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P133" s="10" t="inlineStr">
-        <is>
-          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
-        </is>
-      </c>
+      <c r="P133" s="10" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
         <is>
-          <t>SET-010</t>
+          <t>AI-005</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>AI helpers</t>
         </is>
       </c>
       <c r="C134" s="10" t="inlineStr">
         <is>
-          <t>Setup, Rooms</t>
+          <t>Dashboard, Admin</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
         <is>
-          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
+          <t>The server accepts an AI draft only when every number in it is in the database facts; otherwise it shows the plain figures. The key stays on the server and only the fact lines are sent.</t>
         </is>
       </c>
       <c r="E134" s="10" t="inlineStr">
@@ -11171,33 +11171,33 @@
       </c>
       <c r="H134" s="10" t="inlineStr">
         <is>
-          <t>setup.room.manage</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I134" s="10" t="inlineStr"/>
       <c r="J134" s="10" t="inlineStr">
         <is>
-          <t>a list of room types and rooms</t>
+          <t>a draft that rounds or invents a figure</t>
         </is>
       </c>
       <c r="K134" s="10" t="inlineStr">
         <is>
-          <t>the manager previews and then applies it</t>
+          <t>the brief is written</t>
         </is>
       </c>
       <c r="L134" s="10" t="inlineStr">
         <is>
-          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
+          <t>the plain database lines are shown instead, with a note</t>
         </is>
       </c>
       <c r="M134" s="10" t="inlineStr">
         <is>
-          <t>20261013150000_setup_import.sql: apply_setup_import</t>
+          <t>src/lib/ai-brief.ts, ai-brief.functions.ts, Dashboard morning brief card</t>
         </is>
       </c>
       <c r="N134" s="10" t="inlineStr">
         <is>
-          <t>38_setup_import (29)</t>
+          <t>browser unit: ai-brief-unit (8)</t>
         </is>
       </c>
       <c r="O134" s="10" t="inlineStr">
@@ -11207,19 +11207,19 @@
       </c>
       <c r="P134" s="10" t="inlineStr">
         <is>
-          <t>The AI only drafts the list. This function is the check.</t>
+          <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
         <is>
-          <t>AI-006</t>
+          <t>SET-010</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
         <is>
-          <t>AI helpers</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C135" s="10" t="inlineStr">
@@ -11229,7 +11229,7 @@
       </c>
       <c r="D135" s="10" t="inlineStr">
         <is>
-          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
+          <t>A hotel can add room types and rooms from one checked list: preview first, then all or nothing. Existing codes and room names are skipped, so repeating adds nothing.</t>
         </is>
       </c>
       <c r="E135" s="10" t="inlineStr">
@@ -11255,27 +11255,27 @@
       <c r="I135" s="10" t="inlineStr"/>
       <c r="J135" s="10" t="inlineStr">
         <is>
-          <t>AI switched on with a limit of 1</t>
+          <t>a list of room types and rooms</t>
         </is>
       </c>
       <c r="K135" s="10" t="inlineStr">
         <is>
-          <t>an import draft is started twice</t>
+          <t>the manager previews and then applies it</t>
         </is>
       </c>
       <c r="L135" s="10" t="inlineStr">
         <is>
-          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
+          <t>the preview writes nothing; apply adds every valid item or none (bad name, unknown type, over 500 rooms, over the plan limit); a repeat adds nothing; the import is audited</t>
         </is>
       </c>
       <c r="M135" s="10" t="inlineStr">
         <is>
-          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
+          <t>20261013150000_setup_import.sql: apply_setup_import</t>
         </is>
       </c>
       <c r="N135" s="10" t="inlineStr">
         <is>
-          <t>38_setup_import (8)</t>
+          <t>38_setup_import (29)</t>
         </is>
       </c>
       <c r="O135" s="10" t="inlineStr">
@@ -11283,12 +11283,16 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P135" s="10" t="inlineStr"/>
+      <c r="P135" s="10" t="inlineStr">
+        <is>
+          <t>The AI only drafts the list. This function is the check.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
         <is>
-          <t>AI-007</t>
+          <t>AI-006</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
@@ -11303,7 +11307,7 @@
       </c>
       <c r="D136" s="10" t="inlineStr">
         <is>
-          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
+          <t>The setup import assistant starts only when AI is on and under the monthly limit, and the AI sees only existing room type codes and a room count.</t>
         </is>
       </c>
       <c r="E136" s="10" t="inlineStr">
@@ -11329,27 +11333,27 @@
       <c r="I136" s="10" t="inlineStr"/>
       <c r="J136" s="10" t="inlineStr">
         <is>
-          <t>a pasted list</t>
+          <t>AI switched on with a limit of 1</t>
         </is>
       </c>
       <c r="K136" s="10" t="inlineStr">
         <is>
-          <t>the assistant drafts it</t>
+          <t>an import draft is started twice</t>
         </is>
       </c>
       <c r="L136" s="10" t="inlineStr">
         <is>
-          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
+          <t>the second is refused until the first fails; front desk and other hotels are refused</t>
         </is>
       </c>
       <c r="M136" s="10" t="inlineStr">
         <is>
-          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
+          <t>20261013150000_setup_import.sql: ai_import_start, app.ai_begin</t>
         </is>
       </c>
       <c r="N136" s="10" t="inlineStr">
         <is>
-          <t>browser unit: setup-import-unit (9)</t>
+          <t>38_setup_import (8)</t>
         </is>
       </c>
       <c r="O136" s="10" t="inlineStr">
@@ -11357,36 +11361,32 @@
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P136" s="10" t="inlineStr">
-        <is>
-          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
-        </is>
-      </c>
+      <c r="P136" s="10" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
         <is>
-          <t>SET-011</t>
+          <t>AI-007</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>AI helpers</t>
         </is>
       </c>
       <c r="C137" s="10" t="inlineStr">
         <is>
-          <t>/setup; /dashboard</t>
+          <t>Setup, Rooms</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
         <is>
-          <t>A new hotel sees a checklist of what is left to set up: property details, room types, rooms, rates, taxes, payment methods and staff. Each step says what is missing and links to the right screen. The list comes from the hotel's own data, so it is always current.</t>
+          <t>Pasted text with an email, phone or card number is refused before anything is sent; the draft may only contain rooms, floors, guest limits and type names that are in the pasted text.</t>
         </is>
       </c>
       <c r="E137" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F137" s="10" t="inlineStr">
@@ -11401,37 +11401,33 @@
       </c>
       <c r="H137" s="10" t="inlineStr">
         <is>
-          <t>any setup permission</t>
-        </is>
-      </c>
-      <c r="I137" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>setup.room.manage</t>
+        </is>
+      </c>
+      <c r="I137" s="10" t="inlineStr"/>
       <c r="J137" s="10" t="inlineStr">
         <is>
-          <t>a hotel that is part way through setup</t>
+          <t>a pasted list</t>
         </is>
       </c>
       <c r="K137" s="10" t="inlineStr">
         <is>
-          <t>a manager opens Setup or the Dashboard</t>
+          <t>the assistant drafts it</t>
         </is>
       </c>
       <c r="L137" s="10" t="inlineStr">
         <is>
-          <t>the steps already done are ticked and the next one is linked; once all seven are done the checklist goes away</t>
+          <t>invented rooms, floors and limits are dropped with a note; a draft with no matching rooms is an error</t>
         </is>
       </c>
       <c r="M137" s="10" t="inlineStr">
         <is>
-          <t>setup_progress</t>
+          <t>src/lib/setup-import.ts, setup-import.functions.ts, Import from a list on Setup, Rooms</t>
         </is>
       </c>
       <c r="N137" s="10" t="inlineStr">
         <is>
-          <t>40_guided_setup (30)</t>
+          <t>browser unit: setup-import-unit (9)</t>
         </is>
       </c>
       <c r="O137" s="10" t="inlineStr">
@@ -11441,39 +11437,39 @@
       </c>
       <c r="P137" s="10" t="inlineStr">
         <is>
-          <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
+          <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="10" t="inlineStr">
         <is>
-          <t>NFR-006</t>
+          <t>SET-011</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
         <is>
-          <t>Non-functional</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C138" s="10" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/setup; /dashboard</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr">
         <is>
-          <t>The last room of a type is sold once, however many desks book at the same moment, and a repeated booking never doubles.</t>
+          <t>A new hotel sees a checklist of what is left to set up: property details, room types, rooms, rates, taxes, payment methods and staff. Each step says what is missing and links to the right screen. The list comes from the hotel's own data, so it is always current.</t>
         </is>
       </c>
       <c r="E138" s="10" t="inlineStr">
         <is>
-          <t>BR-001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F138" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G138" s="10" t="inlineStr">
@@ -11483,37 +11479,37 @@
       </c>
       <c r="H138" s="10" t="inlineStr">
         <is>
+          <t>any setup permission</t>
+        </is>
+      </c>
+      <c r="I138" s="10" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I138" s="10" t="inlineStr">
-        <is>
-          <t>Rule: Safe last-room booking</t>
-        </is>
-      </c>
       <c r="J138" s="10" t="inlineStr">
         <is>
-          <t>one room of a type is left and several desks book it together</t>
+          <t>a hotel that is part way through setup</t>
         </is>
       </c>
       <c r="K138" s="10" t="inlineStr">
         <is>
-          <t>all of them submit at the same moment</t>
+          <t>a manager opens Setup or the Dashboard</t>
         </is>
       </c>
       <c r="L138" s="10" t="inlineStr">
         <is>
-          <t>exactly one booking succeeds, the rest get E_NO_AVAILABILITY, and nothing is oversold</t>
+          <t>the steps already done are ticked and the next one is linked; once all seven are done the checklist goes away</t>
         </is>
       </c>
       <c r="M138" s="10" t="inlineStr">
         <is>
-          <t>create_reservation, assert_available</t>
+          <t>setup_progress</t>
         </is>
       </c>
       <c r="N138" s="10" t="inlineStr">
         <is>
-          <t>concurrency/last_room.sh (6)</t>
+          <t>40_guided_setup (30)</t>
         </is>
       </c>
       <c r="O138" s="10" t="inlineStr">
@@ -11523,29 +11519,29 @@
       </c>
       <c r="P138" s="10" t="inlineStr">
         <is>
-          <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
+          <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="10" t="inlineStr">
         <is>
-          <t>SET-012</t>
+          <t>NFR-006</t>
         </is>
       </c>
       <c r="B139" s="10" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Non-functional</t>
         </is>
       </c>
       <c r="C139" s="10" t="inlineStr">
         <is>
-          <t>/setup/property</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr">
         <is>
-          <t>A manager sets the longest stay (1 to 365 nights) and how long a tentative booking holds its room (1 to 720 hours) for each property.</t>
+          <t>The last room of a type is sold once, however many desks book at the same moment, and a repeated booking never doubles.</t>
         </is>
       </c>
       <c r="E139" s="10" t="inlineStr">
@@ -11555,7 +11551,7 @@
       </c>
       <c r="F139" s="10" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G139" s="10" t="inlineStr">
@@ -11565,33 +11561,37 @@
       </c>
       <c r="H139" s="10" t="inlineStr">
         <is>
-          <t>setup.property.edit</t>
-        </is>
-      </c>
-      <c r="I139" s="10" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I139" s="10" t="inlineStr">
+        <is>
+          <t>Rule: Safe last-room booking</t>
+        </is>
+      </c>
       <c r="J139" s="10" t="inlineStr">
         <is>
-          <t>a property with the default rules (30 nights, 24 hours)</t>
+          <t>one room of a type is left and several desks book it together</t>
         </is>
       </c>
       <c r="K139" s="10" t="inlineStr">
         <is>
-          <t>a manager saves new booking rules</t>
+          <t>all of them submit at the same moment</t>
         </is>
       </c>
       <c r="L139" s="10" t="inlineStr">
         <is>
-          <t>new bookings use them, bad values are refused with E_INVALID, and the change is audited with old and new values</t>
+          <t>exactly one booking succeeds, the rest get E_NO_AVAILABILITY, and nothing is oversold</t>
         </is>
       </c>
       <c r="M139" s="10" t="inlineStr">
         <is>
-          <t>set_booking_rules; Booking rules on Setup, Property</t>
+          <t>create_reservation, assert_available</t>
         </is>
       </c>
       <c r="N139" s="10" t="inlineStr">
         <is>
-          <t>42_booking_rules (9)</t>
+          <t>concurrency/last_room.sh (6)</t>
         </is>
       </c>
       <c r="O139" s="10" t="inlineStr">
@@ -11601,39 +11601,39 @@
       </c>
       <c r="P139" s="10" t="inlineStr">
         <is>
-          <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
+          <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="10" t="inlineStr">
         <is>
-          <t>FO-014</t>
+          <t>SET-012</t>
         </is>
       </c>
       <c r="B140" s="10" t="inlineStr">
         <is>
-          <t>Front Office</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C140" s="10" t="inlineStr">
         <is>
-          <t>/downtime</t>
+          <t>/setup/property</t>
         </is>
       </c>
       <c r="D140" s="10" t="inlineStr">
         <is>
-          <t>A printable downtime pack: arrivals due, in-house guests with balance, departures due, ten blank lines for new guests on paper, and a short paper routine. Staff print it when the internet or system is down.</t>
+          <t>A manager sets the longest stay (1 to 365 nights) and how long a tentative booking holds its room (1 to 720 hours) for each property.</t>
         </is>
       </c>
       <c r="E140" s="10" t="inlineStr">
         <is>
-          <t>BR-006</t>
+          <t>BR-001</t>
         </is>
       </c>
       <c r="F140" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G140" s="10" t="inlineStr">
@@ -11643,33 +11643,33 @@
       </c>
       <c r="H140" s="10" t="inlineStr">
         <is>
-          <t>fo.view</t>
+          <t>setup.property.edit</t>
         </is>
       </c>
       <c r="I140" s="10" t="inlineStr"/>
       <c r="J140" s="10" t="inlineStr">
         <is>
-          <t>a hotel with guests in house</t>
+          <t>a property with the default rules (30 nights, 24 hours)</t>
         </is>
       </c>
       <c r="K140" s="10" t="inlineStr">
         <is>
-          <t>a front desk user opens Downtime pack and prints</t>
+          <t>a manager saves new booking rules</t>
         </is>
       </c>
       <c r="L140" s="10" t="inlineStr">
         <is>
-          <t>the lists show room, guest, phone, departure and the folio balance from the database, with blank lines and the paper routine</t>
+          <t>new bookings use them, bad values are refused with E_INVALID, and the change is audited with old and new values</t>
         </is>
       </c>
       <c r="M140" s="10" t="inlineStr">
         <is>
-          <t>src/routes/_authenticated/_app/downtime.tsx</t>
+          <t>set_booking_rules; Booking rules on Setup, Property</t>
         </is>
       </c>
       <c r="N140" s="10" t="inlineStr">
         <is>
-          <t>browser: downtime-pack.spec (1)</t>
+          <t>42_booking_rules (9)</t>
         </is>
       </c>
       <c r="O140" s="10" t="inlineStr">
@@ -11679,87 +11679,165 @@
       </c>
       <c r="P140" s="10" t="inlineStr">
         <is>
-          <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
+          <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="10" t="inlineStr">
         <is>
+          <t>FO-014</t>
+        </is>
+      </c>
+      <c r="B141" s="10" t="inlineStr">
+        <is>
+          <t>Front Office</t>
+        </is>
+      </c>
+      <c r="C141" s="10" t="inlineStr">
+        <is>
+          <t>/downtime</t>
+        </is>
+      </c>
+      <c r="D141" s="10" t="inlineStr">
+        <is>
+          <t>A printable downtime pack: arrivals due, in-house guests with balance, departures due, ten blank lines for new guests on paper, and a short paper routine. Staff print it when the internet or system is down.</t>
+        </is>
+      </c>
+      <c r="E141" s="10" t="inlineStr">
+        <is>
+          <t>BR-006</t>
+        </is>
+      </c>
+      <c r="F141" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G141" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H141" s="10" t="inlineStr">
+        <is>
+          <t>fo.view</t>
+        </is>
+      </c>
+      <c r="I141" s="10" t="inlineStr"/>
+      <c r="J141" s="10" t="inlineStr">
+        <is>
+          <t>a hotel with guests in house</t>
+        </is>
+      </c>
+      <c r="K141" s="10" t="inlineStr">
+        <is>
+          <t>a front desk user opens Downtime pack and prints</t>
+        </is>
+      </c>
+      <c r="L141" s="10" t="inlineStr">
+        <is>
+          <t>the lists show room, guest, phone, departure and the folio balance from the database, with blank lines and the paper routine</t>
+        </is>
+      </c>
+      <c r="M141" s="10" t="inlineStr">
+        <is>
+          <t>src/routes/_authenticated/_app/downtime.tsx</t>
+        </is>
+      </c>
+      <c r="N141" s="10" t="inlineStr">
+        <is>
+          <t>browser: downtime-pack.spec (1)</t>
+        </is>
+      </c>
+      <c r="O141" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P141" s="10" t="inlineStr">
+        <is>
+          <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="10" t="inlineStr">
+        <is>
           <t>DAY-007</t>
         </is>
       </c>
-      <c r="B141" s="10" t="inlineStr">
+      <c r="B142" s="10" t="inlineStr">
         <is>
           <t>Business Date</t>
         </is>
       </c>
-      <c r="C141" s="10" t="inlineStr">
+      <c r="C142" s="10" t="inlineStr">
         <is>
           <t>Notifications bell</t>
         </is>
       </c>
-      <c r="D141" s="10" t="inlineStr">
+      <c r="D142" s="10" t="inlineStr">
         <is>
           <t>In the last hour before a property rolls its business date, if a cashier shift is still open, users who can run the night audit get one warning that night. The roll does not wait.</t>
         </is>
       </c>
-      <c r="E141" s="10" t="inlineStr">
+      <c r="E142" s="10" t="inlineStr">
         <is>
           <t>BR-016</t>
         </is>
       </c>
-      <c r="F141" s="10" t="inlineStr">
+      <c r="F142" s="10" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="G141" s="10" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H141" s="10" t="inlineStr">
+      <c r="G142" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H142" s="10" t="inlineStr">
         <is>
           <t>fin.nightaudit.run</t>
         </is>
       </c>
-      <c r="I141" s="10" t="inlineStr">
+      <c r="I142" s="10" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="J141" s="10" t="inlineStr">
+      <c r="J142" s="10" t="inlineStr">
         <is>
           <t>a cashier shift is still open</t>
         </is>
       </c>
-      <c r="K141" s="10" t="inlineStr">
+      <c r="K142" s="10" t="inlineStr">
         <is>
           <t>the roll time is less than 60 minutes away</t>
         </is>
       </c>
-      <c r="L141" s="10" t="inlineStr">
+      <c r="L142" s="10" t="inlineStr">
         <is>
           <t>each night audit user gets one rollover_warning notification for that business date; none earlier, none after the roll time, none if no shift is open, none twice</t>
         </is>
       </c>
-      <c r="M141" s="10" t="inlineStr">
+      <c r="M142" s="10" t="inlineStr">
         <is>
           <t>app.warn_before_rollover; cron job rollover-warning</t>
         </is>
       </c>
-      <c r="N141" s="10" t="inlineStr">
+      <c r="N142" s="10" t="inlineStr">
         <is>
           <t>43_rollover_warning (9)</t>
         </is>
       </c>
-      <c r="O141" s="10" t="inlineStr">
+      <c r="O142" s="10" t="inlineStr">
         <is>
           <t>Built+tested</t>
         </is>
       </c>
-      <c r="P141" s="10" t="inlineStr">
+      <c r="P142" s="10" t="inlineStr">
         <is>
           <t>Added 8 Oct 2026. Warning only; the hard gate stays in R2 (DAY-005).</t>
         </is>

</xml_diff>

<commit_message>
Ticket photos: a missing assignee must read as no access
An unassigned ticket has a NULL assignee. The permission check returned NULL, which the
function treated as allowed. Every term now defaults to false. Found by running the test
on a scratch database.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -6497,7 +6497,7 @@
       </c>
       <c r="N74" s="10" t="inlineStr">
         <is>
-          <t>48_minibar (16)</t>
+          <t>48_minibar (18)</t>
         </is>
       </c>
       <c r="O74" s="10" t="inlineStr">
@@ -6809,7 +6809,7 @@
       </c>
       <c r="N78" s="10" t="inlineStr">
         <is>
-          <t>49_ticket_photos (17)</t>
+          <t>49_ticket_photos (20)</t>
         </is>
       </c>
       <c r="O78" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Docs: refresh requirements workbook and correct known-issues
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P142"/>
+  <dimension ref="A1:P144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11840,6 +11840,162 @@
       <c r="P142" s="10" t="inlineStr">
         <is>
           <t>Added 8 Oct 2026. Warning only; the hard gate stays in R2 (DAY-005).</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="10" t="inlineStr">
+        <is>
+          <t>RPT-008</t>
+        </is>
+      </c>
+      <c r="B143" s="10" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C143" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D143" s="10" t="inlineStr">
+        <is>
+          <t>A Latest activity feed on the dashboard: new bookings, check-ins, check-outs, payments and rooms marked clean, newest first. Each person sees only the kinds their rights allow.</t>
+        </is>
+      </c>
+      <c r="E143" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F143" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G143" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H143" s="10" t="inlineStr">
+        <is>
+          <t>res.view; fo.view; fin.folio.view; hk.view</t>
+        </is>
+      </c>
+      <c r="I143" s="10" t="inlineStr"/>
+      <c r="J143" s="10" t="inlineStr">
+        <is>
+          <t>a property with recent activity</t>
+        </is>
+      </c>
+      <c r="K143" s="10" t="inlineStr">
+        <is>
+          <t>a signed-in user opens the dashboard</t>
+        </is>
+      </c>
+      <c r="L143" s="10" t="inlineStr">
+        <is>
+          <t>the feed lists up to 8 recent items; payments show only with folio rights; bookings only with reservation rights; no rights is refused with E_FORBIDDEN; a room move adds no second check-in</t>
+        </is>
+      </c>
+      <c r="M143" s="10" t="inlineStr">
+        <is>
+          <t>recent_activity; Latest activity card on the dashboard</t>
+        </is>
+      </c>
+      <c r="N143" s="10" t="inlineStr">
+        <is>
+          <t>50_recent_activity (17)</t>
+        </is>
+      </c>
+      <c r="O143" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P143" s="10" t="inlineStr">
+        <is>
+          <t>Added 9 Oct 2026. Read-only; no money is changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="10" t="inlineStr">
+        <is>
+          <t>RPT-009</t>
+        </is>
+      </c>
+      <c r="B144" s="10" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C144" s="10" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="D144" s="10" t="inlineStr">
+        <is>
+          <t>One rule for money collected. A payment, a refund, and a reversal or transfer that carries a payment method count; the Payments report, the owner summary and the invoice all use it, so a payment reversed the same day shows as zero everywhere.</t>
+        </is>
+      </c>
+      <c r="E144" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F144" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G144" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H144" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view</t>
+        </is>
+      </c>
+      <c r="I144" s="10" t="inlineStr"/>
+      <c r="J144" s="10" t="inlineStr">
+        <is>
+          <t>a payment taken and reversed the same day</t>
+        </is>
+      </c>
+      <c r="K144" s="10" t="inlineStr">
+        <is>
+          <t>a finance user opens the Payments report</t>
+        </is>
+      </c>
+      <c r="L144" s="10" t="inlineStr">
+        <is>
+          <t>the method nets to zero and matches the ledger; front desk without finance reports is refused with E_FORBIDDEN</t>
+        </is>
+      </c>
+      <c r="M144" s="10" t="inlineStr">
+        <is>
+          <t>report_payments; app.is_money_movement</t>
+        </is>
+      </c>
+      <c r="N144" s="10" t="inlineStr">
+        <is>
+          <t>51_money_collected (5)</t>
+        </is>
+      </c>
+      <c r="O144" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P144" s="10" t="inlineStr">
+        <is>
+          <t>Added 10 Oct 2026. The Payments report counted only payments and refunds before this. Cashier shift counts stay separate on purpose: they count what the drawer should hold.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day-in-the-life test and dry-run sheet corrections (DRY-001)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P144"/>
+  <dimension ref="A1:P146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11907,7 +11907,7 @@
       </c>
       <c r="N143" s="10" t="inlineStr">
         <is>
-          <t>50_recent_activity (17)</t>
+          <t>50_recent_activity (17); 52_guest_label_private (3)</t>
         </is>
       </c>
       <c r="O143" s="10" t="inlineStr">
@@ -11996,6 +11996,158 @@
       <c r="P144" s="10" t="inlineStr">
         <is>
           <t>Added 10 Oct 2026. The Payments report counted only payments and refunds before this. Cashier shift counts stay separate on purpose: they count what the drawer should hold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="10" t="inlineStr">
+        <is>
+          <t>FIN-021</t>
+        </is>
+      </c>
+      <c r="B145" s="10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C145" s="10" t="inlineStr">
+        <is>
+          <t>Reports &gt; Collections</t>
+        </is>
+      </c>
+      <c r="D145" s="10" t="inlineStr">
+        <is>
+          <t>Collections list. Departed guests (checked out, no-show, cancelled) who still owe the hotel, with a follow-up log: called, promised, unreachable, disputed or note. Next follow-up is the day after a promised date, or 7 days after the last note.</t>
+        </is>
+      </c>
+      <c r="E145" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F145" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G145" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H145" s="10" t="inlineStr">
+        <is>
+          <t>rpt.finance.view; fin.payment.post</t>
+        </is>
+      </c>
+      <c r="I145" s="10" t="inlineStr"/>
+      <c r="J145" s="10" t="inlineStr">
+        <is>
+          <t>a guest left owing money</t>
+        </is>
+      </c>
+      <c r="K145" s="10" t="inlineStr">
+        <is>
+          <t>finance staff opens Reports &gt; Collections and logs a follow-up</t>
+        </is>
+      </c>
+      <c r="L145" s="10" t="inlineStr">
+        <is>
+          <t>the guest shows with balance and days since departure; a note with a promise needs a future date; guests who owe nothing or have not left are refused; front desk without finance reports is refused</t>
+        </is>
+      </c>
+      <c r="M145" s="10" t="inlineStr">
+        <is>
+          <t>collections_list; add_collection_note; collection_notes</t>
+        </is>
+      </c>
+      <c r="N145" s="10" t="inlineStr">
+        <is>
+          <t>53_collections (20)</t>
+        </is>
+      </c>
+      <c r="O145" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P145" s="10" t="inlineStr">
+        <is>
+          <t>Added 10 Oct 2026. Notes are not ledger rows; they never change a balance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="10" t="inlineStr">
+        <is>
+          <t>DRY-001</t>
+        </is>
+      </c>
+      <c r="B146" s="10" t="inlineStr">
+        <is>
+          <t>Release readiness</t>
+        </is>
+      </c>
+      <c r="C146" s="10" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D146" s="10" t="inlineStr">
+        <is>
+          <t>One full hotel day runs from booking to night roll with the real roles: bookings, deposit, check-in, walk-in, room move, charges, discount approval, service request, extension, maintenance, the night roll, check-out, housekeeping, collections and reports.</t>
+        </is>
+      </c>
+      <c r="E146" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F146" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G146" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H146" s="10" t="inlineStr"/>
+      <c r="I146" s="10" t="inlineStr"/>
+      <c r="J146" s="10" t="inlineStr">
+        <is>
+          <t>a hotel with five kinds of staff</t>
+        </is>
+      </c>
+      <c r="K146" s="10" t="inlineStr">
+        <is>
+          <t>the day is run step by step</t>
+        </is>
+      </c>
+      <c r="L146" s="10" t="inlineStr">
+        <is>
+          <t>each step gives the expected result and each refusal fires for the wrong person; the Payments report matches the ledger</t>
+        </is>
+      </c>
+      <c r="M146" s="10" t="inlineStr">
+        <is>
+          <t>day in the life of a hotel</t>
+        </is>
+      </c>
+      <c r="N146" s="10" t="inlineStr">
+        <is>
+          <t>54_day_in_the_life (49)</t>
+        </is>
+      </c>
+      <c r="O146" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P146" s="10" t="inlineStr">
+        <is>
+          <t>Added 10 Oct 2026. Mirrors docs/pilot-dry-run.md; screens and wording still need people.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix search path on 14 helper functions (QA-07)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P146"/>
+  <dimension ref="A1:P147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12148,6 +12148,88 @@
       <c r="P146" s="10" t="inlineStr">
         <is>
           <t>Added 10 Oct 2026. Mirrors docs/pilot-dry-run.md; screens and wording still need people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="10" t="inlineStr">
+        <is>
+          <t>NFR-007</t>
+        </is>
+      </c>
+      <c r="B147" s="10" t="inlineStr">
+        <is>
+          <t>Non-functional</t>
+        </is>
+      </c>
+      <c r="C147" s="10" t="inlineStr">
+        <is>
+          <t>(all)</t>
+        </is>
+      </c>
+      <c r="D147" s="10" t="inlineStr">
+        <is>
+          <t>Every function we own, helpers included, has a fixed search path so a rogue schema can never change what it does.</t>
+        </is>
+      </c>
+      <c r="E147" s="10" t="inlineStr">
+        <is>
+          <t>BR-017</t>
+        </is>
+      </c>
+      <c r="F147" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G147" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H147" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I147" s="10" t="inlineStr">
+        <is>
+          <t>Rule 4</t>
+        </is>
+      </c>
+      <c r="J147" s="10" t="inlineStr">
+        <is>
+          <t>a migration adds or changes a function</t>
+        </is>
+      </c>
+      <c r="K147" s="10" t="inlineStr">
+        <is>
+          <t>the test suite runs</t>
+        </is>
+      </c>
+      <c r="L147" s="10" t="inlineStr">
+        <is>
+          <t>it fails if any function in app or public has no fixed search path</t>
+        </is>
+      </c>
+      <c r="M147" s="10" t="inlineStr">
+        <is>
+          <t>20261018100000_helper_search_path.sql</t>
+        </is>
+      </c>
+      <c r="N147" s="10" t="inlineStr">
+        <is>
+          <t>50_helper_search_path (1)</t>
+        </is>
+      </c>
+      <c r="O147" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P147" s="10" t="inlineStr">
+        <is>
+          <t>QA-07. Fixes 14 helpers the security advisor listed. Added 10 Oct 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Email hotels before the trial ends and when payment is overdue (QA-05)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P147"/>
+  <dimension ref="A1:P149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12230,6 +12230,170 @@
       <c r="P147" s="10" t="inlineStr">
         <is>
           <t>QA-07. Fixes 14 helpers the security advisor listed. Added 10 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="10" t="inlineStr">
+        <is>
+          <t>PLT-014</t>
+        </is>
+      </c>
+      <c r="B148" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C148" s="10" t="inlineStr">
+        <is>
+          <t>(email)</t>
+        </is>
+      </c>
+      <c r="D148" s="10" t="inlineStr">
+        <is>
+          <t>A hotel is emailed before its free trial ends: 7 days before, 1 day before, and when it ends. The email says what happens, that nothing is deleted, and to contact hello@zikorahq.com. Only the hotel's active System Administrators and General Managers get it, and a hotel that has already chosen a plan gets nothing.</t>
+        </is>
+      </c>
+      <c r="E148" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F148" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G148" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H148" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I148" s="10" t="inlineStr">
+        <is>
+          <t>A13, Decision of 10 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J148" s="10" t="inlineStr">
+        <is>
+          <t>a hotel on a free trial</t>
+        </is>
+      </c>
+      <c r="K148" s="10" t="inlineStr">
+        <is>
+          <t>the daily subscription clock runs</t>
+        </is>
+      </c>
+      <c r="L148" s="10" t="inlineStr">
+        <is>
+          <t>each administrator gets each notice once, however many times the clock runs</t>
+        </is>
+      </c>
+      <c r="M148" s="10" t="inlineStr">
+        <is>
+          <t>app.run_subscription_clock, app.send_subscription_notice</t>
+        </is>
+      </c>
+      <c r="N148" s="10" t="inlineStr">
+        <is>
+          <t>51_subscription_notices (12)</t>
+        </is>
+      </c>
+      <c r="O148" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P148" s="10" t="inlineStr">
+        <is>
+          <t>QA-05. No prices in the email, because billing checkout is not switched on. Product name 'Zikora' in the wording is a draft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="10" t="inlineStr">
+        <is>
+          <t>PLT-015</t>
+        </is>
+      </c>
+      <c r="B149" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C149" s="10" t="inlineStr">
+        <is>
+          <t>(email)</t>
+        </is>
+      </c>
+      <c r="D149" s="10" t="inlineStr">
+        <is>
+          <t>A hotel is emailed when payment is overdue, with 3 days of the 14-day grace left, and when it is suspended. The email says to pay by the date to keep full access, that the hotel then becomes read-only, and to contact hello@zikorahq.com. A hotel that has paid gets nothing.</t>
+        </is>
+      </c>
+      <c r="E149" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F149" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G149" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H149" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I149" s="10" t="inlineStr">
+        <is>
+          <t>D7, Decision of 10 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J149" s="10" t="inlineStr">
+        <is>
+          <t>a hotel whose paid period has ended without payment</t>
+        </is>
+      </c>
+      <c r="K149" s="10" t="inlineStr">
+        <is>
+          <t>the daily subscription clock runs</t>
+        </is>
+      </c>
+      <c r="L149" s="10" t="inlineStr">
+        <is>
+          <t>each administrator gets each notice once, and the clock still marks past due and suspends as before</t>
+        </is>
+      </c>
+      <c r="M149" s="10" t="inlineStr">
+        <is>
+          <t>app.run_subscription_clock, app.send_subscription_notice</t>
+        </is>
+      </c>
+      <c r="N149" s="10" t="inlineStr">
+        <is>
+          <t>51_subscription_notices (10)</t>
+        </is>
+      </c>
+      <c r="O149" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P149" s="10" t="inlineStr">
+        <is>
+          <t>QA-05.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DAY-008: roll records open cashier shifts and notifies night audit users
The date still rolls on its own (DAY-005). The roll result and log now carry open_shifts, and night audit users get one notice.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P146"/>
+  <dimension ref="A1:P147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12148,6 +12148,88 @@
       <c r="P146" s="10" t="inlineStr">
         <is>
           <t>Added 10 Oct 2026. Mirrors docs/pilot-dry-run.md; screens and wording still need people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="10" t="inlineStr">
+        <is>
+          <t>DAY-008</t>
+        </is>
+      </c>
+      <c r="B147" s="10" t="inlineStr">
+        <is>
+          <t>Business Date</t>
+        </is>
+      </c>
+      <c r="C147" s="10" t="inlineStr">
+        <is>
+          <t>Notifications bell</t>
+        </is>
+      </c>
+      <c r="D147" s="10" t="inlineStr">
+        <is>
+          <t>When the business date rolls while a cashier shift is still open, the roll goes ahead, records how many shifts were open, and tells users who can run the night audit once.</t>
+        </is>
+      </c>
+      <c r="E147" s="10" t="inlineStr">
+        <is>
+          <t>BR-016</t>
+        </is>
+      </c>
+      <c r="F147" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G147" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H147" s="10" t="inlineStr">
+        <is>
+          <t>fin.nightaudit.run</t>
+        </is>
+      </c>
+      <c r="I147" s="10" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="J147" s="10" t="inlineStr">
+        <is>
+          <t>a cashier shift is still open at roll time</t>
+        </is>
+      </c>
+      <c r="K147" s="10" t="inlineStr">
+        <is>
+          <t>the date rolls</t>
+        </is>
+      </c>
+      <c r="L147" s="10" t="inlineStr">
+        <is>
+          <t>the roll succeeds; the roll log and result carry open_shifts; each night audit user gets one rollover_open_shifts notice; none if no shift was open</t>
+        </is>
+      </c>
+      <c r="M147" s="10" t="inlineStr">
+        <is>
+          <t>app.roll_property</t>
+        </is>
+      </c>
+      <c r="N147" s="10" t="inlineStr">
+        <is>
+          <t>55_roll_open_shifts (8)</t>
+        </is>
+      </c>
+      <c r="O147" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P147" s="10" t="inlineStr">
+        <is>
+          <t>Added 10 Oct 2026. Decision B: flag, do not stop (DAY-005 gate stays in R2).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RES-014: early departure brings the booking total down to the nights kept
Check-out sets the total to the kept nights (plus the same-day night when charged). Undo check-out restores the old total from the snapshot. Closes QA-12.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P150"/>
+  <dimension ref="A1:P151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12476,6 +12476,88 @@
       <c r="P150" s="10" t="inlineStr">
         <is>
           <t>QA-05.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="10" t="inlineStr">
+        <is>
+          <t>RES-014</t>
+        </is>
+      </c>
+      <c r="B151" s="10" t="inlineStr">
+        <is>
+          <t>Reservations</t>
+        </is>
+      </c>
+      <c r="C151" s="10" t="inlineStr">
+        <is>
+          <t>Front Desk (check-out)</t>
+        </is>
+      </c>
+      <c r="D151" s="10" t="inlineStr">
+        <is>
+          <t>When a guest checks out before the booked departure, the booking total drops to the nights kept (plus the one same-day night when it applies). Undo check-out on the same day restores the old total.</t>
+        </is>
+      </c>
+      <c r="E151" s="10" t="inlineStr">
+        <is>
+          <t>BR-006</t>
+        </is>
+      </c>
+      <c r="F151" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G151" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H151" s="10" t="inlineStr">
+        <is>
+          <t>fo.checkout</t>
+        </is>
+      </c>
+      <c r="I151" s="10" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="J151" s="10" t="inlineStr">
+        <is>
+          <t>a guest leaves before the booked departure</t>
+        </is>
+      </c>
+      <c r="K151" s="10" t="inlineStr">
+        <is>
+          <t>the check-out is made</t>
+        </is>
+      </c>
+      <c r="L151" s="10" t="inlineStr">
+        <is>
+          <t>total_amount equals the kept nights; undo check-out restores it</t>
+        </is>
+      </c>
+      <c r="M151" s="10" t="inlineStr">
+        <is>
+          <t>public.check_out; public.undo_checkout</t>
+        </is>
+      </c>
+      <c r="N151" s="10" t="inlineStr">
+        <is>
+          <t>56_early_departure_total (4)</t>
+        </is>
+      </c>
+      <c r="O151" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P151" s="10" t="inlineStr">
+        <is>
+          <t>Added 10 Oct 2026 (QA-12).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: fix register notes (SET-002, RES-012, RES-013), screens list, known issues and status report banner
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P151"/>
+  <dimension ref="A1:Q151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -760,6 +760,7 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -838,6 +839,7 @@
         </is>
       </c>
       <c r="P2" s="10" t="inlineStr"/>
+      <c r="Q2" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -916,6 +918,7 @@
         </is>
       </c>
       <c r="P3" s="10" t="inlineStr"/>
+      <c r="Q3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -994,6 +997,7 @@
         </is>
       </c>
       <c r="P4" s="10" t="inlineStr"/>
+      <c r="Q4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1072,6 +1076,7 @@
         </is>
       </c>
       <c r="P5" s="10" t="inlineStr"/>
+      <c r="Q5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -1150,6 +1155,7 @@
         </is>
       </c>
       <c r="P6" s="10" t="inlineStr"/>
+      <c r="Q6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -1228,6 +1234,7 @@
         </is>
       </c>
       <c r="P7" s="10" t="inlineStr"/>
+      <c r="Q7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1310,6 +1317,7 @@
           <t>Adding a property: System Administrator and General Manager (ADM-002), within plans.max_properties.</t>
         </is>
       </c>
+      <c r="Q8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -1392,6 +1400,7 @@
           <t>Platform console /platform (wave 2 item 2): extend trial, activate or extend paid period, suspend, change plan, cancel; each with a reason, logged in subscription_history with the operator.</t>
         </is>
       </c>
+      <c r="Q9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -1474,6 +1483,7 @@
           <t>Corrected 6 Oct 2026: before wave 2 item 2 there was no platform staff role at all; the earlier "Built, no tagged test" was wrong.</t>
         </is>
       </c>
+      <c r="Q10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -1556,6 +1566,7 @@
           <t>Database done 8 Oct 2026. Screens for the hotel (Admin) and the operator (platform console) follow. New permission adm.support.manage reaches System Administrator and General Manager only.</t>
         </is>
       </c>
+      <c r="Q11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -1634,6 +1645,7 @@
         </is>
       </c>
       <c r="P12" s="10" t="inlineStr"/>
+      <c r="Q12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -1716,6 +1728,7 @@
           <t>Needs PAYSTACK_SECRET_KEY and the webhook address set in Paystack. Prices are empty until A16 is decided.</t>
         </is>
       </c>
+      <c r="Q13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -1794,6 +1807,7 @@
         </is>
       </c>
       <c r="P14" s="10" t="inlineStr"/>
+      <c r="Q14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -1876,6 +1890,7 @@
           <t>Invites are sent by a Vercel server function (not an Edge Function).</t>
         </is>
       </c>
+      <c r="Q15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -1954,6 +1969,7 @@
         </is>
       </c>
       <c r="P16" s="10" t="inlineStr"/>
+      <c r="Q16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -2032,6 +2048,7 @@
         </is>
       </c>
       <c r="P17" s="10" t="inlineStr"/>
+      <c r="Q17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -2110,6 +2127,7 @@
         </is>
       </c>
       <c r="P18" s="10" t="inlineStr"/>
+      <c r="Q18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -2188,6 +2206,7 @@
         </is>
       </c>
       <c r="P19" s="10" t="inlineStr"/>
+      <c r="Q19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -2266,6 +2285,7 @@
         </is>
       </c>
       <c r="P20" s="10" t="inlineStr"/>
+      <c r="Q20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
@@ -2344,6 +2364,7 @@
         </is>
       </c>
       <c r="P21" s="10" t="inlineStr"/>
+      <c r="Q21" s="10" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
@@ -2422,6 +2443,7 @@
         </is>
       </c>
       <c r="P22" s="10" t="inlineStr"/>
+      <c r="Q22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
@@ -2504,6 +2526,7 @@
           <t>export_data (audited), Reports &gt; Export.</t>
         </is>
       </c>
+      <c r="Q23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
@@ -2582,6 +2605,7 @@
         </is>
       </c>
       <c r="P24" s="10" t="inlineStr"/>
+      <c r="Q24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
@@ -2661,9 +2685,10 @@
       </c>
       <c r="P25" s="10" t="inlineStr">
         <is>
-          <t>Corrected 6 Oct 2026: room types and occupancy limits (save_room_type, max adults and children; Setup, Room types) exist; the overbooking allowance does not exist anywhere in the app.</t>
-        </is>
-      </c>
+          <t>Room types and occupancy limits are built (save_room_type: max adults and children; Setup, Room types). The overbooking allowance is not built: decision pending (QA-17, 11 Oct 2026). Recommended: skip it for the pilot.</t>
+        </is>
+      </c>
+      <c r="Q25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
@@ -2746,6 +2771,7 @@
           <t>A room cannot be retired while a guest is in it ([E_ROOM_OCCUPIED], checked first) or while upcoming bookings are assigned to it ([E_ROOM_BOOKED], names up to 5 booking numbers): confirmed, or tentative with an unexpired hold, from the business date forward (decisions of 6 Oct 2026). Retiring a room that is already retired is safe to repeat; renaming and floor changes still work.</t>
         </is>
       </c>
+      <c r="Q26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
@@ -2824,6 +2850,7 @@
         </is>
       </c>
       <c r="P27" s="10" t="inlineStr"/>
+      <c r="Q27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
@@ -2902,6 +2929,7 @@
         </is>
       </c>
       <c r="P28" s="10" t="inlineStr"/>
+      <c r="Q28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
@@ -2980,6 +3008,7 @@
         </is>
       </c>
       <c r="P29" s="10" t="inlineStr"/>
+      <c r="Q29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
@@ -3058,6 +3087,7 @@
         </is>
       </c>
       <c r="P30" s="10" t="inlineStr"/>
+      <c r="Q30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
@@ -3136,6 +3166,7 @@
         </is>
       </c>
       <c r="P31" s="10" t="inlineStr"/>
+      <c r="Q31" s="10" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
@@ -3214,6 +3245,7 @@
         </is>
       </c>
       <c r="P32" s="10" t="inlineStr"/>
+      <c r="Q32" s="10" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
@@ -3292,6 +3324,7 @@
         </is>
       </c>
       <c r="P33" s="10" t="inlineStr"/>
+      <c r="Q33" s="10" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
@@ -3370,6 +3403,7 @@
         </is>
       </c>
       <c r="P34" s="10" t="inlineStr"/>
+      <c r="Q34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
@@ -3448,6 +3482,7 @@
         </is>
       </c>
       <c r="P35" s="10" t="inlineStr"/>
+      <c r="Q35" s="10" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
@@ -3526,6 +3561,7 @@
         </is>
       </c>
       <c r="P36" s="10" t="inlineStr"/>
+      <c r="Q36" s="10" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
@@ -3604,6 +3640,7 @@
         </is>
       </c>
       <c r="P37" s="10" t="inlineStr"/>
+      <c r="Q37" s="10" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
@@ -3682,6 +3719,7 @@
         </is>
       </c>
       <c r="P38" s="10" t="inlineStr"/>
+      <c r="Q38" s="10" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
@@ -3760,6 +3798,7 @@
         </is>
       </c>
       <c r="P39" s="10" t="inlineStr"/>
+      <c r="Q39" s="10" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
@@ -3838,6 +3877,7 @@
         </is>
       </c>
       <c r="P40" s="10" t="inlineStr"/>
+      <c r="Q40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
@@ -3916,6 +3956,7 @@
         </is>
       </c>
       <c r="P41" s="10" t="inlineStr"/>
+      <c r="Q41" s="10" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
@@ -3994,6 +4035,7 @@
         </is>
       </c>
       <c r="P42" s="10" t="inlineStr"/>
+      <c r="Q42" s="10" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
@@ -4073,7 +4115,12 @@
       </c>
       <c r="P43" s="10" t="inlineStr">
         <is>
-          <t>save_group_booking exists and the booking form picks a group; there is no screen to create a group.</t>
+          <t>save_group_booking exists. The booking form creates a group (Add group) and picks one; Reservations</t>
+        </is>
+      </c>
+      <c r="Q43" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Groups lists each group and opens it with its rooms and totals. Browser test: e2e/group-bookings.spec.ts.</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4202,12 @@
       </c>
       <c r="P44" s="10" t="inlineStr">
         <is>
-          <t>set_arrival_ready exists; no screen shows the flag yet (skipped 6 Oct 2026).</t>
+          <t>set_arrival_ready exists. The booking page has Mark ready and Not ready; the Front Desk arrivals list and the group page show Ready (QA-15</t>
+        </is>
+      </c>
+      <c r="Q44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11 Oct 2026).</t>
         </is>
       </c>
     </row>
@@ -4236,6 +4288,7 @@
         </is>
       </c>
       <c r="P45" s="10" t="inlineStr"/>
+      <c r="Q45" s="10" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
@@ -4314,6 +4367,7 @@
         </is>
       </c>
       <c r="P46" s="10" t="inlineStr"/>
+      <c r="Q46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
@@ -4396,6 +4450,7 @@
           <t>The check-in and walk-in screens force the registration card tick; a direct database call that omits it is not refused (decision 6 Oct 2026). Drawn signature later.</t>
         </is>
       </c>
+      <c r="Q47" s="10" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
@@ -4474,6 +4529,7 @@
         </is>
       </c>
       <c r="P48" s="10" t="inlineStr"/>
+      <c r="Q48" s="10" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
@@ -4552,6 +4608,7 @@
         </is>
       </c>
       <c r="P49" s="10" t="inlineStr"/>
+      <c r="Q49" s="10" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
@@ -4630,6 +4687,7 @@
         </is>
       </c>
       <c r="P50" s="10" t="inlineStr"/>
+      <c r="Q50" s="10" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
@@ -4712,6 +4770,7 @@
           <t>Dearer room type: front desk charges the new rate; keeping it needs fo.upgrade.complimentary (SYSADMIN, GM, FOM), audited.</t>
         </is>
       </c>
+      <c r="Q51" s="10" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
@@ -4790,6 +4849,7 @@
         </is>
       </c>
       <c r="P52" s="10" t="inlineStr"/>
+      <c r="Q52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
@@ -4868,6 +4928,7 @@
         </is>
       </c>
       <c r="P53" s="10" t="inlineStr"/>
+      <c r="Q53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
@@ -4946,6 +5007,7 @@
         </is>
       </c>
       <c r="P54" s="10" t="inlineStr"/>
+      <c r="Q54" s="10" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
@@ -5024,6 +5086,7 @@
         </is>
       </c>
       <c r="P55" s="10" t="inlineStr"/>
+      <c r="Q55" s="10" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
@@ -5102,6 +5165,7 @@
         </is>
       </c>
       <c r="P56" s="10" t="inlineStr"/>
+      <c r="Q56" s="10" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
@@ -5180,6 +5244,7 @@
         </is>
       </c>
       <c r="P57" s="10" t="inlineStr"/>
+      <c r="Q57" s="10" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
@@ -5258,6 +5323,7 @@
         </is>
       </c>
       <c r="P58" s="10" t="inlineStr"/>
+      <c r="Q58" s="10" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
@@ -5336,6 +5402,7 @@
         </is>
       </c>
       <c r="P59" s="10" t="inlineStr"/>
+      <c r="Q59" s="10" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
@@ -5414,6 +5481,7 @@
         </is>
       </c>
       <c r="P60" s="10" t="inlineStr"/>
+      <c r="Q60" s="10" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
@@ -5492,6 +5560,7 @@
         </is>
       </c>
       <c r="P61" s="10" t="inlineStr"/>
+      <c r="Q61" s="10" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
@@ -5570,6 +5639,7 @@
         </is>
       </c>
       <c r="P62" s="10" t="inlineStr"/>
+      <c r="Q62" s="10" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
@@ -5648,6 +5718,7 @@
         </is>
       </c>
       <c r="P63" s="10" t="inlineStr"/>
+      <c r="Q63" s="10" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
@@ -5726,6 +5797,7 @@
         </is>
       </c>
       <c r="P64" s="10" t="inlineStr"/>
+      <c r="Q64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
@@ -5804,6 +5876,7 @@
         </is>
       </c>
       <c r="P65" s="10" t="inlineStr"/>
+      <c r="Q65" s="10" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
@@ -5882,6 +5955,7 @@
         </is>
       </c>
       <c r="P66" s="10" t="inlineStr"/>
+      <c r="Q66" s="10" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
@@ -5960,6 +6034,7 @@
         </is>
       </c>
       <c r="P67" s="10" t="inlineStr"/>
+      <c r="Q67" s="10" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
@@ -6038,6 +6113,7 @@
         </is>
       </c>
       <c r="P68" s="10" t="inlineStr"/>
+      <c r="Q68" s="10" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
@@ -6116,6 +6192,7 @@
         </is>
       </c>
       <c r="P69" s="10" t="inlineStr"/>
+      <c r="Q69" s="10" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
@@ -6194,6 +6271,7 @@
         </is>
       </c>
       <c r="P70" s="10" t="inlineStr"/>
+      <c r="Q70" s="10" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
@@ -6272,6 +6350,7 @@
         </is>
       </c>
       <c r="P71" s="10" t="inlineStr"/>
+      <c r="Q71" s="10" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
@@ -6350,6 +6429,7 @@
         </is>
       </c>
       <c r="P72" s="10" t="inlineStr"/>
+      <c r="Q72" s="10" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
@@ -6428,6 +6508,7 @@
         </is>
       </c>
       <c r="P73" s="10" t="inlineStr"/>
+      <c r="Q73" s="10" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
@@ -6506,6 +6587,7 @@
         </is>
       </c>
       <c r="P74" s="10" t="inlineStr"/>
+      <c r="Q74" s="10" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
@@ -6584,6 +6666,7 @@
         </is>
       </c>
       <c r="P75" s="10" t="inlineStr"/>
+      <c r="Q75" s="10" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
@@ -6662,6 +6745,7 @@
         </is>
       </c>
       <c r="P76" s="10" t="inlineStr"/>
+      <c r="Q76" s="10" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
@@ -6740,6 +6824,7 @@
         </is>
       </c>
       <c r="P77" s="10" t="inlineStr"/>
+      <c r="Q77" s="10" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
@@ -6818,6 +6903,7 @@
         </is>
       </c>
       <c r="P78" s="10" t="inlineStr"/>
+      <c r="Q78" s="10" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
@@ -6896,6 +6982,7 @@
         </is>
       </c>
       <c r="P79" s="10" t="inlineStr"/>
+      <c r="Q79" s="10" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
@@ -6974,6 +7061,7 @@
         </is>
       </c>
       <c r="P80" s="10" t="inlineStr"/>
+      <c r="Q80" s="10" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
@@ -7052,6 +7140,7 @@
         </is>
       </c>
       <c r="P81" s="10" t="inlineStr"/>
+      <c r="Q81" s="10" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
@@ -7130,6 +7219,7 @@
         </is>
       </c>
       <c r="P82" s="10" t="inlineStr"/>
+      <c r="Q82" s="10" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
@@ -7208,6 +7298,7 @@
         </is>
       </c>
       <c r="P83" s="10" t="inlineStr"/>
+      <c r="Q83" s="10" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
@@ -7286,6 +7377,7 @@
         </is>
       </c>
       <c r="P84" s="10" t="inlineStr"/>
+      <c r="Q84" s="10" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
@@ -7364,6 +7456,7 @@
         </is>
       </c>
       <c r="P85" s="10" t="inlineStr"/>
+      <c r="Q85" s="10" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
@@ -7442,6 +7535,7 @@
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr"/>
+      <c r="Q86" s="10" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
@@ -7520,6 +7614,7 @@
         </is>
       </c>
       <c r="P87" s="10" t="inlineStr"/>
+      <c r="Q87" s="10" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
@@ -7598,6 +7693,7 @@
         </is>
       </c>
       <c r="P88" s="10" t="inlineStr"/>
+      <c r="Q88" s="10" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
@@ -7676,6 +7772,7 @@
         </is>
       </c>
       <c r="P89" s="10" t="inlineStr"/>
+      <c r="Q89" s="10" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
@@ -7754,6 +7851,7 @@
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr"/>
+      <c r="Q90" s="10" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
@@ -7832,6 +7930,7 @@
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr"/>
+      <c r="Q91" s="10" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
@@ -7910,6 +8009,7 @@
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr"/>
+      <c r="Q92" s="10" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
@@ -7988,6 +8088,7 @@
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr"/>
+      <c r="Q93" s="10" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
@@ -8066,6 +8167,7 @@
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr"/>
+      <c r="Q94" s="10" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
@@ -8144,6 +8246,7 @@
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr"/>
+      <c r="Q95" s="10" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
@@ -8226,6 +8329,7 @@
           <t>Cashier shift page built (open, close with counts, review, reconcile). Not covered by a browser test yet. New permission fin.shift.reconcile goes to built-in roles only.</t>
         </is>
       </c>
+      <c r="Q96" s="10" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
@@ -8304,6 +8408,7 @@
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr"/>
+      <c r="Q97" s="10" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
@@ -8382,6 +8487,7 @@
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr"/>
+      <c r="Q98" s="10" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
@@ -8460,6 +8566,7 @@
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr"/>
+      <c r="Q99" s="10" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
@@ -8538,6 +8645,7 @@
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr"/>
+      <c r="Q100" s="10" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
@@ -8620,6 +8728,7 @@
           <t>Flags shown in Admin, Business date. The gate that stops the roll while a blocking flag is open is not built.</t>
         </is>
       </c>
+      <c r="Q101" s="10" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
@@ -8702,6 +8811,7 @@
           <t>Decided by Peter on 30 Sep 2026 (answer 5) and confirmed on 1 Oct 2026: same-day stays are charged one night; a manager can waive it with a reason.</t>
         </is>
       </c>
+      <c r="Q102" s="10" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
@@ -8780,6 +8890,7 @@
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr"/>
+      <c r="Q103" s="10" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
@@ -8858,6 +8969,7 @@
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr"/>
+      <c r="Q104" s="10" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
@@ -8936,6 +9048,7 @@
         </is>
       </c>
       <c r="P105" s="10" t="inlineStr"/>
+      <c r="Q105" s="10" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
@@ -9018,6 +9131,7 @@
           <t>Reports screen: KPIs, revenue by charge code, outstanding balances, payments, cancellations and stay length, balances by guest, export.</t>
         </is>
       </c>
+      <c r="Q106" s="10" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
@@ -9096,6 +9210,7 @@
         </is>
       </c>
       <c r="P107" s="10" t="inlineStr"/>
+      <c r="Q107" s="10" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
@@ -9174,6 +9289,7 @@
         </is>
       </c>
       <c r="P108" s="10" t="inlineStr"/>
+      <c r="Q108" s="10" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
@@ -9252,6 +9368,7 @@
         </is>
       </c>
       <c r="P109" s="10" t="inlineStr"/>
+      <c r="Q109" s="10" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
@@ -9330,6 +9447,7 @@
         </is>
       </c>
       <c r="P110" s="10" t="inlineStr"/>
+      <c r="Q110" s="10" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
@@ -9408,6 +9526,7 @@
         </is>
       </c>
       <c r="P111" s="10" t="inlineStr"/>
+      <c r="Q111" s="10" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
@@ -9486,6 +9605,7 @@
         </is>
       </c>
       <c r="P112" s="10" t="inlineStr"/>
+      <c r="Q112" s="10" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
@@ -9564,6 +9684,7 @@
         </is>
       </c>
       <c r="P113" s="10" t="inlineStr"/>
+      <c r="Q113" s="10" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
@@ -9646,6 +9767,7 @@
           <t>Method only; the accountant still signs off the rates (A11)</t>
         </is>
       </c>
+      <c r="Q114" s="10" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
@@ -9728,6 +9850,7 @@
           <t>Day totals and fields are stored in the invoice header when it is issued</t>
         </is>
       </c>
+      <c r="Q115" s="10" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
@@ -9810,6 +9933,7 @@
           <t>Month comes from the business date, not the clock. No hotel code in the number yet.</t>
         </is>
       </c>
+      <c r="Q116" s="10" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
@@ -9888,6 +10012,7 @@
         </is>
       </c>
       <c r="P117" s="10" t="inlineStr"/>
+      <c r="Q117" s="10" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
@@ -9966,6 +10091,7 @@
         </is>
       </c>
       <c r="P118" s="10" t="inlineStr"/>
+      <c r="Q118" s="10" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
@@ -10044,6 +10170,7 @@
         </is>
       </c>
       <c r="P119" s="10" t="inlineStr"/>
+      <c r="Q119" s="10" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
@@ -10122,6 +10249,7 @@
         </is>
       </c>
       <c r="P120" s="10" t="inlineStr"/>
+      <c r="Q120" s="10" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
@@ -10200,6 +10328,7 @@
         </is>
       </c>
       <c r="P121" s="10" t="inlineStr"/>
+      <c r="Q121" s="10" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="10" t="inlineStr">
@@ -10278,6 +10407,7 @@
         </is>
       </c>
       <c r="P122" s="10" t="inlineStr"/>
+      <c r="Q122" s="10" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
@@ -10356,6 +10486,7 @@
           <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
         </is>
       </c>
+      <c r="Q123" s="10" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="10" t="inlineStr">
@@ -10434,6 +10565,7 @@
           <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
         </is>
       </c>
+      <c r="Q124" s="10" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
@@ -10512,6 +10644,7 @@
           <t>Access is per branch, using the existing role assignment screen.</t>
         </is>
       </c>
+      <c r="Q125" s="10" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="10" t="inlineStr">
@@ -10590,6 +10723,7 @@
           <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
         </is>
       </c>
+      <c r="Q126" s="10" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
@@ -10668,6 +10802,7 @@
           <t>Bookings counted by arrival date; revenue by posting date.</t>
         </is>
       </c>
+      <c r="Q127" s="10" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
@@ -10746,6 +10881,7 @@
           <t>Guests still staying count as current.</t>
         </is>
       </c>
+      <c r="Q128" s="10" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
@@ -10828,6 +10964,7 @@
           <t>Email delivery waits on the sending domain and email account. Collected money nets payment reversals the same day (migration 20261015130000).</t>
         </is>
       </c>
+      <c r="Q129" s="10" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
@@ -10906,6 +11043,7 @@
           <t>Custom roles copied earlier do not get adm.ai.manage.</t>
         </is>
       </c>
+      <c r="Q130" s="10" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
@@ -10984,6 +11122,7 @@
           <t>Overdue means unpaid more than 30 days after departure.</t>
         </is>
       </c>
+      <c r="Q131" s="10" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="10" t="inlineStr">
@@ -11058,6 +11197,7 @@
         </is>
       </c>
       <c r="P132" s="10" t="inlineStr"/>
+      <c r="Q132" s="10" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
@@ -11132,6 +11272,7 @@
         </is>
       </c>
       <c r="P133" s="10" t="inlineStr"/>
+      <c r="Q133" s="10" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
@@ -11210,6 +11351,7 @@
           <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
         </is>
       </c>
+      <c r="Q134" s="10" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
@@ -11288,6 +11430,7 @@
           <t>The AI only drafts the list. This function is the check.</t>
         </is>
       </c>
+      <c r="Q135" s="10" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
@@ -11362,6 +11505,7 @@
         </is>
       </c>
       <c r="P136" s="10" t="inlineStr"/>
+      <c r="Q136" s="10" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
@@ -11440,6 +11584,7 @@
           <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
         </is>
       </c>
+      <c r="Q137" s="10" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="10" t="inlineStr">
@@ -11522,6 +11667,7 @@
           <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
         </is>
       </c>
+      <c r="Q138" s="10" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="10" t="inlineStr">
@@ -11604,6 +11750,7 @@
           <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
         </is>
       </c>
+      <c r="Q139" s="10" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="10" t="inlineStr">
@@ -11682,6 +11829,7 @@
           <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
         </is>
       </c>
+      <c r="Q140" s="10" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="10" t="inlineStr">
@@ -11760,6 +11908,7 @@
           <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
         </is>
       </c>
+      <c r="Q141" s="10" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="10" t="inlineStr">
@@ -11842,6 +11991,7 @@
           <t>Added 8 Oct 2026. Warning only; the hard gate stays in R2 (DAY-005).</t>
         </is>
       </c>
+      <c r="Q142" s="10" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="10" t="inlineStr">
@@ -11920,6 +12070,7 @@
           <t>Added 9 Oct 2026. Read-only; no money is changed.</t>
         </is>
       </c>
+      <c r="Q143" s="10" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="10" t="inlineStr">
@@ -11998,6 +12149,7 @@
           <t>Added 10 Oct 2026. The Payments report counted only payments and refunds before this. Cashier shift counts stay separate on purpose: they count what the drawer should hold.</t>
         </is>
       </c>
+      <c r="Q144" s="10" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="10" t="inlineStr">
@@ -12076,6 +12228,7 @@
           <t>Added 10 Oct 2026. Notes are not ledger rows; they never change a balance.</t>
         </is>
       </c>
+      <c r="Q145" s="10" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="10" t="inlineStr">
@@ -12150,6 +12303,7 @@
           <t>Added 10 Oct 2026. Mirrors docs/pilot-dry-run.md; screens and wording still need people.</t>
         </is>
       </c>
+      <c r="Q146" s="10" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="10" t="inlineStr">
@@ -12232,6 +12386,7 @@
           <t>Added 10 Oct 2026. Decision B: flag, do not stop (DAY-005 gate stays in R2).</t>
         </is>
       </c>
+      <c r="Q147" s="10" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="10" t="inlineStr">
@@ -12314,6 +12469,7 @@
           <t>QA-07. Fixes 14 helpers the security advisor listed. Added 10 Oct 2026.</t>
         </is>
       </c>
+      <c r="Q148" s="10" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="10" t="inlineStr">
@@ -12396,6 +12552,7 @@
           <t>QA-05. No prices in the email, because billing checkout is not switched on. Product name 'Zikora' in the wording is a draft.</t>
         </is>
       </c>
+      <c r="Q149" s="10" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="10" t="inlineStr">
@@ -12478,6 +12635,7 @@
           <t>QA-05.</t>
         </is>
       </c>
+      <c r="Q150" s="10" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="10" t="inlineStr">
@@ -12560,6 +12718,7 @@
           <t>Added 10 Oct 2026 (QA-12).</t>
         </is>
       </c>
+      <c r="Q151" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Offline stages 1 and 2: public page wording, register rows OFF-001 to OFF-004, roadmap
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q151"/>
+  <dimension ref="A1:Q155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12719,6 +12719,338 @@
         </is>
       </c>
       <c r="Q151" s="10" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="10" t="inlineStr">
+        <is>
+          <t>OFF-001</t>
+        </is>
+      </c>
+      <c r="B152" s="10" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C152" s="10" t="inlineStr">
+        <is>
+          <t>(all signed-in screens)</t>
+        </is>
+      </c>
+      <c r="D152" s="10" t="inlineStr">
+        <is>
+          <t>When the connection drops, the lists a signed-in user last loaded (arrivals, in house, room board, housekeeping tasks, open folios) stay readable on that device. A bar says 'No connection'.</t>
+        </is>
+      </c>
+      <c r="E152" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F152" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G152" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H152" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I152" s="10" t="inlineStr">
+        <is>
+          <t>A12; docs/offline-design.md</t>
+        </is>
+      </c>
+      <c r="J152" s="10" t="inlineStr">
+        <is>
+          <t>a user signed in on this device who loaded the front desk</t>
+        </is>
+      </c>
+      <c r="K152" s="10" t="inlineStr">
+        <is>
+          <t>the connection drops and the page is reloaded</t>
+        </is>
+      </c>
+      <c r="L152" s="10" t="inlineStr">
+        <is>
+          <t>the saved lists show and the No connection bar appears</t>
+        </is>
+      </c>
+      <c r="M152" s="10" t="inlineStr">
+        <is>
+          <t>public/sw.js; src/lib/offline/cache.ts; src/components/offline-banner.tsx</t>
+        </is>
+      </c>
+      <c r="N152" s="10" t="inlineStr">
+        <is>
+          <t>e2e/offline-read.spec.ts</t>
+        </is>
+      </c>
+      <c r="O152" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P152" s="10" t="inlineStr">
+        <is>
+          <t>Stage 1. Only data the user's role may see is saved. ID numbers and photos are never saved.</t>
+        </is>
+      </c>
+      <c r="Q152" s="10" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="10" t="inlineStr">
+        <is>
+          <t>OFF-002</t>
+        </is>
+      </c>
+      <c r="B153" s="10" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C153" s="10" t="inlineStr">
+        <is>
+          <t>(sign-out)</t>
+        </is>
+      </c>
+      <c r="D153" s="10" t="inlineStr">
+        <is>
+          <t>Saved offline data is removed from the device on sign-out.</t>
+        </is>
+      </c>
+      <c r="E153" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F153" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G153" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H153" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I153" s="10" t="inlineStr">
+        <is>
+          <t>docs/offline-design.md</t>
+        </is>
+      </c>
+      <c r="J153" s="10" t="inlineStr">
+        <is>
+          <t>a device holding saved lists</t>
+        </is>
+      </c>
+      <c r="K153" s="10" t="inlineStr">
+        <is>
+          <t>the user signs out</t>
+        </is>
+      </c>
+      <c r="L153" s="10" t="inlineStr">
+        <is>
+          <t>the saved lists are gone</t>
+        </is>
+      </c>
+      <c r="M153" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/offline/cache.ts clearOfflineData; src/routes/__root.tsx</t>
+        </is>
+      </c>
+      <c r="N153" s="10" t="inlineStr">
+        <is>
+          <t>e2e/offline-read.spec.ts</t>
+        </is>
+      </c>
+      <c r="O153" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P153" s="10" t="inlineStr">
+        <is>
+          <t>Stage 1. Sign-out is refused while actions still wait to send (OFF-004).</t>
+        </is>
+      </c>
+      <c r="Q153" s="10" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="10" t="inlineStr">
+        <is>
+          <t>OFF-003</t>
+        </is>
+      </c>
+      <c r="B154" s="10" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C154" s="10" t="inlineStr">
+        <is>
+          <t>Folio; My tasks</t>
+        </is>
+      </c>
+      <c r="D154" s="10" t="inlineStr">
+        <is>
+          <t>A charge, a payment, a cleaning task start and a cleaning task completion entered with no connection wait on the device and are sent oldest first when the connection returns. The bar shows how many wait and any that were refused, with Try again and Remove.</t>
+        </is>
+      </c>
+      <c r="E154" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F154" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G154" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H154" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I154" s="10" t="inlineStr">
+        <is>
+          <t>A12; docs/offline-design.md</t>
+        </is>
+      </c>
+      <c r="J154" s="10" t="inlineStr">
+        <is>
+          <t>no connection</t>
+        </is>
+      </c>
+      <c r="K154" s="10" t="inlineStr">
+        <is>
+          <t>a clerk posts a charge or starts a cleaning task</t>
+        </is>
+      </c>
+      <c r="L154" s="10" t="inlineStr">
+        <is>
+          <t>it waits on the device, then posts once when the connection returns</t>
+        </is>
+      </c>
+      <c r="M154" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/offline/queue.ts; src/lib/folios.tsx; src/lib/housekeeping.tsx</t>
+        </is>
+      </c>
+      <c r="N154" s="10" t="inlineStr">
+        <is>
+          <t>e2e/offline-write.spec.ts</t>
+        </is>
+      </c>
+      <c r="O154" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P154" s="10" t="inlineStr">
+        <is>
+          <t>Stage 2. Approvals, check-in, check-out and room moves stay online only (stage 3 is not built).</t>
+        </is>
+      </c>
+      <c r="Q154" s="10" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="10" t="inlineStr">
+        <is>
+          <t>OFF-004</t>
+        </is>
+      </c>
+      <c r="B155" s="10" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C155" s="10" t="inlineStr">
+        <is>
+          <t>Folio</t>
+        </is>
+      </c>
+      <c r="D155" s="10" t="inlineStr">
+        <is>
+          <t>A charge or payment that waits on the device carries its repeat-safe key, so sending it twice never posts twice.</t>
+        </is>
+      </c>
+      <c r="E155" s="10" t="inlineStr">
+        <is>
+          <t>FIN-008</t>
+        </is>
+      </c>
+      <c r="F155" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G155" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H155" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I155" s="10" t="inlineStr">
+        <is>
+          <t>Rule: idempotency keys</t>
+        </is>
+      </c>
+      <c r="J155" s="10" t="inlineStr">
+        <is>
+          <t>a queued charge</t>
+        </is>
+      </c>
+      <c r="K155" s="10" t="inlineStr">
+        <is>
+          <t>it is sent twice</t>
+        </is>
+      </c>
+      <c r="L155" s="10" t="inlineStr">
+        <is>
+          <t>the balance rises once</t>
+        </is>
+      </c>
+      <c r="M155" s="10" t="inlineStr">
+        <is>
+          <t>queue keeps the idempotency key; post_charge key check</t>
+        </is>
+      </c>
+      <c r="N155" s="10" t="inlineStr">
+        <is>
+          <t>e2e/offline-write.spec.ts</t>
+        </is>
+      </c>
+      <c r="O155" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P155" s="10" t="inlineStr">
+        <is>
+          <t>Stage 2.</t>
+        </is>
+      </c>
+      <c r="Q155" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
New hotels get a 60-day free trial (PLT-016)
create_hotel now sets the trial to 60 days (was 30). The pricing page,
signup page and terms say so, and the pricing button opens Create account.
Existing trials keep their dates. Test 17_more_features changed from 30 to 60.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'R1 Requirements'!$A$1:$O$108</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q158"/>
+  <dimension ref="A1:Q159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>a tenant, a 30-day trial, one property with country defaults, and the System Administrator and General Manager roles exist for them</t>
+          <t>a tenant, a 60-day trial, one property with country defaults, and the System Administrator and General Manager roles exist for them</t>
         </is>
       </c>
       <c r="M2" s="10" t="inlineStr">
@@ -13300,6 +13300,89 @@
         </is>
       </c>
       <c r="Q158" s="10" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="10" t="inlineStr">
+        <is>
+          <t>PLT-016</t>
+        </is>
+      </c>
+      <c r="B159" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C159" s="10" t="inlineStr">
+        <is>
+          <t>(signup page), (banner), pricing page</t>
+        </is>
+      </c>
+      <c r="D159" s="10" t="inlineStr">
+        <is>
+          <t>A new hotel gets a 60-day free trial with every feature and no card. After it, the hotel becomes read-only until a plan is switched on.</t>
+        </is>
+      </c>
+      <c r="E159" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F159" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G159" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H159" s="10" t="inlineStr">
+        <is>
+          <t>(any signed-in user)</t>
+        </is>
+      </c>
+      <c r="I159" s="10" t="inlineStr">
+        <is>
+          <t>A13, Decision of 12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J159" s="10" t="inlineStr">
+        <is>
+          <t>a signed-in user with a confirmed email and no hotel</t>
+        </is>
+      </c>
+      <c r="K159" s="10" t="inlineStr">
+        <is>
+          <t>they create their hotel</t>
+        </is>
+      </c>
+      <c r="L159" s="10" t="inlineStr">
+        <is>
+          <t>the trial ends 60 days after the hotel was created, and the status is trial</t>
+        </is>
+      </c>
+      <c r="M159" s="10" t="inlineStr">
+        <is>
+          <t>create_hotel</t>
+        </is>
+      </c>
+      <c r="N159" s="10" t="inlineStr">
+        <is>
+          <t>17_more_features (1)</t>
+        </is>
+      </c>
+      <c r="O159" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P159" s="10" t="inlineStr">
+        <is>
+          <t>Peter decided on 12 Oct 2026 (was 30 days). Hotels already on trial keep their dates; platform staff can extend one by hand. Plan choice at signup is not built: every new hotel starts on Starter (20 rooms).</t>
+        </is>
+      </c>
+      <c r="Q159" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Plan prices in naira: Starter 20,000, Standard 45,000, Pro 80,000 (PLT-017)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q159"/>
+  <dimension ref="A1:Q160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13383,6 +13383,89 @@
         </is>
       </c>
       <c r="Q159" s="10" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="10" t="inlineStr">
+        <is>
+          <t>PLT-017</t>
+        </is>
+      </c>
+      <c r="B160" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C160" s="10" t="inlineStr">
+        <is>
+          <t>(signup page), (banner), pricing page</t>
+        </is>
+      </c>
+      <c r="D160" s="10" t="inlineStr">
+        <is>
+          <t>Plan prices are set in naira: Starter 20,000, Standard 45,000, Pro 80,000 a month; a year costs ten months; Enterprise is quoted and has no online price.</t>
+        </is>
+      </c>
+      <c r="E160" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F160" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G160" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H160" s="10" t="inlineStr">
+        <is>
+          <t>(any signed-in user)</t>
+        </is>
+      </c>
+      <c r="I160" s="10" t="inlineStr">
+        <is>
+          <t>A16, Decision of 12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J160" s="10" t="inlineStr">
+        <is>
+          <t>a hotel administrator on trial</t>
+        </is>
+      </c>
+      <c r="K160" s="10" t="inlineStr">
+        <is>
+          <t>they start a payment for a plan</t>
+        </is>
+      </c>
+      <c r="L160" s="10" t="inlineStr">
+        <is>
+          <t>the amount comes from the plans table in kobo; Enterprise is refused with E_NO_PRICE</t>
+        </is>
+      </c>
+      <c r="M160" s="10" t="inlineStr">
+        <is>
+          <t>start_subscription_payment (migration 20261020130000)</t>
+        </is>
+      </c>
+      <c r="N160" s="10" t="inlineStr">
+        <is>
+          <t>59_plan_prices (1)</t>
+        </is>
+      </c>
+      <c r="O160" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P160" s="10" t="inlineStr">
+        <is>
+          <t>Starter 20,000 is the launch price. List price 30,000 and the 12-month lock for early hotels are not built: raising the price later raises it for every hotel. Features by plan are not built; plans cap rooms, properties and users only. Billing stays off until the Paystack key and webhook are set.</t>
+        </is>
+      </c>
+      <c r="Q160" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Starter plan is 30,000 naira; no launch price or price lock (A16)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -13402,7 +13402,7 @@
       </c>
       <c r="D160" s="10" t="inlineStr">
         <is>
-          <t>Plan prices are set in naira: Starter 20,000, Standard 45,000, Pro 80,000 a month; a year costs ten months; Enterprise is quoted and has no online price.</t>
+          <t>Plan prices are set in naira: Starter 30,000, Standard 45,000, Pro 80,000 a month; a year costs ten months; Enterprise is quoted and has no online price.</t>
         </is>
       </c>
       <c r="E160" s="10" t="inlineStr">
@@ -13462,7 +13462,7 @@
       </c>
       <c r="P160" s="10" t="inlineStr">
         <is>
-          <t>Starter 20,000 is the launch price. List price 30,000 and the 12-month lock for early hotels are not built: raising the price later raises it for every hotel. Features by plan are not built; plans cap rooms, properties and users only. Billing stays off until the Paystack key and webhook are set.</t>
+          <t>One price for every hotel: no launch price and no price lock (Peter, 12 Oct 2026). Features by plan are not built; plans cap rooms, properties and users only. Billing stays off until the Paystack key and webhook are set.</t>
         </is>
       </c>
       <c r="Q160" s="10" t="n"/>

</xml_diff>

<commit_message>
Offline stage 3a: check-out and room moves wait on the device (OFF-005, OFF-006)
No database change. Both functions already tolerate a repeat. A check-out with a
balance is accepted at send time only for staff who may check out with a balance.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q160"/>
+  <dimension ref="A1:Q162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12964,7 +12964,7 @@
       </c>
       <c r="P154" s="10" t="inlineStr">
         <is>
-          <t>Stage 2. Approvals, check-in, check-out and room moves stay online only (stage 3 is not built).</t>
+          <t>Stage 2. Approvals and check-in stay online only. Check-out and room moves: see OFF-005 and OFF-006.</t>
         </is>
       </c>
       <c r="Q154" s="10" t="n"/>
@@ -13466,6 +13466,172 @@
         </is>
       </c>
       <c r="Q160" s="10" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="10" t="inlineStr">
+        <is>
+          <t>OFF-005</t>
+        </is>
+      </c>
+      <c r="B161" s="10" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C161" s="10" t="inlineStr">
+        <is>
+          <t>Check-out</t>
+        </is>
+      </c>
+      <c r="D161" s="10" t="inlineStr">
+        <is>
+          <t>A check-out entered with no connection waits on the device and is sent when the connection returns. The screen does not offer it twice while it waits. The database applies its usual rule at send time: a balance that is not zero is accepted only from someone who may check out with a balance, and it then appears in Collections for Finance. Anyone else sees it under Needs attention.</t>
+        </is>
+      </c>
+      <c r="E161" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F161" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G161" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H161" s="10" t="inlineStr">
+        <is>
+          <t>fo.checkout; fo.checkout.unsettled</t>
+        </is>
+      </c>
+      <c r="I161" s="10" t="inlineStr">
+        <is>
+          <t>A12; docs/offline-design.md</t>
+        </is>
+      </c>
+      <c r="J161" s="10" t="inlineStr">
+        <is>
+          <t>no connection and a guest in house</t>
+        </is>
+      </c>
+      <c r="K161" s="10" t="inlineStr">
+        <is>
+          <t>a clerk checks the guest out</t>
+        </is>
+      </c>
+      <c r="L161" s="10" t="inlineStr">
+        <is>
+          <t>it waits on the device, then the guest is checked out once when the connection returns</t>
+        </is>
+      </c>
+      <c r="M161" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/offline/queue.ts; src/lib/checkout.tsx; src/lib/offline/warm.ts</t>
+        </is>
+      </c>
+      <c r="N161" s="10" t="inlineStr">
+        <is>
+          <t>e2e/offline-stage3.spec.ts</t>
+        </is>
+      </c>
+      <c r="O161" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P161" s="10" t="inlineStr">
+        <is>
+          <t>Stage 3a. Reason recorded: Checked out with no connection. Approvals stay online only.</t>
+        </is>
+      </c>
+      <c r="Q161" s="10" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="10" t="inlineStr">
+        <is>
+          <t>OFF-006</t>
+        </is>
+      </c>
+      <c r="B162" s="10" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C162" s="10" t="inlineStr">
+        <is>
+          <t>Front Desk</t>
+        </is>
+      </c>
+      <c r="D162" s="10" t="inlineStr">
+        <is>
+          <t>A room move entered with no connection waits on the device and is sent when the connection returns. If the database refuses it (for example the room was taken), it moves to Needs attention with the plain message and nothing is lost.</t>
+        </is>
+      </c>
+      <c r="E162" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F162" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G162" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H162" s="10" t="inlineStr">
+        <is>
+          <t>fo.room.move</t>
+        </is>
+      </c>
+      <c r="I162" s="10" t="inlineStr">
+        <is>
+          <t>A12; docs/offline-design.md</t>
+        </is>
+      </c>
+      <c r="J162" s="10" t="inlineStr">
+        <is>
+          <t>no connection and a guest in house</t>
+        </is>
+      </c>
+      <c r="K162" s="10" t="inlineStr">
+        <is>
+          <t>a clerk moves the guest to another room</t>
+        </is>
+      </c>
+      <c r="L162" s="10" t="inlineStr">
+        <is>
+          <t>it waits on the device and moves the guest when the connection returns, or shows Needs attention if refused</t>
+        </is>
+      </c>
+      <c r="M162" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/offline/queue.ts; src/lib/front-desk.tsx; src/lib/offline/warm.ts</t>
+        </is>
+      </c>
+      <c r="N162" s="10" t="inlineStr">
+        <is>
+          <t>e2e/offline-stage3.spec.ts</t>
+        </is>
+      </c>
+      <c r="O162" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P162" s="10" t="inlineStr">
+        <is>
+          <t>Stage 3a. Check-in and walk-in are stage 3b (waiting on the ID number decision).</t>
+        </is>
+      </c>
+      <c r="Q162" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Day 61: a trial that ends moves the hotel to its paid plan with 14 days to pay (PLT-018)
Migration 20261021100000. Tests 15, 51 changed with Peter's yes (past_due, price in email). New test 60.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q160"/>
+  <dimension ref="A1:Q161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>A trial ends automatically and the hotel becomes read-only.</t>
+          <t>A trial ends automatically. The hotel moves to a paid plan and has 14 days to pay (see PLT-018).</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="L6" s="10" t="inlineStr">
         <is>
-          <t>the subscription is Expired, the change is in the subscription history, and the hotel can read but not create</t>
+          <t>the subscription is Past due, the change is in the subscription history, and the hotel keeps working during the 14 days</t>
         </is>
       </c>
       <c r="M6" s="10" t="inlineStr">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="P149" s="10" t="inlineStr">
         <is>
-          <t>QA-05. No prices in the email, because billing checkout is not switched on. Product name 'Zikora' in the wording is a draft.</t>
+          <t>QA-05. The warnings name the plan and price (PLT-018). Product name 'Zikora' in the wording is a draft.</t>
         </is>
       </c>
       <c r="Q149" s="10" t="n"/>
@@ -13319,7 +13319,7 @@
       </c>
       <c r="D159" s="10" t="inlineStr">
         <is>
-          <t>A new hotel gets a 60-day free trial with every feature and no card. After it, the hotel becomes read-only until a plan is switched on.</t>
+          <t>A new hotel gets a 60-day free trial with every feature and no card. After it, the hotel moves to a paid plan with 14 days to pay (PLT-018).</t>
         </is>
       </c>
       <c r="E159" s="10" t="inlineStr">
@@ -13466,6 +13466,89 @@
         </is>
       </c>
       <c r="Q160" s="10" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="10" t="inlineStr">
+        <is>
+          <t>PLT-018</t>
+        </is>
+      </c>
+      <c r="B161" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C161" s="10" t="inlineStr">
+        <is>
+          <t>(email), (banner), pricing page</t>
+        </is>
+      </c>
+      <c r="D161" s="10" t="inlineStr">
+        <is>
+          <t>When the 60-day trial ends, the hotel moves to the cheapest plan it fits (Starter, Standard, Pro, else Enterprise), becomes Past due and has 14 days to pay, counted from the day the trial ended. It keeps working. One email names the plan and the monthly price from the plans table; a hotel too big for every priced plan is told to contact us for a quote. Unpaid after 14 days, the hotel becomes read-only (suspended). Nothing is deleted. The 7 and 1 day warnings name the plan and price.</t>
+        </is>
+      </c>
+      <c r="E161" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F161" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G161" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H161" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I161" s="10" t="inlineStr">
+        <is>
+          <t>A13, A16, Decision of 12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J161" s="10" t="inlineStr">
+        <is>
+          <t>a hotel whose trial end date has passed</t>
+        </is>
+      </c>
+      <c r="K161" s="10" t="inlineStr">
+        <is>
+          <t>the daily clock runs</t>
+        </is>
+      </c>
+      <c r="L161" s="10" t="inlineStr">
+        <is>
+          <t>the hotel is on its plan, Past due, still working, with one email; after 14 days unpaid it is read-only</t>
+        </is>
+      </c>
+      <c r="M161" s="10" t="inlineStr">
+        <is>
+          <t>app.run_subscription_clock; app.trial_plan; app.plan_price_text; app.trial_plan_sentence</t>
+        </is>
+      </c>
+      <c r="N161" s="10" t="inlineStr">
+        <is>
+          <t>60_trial_to_paid_plan; 15_accounts; 51_subscription_notices</t>
+        </is>
+      </c>
+      <c r="O161" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P161" s="10" t="inlineStr">
+        <is>
+          <t>Billing checkout (Paystack) is off until the key and webhook are set, so payment is arranged by email to hello@zikorahq.com. The Terms (section 4) still say read-only at trial end and need counsel to reword.</t>
+        </is>
+      </c>
+      <c r="Q161" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Offline stage 3b: check-in waits on the device; the ID number stays only until it is sent (OFF-007, OFF-008)
No database change. check_in already returns the first stay on a repeat.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q162"/>
+  <dimension ref="A1:Q164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13628,10 +13628,176 @@
       </c>
       <c r="P162" s="10" t="inlineStr">
         <is>
-          <t>Stage 3a. Check-in and walk-in are stage 3b (waiting on the ID number decision).</t>
+          <t>Stage 3a. Check-in is OFF-007 and OFF-008. Walk-in is not built.</t>
         </is>
       </c>
       <c r="Q162" s="10" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="10" t="inlineStr">
+        <is>
+          <t>OFF-007</t>
+        </is>
+      </c>
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C163" s="10" t="inlineStr">
+        <is>
+          <t>Front Desk</t>
+        </is>
+      </c>
+      <c r="D163" s="10" t="inlineStr">
+        <is>
+          <t>A check-in entered with no connection waits on the device and is sent when the connection returns. The guest's ID number waits on the device only until the entry is sent, then it is gone.</t>
+        </is>
+      </c>
+      <c r="E163" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F163" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G163" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H163" s="10" t="inlineStr">
+        <is>
+          <t>fo.checkin</t>
+        </is>
+      </c>
+      <c r="I163" s="10" t="inlineStr">
+        <is>
+          <t>A12; docs/offline-design.md; Peter 12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J163" s="10" t="inlineStr">
+        <is>
+          <t>no connection and an arrival today</t>
+        </is>
+      </c>
+      <c r="K163" s="10" t="inlineStr">
+        <is>
+          <t>a clerk checks the guest in</t>
+        </is>
+      </c>
+      <c r="L163" s="10" t="inlineStr">
+        <is>
+          <t>it waits on the device, then the guest is checked in once when the connection returns, and the ID number is no longer saved on the device</t>
+        </is>
+      </c>
+      <c r="M163" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/offline/queue.ts; src/lib/front-desk.tsx; src/lib/offline/warm.ts</t>
+        </is>
+      </c>
+      <c r="N163" s="10" t="inlineStr">
+        <is>
+          <t>e2e/offline-stage3.spec.ts</t>
+        </is>
+      </c>
+      <c r="O163" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P163" s="10" t="inlineStr">
+        <is>
+          <t>Stage 3b, check-in of an existing booking. Walk-in is not built (needs a new guest to be made offline). ID photos need a connection.</t>
+        </is>
+      </c>
+      <c r="Q163" s="10" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="10" t="inlineStr">
+        <is>
+          <t>OFF-008</t>
+        </is>
+      </c>
+      <c r="B164" s="10" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C164" s="10" t="inlineStr">
+        <is>
+          <t>Front Desk</t>
+        </is>
+      </c>
+      <c r="D164" s="10" t="inlineStr">
+        <is>
+          <t>A check-in the database refuses (for example the room is taken) moves to Needs attention with the plain message. Its ID number is erased from the device at that moment, it cannot be sent again as it was, and staff check the guest in again online.</t>
+        </is>
+      </c>
+      <c r="E164" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F164" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G164" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H164" s="10" t="inlineStr">
+        <is>
+          <t>fo.checkin</t>
+        </is>
+      </c>
+      <c r="I164" s="10" t="inlineStr">
+        <is>
+          <t>docs/offline-design.md; Peter 12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J164" s="10" t="inlineStr">
+        <is>
+          <t>a check-in waiting on the device</t>
+        </is>
+      </c>
+      <c r="K164" s="10" t="inlineStr">
+        <is>
+          <t>the database refuses it</t>
+        </is>
+      </c>
+      <c r="L164" s="10" t="inlineStr">
+        <is>
+          <t>the entry shows Needs attention with Remove only, and no ID number is saved on the device</t>
+        </is>
+      </c>
+      <c r="M164" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/offline/queue.ts; src/components/offline-banner.tsx</t>
+        </is>
+      </c>
+      <c r="N164" s="10" t="inlineStr">
+        <is>
+          <t>e2e/offline-stage3.spec.ts</t>
+        </is>
+      </c>
+      <c r="O164" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P164" s="10" t="inlineStr">
+        <is>
+          <t>Stage 3b.</t>
+        </is>
+      </c>
+      <c r="Q164" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Contact form sends through the server, with an email app fallback (PLT-019)
The form now asks the server to email hello@zikorahq.com through Resend and says thank you only when the service confirms. With no key set, or if sending fails, it opens the visitor's email app and says nothing has been received. A hidden field turns bots away.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q165"/>
+  <dimension ref="A1:Q166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13881,6 +13881,89 @@
         </is>
       </c>
       <c r="Q165" s="10" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="10" t="inlineStr">
+        <is>
+          <t>PLT-019</t>
+        </is>
+      </c>
+      <c r="B166" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C166" s="10" t="inlineStr">
+        <is>
+          <t>Contact page</t>
+        </is>
+      </c>
+      <c r="D166" s="10" t="inlineStr">
+        <is>
+          <t>The website contact form emails the enquiry to hello@zikorahq.com through the email service and says thank you only when the service confirms. If the service is not set up or fails, the form opens the visitor's email app and says nothing has been received. A hidden field turns bots away. Nothing is stored.</t>
+        </is>
+      </c>
+      <c r="E166" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F166" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G166" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H166" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I166" s="10" t="inlineStr">
+        <is>
+          <t>Audit 12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J166" s="10" t="inlineStr">
+        <is>
+          <t>a visitor fills the contact form</t>
+        </is>
+      </c>
+      <c r="K166" s="10" t="inlineStr">
+        <is>
+          <t>they send it</t>
+        </is>
+      </c>
+      <c r="L166" s="10" t="inlineStr">
+        <is>
+          <t>one email reaches the contact address with the visitor as reply-to; with no email key the form says it did not send</t>
+        </is>
+      </c>
+      <c r="M166" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/enquiry.ts; src/lib/enquiry.functions.ts; src/components/public/enquiry-form.tsx</t>
+        </is>
+      </c>
+      <c r="N166" s="10" t="inlineStr">
+        <is>
+          <t>e2e/enquiry-unit.spec.ts</t>
+        </is>
+      </c>
+      <c r="O166" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P166" s="10" t="inlineStr">
+        <is>
+          <t>Real sending starts when RESEND_API_KEY and OUTBOX_FROM_EMAIL are set in Vercel. Until then the form uses the email app fallback. No rate limit yet.</t>
+        </is>
+      </c>
+      <c r="Q166" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Security headers on every page (PLT-020)
No framing by other sites, no file type guessing, limited referrer, microphone and location off, camera for the same site only. No script policy yet.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q166"/>
+  <dimension ref="A1:Q167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13964,6 +13964,89 @@
         </is>
       </c>
       <c r="Q166" s="10" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="10" t="inlineStr">
+        <is>
+          <t>PLT-020</t>
+        </is>
+      </c>
+      <c r="B167" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C167" s="10" t="inlineStr">
+        <is>
+          <t>All pages</t>
+        </is>
+      </c>
+      <c r="D167" s="10" t="inlineStr">
+        <is>
+          <t>Every page and answer from the live site carries security headers: no framing by other sites, no file type guessing, limited referrer, microphone and location off, camera allowed for the same site only (ID and ticket photos). No script policy yet, because the app needs inline scripts to start.</t>
+        </is>
+      </c>
+      <c r="E167" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F167" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G167" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H167" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I167" s="10" t="inlineStr">
+        <is>
+          <t>Audit 12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J167" s="10" t="inlineStr">
+        <is>
+          <t>a visitor or a hijacking site loads Zikora</t>
+        </is>
+      </c>
+      <c r="K167" s="10" t="inlineStr">
+        <is>
+          <t>the page is served</t>
+        </is>
+      </c>
+      <c r="L167" s="10" t="inlineStr">
+        <is>
+          <t>other sites cannot frame it and the browser applies the limits</t>
+        </is>
+      </c>
+      <c r="M167" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/security-headers.ts; vite.config.ts</t>
+        </is>
+      </c>
+      <c r="N167" s="10" t="inlineStr">
+        <is>
+          <t>e2e/security-headers-unit.spec.ts</t>
+        </is>
+      </c>
+      <c r="O167" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P167" s="10" t="inlineStr">
+        <is>
+          <t>Headers apply on the Vercel build only (not the local dev server). Full script policy (CSP) is a later job.</t>
+        </is>
+      </c>
+      <c r="Q167" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Web app manifest so Zikora can be added to a phone home screen (PLT-021)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q166"/>
+  <dimension ref="A1:Q167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13553,22 +13553,22 @@
     <row r="162">
       <c r="A162" s="10" t="inlineStr">
         <is>
-          <t>OFF-005</t>
+          <t>PLT-021</t>
         </is>
       </c>
       <c r="B162" s="10" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Platform &amp; Tenancy</t>
         </is>
       </c>
       <c r="C162" s="10" t="inlineStr">
         <is>
-          <t>Check-out</t>
+          <t>All pages</t>
         </is>
       </c>
       <c r="D162" s="10" t="inlineStr">
         <is>
-          <t>A check-out entered with no connection waits on the device and is sent when the connection returns. The screen does not offer it twice while it waits. The database applies its usual rule at send time: a balance that is not zero is accepted only from someone who may check out with a balance, and it then appears in Collections for Finance. Anyone else sees it under Needs attention.</t>
+          <t>Zikora can be added to a phone or tablet home screen and opens as its own app window, with the Zikora name, icon and colours. It opens on the sign-in page.</t>
         </is>
       </c>
       <c r="E162" s="10" t="inlineStr">
@@ -13588,37 +13588,37 @@
       </c>
       <c r="H162" s="10" t="inlineStr">
         <is>
-          <t>fo.checkout; fo.checkout.unsettled</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I162" s="10" t="inlineStr">
         <is>
-          <t>A12; docs/offline-design.md</t>
+          <t>Audit 12 Oct 2026</t>
         </is>
       </c>
       <c r="J162" s="10" t="inlineStr">
         <is>
-          <t>no connection and a guest in house</t>
+          <t>a staff member opens Zikora on a phone</t>
         </is>
       </c>
       <c r="K162" s="10" t="inlineStr">
         <is>
-          <t>a clerk checks the guest out</t>
+          <t>they choose Add to home screen (or Install)</t>
         </is>
       </c>
       <c r="L162" s="10" t="inlineStr">
         <is>
-          <t>it waits on the device, then the guest is checked out once when the connection returns</t>
+          <t>the icon appears with the name Zikora and it opens full screen on the sign-in page</t>
         </is>
       </c>
       <c r="M162" s="10" t="inlineStr">
         <is>
-          <t>src/lib/offline/queue.ts; src/lib/checkout.tsx; src/lib/offline/warm.ts</t>
+          <t>public/manifest.webmanifest; src/routes/__root.tsx</t>
         </is>
       </c>
       <c r="N162" s="10" t="inlineStr">
         <is>
-          <t>e2e/offline-stage3.spec.ts</t>
+          <t>e2e/web-manifest-unit.spec.ts</t>
         </is>
       </c>
       <c r="O162" s="10" t="inlineStr">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="P162" s="10" t="inlineStr">
         <is>
-          <t>Stage 3a. Reason recorded: Checked out with no connection. Approvals stay online only.</t>
+          <t>Needs a real phone check (iPhone Safari and Android Chrome). Works with the offline service worker already in place.</t>
         </is>
       </c>
       <c r="Q162" s="10" t="n"/>
@@ -13636,7 +13636,7 @@
     <row r="163">
       <c r="A163" s="10" t="inlineStr">
         <is>
-          <t>OFF-006</t>
+          <t>OFF-005</t>
         </is>
       </c>
       <c r="B163" s="10" t="inlineStr">
@@ -13646,12 +13646,12 @@
       </c>
       <c r="C163" s="10" t="inlineStr">
         <is>
-          <t>Front Desk</t>
+          <t>Check-out</t>
         </is>
       </c>
       <c r="D163" s="10" t="inlineStr">
         <is>
-          <t>A room move entered with no connection waits on the device and is sent when the connection returns. If the database refuses it (for example the room was taken), it moves to Needs attention with the plain message and nothing is lost.</t>
+          <t>A check-out entered with no connection waits on the device and is sent when the connection returns. The screen does not offer it twice while it waits. The database applies its usual rule at send time: a balance that is not zero is accepted only from someone who may check out with a balance, and it then appears in Collections for Finance. Anyone else sees it under Needs attention.</t>
         </is>
       </c>
       <c r="E163" s="10" t="inlineStr">
@@ -13671,7 +13671,7 @@
       </c>
       <c r="H163" s="10" t="inlineStr">
         <is>
-          <t>fo.room.move</t>
+          <t>fo.checkout; fo.checkout.unsettled</t>
         </is>
       </c>
       <c r="I163" s="10" t="inlineStr">
@@ -13686,17 +13686,17 @@
       </c>
       <c r="K163" s="10" t="inlineStr">
         <is>
-          <t>a clerk moves the guest to another room</t>
+          <t>a clerk checks the guest out</t>
         </is>
       </c>
       <c r="L163" s="10" t="inlineStr">
         <is>
-          <t>it waits on the device and moves the guest when the connection returns, or shows Needs attention if refused</t>
+          <t>it waits on the device, then the guest is checked out once when the connection returns</t>
         </is>
       </c>
       <c r="M163" s="10" t="inlineStr">
         <is>
-          <t>src/lib/offline/queue.ts; src/lib/front-desk.tsx; src/lib/offline/warm.ts</t>
+          <t>src/lib/offline/queue.ts; src/lib/checkout.tsx; src/lib/offline/warm.ts</t>
         </is>
       </c>
       <c r="N163" s="10" t="inlineStr">
@@ -13711,7 +13711,7 @@
       </c>
       <c r="P163" s="10" t="inlineStr">
         <is>
-          <t>Stage 3a. Check-in is OFF-007 and OFF-008. Walk-in is not built.</t>
+          <t>Stage 3a. Reason recorded: Checked out with no connection. Approvals stay online only.</t>
         </is>
       </c>
       <c r="Q163" s="10" t="n"/>
@@ -13719,7 +13719,7 @@
     <row r="164">
       <c r="A164" s="10" t="inlineStr">
         <is>
-          <t>OFF-007</t>
+          <t>OFF-006</t>
         </is>
       </c>
       <c r="B164" s="10" t="inlineStr">
@@ -13734,7 +13734,7 @@
       </c>
       <c r="D164" s="10" t="inlineStr">
         <is>
-          <t>A check-in entered with no connection waits on the device and is sent when the connection returns. The guest's ID number waits on the device only until the entry is sent, then it is gone.</t>
+          <t>A room move entered with no connection waits on the device and is sent when the connection returns. If the database refuses it (for example the room was taken), it moves to Needs attention with the plain message and nothing is lost.</t>
         </is>
       </c>
       <c r="E164" s="10" t="inlineStr">
@@ -13754,27 +13754,27 @@
       </c>
       <c r="H164" s="10" t="inlineStr">
         <is>
-          <t>fo.checkin</t>
+          <t>fo.room.move</t>
         </is>
       </c>
       <c r="I164" s="10" t="inlineStr">
         <is>
-          <t>A12; docs/offline-design.md; Peter 12 Oct 2026</t>
+          <t>A12; docs/offline-design.md</t>
         </is>
       </c>
       <c r="J164" s="10" t="inlineStr">
         <is>
-          <t>no connection and an arrival today</t>
+          <t>no connection and a guest in house</t>
         </is>
       </c>
       <c r="K164" s="10" t="inlineStr">
         <is>
-          <t>a clerk checks the guest in</t>
+          <t>a clerk moves the guest to another room</t>
         </is>
       </c>
       <c r="L164" s="10" t="inlineStr">
         <is>
-          <t>it waits on the device, then the guest is checked in once when the connection returns, and the ID number is no longer saved on the device</t>
+          <t>it waits on the device and moves the guest when the connection returns, or shows Needs attention if refused</t>
         </is>
       </c>
       <c r="M164" s="10" t="inlineStr">
@@ -13794,7 +13794,7 @@
       </c>
       <c r="P164" s="10" t="inlineStr">
         <is>
-          <t>Stage 3b, check-in of an existing booking. Walk-in is not built (needs a new guest to be made offline). ID photos need a connection.</t>
+          <t>Stage 3a. Check-in is OFF-007 and OFF-008. Walk-in is not built.</t>
         </is>
       </c>
       <c r="Q164" s="10" t="n"/>
@@ -13802,7 +13802,7 @@
     <row r="165">
       <c r="A165" s="10" t="inlineStr">
         <is>
-          <t>OFF-008</t>
+          <t>OFF-007</t>
         </is>
       </c>
       <c r="B165" s="10" t="inlineStr">
@@ -13817,7 +13817,7 @@
       </c>
       <c r="D165" s="10" t="inlineStr">
         <is>
-          <t>A check-in the database refuses (for example the room is taken) moves to Needs attention with the plain message. Its ID number is erased from the device at that moment, it cannot be sent again as it was, and staff check the guest in again online.</t>
+          <t>A check-in entered with no connection waits on the device and is sent when the connection returns. The guest's ID number waits on the device only until the entry is sent, then it is gone.</t>
         </is>
       </c>
       <c r="E165" s="10" t="inlineStr">
@@ -13827,7 +13827,7 @@
       </c>
       <c r="F165" s="10" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="G165" s="10" t="inlineStr">
@@ -13842,27 +13842,27 @@
       </c>
       <c r="I165" s="10" t="inlineStr">
         <is>
-          <t>docs/offline-design.md; Peter 12 Oct 2026</t>
+          <t>A12; docs/offline-design.md; Peter 12 Oct 2026</t>
         </is>
       </c>
       <c r="J165" s="10" t="inlineStr">
         <is>
-          <t>a check-in waiting on the device</t>
+          <t>no connection and an arrival today</t>
         </is>
       </c>
       <c r="K165" s="10" t="inlineStr">
         <is>
-          <t>the database refuses it</t>
+          <t>a clerk checks the guest in</t>
         </is>
       </c>
       <c r="L165" s="10" t="inlineStr">
         <is>
-          <t>the entry shows Needs attention with Remove only, and no ID number is saved on the device</t>
+          <t>it waits on the device, then the guest is checked in once when the connection returns, and the ID number is no longer saved on the device</t>
         </is>
       </c>
       <c r="M165" s="10" t="inlineStr">
         <is>
-          <t>src/lib/offline/queue.ts; src/components/offline-banner.tsx</t>
+          <t>src/lib/offline/queue.ts; src/lib/front-desk.tsx; src/lib/offline/warm.ts</t>
         </is>
       </c>
       <c r="N165" s="10" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="P165" s="10" t="inlineStr">
         <is>
-          <t>Stage 3b.</t>
+          <t>Stage 3b, check-in of an existing booking. Walk-in is not built (needs a new guest to be made offline). ID photos need a connection.</t>
         </is>
       </c>
       <c r="Q165" s="10" t="n"/>
@@ -13885,85 +13885,168 @@
     <row r="166">
       <c r="A166" s="10" t="inlineStr">
         <is>
+          <t>OFF-008</t>
+        </is>
+      </c>
+      <c r="B166" s="10" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C166" s="10" t="inlineStr">
+        <is>
+          <t>Front Desk</t>
+        </is>
+      </c>
+      <c r="D166" s="10" t="inlineStr">
+        <is>
+          <t>A check-in the database refuses (for example the room is taken) moves to Needs attention with the plain message. Its ID number is erased from the device at that moment, it cannot be sent again as it was, and staff check the guest in again online.</t>
+        </is>
+      </c>
+      <c r="E166" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F166" s="10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G166" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H166" s="10" t="inlineStr">
+        <is>
+          <t>fo.checkin</t>
+        </is>
+      </c>
+      <c r="I166" s="10" t="inlineStr">
+        <is>
+          <t>docs/offline-design.md; Peter 12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J166" s="10" t="inlineStr">
+        <is>
+          <t>a check-in waiting on the device</t>
+        </is>
+      </c>
+      <c r="K166" s="10" t="inlineStr">
+        <is>
+          <t>the database refuses it</t>
+        </is>
+      </c>
+      <c r="L166" s="10" t="inlineStr">
+        <is>
+          <t>the entry shows Needs attention with Remove only, and no ID number is saved on the device</t>
+        </is>
+      </c>
+      <c r="M166" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/offline/queue.ts; src/components/offline-banner.tsx</t>
+        </is>
+      </c>
+      <c r="N166" s="10" t="inlineStr">
+        <is>
+          <t>e2e/offline-stage3.spec.ts</t>
+        </is>
+      </c>
+      <c r="O166" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P166" s="10" t="inlineStr">
+        <is>
+          <t>Stage 3b.</t>
+        </is>
+      </c>
+      <c r="Q166" s="10" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="10" t="inlineStr">
+        <is>
           <t>PLT-019</t>
         </is>
       </c>
-      <c r="B166" s="10" t="inlineStr">
+      <c r="B167" s="10" t="inlineStr">
         <is>
           <t>Platform &amp; Tenancy</t>
         </is>
       </c>
-      <c r="C166" s="10" t="inlineStr">
+      <c r="C167" s="10" t="inlineStr">
         <is>
           <t>Contact page</t>
         </is>
       </c>
-      <c r="D166" s="10" t="inlineStr">
+      <c r="D167" s="10" t="inlineStr">
         <is>
           <t>The website contact form emails the enquiry to hello@zikorahq.com through the email service and says thank you only when the service confirms. If the service is not set up or fails, the form opens the visitor's email app and says nothing has been received. A hidden field turns bots away. Nothing is stored.</t>
         </is>
       </c>
-      <c r="E166" s="10" t="inlineStr">
+      <c r="E167" s="10" t="inlineStr">
         <is>
           <t>BR-001</t>
         </is>
       </c>
-      <c r="F166" s="10" t="inlineStr">
+      <c r="F167" s="10" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="G166" s="10" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H166" s="10" t="inlineStr">
+      <c r="G167" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H167" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I166" s="10" t="inlineStr">
+      <c r="I167" s="10" t="inlineStr">
         <is>
           <t>Audit 12 Oct 2026</t>
         </is>
       </c>
-      <c r="J166" s="10" t="inlineStr">
+      <c r="J167" s="10" t="inlineStr">
         <is>
           <t>a visitor fills the contact form</t>
         </is>
       </c>
-      <c r="K166" s="10" t="inlineStr">
+      <c r="K167" s="10" t="inlineStr">
         <is>
           <t>they send it</t>
         </is>
       </c>
-      <c r="L166" s="10" t="inlineStr">
+      <c r="L167" s="10" t="inlineStr">
         <is>
           <t>one email reaches the contact address with the visitor as reply-to; with no email key the form says it did not send</t>
         </is>
       </c>
-      <c r="M166" s="10" t="inlineStr">
+      <c r="M167" s="10" t="inlineStr">
         <is>
           <t>src/lib/enquiry.ts; src/lib/enquiry.functions.ts; src/components/public/enquiry-form.tsx</t>
         </is>
       </c>
-      <c r="N166" s="10" t="inlineStr">
+      <c r="N167" s="10" t="inlineStr">
         <is>
           <t>e2e/enquiry-unit.spec.ts</t>
         </is>
       </c>
-      <c r="O166" s="10" t="inlineStr">
-        <is>
-          <t>Built+tested</t>
-        </is>
-      </c>
-      <c r="P166" s="10" t="inlineStr">
+      <c r="O167" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P167" s="10" t="inlineStr">
         <is>
           <t>Real sending starts when RESEND_API_KEY and OUTBOX_FROM_EMAIL are set in Vercel. Until then the form uses the email app fallback. No rate limit yet.</t>
         </is>
       </c>
-      <c r="Q166" s="10" t="n"/>
+      <c r="Q167" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Website: canonical links on Privacy and Terms, and a security.txt (PLT-022)
Small website fixes found in the 12 Oct 2026 audit. No database change.
- Privacy and Terms now name their own canonical address and og:url, like every other public page.
- /.well-known/security.txt added (RFC 9116). Contact is the website contact page until hello@ can receive mail.
  It expires 1 Oct 2026 + 1 year; known-issues notes the renewal and the test fails when under 30 days remain.
- New test e2e/site-basics.spec.ts [PLT-022]: every sitemap page is canonical to itself; security.txt is valid.
- Register row PLT-022 added, workbook rebuilt (168 requirements).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'R1 Requirements'!$A$1:$O$108</definedName>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q168"/>
+  <dimension ref="A1:Q169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14130,6 +14130,89 @@
         </is>
       </c>
       <c r="Q168" s="10" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="10" t="inlineStr">
+        <is>
+          <t>PLT-022</t>
+        </is>
+      </c>
+      <c r="B169" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C169" s="10" t="inlineStr">
+        <is>
+          <t>All public pages</t>
+        </is>
+      </c>
+      <c r="D169" s="10" t="inlineStr">
+        <is>
+          <t>Every public page names its own canonical address, and the site publishes a security.txt so a researcher knows how to report a problem.</t>
+        </is>
+      </c>
+      <c r="E169" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F169" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G169" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H169" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I169" s="10" t="inlineStr">
+        <is>
+          <t>Audit 12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J169" s="10" t="inlineStr">
+        <is>
+          <t>a search engine or a security researcher visits the site</t>
+        </is>
+      </c>
+      <c r="K169" s="10" t="inlineStr">
+        <is>
+          <t>it reads a public page or /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="L169" s="10" t="inlineStr">
+        <is>
+          <t>each indexed page names itself as canonical (Privacy and Terms did not), and security.txt gives a contact, an expiry date within a year and its own address</t>
+        </is>
+      </c>
+      <c r="M169" s="10" t="inlineStr">
+        <is>
+          <t>pageHead path on Privacy and Terms; public/.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="N169" s="10" t="inlineStr">
+        <is>
+          <t>site-basics (2)</t>
+        </is>
+      </c>
+      <c r="O169" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P169" s="10" t="inlineStr">
+        <is>
+          <t>Added 12 Oct 2026. security.txt expires 1 Oct 2027: renew it before then. Its contact is the website contact page until the hello@ mailbox can receive mail.</t>
+        </is>
+      </c>
+      <c r="Q169" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Register: RES-012 and RES-013 now have browser tests; FIN-016 says what is and is not covered
Adds e2e/arrival-ready.spec.ts for RES-013. Fixes two rows whose Notes had an unquoted comma.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="R1 Requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BR Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Build Gaps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'R1 Requirements'!$A$1:$O$108</definedName>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q168"/>
+  <dimension ref="A1:P168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -760,7 +760,6 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -839,7 +838,6 @@
         </is>
       </c>
       <c r="P2" s="10" t="inlineStr"/>
-      <c r="Q2" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -918,7 +916,6 @@
         </is>
       </c>
       <c r="P3" s="10" t="inlineStr"/>
-      <c r="Q3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -997,7 +994,6 @@
         </is>
       </c>
       <c r="P4" s="10" t="inlineStr"/>
-      <c r="Q4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1076,7 +1072,6 @@
         </is>
       </c>
       <c r="P5" s="10" t="inlineStr"/>
-      <c r="Q5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -1155,7 +1150,6 @@
         </is>
       </c>
       <c r="P6" s="10" t="inlineStr"/>
-      <c r="Q6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -1234,7 +1228,6 @@
         </is>
       </c>
       <c r="P7" s="10" t="inlineStr"/>
-      <c r="Q7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1317,7 +1310,6 @@
           <t>Adding a property: System Administrator and General Manager (ADM-002), within plans.max_properties.</t>
         </is>
       </c>
-      <c r="Q8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -1400,7 +1392,6 @@
           <t>Platform console /platform (wave 2 item 2): extend trial, activate or extend paid period, suspend, change plan, cancel; each with a reason, logged in subscription_history with the operator.</t>
         </is>
       </c>
-      <c r="Q9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -1483,7 +1474,6 @@
           <t>Corrected 6 Oct 2026: before wave 2 item 2 there was no platform staff role at all; the earlier "Built, no tagged test" was wrong.</t>
         </is>
       </c>
-      <c r="Q10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -1566,7 +1556,6 @@
           <t>Database done 8 Oct 2026. Screens for the hotel (Admin) and the operator (platform console) follow. New permission adm.support.manage reaches System Administrator and General Manager only.</t>
         </is>
       </c>
-      <c r="Q11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -1645,7 +1634,6 @@
         </is>
       </c>
       <c r="P12" s="10" t="inlineStr"/>
-      <c r="Q12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -1728,7 +1716,6 @@
           <t>Needs PAYSTACK_SECRET_KEY and the webhook address set in Paystack. Prices are empty until A16 is decided.</t>
         </is>
       </c>
-      <c r="Q13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -1807,7 +1794,6 @@
         </is>
       </c>
       <c r="P14" s="10" t="inlineStr"/>
-      <c r="Q14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -1890,7 +1876,6 @@
           <t>Invites are sent by a Vercel server function (not an Edge Function).</t>
         </is>
       </c>
-      <c r="Q15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -1969,7 +1954,6 @@
         </is>
       </c>
       <c r="P16" s="10" t="inlineStr"/>
-      <c r="Q16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -2048,7 +2032,6 @@
         </is>
       </c>
       <c r="P17" s="10" t="inlineStr"/>
-      <c r="Q17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -2127,7 +2110,6 @@
         </is>
       </c>
       <c r="P18" s="10" t="inlineStr"/>
-      <c r="Q18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -2206,7 +2188,6 @@
         </is>
       </c>
       <c r="P19" s="10" t="inlineStr"/>
-      <c r="Q19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -2285,7 +2266,6 @@
         </is>
       </c>
       <c r="P20" s="10" t="inlineStr"/>
-      <c r="Q20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
@@ -2364,7 +2344,6 @@
         </is>
       </c>
       <c r="P21" s="10" t="inlineStr"/>
-      <c r="Q21" s="10" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
@@ -2443,7 +2422,6 @@
         </is>
       </c>
       <c r="P22" s="10" t="inlineStr"/>
-      <c r="Q22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
@@ -2526,7 +2504,6 @@
           <t>export_data (audited), Reports &gt; Export.</t>
         </is>
       </c>
-      <c r="Q23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
@@ -2605,7 +2582,6 @@
         </is>
       </c>
       <c r="P24" s="10" t="inlineStr"/>
-      <c r="Q24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
@@ -2688,7 +2664,6 @@
           <t>Room types and occupancy limits are built (save_room_type: max adults and children; Setup, Room types). The overbooking allowance is not built: decision pending (QA-17, 11 Oct 2026). Recommended: skip it for the pilot.</t>
         </is>
       </c>
-      <c r="Q25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
@@ -2771,7 +2746,6 @@
           <t>A room cannot be retired while a guest is in it ([E_ROOM_OCCUPIED], checked first) or while upcoming bookings are assigned to it ([E_ROOM_BOOKED], names up to 5 booking numbers): confirmed, or tentative with an unexpired hold, from the business date forward (decisions of 6 Oct 2026). Retiring a room that is already retired is safe to repeat; renaming and floor changes still work.</t>
         </is>
       </c>
-      <c r="Q26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
@@ -2850,7 +2824,6 @@
         </is>
       </c>
       <c r="P27" s="10" t="inlineStr"/>
-      <c r="Q27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
@@ -2929,7 +2902,6 @@
         </is>
       </c>
       <c r="P28" s="10" t="inlineStr"/>
-      <c r="Q28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
@@ -3008,7 +2980,6 @@
         </is>
       </c>
       <c r="P29" s="10" t="inlineStr"/>
-      <c r="Q29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
@@ -3087,7 +3058,6 @@
         </is>
       </c>
       <c r="P30" s="10" t="inlineStr"/>
-      <c r="Q30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
@@ -3166,7 +3136,6 @@
         </is>
       </c>
       <c r="P31" s="10" t="inlineStr"/>
-      <c r="Q31" s="10" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
@@ -3245,7 +3214,6 @@
         </is>
       </c>
       <c r="P32" s="10" t="inlineStr"/>
-      <c r="Q32" s="10" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
@@ -3324,7 +3292,6 @@
         </is>
       </c>
       <c r="P33" s="10" t="inlineStr"/>
-      <c r="Q33" s="10" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
@@ -3403,7 +3370,6 @@
         </is>
       </c>
       <c r="P34" s="10" t="inlineStr"/>
-      <c r="Q34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
@@ -3482,7 +3448,6 @@
         </is>
       </c>
       <c r="P35" s="10" t="inlineStr"/>
-      <c r="Q35" s="10" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
@@ -3561,7 +3526,6 @@
         </is>
       </c>
       <c r="P36" s="10" t="inlineStr"/>
-      <c r="Q36" s="10" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
@@ -3640,7 +3604,6 @@
         </is>
       </c>
       <c r="P37" s="10" t="inlineStr"/>
-      <c r="Q37" s="10" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
@@ -3719,7 +3682,6 @@
         </is>
       </c>
       <c r="P38" s="10" t="inlineStr"/>
-      <c r="Q38" s="10" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
@@ -3798,7 +3760,6 @@
         </is>
       </c>
       <c r="P39" s="10" t="inlineStr"/>
-      <c r="Q39" s="10" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
@@ -3877,7 +3838,6 @@
         </is>
       </c>
       <c r="P40" s="10" t="inlineStr"/>
-      <c r="Q40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
@@ -3956,7 +3916,6 @@
         </is>
       </c>
       <c r="P41" s="10" t="inlineStr"/>
-      <c r="Q41" s="10" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
@@ -4035,7 +3994,6 @@
         </is>
       </c>
       <c r="P42" s="10" t="inlineStr"/>
-      <c r="Q42" s="10" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
@@ -4105,22 +4063,17 @@
       </c>
       <c r="N43" s="10" t="inlineStr">
         <is>
-          <t>29_untagged_rows (7)</t>
+          <t>29_untagged_rows (7); browser: group-bookings (QA-11)</t>
         </is>
       </c>
       <c r="O43" s="10" t="inlineStr">
         <is>
-          <t>Built+tested (database only)</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P43" s="10" t="inlineStr">
         <is>
-          <t>save_group_booking exists. The booking form creates a group (Add group) and picks one; Reservations</t>
-        </is>
-      </c>
-      <c r="Q43" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Groups lists each group and opens it with its rooms and totals. Browser test: e2e/group-bookings.spec.ts.</t>
+          <t>save_group_booking exists. The booking form creates a group (Add group) and picks one; Reservations, Groups lists each group and opens it with its rooms and totals. Browser test: e2e/group-bookings.spec.ts.</t>
         </is>
       </c>
     </row>
@@ -4192,22 +4145,17 @@
       </c>
       <c r="N44" s="10" t="inlineStr">
         <is>
-          <t>17_more_features (2); 26_small_fixes (4); 29_untagged_rows (6)</t>
+          <t>17_more_features (2); 26_small_fixes (4); 29_untagged_rows (6); browser: arrival-ready</t>
         </is>
       </c>
       <c r="O44" s="10" t="inlineStr">
         <is>
-          <t>Built+tested (database only)</t>
+          <t>Built+tested</t>
         </is>
       </c>
       <c r="P44" s="10" t="inlineStr">
         <is>
-          <t>set_arrival_ready exists. The booking page has Mark ready and Not ready; the Front Desk arrivals list and the group page show Ready (QA-15</t>
-        </is>
-      </c>
-      <c r="Q44" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 11 Oct 2026).</t>
+          <t>set_arrival_ready exists. The booking page has Mark ready and Not ready; the Front Desk arrivals list and the group page show Ready (QA-15, 11 Oct 2026). Browser test e2e/arrival-ready.spec.ts (12 Oct 2026): Mark ready shows Ready for arrival on the booking page and Ready on the Front Desk arrivals list; Not ready clears it.</t>
         </is>
       </c>
     </row>
@@ -4288,7 +4236,6 @@
         </is>
       </c>
       <c r="P45" s="10" t="inlineStr"/>
-      <c r="Q45" s="10" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
@@ -4367,7 +4314,6 @@
         </is>
       </c>
       <c r="P46" s="10" t="inlineStr"/>
-      <c r="Q46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
@@ -4450,7 +4396,6 @@
           <t>The check-in and walk-in screens force the registration card tick; a direct database call that omits it is not refused (decision 6 Oct 2026). Drawn signature later.</t>
         </is>
       </c>
-      <c r="Q47" s="10" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
@@ -4529,7 +4474,6 @@
         </is>
       </c>
       <c r="P48" s="10" t="inlineStr"/>
-      <c r="Q48" s="10" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
@@ -4608,7 +4552,6 @@
         </is>
       </c>
       <c r="P49" s="10" t="inlineStr"/>
-      <c r="Q49" s="10" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
@@ -4687,7 +4630,6 @@
         </is>
       </c>
       <c r="P50" s="10" t="inlineStr"/>
-      <c r="Q50" s="10" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
@@ -4770,7 +4712,6 @@
           <t>Dearer room type: front desk charges the new rate; keeping it needs fo.upgrade.complimentary (SYSADMIN, GM, FOM), audited.</t>
         </is>
       </c>
-      <c r="Q51" s="10" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
@@ -4849,7 +4790,6 @@
         </is>
       </c>
       <c r="P52" s="10" t="inlineStr"/>
-      <c r="Q52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
@@ -4928,7 +4868,6 @@
         </is>
       </c>
       <c r="P53" s="10" t="inlineStr"/>
-      <c r="Q53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
@@ -5007,7 +4946,6 @@
         </is>
       </c>
       <c r="P54" s="10" t="inlineStr"/>
-      <c r="Q54" s="10" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
@@ -5086,7 +5024,6 @@
         </is>
       </c>
       <c r="P55" s="10" t="inlineStr"/>
-      <c r="Q55" s="10" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
@@ -5165,7 +5102,6 @@
         </is>
       </c>
       <c r="P56" s="10" t="inlineStr"/>
-      <c r="Q56" s="10" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
@@ -5244,7 +5180,6 @@
         </is>
       </c>
       <c r="P57" s="10" t="inlineStr"/>
-      <c r="Q57" s="10" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
@@ -5323,7 +5258,6 @@
         </is>
       </c>
       <c r="P58" s="10" t="inlineStr"/>
-      <c r="Q58" s="10" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
@@ -5402,7 +5336,6 @@
         </is>
       </c>
       <c r="P59" s="10" t="inlineStr"/>
-      <c r="Q59" s="10" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
@@ -5481,7 +5414,6 @@
         </is>
       </c>
       <c r="P60" s="10" t="inlineStr"/>
-      <c r="Q60" s="10" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
@@ -5560,7 +5492,6 @@
         </is>
       </c>
       <c r="P61" s="10" t="inlineStr"/>
-      <c r="Q61" s="10" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
@@ -5639,7 +5570,6 @@
         </is>
       </c>
       <c r="P62" s="10" t="inlineStr"/>
-      <c r="Q62" s="10" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
@@ -5718,7 +5648,6 @@
         </is>
       </c>
       <c r="P63" s="10" t="inlineStr"/>
-      <c r="Q63" s="10" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
@@ -5797,7 +5726,6 @@
         </is>
       </c>
       <c r="P64" s="10" t="inlineStr"/>
-      <c r="Q64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
@@ -5876,7 +5804,6 @@
         </is>
       </c>
       <c r="P65" s="10" t="inlineStr"/>
-      <c r="Q65" s="10" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
@@ -5955,7 +5882,6 @@
         </is>
       </c>
       <c r="P66" s="10" t="inlineStr"/>
-      <c r="Q66" s="10" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
@@ -6034,7 +5960,6 @@
         </is>
       </c>
       <c r="P67" s="10" t="inlineStr"/>
-      <c r="Q67" s="10" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
@@ -6113,7 +6038,6 @@
         </is>
       </c>
       <c r="P68" s="10" t="inlineStr"/>
-      <c r="Q68" s="10" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
@@ -6192,7 +6116,6 @@
         </is>
       </c>
       <c r="P69" s="10" t="inlineStr"/>
-      <c r="Q69" s="10" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
@@ -6271,7 +6194,6 @@
         </is>
       </c>
       <c r="P70" s="10" t="inlineStr"/>
-      <c r="Q70" s="10" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
@@ -6350,7 +6272,6 @@
         </is>
       </c>
       <c r="P71" s="10" t="inlineStr"/>
-      <c r="Q71" s="10" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
@@ -6429,7 +6350,6 @@
         </is>
       </c>
       <c r="P72" s="10" t="inlineStr"/>
-      <c r="Q72" s="10" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
@@ -6508,7 +6428,6 @@
         </is>
       </c>
       <c r="P73" s="10" t="inlineStr"/>
-      <c r="Q73" s="10" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
@@ -6587,7 +6506,6 @@
         </is>
       </c>
       <c r="P74" s="10" t="inlineStr"/>
-      <c r="Q74" s="10" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
@@ -6666,7 +6584,6 @@
         </is>
       </c>
       <c r="P75" s="10" t="inlineStr"/>
-      <c r="Q75" s="10" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
@@ -6745,7 +6662,6 @@
         </is>
       </c>
       <c r="P76" s="10" t="inlineStr"/>
-      <c r="Q76" s="10" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
@@ -6824,7 +6740,6 @@
         </is>
       </c>
       <c r="P77" s="10" t="inlineStr"/>
-      <c r="Q77" s="10" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
@@ -6903,7 +6818,6 @@
         </is>
       </c>
       <c r="P78" s="10" t="inlineStr"/>
-      <c r="Q78" s="10" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
@@ -6982,7 +6896,6 @@
         </is>
       </c>
       <c r="P79" s="10" t="inlineStr"/>
-      <c r="Q79" s="10" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
@@ -7061,7 +6974,6 @@
         </is>
       </c>
       <c r="P80" s="10" t="inlineStr"/>
-      <c r="Q80" s="10" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
@@ -7140,7 +7052,6 @@
         </is>
       </c>
       <c r="P81" s="10" t="inlineStr"/>
-      <c r="Q81" s="10" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
@@ -7219,7 +7130,6 @@
         </is>
       </c>
       <c r="P82" s="10" t="inlineStr"/>
-      <c r="Q82" s="10" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
@@ -7298,7 +7208,6 @@
         </is>
       </c>
       <c r="P83" s="10" t="inlineStr"/>
-      <c r="Q83" s="10" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
@@ -7377,7 +7286,6 @@
         </is>
       </c>
       <c r="P84" s="10" t="inlineStr"/>
-      <c r="Q84" s="10" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
@@ -7456,7 +7364,6 @@
         </is>
       </c>
       <c r="P85" s="10" t="inlineStr"/>
-      <c r="Q85" s="10" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
@@ -7535,7 +7442,6 @@
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr"/>
-      <c r="Q86" s="10" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
@@ -7614,7 +7520,6 @@
         </is>
       </c>
       <c r="P87" s="10" t="inlineStr"/>
-      <c r="Q87" s="10" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
@@ -7693,7 +7598,6 @@
         </is>
       </c>
       <c r="P88" s="10" t="inlineStr"/>
-      <c r="Q88" s="10" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
@@ -7772,7 +7676,6 @@
         </is>
       </c>
       <c r="P89" s="10" t="inlineStr"/>
-      <c r="Q89" s="10" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
@@ -7851,7 +7754,6 @@
         </is>
       </c>
       <c r="P90" s="10" t="inlineStr"/>
-      <c r="Q90" s="10" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
@@ -7930,7 +7832,6 @@
         </is>
       </c>
       <c r="P91" s="10" t="inlineStr"/>
-      <c r="Q91" s="10" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
@@ -8009,7 +7910,6 @@
         </is>
       </c>
       <c r="P92" s="10" t="inlineStr"/>
-      <c r="Q92" s="10" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
@@ -8088,7 +7988,6 @@
         </is>
       </c>
       <c r="P93" s="10" t="inlineStr"/>
-      <c r="Q93" s="10" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
@@ -8167,7 +8066,6 @@
         </is>
       </c>
       <c r="P94" s="10" t="inlineStr"/>
-      <c r="Q94" s="10" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
@@ -8246,7 +8144,6 @@
         </is>
       </c>
       <c r="P95" s="10" t="inlineStr"/>
-      <c r="Q95" s="10" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
@@ -8316,7 +8213,7 @@
       </c>
       <c r="N96" s="10" t="inlineStr">
         <is>
-          <t>34_cashier_shifts (45)</t>
+          <t>34_cashier_shifts (45); browser: screens-actions (opening a shift)</t>
         </is>
       </c>
       <c r="O96" s="10" t="inlineStr">
@@ -8326,10 +8223,9 @@
       </c>
       <c r="P96" s="10" t="inlineStr">
         <is>
-          <t>Cashier shift page built (open, close with counts, review, reconcile). Not covered by a browser test yet. New permission fin.shift.reconcile goes to built-in roles only.</t>
-        </is>
-      </c>
-      <c r="Q96" s="10" t="n"/>
+          <t>Cashier shift page built (open, close with counts, review, reconcile). A browser test (QA-11) covers opening a shift. Closing with counts, review and reconcile are covered by the database tests only (checked 12 Oct 2026). New permission fin.shift.reconcile goes to built-in roles only.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
@@ -8408,7 +8304,6 @@
         </is>
       </c>
       <c r="P97" s="10" t="inlineStr"/>
-      <c r="Q97" s="10" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
@@ -8487,7 +8382,6 @@
         </is>
       </c>
       <c r="P98" s="10" t="inlineStr"/>
-      <c r="Q98" s="10" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
@@ -8566,7 +8460,6 @@
         </is>
       </c>
       <c r="P99" s="10" t="inlineStr"/>
-      <c r="Q99" s="10" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
@@ -8645,7 +8538,6 @@
         </is>
       </c>
       <c r="P100" s="10" t="inlineStr"/>
-      <c r="Q100" s="10" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
@@ -8728,7 +8620,6 @@
           <t>Flags shown in Admin, Business date. The gate that stops the roll while a blocking flag is open is not built.</t>
         </is>
       </c>
-      <c r="Q101" s="10" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
@@ -8811,7 +8702,6 @@
           <t>Decided by Peter on 30 Sep 2026 (answer 5) and confirmed on 1 Oct 2026: same-day stays are charged one night; a manager can waive it with a reason.</t>
         </is>
       </c>
-      <c r="Q102" s="10" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
@@ -8890,7 +8780,6 @@
         </is>
       </c>
       <c r="P103" s="10" t="inlineStr"/>
-      <c r="Q103" s="10" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
@@ -8969,7 +8858,6 @@
         </is>
       </c>
       <c r="P104" s="10" t="inlineStr"/>
-      <c r="Q104" s="10" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
@@ -9048,7 +8936,6 @@
         </is>
       </c>
       <c r="P105" s="10" t="inlineStr"/>
-      <c r="Q105" s="10" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
@@ -9131,7 +9018,6 @@
           <t>Reports screen: KPIs, revenue by charge code, outstanding balances, payments, cancellations and stay length, balances by guest, export.</t>
         </is>
       </c>
-      <c r="Q106" s="10" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
@@ -9210,7 +9096,6 @@
         </is>
       </c>
       <c r="P107" s="10" t="inlineStr"/>
-      <c r="Q107" s="10" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
@@ -9289,7 +9174,6 @@
         </is>
       </c>
       <c r="P108" s="10" t="inlineStr"/>
-      <c r="Q108" s="10" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
@@ -9368,7 +9252,6 @@
         </is>
       </c>
       <c r="P109" s="10" t="inlineStr"/>
-      <c r="Q109" s="10" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
@@ -9447,7 +9330,6 @@
         </is>
       </c>
       <c r="P110" s="10" t="inlineStr"/>
-      <c r="Q110" s="10" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
@@ -9526,7 +9408,6 @@
         </is>
       </c>
       <c r="P111" s="10" t="inlineStr"/>
-      <c r="Q111" s="10" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
@@ -9605,7 +9486,6 @@
         </is>
       </c>
       <c r="P112" s="10" t="inlineStr"/>
-      <c r="Q112" s="10" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
@@ -9684,7 +9564,6 @@
         </is>
       </c>
       <c r="P113" s="10" t="inlineStr"/>
-      <c r="Q113" s="10" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
@@ -9767,7 +9646,6 @@
           <t>Method only; the accountant still signs off the rates (A11)</t>
         </is>
       </c>
-      <c r="Q114" s="10" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
@@ -9850,7 +9728,6 @@
           <t>Day totals and fields are stored in the invoice header when it is issued</t>
         </is>
       </c>
-      <c r="Q115" s="10" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
@@ -9933,7 +9810,6 @@
           <t>Month comes from the business date, not the clock. No hotel code in the number yet.</t>
         </is>
       </c>
-      <c r="Q116" s="10" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
@@ -10012,7 +9888,6 @@
         </is>
       </c>
       <c r="P117" s="10" t="inlineStr"/>
-      <c r="Q117" s="10" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
@@ -10091,7 +9966,6 @@
         </is>
       </c>
       <c r="P118" s="10" t="inlineStr"/>
-      <c r="Q118" s="10" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
@@ -10170,7 +10044,6 @@
         </is>
       </c>
       <c r="P119" s="10" t="inlineStr"/>
-      <c r="Q119" s="10" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
@@ -10249,7 +10122,6 @@
         </is>
       </c>
       <c r="P120" s="10" t="inlineStr"/>
-      <c r="Q120" s="10" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
@@ -10328,7 +10200,6 @@
         </is>
       </c>
       <c r="P121" s="10" t="inlineStr"/>
-      <c r="Q121" s="10" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="10" t="inlineStr">
@@ -10407,7 +10278,6 @@
         </is>
       </c>
       <c r="P122" s="10" t="inlineStr"/>
-      <c r="Q122" s="10" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
@@ -10486,7 +10356,6 @@
           <t>Custom roles copied earlier do not get the new permission; say so when releasing.</t>
         </is>
       </c>
-      <c r="Q123" s="10" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="10" t="inlineStr">
@@ -10565,7 +10434,6 @@
           <t>Figures are read from each branch own business date. No arithmetic in the browser.</t>
         </is>
       </c>
-      <c r="Q124" s="10" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
@@ -10644,7 +10512,6 @@
           <t>Access is per branch, using the existing role assignment screen.</t>
         </is>
       </c>
-      <c r="Q125" s="10" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="10" t="inlineStr">
@@ -10723,7 +10590,6 @@
           <t>Taxes, charge codes and payment methods already arrive with every new branch.</t>
         </is>
       </c>
-      <c r="Q126" s="10" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
@@ -10802,7 +10668,6 @@
           <t>Bookings counted by arrival date; revenue by posting date.</t>
         </is>
       </c>
-      <c r="Q127" s="10" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
@@ -10881,7 +10746,6 @@
           <t>Guests still staying count as current.</t>
         </is>
       </c>
-      <c r="Q128" s="10" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
@@ -10964,7 +10828,6 @@
           <t>Email delivery waits on the sending domain and email account. Collected money nets payment reversals the same day (migration 20261015130000).</t>
         </is>
       </c>
-      <c r="Q129" s="10" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
@@ -11043,7 +10906,6 @@
           <t>Custom roles copied earlier do not get adm.ai.manage.</t>
         </is>
       </c>
-      <c r="Q130" s="10" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
@@ -11122,7 +10984,6 @@
           <t>Overdue means unpaid more than 30 days after departure.</t>
         </is>
       </c>
-      <c r="Q131" s="10" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="10" t="inlineStr">
@@ -11197,7 +11058,6 @@
         </is>
       </c>
       <c r="P132" s="10" t="inlineStr"/>
-      <c r="Q132" s="10" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
@@ -11272,7 +11132,6 @@
         </is>
       </c>
       <c r="P133" s="10" t="inlineStr"/>
-      <c r="Q133" s="10" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
@@ -11351,7 +11210,6 @@
           <t>Needs ANTHROPIC_API_KEY on the server (Vercel settings). Not set yet.</t>
         </is>
       </c>
-      <c r="Q134" s="10" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
@@ -11430,7 +11288,6 @@
           <t>The AI only drafts the list. This function is the check.</t>
         </is>
       </c>
-      <c r="Q135" s="10" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
@@ -11505,7 +11362,6 @@
         </is>
       </c>
       <c r="P136" s="10" t="inlineStr"/>
-      <c r="Q136" s="10" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
@@ -11584,7 +11440,6 @@
           <t>Needs ANTHROPIC_API_KEY on the server. Not set yet.</t>
         </is>
       </c>
-      <c r="Q137" s="10" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="10" t="inlineStr">
@@ -11667,7 +11522,6 @@
           <t>Read-only function, no stored progress. Staff step counts people with a role at the property (two or more).</t>
         </is>
       </c>
-      <c r="Q138" s="10" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="10" t="inlineStr">
@@ -11750,7 +11604,6 @@
           <t>Runs 8 separate database sessions at once. Added 7 Oct 2026.</t>
         </is>
       </c>
-      <c r="Q139" s="10" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="10" t="inlineStr">
@@ -11829,7 +11682,6 @@
           <t>Added 8 Oct 2026. The columns existed since the reservations release; this adds the screen and the function.</t>
         </is>
       </c>
-      <c r="Q140" s="10" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="10" t="inlineStr">
@@ -11908,7 +11760,6 @@
           <t>No database change. Reads v_arrivals, v_in_house and v_folio_balances. Added 8 Oct 2026.</t>
         </is>
       </c>
-      <c r="Q141" s="10" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="10" t="inlineStr">
@@ -11991,7 +11842,6 @@
           <t>Added 8 Oct 2026. Warning only; the hard gate stays in R2 (DAY-005).</t>
         </is>
       </c>
-      <c r="Q142" s="10" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="10" t="inlineStr">
@@ -12070,7 +11920,6 @@
           <t>Added 9 Oct 2026. Read-only; no money is changed.</t>
         </is>
       </c>
-      <c r="Q143" s="10" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="10" t="inlineStr">
@@ -12149,7 +11998,6 @@
           <t>Added 10 Oct 2026. The Payments report counted only payments and refunds before this. Cashier shift counts stay separate on purpose: they count what the drawer should hold.</t>
         </is>
       </c>
-      <c r="Q144" s="10" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="10" t="inlineStr">
@@ -12228,7 +12076,6 @@
           <t>Added 10 Oct 2026. Notes are not ledger rows; they never change a balance.</t>
         </is>
       </c>
-      <c r="Q145" s="10" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="10" t="inlineStr">
@@ -12303,7 +12150,6 @@
           <t>Added 10 Oct 2026. Mirrors docs/pilot-dry-run.md; screens and wording still need people.</t>
         </is>
       </c>
-      <c r="Q146" s="10" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="10" t="inlineStr">
@@ -12386,7 +12232,6 @@
           <t>Added 10 Oct 2026. Decision B: flag, do not stop (DAY-005 gate stays in R2).</t>
         </is>
       </c>
-      <c r="Q147" s="10" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="10" t="inlineStr">
@@ -12469,7 +12314,6 @@
           <t>QA-07. Fixes 14 helpers the security advisor listed. Added 10 Oct 2026.</t>
         </is>
       </c>
-      <c r="Q148" s="10" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="10" t="inlineStr">
@@ -12552,7 +12396,6 @@
           <t>QA-05. The warnings name the plan and price (PLT-018). Product name 'Zikora' in the wording is a draft.</t>
         </is>
       </c>
-      <c r="Q149" s="10" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="10" t="inlineStr">
@@ -12635,7 +12478,6 @@
           <t>QA-05.</t>
         </is>
       </c>
-      <c r="Q150" s="10" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="10" t="inlineStr">
@@ -12718,7 +12560,6 @@
           <t>Added 10 Oct 2026 (QA-12).</t>
         </is>
       </c>
-      <c r="Q151" s="10" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="10" t="inlineStr">
@@ -12801,7 +12642,6 @@
           <t>Stage 1. Only data the user's role may see is saved. ID numbers and photos are never saved.</t>
         </is>
       </c>
-      <c r="Q152" s="10" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="10" t="inlineStr">
@@ -12884,7 +12724,6 @@
           <t>Stage 1. Sign-out is refused while actions still wait to send (OFF-004).</t>
         </is>
       </c>
-      <c r="Q153" s="10" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="10" t="inlineStr">
@@ -12967,7 +12806,6 @@
           <t>Stage 2. Approvals and check-in stay online only. Check-out and room moves: see OFF-005 and OFF-006.</t>
         </is>
       </c>
-      <c r="Q154" s="10" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="10" t="inlineStr">
@@ -13050,7 +12888,6 @@
           <t>Stage 2.</t>
         </is>
       </c>
-      <c r="Q155" s="10" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="10" t="inlineStr">
@@ -13133,7 +12970,6 @@
           <t>QA-22. Page sizes: 100 bookings, 50 guests, 200 folios, 100 audit rows.</t>
         </is>
       </c>
-      <c r="Q156" s="10" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="10" t="inlineStr">
@@ -13216,7 +13052,6 @@
           <t>Needs a connection. Not saved for offline use.</t>
         </is>
       </c>
-      <c r="Q157" s="10" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="10" t="inlineStr">
@@ -13299,7 +13134,6 @@
           <t>Added 11 Oct 2026. The availability calendar and the downtime pack are true grids and scroll inside their own box on purpose.</t>
         </is>
       </c>
-      <c r="Q158" s="10" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="10" t="inlineStr">
@@ -13382,7 +13216,6 @@
           <t>Peter decided on 12 Oct 2026 (was 30 days). Hotels already on trial keep their dates; platform staff can extend one by hand. Plan choice at signup is not built: every new hotel starts on Starter (20 rooms).</t>
         </is>
       </c>
-      <c r="Q159" s="10" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="10" t="inlineStr">
@@ -13465,7 +13298,6 @@
           <t>One price for every hotel: no launch price and no price lock (Peter, 12 Oct 2026). Features by plan are not built; plans cap rooms, properties and users only. Billing stays off until the Paystack key and webhook are set.</t>
         </is>
       </c>
-      <c r="Q160" s="10" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="10" t="inlineStr">
@@ -13548,7 +13380,6 @@
           <t>Billing checkout (Paystack) is off until the key and webhook are set, so payment is arranged by email to hello@zikorahq.com. The Terms (section 4) still say read-only at trial end and need counsel to reword.</t>
         </is>
       </c>
-      <c r="Q161" s="10" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="10" t="inlineStr">
@@ -13631,7 +13462,6 @@
           <t>Needs a real phone check (iPhone Safari and Android Chrome). Works with the offline service worker already in place.</t>
         </is>
       </c>
-      <c r="Q162" s="10" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="10" t="inlineStr">
@@ -13714,7 +13544,6 @@
           <t>Stage 3a. Reason recorded: Checked out with no connection. Approvals stay online only.</t>
         </is>
       </c>
-      <c r="Q163" s="10" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="10" t="inlineStr">
@@ -13797,7 +13626,6 @@
           <t>Stage 3a. Check-in is OFF-007 and OFF-008. Walk-in is not built.</t>
         </is>
       </c>
-      <c r="Q164" s="10" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="10" t="inlineStr">
@@ -13880,7 +13708,6 @@
           <t>Stage 3b, check-in of an existing booking. Walk-in is not built (needs a new guest to be made offline). ID photos need a connection.</t>
         </is>
       </c>
-      <c r="Q165" s="10" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="10" t="inlineStr">
@@ -13963,7 +13790,6 @@
           <t>Stage 3b.</t>
         </is>
       </c>
-      <c r="Q166" s="10" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="10" t="inlineStr">
@@ -14046,7 +13872,6 @@
           <t>Real sending starts when RESEND_API_KEY and OUTBOX_FROM_EMAIL are set in Vercel. Until then the form uses the email app fallback. No rate limit yet.</t>
         </is>
       </c>
-      <c r="Q167" s="10" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="10" t="inlineStr">
@@ -14129,7 +13954,6 @@
           <t>Headers apply on the Vercel build only (not the local dev server). Full script policy (CSP) is a later job.</t>
         </is>
       </c>
-      <c r="Q168" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O108"/>

</xml_diff>

<commit_message>
Trim the first page load from 823 KB to 423 KB
Public pages no longer download the sign-in library, the form checker or the toast library.
They load when someone signs in, sends a form or reaches a signed-in screen. Adds a size check (PLT-023).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P169"/>
+  <dimension ref="A1:P170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14034,6 +14034,88 @@
       <c r="P169" s="10" t="inlineStr">
         <is>
           <t>Added 12 Oct 2026. security.txt expires 1 Oct 2027: renew it before then. Its contact is the website contact page until the hello@ mailbox can receive mail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="10" t="inlineStr">
+        <is>
+          <t>PLT-023</t>
+        </is>
+      </c>
+      <c r="B170" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C170" s="10" t="inlineStr">
+        <is>
+          <t>All pages</t>
+        </is>
+      </c>
+      <c r="D170" s="10" t="inlineStr">
+        <is>
+          <t>The first page load stays small. Public pages do not download the sign-in library, the form checker or the toast library; those load only when someone signs in, sends a form or reaches a signed-in screen. The first load went from 823 KB to 423 KB (243 KB to 134 KB compressed).</t>
+        </is>
+      </c>
+      <c r="E170" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F170" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G170" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H170" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I170" s="10" t="inlineStr">
+        <is>
+          <t>Audit 12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J170" s="10" t="inlineStr">
+        <is>
+          <t>a hotel owner opens the home page on mobile data</t>
+        </is>
+      </c>
+      <c r="K170" s="10" t="inlineStr">
+        <is>
+          <t>the page loads</t>
+        </is>
+      </c>
+      <c r="L170" s="10" t="inlineStr">
+        <is>
+          <t>the first scripts total under 470 KB and include none of the app-only libraries</t>
+        </is>
+      </c>
+      <c r="M170" s="10" t="inlineStr">
+        <is>
+          <t>scripts/bundle-size.mjs; scripts/check-bundle.mjs; src/lib/auth-watch.ts; src/lib/queries.ts; src/routes/__root.tsx</t>
+        </is>
+      </c>
+      <c r="N170" s="10" t="inlineStr">
+        <is>
+          <t>e2e/bundle-size-unit.spec.ts</t>
+        </is>
+      </c>
+      <c r="O170" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P170" s="10" t="inlineStr">
+        <is>
+          <t>Checked in CI after the build (npm run check:bundle). The 470 KB limit is raw size. React itself is about 200 KB of it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Platform console: owner summary (hotels by status, new, trials ending, quiet, monthly value)
Adds public.platform_summary (operator + two-step sign-in), a summary block at the top of /platform, test 62_platform_summary, requirement PLT-024.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P170"/>
+  <dimension ref="A1:P171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14116,6 +14116,88 @@
       <c r="P170" s="10" t="inlineStr">
         <is>
           <t>Checked in CI after the build (npm run check:bundle). The 470 KB limit is raw size. React itself is about 200 KB of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="10" t="inlineStr">
+        <is>
+          <t>PLT-024</t>
+        </is>
+      </c>
+      <c r="B171" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C171" s="10" t="inlineStr">
+        <is>
+          <t>Platform console</t>
+        </is>
+      </c>
+      <c r="D171" s="10" t="inlineStr">
+        <is>
+          <t>The owner sees a summary at the top of the platform console: hotels by status, new hotels this week and month, trials ending within 14 days, hotels gone quiet, and the monthly list price of active hotels. Account data only.</t>
+        </is>
+      </c>
+      <c r="E171" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F171" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G171" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H171" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I171" s="10" t="inlineStr">
+        <is>
+          <t>Owner request 13 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J171" s="10" t="inlineStr">
+        <is>
+          <t>a platform operator signed in with two-step sign-in</t>
+        </is>
+      </c>
+      <c r="K171" s="10" t="inlineStr">
+        <is>
+          <t>they open the platform console</t>
+        </is>
+      </c>
+      <c r="L171" s="10" t="inlineStr">
+        <is>
+          <t>they see the counts, the trials about to end, the quiet hotels and the monthly value of active hotels, with no guest, booking or balance data</t>
+        </is>
+      </c>
+      <c r="M171" s="10" t="inlineStr">
+        <is>
+          <t>platform_summary; src/routes/_authenticated/platform.tsx; src/components/platform-summary.tsx</t>
+        </is>
+      </c>
+      <c r="N171" s="10" t="inlineStr">
+        <is>
+          <t>supabase/tests/db/62_platform_summary.sql</t>
+        </is>
+      </c>
+      <c r="O171" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P171" s="10" t="inlineStr">
+        <is>
+          <t>Monthly value is list price of hotels with Active status. Pilot hotels invoiced by hand or free still count if set to Active.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add one-time script to remove demo hotels, with test and runbook (PLT-025)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P171"/>
+  <dimension ref="A1:P172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14198,6 +14198,88 @@
       <c r="P171" s="10" t="inlineStr">
         <is>
           <t>Monthly value is list price of hotels with Active status. Pilot hotels invoiced by hand or free still count if set to Active.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="10" t="inlineStr">
+        <is>
+          <t>PLT-025</t>
+        </is>
+      </c>
+      <c r="B172" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C172" s="10" t="inlineStr">
+        <is>
+          <t>Operations (not a screen)</t>
+        </is>
+      </c>
+      <c r="D172" s="10" t="inlineStr">
+        <is>
+          <t>Demo hotels can be removed completely, with their ledger, audit log and staff sign-ins, by a one-time script that Claude prepares and the owner runs. A dry run shows every count and changes nothing. It never touches other hotels or platform operators, and it rolls back if anything is left behind.</t>
+        </is>
+      </c>
+      <c r="E172" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F172" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G172" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H172" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I172" s="10" t="inlineStr">
+        <is>
+          <t>Owner request 13 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J172" s="10" t="inlineStr">
+        <is>
+          <t>a demo hotel that holds no real guest or money data</t>
+        </is>
+      </c>
+      <c r="K172" s="10" t="inlineStr">
+        <is>
+          <t>the owner runs the removal script with the hotel id</t>
+        </is>
+      </c>
+      <c r="L172" s="10" t="inlineStr">
+        <is>
+          <t>the hotel and everything it owns is gone, other hotels and operators are unchanged, and the ledger locks are back on</t>
+        </is>
+      </c>
+      <c r="M172" s="10" t="inlineStr">
+        <is>
+          <t>scripts/remove-hotels.sql; docs/runbook-remove-hotels.md</t>
+        </is>
+      </c>
+      <c r="N172" s="10" t="inlineStr">
+        <is>
+          <t>supabase/tests/db/63_remove_hotels.sql</t>
+        </is>
+      </c>
+      <c r="O172" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P172" s="10" t="inlineStr">
+        <is>
+          <t>One-time tool, not a migration. Live needs a backup first and the owner's typed yes, live.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove-hotels script: add remove_operator, test and runbook (PLT-025)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -14219,7 +14219,7 @@
       </c>
       <c r="D172" s="10" t="inlineStr">
         <is>
-          <t>Demo hotels can be removed completely, with their ledger, audit log and staff sign-ins, by a one-time script that Claude prepares and the owner runs. A dry run shows every count and changes nothing. It never touches other hotels or platform operators, and it rolls back if anything is left behind.</t>
+          <t>Demo hotels can be removed completely, with their ledger, audit log and staff sign-ins, by a one-time script that Claude prepares and the owner runs. A dry run shows every count and changes nothing. A second function removes a named platform operator on request. Hotel removal never touches other hotels or operators, and it rolls back if anything is left behind.</t>
         </is>
       </c>
       <c r="E172" s="10" t="inlineStr">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="L172" s="10" t="inlineStr">
         <is>
-          <t>the hotel and everything it owns is gone, other hotels and operators are unchanged, and the ledger locks are back on</t>
+          <t>the hotel and everything it owns is gone, other hotels and operators are unchanged, and a named operator can be removed on its own, and the ledger locks are back on</t>
         </is>
       </c>
       <c r="M172" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Sign-up safety check with Cloudflare Turnstile, off until a site key is set (PLT-026)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fzvY8u15ZSmsSpkvwn7gE
</commit_message>
<xml_diff>
--- a/docs/HMS_R1_Requirements.xlsx
+++ b/docs/HMS_R1_Requirements.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="13">
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P172"/>
+  <dimension ref="A1:P173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14280,6 +14280,88 @@
       <c r="P172" s="10" t="inlineStr">
         <is>
           <t>One-time tool, not a migration. Live needs a backup first and the owner's typed yes, live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="10" t="inlineStr">
+        <is>
+          <t>PLT-026</t>
+        </is>
+      </c>
+      <c r="B173" s="10" t="inlineStr">
+        <is>
+          <t>Platform &amp; Tenancy</t>
+        </is>
+      </c>
+      <c r="C173" s="10" t="inlineStr">
+        <is>
+          <t>Sign up, Sign in, Reset password</t>
+        </is>
+      </c>
+      <c r="D173" s="10" t="inlineStr">
+        <is>
+          <t>Open sign-up has a safety check (Cloudflare Turnstile) that stops bots from creating accounts in bulk. The check also guards sign-in and password reset, because Supabase applies it to all three. It is off until a site key is set, and the secret key stays in the Supabase dashboard only.</t>
+        </is>
+      </c>
+      <c r="E173" s="10" t="inlineStr">
+        <is>
+          <t>BR-001</t>
+        </is>
+      </c>
+      <c r="F173" s="10" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G173" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H173" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I173" s="10" t="inlineStr">
+        <is>
+          <t>Owner decision 13 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J173" s="10" t="inlineStr">
+        <is>
+          <t>a visitor on the sign-up page with the check switched on</t>
+        </is>
+      </c>
+      <c r="K173" s="10" t="inlineStr">
+        <is>
+          <t>they send the form</t>
+        </is>
+      </c>
+      <c r="L173" s="10" t="inlineStr">
+        <is>
+          <t>the safety check token goes with the request and the account is created only if it passes; with no site key the form works as before</t>
+        </is>
+      </c>
+      <c r="M173" s="10" t="inlineStr">
+        <is>
+          <t>src/lib/captcha.ts; src/components/turnstile.tsx; src/routes/auth.tsx; src/routes/forgot-password.tsx</t>
+        </is>
+      </c>
+      <c r="N173" s="10" t="inlineStr">
+        <is>
+          <t>e2e/captcha-unit.spec.ts</t>
+        </is>
+      </c>
+      <c r="O173" s="10" t="inlineStr">
+        <is>
+          <t>Built+tested</t>
+        </is>
+      </c>
+      <c r="P173" s="10" t="inlineStr">
+        <is>
+          <t>Switch-on order matters: set the site key in Vercel and deploy first, then turn on CAPTCHA protection in Supabase. The other way round, nobody can sign in. See docs/setup-checklist.md.</t>
         </is>
       </c>
     </row>

</xml_diff>